<commit_message>
classes + planif 2.0
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8FB0A2-CF35-4336-86E8-6FC5E284924D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786CC19C-4F78-4E7F-88C4-8A344D9C5BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="23160" windowHeight="13040" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="89">
   <si>
     <t>Planification globale</t>
   </si>
@@ -176,9 +176,6 @@
     <t xml:space="preserve">Créer game.php  </t>
   </si>
   <si>
-    <t>Créer ganeAction:executeAction, movePiece</t>
-  </si>
-  <si>
     <t>Créer le composant : Board(grille 10x10, zones infranchissables)</t>
   </si>
   <si>
@@ -258,6 +255,48 @@
   </si>
   <si>
     <t>Dans la page index.jsx : ajout du formulaire (signup, signin, signout)</t>
+  </si>
+  <si>
+    <t>Implémentation du LobbyManager</t>
+  </si>
+  <si>
+    <t>Implémentation du Controleur</t>
+  </si>
+  <si>
+    <t>Implémentation du GameManager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Développement de l'IA - Algorithme MCTS </t>
+  </si>
+  <si>
+    <t>Créer la classe Board</t>
+  </si>
+  <si>
+    <t>Créer la classe User/Player</t>
+  </si>
+  <si>
+    <t>Créer la classe Move</t>
+  </si>
+  <si>
+    <t>Créer la classe Piece</t>
+  </si>
+  <si>
+    <t>Créer gameAction:executeAction, movePiece</t>
+  </si>
+  <si>
+    <t>Créer la classe AIPlayer</t>
+  </si>
+  <si>
+    <t>Créer la classe ObservedPiece/BeliefPiece</t>
+  </si>
+  <si>
+    <t>Créer la classe Node et la classe InfoSet</t>
+  </si>
+  <si>
+    <t>Créer la classe MCTS</t>
+  </si>
+  <si>
+    <t>Communication entre le serveur et le client (envois/réceptions)</t>
   </si>
 </sst>
 </file>
@@ -384,9 +423,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -424,7 +463,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -530,7 +569,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -672,7 +711,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -680,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2A98864-B157-464B-9C9C-D10C2E7AC6B8}">
-  <dimension ref="B1:F102"/>
+  <dimension ref="B1:F101"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.1796875" customWidth="1"/>
@@ -704,7 +743,7 @@
     </row>
     <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>28</v>
@@ -842,7 +881,7 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>34</v>
@@ -963,7 +1002,7 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>34</v>
@@ -974,7 +1013,7 @@
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>34</v>
@@ -985,7 +1024,7 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>34</v>
@@ -996,7 +1035,7 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>34</v>
@@ -1007,7 +1046,7 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>34</v>
@@ -1018,7 +1057,7 @@
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>28</v>
@@ -1029,10 +1068,10 @@
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
@@ -1040,7 +1079,7 @@
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>34</v>
@@ -1051,7 +1090,7 @@
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>34</v>
@@ -1062,7 +1101,7 @@
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>34</v>
@@ -1073,7 +1112,7 @@
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>28</v>
@@ -1084,7 +1123,7 @@
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>28</v>
@@ -1095,7 +1134,7 @@
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>32</v>
@@ -1106,7 +1145,7 @@
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>32</v>
@@ -1117,7 +1156,7 @@
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>32</v>
@@ -1128,7 +1167,7 @@
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>34</v>
@@ -1139,7 +1178,7 @@
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>28</v>
@@ -1175,7 +1214,7 @@
         <v>67</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
@@ -1186,7 +1225,7 @@
         <v>68</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>28</v>
+        <v>69</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
@@ -1194,10 +1233,10 @@
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C49" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
@@ -1208,7 +1247,7 @@
         <v>71</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
@@ -1219,7 +1258,7 @@
         <v>72</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
@@ -1227,95 +1266,143 @@
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
+      <c r="B54" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
+      <c r="B55" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
+      <c r="B56" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
+      <c r="B57" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
+      <c r="B58" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
+      <c r="B59" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
+      <c r="B60" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D60" s="3"/>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
+      <c r="B61" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D61" s="3"/>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
+      <c r="B62" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
+      <c r="B63" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D63" s="3"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
+      <c r="B64" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>32</v>
+      </c>
       <c r="D64" s="3"/>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
@@ -1579,19 +1666,12 @@
       <c r="E101" s="3"/>
       <c r="F101" s="3"/>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.35">
-      <c r="B102" s="3"/>
-      <c r="C102" s="3"/>
-      <c r="D102" s="3"/>
-      <c r="E102" s="3"/>
-      <c r="F102" s="3"/>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E102" xr:uid="{C1E49912-FB61-4F2F-8F8F-588FF6944C57}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E44 E45:E101" xr:uid="{C1E49912-FB61-4F2F-8F8F-588FF6944C57}">
       <formula1>"Haute,Moyenne,Basse,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D102" xr:uid="{A1B83402-03F9-4A0F-BE40-AAB54D35ECC4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D44 D45:D101" xr:uid="{A1B83402-03F9-4A0F-BE40-AAB54D35ECC4}">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Mise a jour diagramme de classe
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45F7176B-92F4-4BA7-B806-AACEA65B28BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C408D2F2-66B1-46D2-99B1-41876276B4C3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,10 +37,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -943,9 +943,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -983,7 +983,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1089,7 +1089,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1231,7 +1231,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2901,6 +2901,10 @@
     <col min="10" max="10" width="9.54296875" customWidth="1"/>
     <col min="11" max="11" width="16.1796875" customWidth="1"/>
     <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">

</xml_diff>

<commit_message>
debut backend (rules, lobbymanager)
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E1F0310-2F9A-45FC-BF67-D89F89492E03}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB607E7-C505-4FCB-9ED9-8BCDDF6C2399}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,22 +27,17 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planification!$B$5:$E$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="162">
   <si>
     <t>Planification globale</t>
   </si>
@@ -522,6 +517,12 @@
   </si>
   <si>
     <t>des pertes de connexions aléatoires</t>
+  </si>
+  <si>
+    <t>Plus long que prévu, créé plusieurs autres classes nécessaires</t>
+  </si>
+  <si>
+    <t>Reste à créér la classe user et à mettre des choses dans la classe Player</t>
   </si>
 </sst>
 </file>
@@ -979,14 +980,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor theme="7" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1304,26 +1305,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:5" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1337,7 +1338,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B6" s="21" t="s">
         <v>153</v>
       </c>
@@ -1351,7 +1352,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="18" t="s">
         <v>123</v>
       </c>
@@ -1365,7 +1366,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>124</v>
       </c>
@@ -1379,7 +1380,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="18" t="s">
         <v>125</v>
       </c>
@@ -1393,7 +1394,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="18" t="s">
         <v>126</v>
       </c>
@@ -1407,7 +1408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="18" t="s">
         <v>128</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="18" t="s">
         <v>129</v>
       </c>
@@ -1435,7 +1436,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="18" t="s">
         <v>130</v>
       </c>
@@ -1449,7 +1450,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>157</v>
       </c>
@@ -1463,7 +1464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="18" t="s">
         <v>133</v>
       </c>
@@ -1477,7 +1478,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="18" t="s">
         <v>134</v>
       </c>
@@ -1491,7 +1492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="18" t="s">
         <v>136</v>
       </c>
@@ -1505,7 +1506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="18" t="s">
         <v>142</v>
       </c>
@@ -1519,7 +1520,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B19" s="18" t="s">
         <v>131</v>
       </c>
@@ -1533,7 +1534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
         <v>132</v>
       </c>
@@ -1547,7 +1548,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B21" s="18" t="s">
         <v>137</v>
       </c>
@@ -1561,7 +1562,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B22" s="18" t="s">
         <v>138</v>
       </c>
@@ -1575,7 +1576,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B23" s="18" t="s">
         <v>139</v>
       </c>
@@ -1589,7 +1590,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B24" s="18" t="s">
         <v>141</v>
       </c>
@@ -1603,7 +1604,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B25" s="18" t="s">
         <v>145</v>
       </c>
@@ -1617,7 +1618,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>146</v>
       </c>
@@ -1631,7 +1632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B27" s="18" t="s">
         <v>147</v>
       </c>
@@ -1645,7 +1646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B28" s="18" t="s">
         <v>140</v>
       </c>
@@ -1659,7 +1660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B29" s="18" t="s">
         <v>143</v>
       </c>
@@ -1673,7 +1674,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B30" s="18" t="s">
         <v>135</v>
       </c>
@@ -1687,7 +1688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>144</v>
       </c>
@@ -1701,7 +1702,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>148</v>
       </c>
@@ -1715,7 +1716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B33" s="18" t="s">
         <v>149</v>
       </c>
@@ -1729,7 +1730,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B34" s="18" t="s">
         <v>150</v>
       </c>
@@ -1743,7 +1744,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="18" t="s">
         <v>151</v>
       </c>
@@ -1757,7 +1758,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="18" t="s">
         <v>152</v>
       </c>
@@ -1771,7 +1772,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="22" t="s">
         <v>127</v>
       </c>
@@ -1785,8 +1786,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="41" t="s">
         <v>158</v>
       </c>
@@ -1822,32 +1823,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1877,7 +1878,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -1931,7 +1932,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="23" t="s">
         <v>97</v>
       </c>
@@ -1958,7 +1959,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="26" t="s">
         <v>96</v>
       </c>
@@ -1980,7 +1981,7 @@
       <c r="P6" s="31"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="26" t="s">
         <v>98</v>
       </c>
@@ -2007,7 +2008,7 @@
       <c r="P7" s="31"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="26" t="s">
         <v>104</v>
       </c>
@@ -2040,7 +2041,7 @@
       <c r="P8" s="31"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="26" t="s">
         <v>99</v>
       </c>
@@ -2077,7 +2078,7 @@
       </c>
       <c r="R9" s="28"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="26" t="s">
         <v>103</v>
       </c>
@@ -2114,7 +2115,7 @@
       </c>
       <c r="R10" s="28"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="26" t="s">
         <v>101</v>
       </c>
@@ -2146,7 +2147,7 @@
       </c>
       <c r="R11" s="28"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="26" t="s">
         <v>102</v>
       </c>
@@ -2174,7 +2175,7 @@
       <c r="P12" s="31"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="47" t="s">
         <v>100</v>
       </c>
@@ -2201,15 +2202,15 @@
       <c r="Q13" s="46"/>
       <c r="R13" s="17"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="20"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="20"/>
       <c r="P25" s="20"/>
       <c r="S25" s="20"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="20"/>
       <c r="P26" s="20"/>
       <c r="S26" s="20"/>
@@ -2225,23 +2226,24 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B3:L35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.453125" customWidth="1"/>
+    <col min="9" max="9" width="52.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="3" spans="2:12" ht="46" x14ac:dyDescent="1">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B5" s="7"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
@@ -2266,7 +2268,7 @@
       </c>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="7" t="s">
         <v>1</v>
       </c>
@@ -2301,7 +2303,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
         <v>24</v>
       </c>
@@ -2324,7 +2326,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="36" t="s">
         <v>35</v>
       </c>
@@ -2342,7 +2344,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
@@ -2360,22 +2362,25 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="36" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>89</v>
+      <c r="D10" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
       </c>
       <c r="F10" s="14"/>
       <c r="G10" s="18"/>
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="36" t="s">
         <v>122</v>
       </c>
@@ -2390,7 +2395,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="36" t="s">
         <v>25</v>
       </c>
@@ -2405,7 +2410,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="36" t="s">
         <v>26</v>
       </c>
@@ -2420,7 +2425,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="36" t="s">
         <v>27</v>
       </c>
@@ -2435,7 +2440,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="36" t="s">
         <v>29</v>
       </c>
@@ -2450,7 +2455,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="36" t="s">
         <v>30</v>
       </c>
@@ -2465,7 +2470,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="36" t="s">
         <v>92</v>
       </c>
@@ -2474,13 +2479,18 @@
       </c>
       <c r="D17" s="18"/>
       <c r="F17" s="14"/>
-      <c r="G17" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="I17" s="14"/>
+      <c r="G17" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="H17">
+        <v>100</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>160</v>
+      </c>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="36" t="s">
         <v>51</v>
       </c>
@@ -2489,13 +2499,16 @@
       </c>
       <c r="D18" s="18"/>
       <c r="F18" s="14"/>
-      <c r="G18" s="18" t="s">
-        <v>89</v>
+      <c r="G18" s="18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>100</v>
       </c>
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="36" t="s">
         <v>90</v>
       </c>
@@ -2510,22 +2523,24 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="36" t="s">
         <v>74</v>
       </c>
       <c r="C20" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="18"/>
       <c r="F20" s="14"/>
-      <c r="G20" s="18" t="s">
-        <v>89</v>
+      <c r="G20" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H20">
+        <v>100</v>
       </c>
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="36" t="s">
         <v>80</v>
       </c>
@@ -2534,14 +2549,19 @@
       </c>
       <c r="D21" s="18"/>
       <c r="F21" s="14"/>
-      <c r="G21" s="18"/>
+      <c r="G21" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H21">
+        <v>100</v>
+      </c>
       <c r="I21" s="14"/>
       <c r="J21" t="s">
         <v>89</v>
       </c>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="36" t="s">
         <v>93</v>
       </c>
@@ -2557,7 +2577,7 @@
       </c>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="36" t="s">
         <v>94</v>
       </c>
@@ -2573,7 +2593,7 @@
       </c>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="36" t="s">
         <v>79</v>
       </c>
@@ -2582,14 +2602,21 @@
       </c>
       <c r="D24" s="18"/>
       <c r="F24" s="14"/>
-      <c r="G24" s="18"/>
-      <c r="I24" s="14"/>
+      <c r="G24" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H24">
+        <v>25</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>161</v>
+      </c>
       <c r="J24" t="s">
         <v>89</v>
       </c>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="18" t="s">
         <v>76</v>
       </c>
@@ -2605,7 +2632,7 @@
       </c>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="36" t="s">
         <v>31</v>
       </c>
@@ -2621,7 +2648,7 @@
       </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="18" t="s">
         <v>44</v>
       </c>
@@ -2637,7 +2664,7 @@
       </c>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="36" t="s">
         <v>37</v>
       </c>
@@ -2653,7 +2680,7 @@
       </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="36" t="s">
         <v>73</v>
       </c>
@@ -2669,7 +2696,7 @@
       </c>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="36" t="s">
         <v>38</v>
       </c>
@@ -2685,7 +2712,7 @@
       </c>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="36" t="s">
         <v>39</v>
       </c>
@@ -2701,7 +2728,7 @@
       </c>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="36" t="s">
         <v>42</v>
       </c>
@@ -2717,7 +2744,7 @@
       </c>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="36" t="s">
         <v>43</v>
       </c>
@@ -2733,7 +2760,7 @@
       </c>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="36" t="s">
         <v>61</v>
       </c>
@@ -2749,7 +2776,7 @@
       </c>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="37" t="s">
         <v>56</v>
       </c>
@@ -2779,27 +2806,27 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.21875" customWidth="1"/>
-    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.21875" customWidth="1"/>
-    <col min="9" max="9" width="19.77734375" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="2.1796875" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.54296875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.1796875" customWidth="1"/>
+    <col min="9" max="9" width="19.81640625" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="19.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -2818,7 +2845,7 @@
       <c r="K3" s="4"/>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -2853,7 +2880,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="35"/>
       <c r="C5" s="12"/>
       <c r="D5" s="49"/>
@@ -2866,7 +2893,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="36"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -2875,7 +2902,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="36"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -2884,7 +2911,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="36"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -2893,7 +2920,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="36"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -2902,7 +2929,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="36"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -2911,7 +2938,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="36"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -2920,7 +2947,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="36"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -2929,7 +2956,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="36"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -2938,7 +2965,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="36"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -2947,7 +2974,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="36"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -2956,7 +2983,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="36"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -2965,7 +2992,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="36"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -2974,7 +3001,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="36"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -2983,7 +3010,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="36"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -2992,7 +3019,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="36"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3001,7 +3028,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="36"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3010,7 +3037,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="36"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3019,7 +3046,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="36"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3028,7 +3055,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="36"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3037,7 +3064,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="36"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3046,7 +3073,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="36"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3055,7 +3082,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="36"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3064,7 +3091,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="36"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3073,7 +3100,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="36"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3082,7 +3109,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="36"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3091,7 +3118,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="36"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3100,7 +3127,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="36"/>
       <c r="C32" s="14"/>
       <c r="D32" s="50"/>
@@ -3109,7 +3136,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="36"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3118,7 +3145,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="36"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3127,7 +3154,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="36"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3136,7 +3163,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="36"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3145,7 +3172,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="36"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3154,7 +3181,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="36"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3163,7 +3190,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="36"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3172,7 +3199,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B40" s="37"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3187,11 +3214,11 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:B40">
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>COUNTIF(D5:L5,100%)=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>COUNTIF(D5:L5,100%)&gt;0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>COUNTIF(D5:L5,100%)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3205,21 +3232,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="70.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="70.81640625" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" customWidth="1"/>
+    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="9" t="s">
         <v>22</v>
       </c>
@@ -3233,151 +3260,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -3393,28 +3420,28 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -3439,7 +3466,7 @@
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -3474,7 +3501,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="51"/>
       <c r="C5" s="12"/>
       <c r="D5" s="21"/>
@@ -3487,7 +3514,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="52"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -3496,7 +3523,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="52"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -3505,7 +3532,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="52"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -3514,7 +3541,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="52"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -3523,7 +3550,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="52"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -3532,7 +3559,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="52"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -3541,7 +3568,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="52"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -3550,7 +3577,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="52"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -3559,7 +3586,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="52"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -3568,7 +3595,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="52"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -3577,7 +3604,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="52"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -3586,7 +3613,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="52"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -3595,7 +3622,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="52"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -3604,7 +3631,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="52"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -3613,7 +3640,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="52"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3622,7 +3649,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="52"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3631,7 +3658,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="52"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3640,7 +3667,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="52"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3649,7 +3676,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="52"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3658,7 +3685,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="52"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3667,7 +3694,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="52"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3676,7 +3703,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="52"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3685,7 +3712,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="52"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3694,7 +3721,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="52"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3703,7 +3730,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="52"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3712,7 +3739,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="52"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3721,7 +3748,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="52"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -3730,7 +3757,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="52"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3739,7 +3766,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="52"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3748,7 +3775,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="52"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3757,7 +3784,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="52"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3766,7 +3793,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="52"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3775,7 +3802,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="52"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3784,7 +3811,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="52"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3793,7 +3820,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B40" s="53"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3826,18 +3853,18 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B2:O56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -3861,7 +3888,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -3905,7 +3932,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="10" t="s">
         <v>95</v>
       </c>
@@ -3927,7 +3954,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -3945,7 +3972,7 @@
       <c r="M7" s="18"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="13" t="s">
         <v>84</v>
       </c>
@@ -3963,7 +3990,7 @@
       <c r="M8" s="18"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
@@ -3981,7 +4008,7 @@
       <c r="M9" s="18"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="13" t="s">
         <v>83</v>
       </c>
@@ -3999,7 +4026,7 @@
       <c r="M10" s="18"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="13" t="s">
         <v>62</v>
       </c>
@@ -4017,7 +4044,7 @@
       <c r="M11" s="18"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
@@ -4035,7 +4062,7 @@
       <c r="M12" s="18"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="13" t="s">
         <v>86</v>
       </c>
@@ -4053,7 +4080,7 @@
       <c r="M13" s="18"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="13" t="s">
         <v>54</v>
       </c>
@@ -4071,7 +4098,7 @@
       <c r="M14" s="18"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="13" t="s">
         <v>58</v>
       </c>
@@ -4089,7 +4116,7 @@
       <c r="M15" s="18"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="13" t="s">
         <v>59</v>
       </c>
@@ -4107,7 +4134,7 @@
       <c r="M16" s="18"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="13" t="s">
         <v>60</v>
       </c>
@@ -4125,7 +4152,7 @@
       <c r="M17" s="18"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="13" t="s">
         <v>63</v>
       </c>
@@ -4143,7 +4170,7 @@
       <c r="M18" s="18"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="13" t="s">
         <v>46</v>
       </c>
@@ -4161,7 +4188,7 @@
       <c r="M19" s="18"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="13" t="s">
         <v>45</v>
       </c>
@@ -4179,7 +4206,7 @@
       <c r="M20" s="18"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="13" t="s">
         <v>82</v>
       </c>
@@ -4197,7 +4224,7 @@
       <c r="M21" s="18"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
         <v>40</v>
       </c>
@@ -4215,7 +4242,7 @@
       <c r="M22" s="18"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="13" t="s">
         <v>41</v>
       </c>
@@ -4233,7 +4260,7 @@
       <c r="M23" s="18"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="13" t="s">
         <v>57</v>
       </c>
@@ -4251,7 +4278,7 @@
       <c r="M24" s="18"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="13" t="s">
         <v>53</v>
       </c>
@@ -4269,7 +4296,7 @@
       <c r="M25" s="18"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="13" t="s">
         <v>72</v>
       </c>
@@ -4287,7 +4314,7 @@
       <c r="M26" s="18"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
@@ -4305,7 +4332,7 @@
       <c r="M27" s="18"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="13" t="s">
         <v>69</v>
       </c>
@@ -4323,7 +4350,7 @@
       <c r="M28" s="18"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="13" t="s">
         <v>71</v>
       </c>
@@ -4341,7 +4368,7 @@
       <c r="M29" s="18"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>67</v>
       </c>
@@ -4359,7 +4386,7 @@
       </c>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="13" t="s">
         <v>65</v>
       </c>
@@ -4377,7 +4404,7 @@
       </c>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="13" t="s">
         <v>66</v>
       </c>
@@ -4395,7 +4422,7 @@
       </c>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="13" t="s">
         <v>114</v>
       </c>
@@ -4413,7 +4440,7 @@
       </c>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="13" t="s">
         <v>88</v>
       </c>
@@ -4431,7 +4458,7 @@
       </c>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="15" t="s">
         <v>70</v>
       </c>
@@ -4453,47 +4480,47 @@
       <c r="N35" s="16"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="40" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B48" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" s="36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" s="36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" s="36" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B54" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4505,29 +4532,29 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="51.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.21875" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" customWidth="1"/>
-    <col min="7" max="7" width="20.44140625" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.21875" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.21875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="51.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -4559,7 +4586,7 @@
       </c>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -4603,7 +4630,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="51"/>
       <c r="C6" s="12"/>
       <c r="D6" s="21"/>
@@ -4619,7 +4646,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="52"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -4629,7 +4656,7 @@
       <c r="L7" s="14"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="52"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -4639,7 +4666,7 @@
       <c r="L8" s="14"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="52"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -4649,7 +4676,7 @@
       <c r="L9" s="14"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="52"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -4659,7 +4686,7 @@
       <c r="L10" s="14"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="52"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -4669,7 +4696,7 @@
       <c r="L11" s="14"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="52"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -4679,7 +4706,7 @@
       <c r="L12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="52"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -4689,7 +4716,7 @@
       <c r="L13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="52"/>
       <c r="C14" s="14"/>
       <c r="D14" s="50"/>
@@ -4699,7 +4726,7 @@
       <c r="L14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="52"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -4709,7 +4736,7 @@
       <c r="L15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="52"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -4719,7 +4746,7 @@
       <c r="L16" s="14"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="52"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -4729,7 +4756,7 @@
       <c r="L17" s="14"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="52"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -4739,7 +4766,7 @@
       <c r="L18" s="14"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="52"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -4749,7 +4776,7 @@
       <c r="L19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="52"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -4759,7 +4786,7 @@
       <c r="L20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="52"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -4769,7 +4796,7 @@
       <c r="L21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="52"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -4779,7 +4806,7 @@
       <c r="L22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="52"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -4789,7 +4816,7 @@
       <c r="L23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="52"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -4799,7 +4826,7 @@
       <c r="L24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="52"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -4809,7 +4836,7 @@
       <c r="L25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="52"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -4819,7 +4846,7 @@
       <c r="L26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="52"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -4829,7 +4856,7 @@
       <c r="L27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="52"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -4839,7 +4866,7 @@
       <c r="L28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="52"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -4849,7 +4876,7 @@
       <c r="L29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="52"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -4859,7 +4886,7 @@
       <c r="L30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="52"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -4869,7 +4896,7 @@
       <c r="L31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="52"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -4879,7 +4906,7 @@
       <c r="L32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="52"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -4889,7 +4916,7 @@
       <c r="L33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="52"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -4899,7 +4926,7 @@
       <c r="L34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B35" s="52"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -4909,7 +4936,7 @@
       <c r="L35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B36" s="52"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -4919,7 +4946,7 @@
       <c r="L36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B37" s="52"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -4929,7 +4956,7 @@
       <c r="L37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B38" s="52"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -4939,7 +4966,7 @@
       <c r="L38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B39" s="52"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -4949,7 +4976,7 @@
       <c r="L39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B40" s="52"/>
       <c r="C40" s="14"/>
       <c r="D40" s="18"/>
@@ -4959,7 +4986,7 @@
       <c r="L40" s="14"/>
       <c r="O40" s="14"/>
     </row>
-    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B41" s="53"/>
       <c r="C41" s="17"/>
       <c r="D41" s="22"/>
@@ -4975,7 +5002,7 @@
       <c r="N41" s="16"/>
       <c r="O41" s="17"/>
     </row>
-    <row r="64" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" t="s">
@@ -4984,7 +5011,7 @@
       <c r="J64" s="5"/>
       <c r="M64" s="5"/>
     </row>
-    <row r="65" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" t="s">
@@ -4993,7 +5020,7 @@
       <c r="J65" s="5"/>
       <c r="M65" s="5"/>
     </row>
-    <row r="67" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" t="s">
@@ -5002,7 +5029,7 @@
       <c r="J67" s="5"/>
       <c r="M67" s="5"/>
     </row>
-    <row r="68" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D68" s="5"/>
       <c r="G68" s="5"/>
       <c r="J68" s="5"/>
@@ -5011,17 +5038,17 @@
       </c>
       <c r="M68" s="5"/>
     </row>
-    <row r="71" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:13" x14ac:dyDescent="0.35">
       <c r="H71" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:13" x14ac:dyDescent="0.35">
       <c r="K72" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D73" s="5"/>
       <c r="G73" s="5"/>
       <c r="J73" s="5"/>
@@ -5049,28 +5076,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
-    <col min="2" max="2" width="93.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1796875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:6" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -5087,7 +5114,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -5100,7 +5127,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -5113,7 +5140,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -5126,7 +5153,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -5139,7 +5166,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -5152,7 +5179,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -5165,7 +5192,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -5178,7 +5205,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -5191,7 +5218,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5204,7 +5231,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -5217,7 +5244,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -5230,7 +5257,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5243,7 +5270,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -5256,7 +5283,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -5269,7 +5296,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -5282,7 +5309,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -5295,7 +5322,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -5308,7 +5335,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -5321,7 +5348,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -5334,7 +5361,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -5347,7 +5374,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5360,7 +5387,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -5373,7 +5400,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -5386,7 +5413,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -5399,7 +5426,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -5412,7 +5439,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -5425,7 +5452,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -5438,7 +5465,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -5451,7 +5478,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -5464,7 +5491,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -5477,7 +5504,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -5490,7 +5517,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -5503,7 +5530,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -5516,7 +5543,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -5529,7 +5556,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -5542,7 +5569,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -5555,7 +5582,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -5568,7 +5595,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -5581,7 +5608,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -5594,7 +5621,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -5607,7 +5634,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -5620,7 +5647,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -5633,7 +5660,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -5646,7 +5673,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -5659,7 +5686,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -5672,7 +5699,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -5685,7 +5712,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -5698,7 +5725,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -5711,7 +5738,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -5724,7 +5751,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -5737,7 +5764,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -5750,7 +5777,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -5763,7 +5790,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -5776,7 +5803,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -5789,7 +5816,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -5802,7 +5829,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -5815,7 +5842,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -5828,7 +5855,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -5841,7 +5868,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -5854,7 +5881,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>96</v>
       </c>
@@ -5865,7 +5892,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>97</v>
       </c>
@@ -5876,7 +5903,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>98</v>
       </c>
@@ -5887,7 +5914,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>99</v>
       </c>
@@ -5898,7 +5925,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>100</v>
       </c>
@@ -5909,7 +5936,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>101</v>
       </c>
@@ -5920,7 +5947,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>102</v>
       </c>
@@ -5931,7 +5958,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>103</v>
       </c>
@@ -5942,7 +5969,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>104</v>
       </c>
@@ -5953,7 +5980,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
         <v>120</v>
       </c>
@@ -5964,7 +5991,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
         <v>121</v>
       </c>
@@ -5975,182 +6002,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Ajout des pages dans main.jsx
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB607E7-C505-4FCB-9ED9-8BCDDF6C2399}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C95E976-A156-410F-8D3B-FFCC70E3A401}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,17 +27,22 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planification!$B$5:$E$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="647" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="166">
   <si>
     <t>Planification globale</t>
   </si>
@@ -523,6 +528,18 @@
   </si>
   <si>
     <t>Reste à créér la classe user et à mettre des choses dans la classe Player</t>
+  </si>
+  <si>
+    <t>Créer le routage vers les differentes pages: index,lobby,game</t>
+  </si>
+  <si>
+    <t>Créer la page main.jsx</t>
+  </si>
+  <si>
+    <t>Tests: acces pages web:frontend et backend du client</t>
+  </si>
+  <si>
+    <t>Créer IndexAction: signup, signin,signout</t>
   </si>
 </sst>
 </file>
@@ -873,7 +890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -944,6 +961,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1305,26 +1328,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" customWidth="1"/>
-    <col min="5" max="5" width="42.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.75" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:5" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1338,7 +1361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
         <v>153</v>
       </c>
@@ -1352,7 +1375,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="18" t="s">
         <v>123</v>
       </c>
@@ -1366,7 +1389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="18" t="s">
         <v>124</v>
       </c>
@@ -1380,7 +1403,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
         <v>125</v>
       </c>
@@ -1394,7 +1417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
         <v>126</v>
       </c>
@@ -1408,7 +1431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="18" t="s">
         <v>128</v>
       </c>
@@ -1422,7 +1445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="18" t="s">
         <v>129</v>
       </c>
@@ -1436,7 +1459,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="18" t="s">
         <v>130</v>
       </c>
@@ -1450,7 +1473,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="18" t="s">
         <v>157</v>
       </c>
@@ -1464,7 +1487,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
         <v>133</v>
       </c>
@@ -1478,7 +1501,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="18" t="s">
         <v>134</v>
       </c>
@@ -1492,7 +1515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="18" t="s">
         <v>136</v>
       </c>
@@ -1506,7 +1529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="18" t="s">
         <v>142</v>
       </c>
@@ -1520,7 +1543,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" s="18" t="s">
         <v>131</v>
       </c>
@@ -1534,7 +1557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B20" s="18" t="s">
         <v>132</v>
       </c>
@@ -1548,7 +1571,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
         <v>137</v>
       </c>
@@ -1562,7 +1585,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B22" s="18" t="s">
         <v>138</v>
       </c>
@@ -1576,7 +1599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B23" s="18" t="s">
         <v>139</v>
       </c>
@@ -1590,7 +1613,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B24" s="18" t="s">
         <v>141</v>
       </c>
@@ -1604,7 +1627,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B25" s="18" t="s">
         <v>145</v>
       </c>
@@ -1618,7 +1641,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B26" s="18" t="s">
         <v>146</v>
       </c>
@@ -1632,7 +1655,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B27" s="18" t="s">
         <v>147</v>
       </c>
@@ -1646,7 +1669,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B28" s="18" t="s">
         <v>140</v>
       </c>
@@ -1660,7 +1683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B29" s="18" t="s">
         <v>143</v>
       </c>
@@ -1674,7 +1697,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B30" s="18" t="s">
         <v>135</v>
       </c>
@@ -1688,7 +1711,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="18" t="s">
         <v>144</v>
       </c>
@@ -1702,7 +1725,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B32" s="18" t="s">
         <v>148</v>
       </c>
@@ -1716,7 +1739,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B33" s="18" t="s">
         <v>149</v>
       </c>
@@ -1730,7 +1753,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B34" s="18" t="s">
         <v>150</v>
       </c>
@@ -1744,7 +1767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="18" t="s">
         <v>151</v>
       </c>
@@ -1758,7 +1781,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="18" t="s">
         <v>152</v>
       </c>
@@ -1772,7 +1795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="22" t="s">
         <v>127</v>
       </c>
@@ -1786,8 +1809,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="41" t="s">
         <v>158</v>
       </c>
@@ -1823,32 +1846,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" customWidth="1"/>
-    <col min="6" max="6" width="18.81640625" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" customWidth="1"/>
-    <col min="8" max="8" width="16.08984375" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
-    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -1878,7 +1901,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -1932,7 +1955,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
         <v>97</v>
       </c>
@@ -1959,7 +1982,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="26" t="s">
         <v>96</v>
       </c>
@@ -1981,7 +2004,7 @@
       <c r="P6" s="31"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="26" t="s">
         <v>98</v>
       </c>
@@ -2008,7 +2031,7 @@
       <c r="P7" s="31"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="26" t="s">
         <v>104</v>
       </c>
@@ -2041,7 +2064,7 @@
       <c r="P8" s="31"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="26" t="s">
         <v>99</v>
       </c>
@@ -2078,7 +2101,7 @@
       </c>
       <c r="R9" s="28"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="26" t="s">
         <v>103</v>
       </c>
@@ -2115,7 +2138,7 @@
       </c>
       <c r="R10" s="28"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="26" t="s">
         <v>101</v>
       </c>
@@ -2147,7 +2170,7 @@
       </c>
       <c r="R11" s="28"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="26" t="s">
         <v>102</v>
       </c>
@@ -2175,7 +2198,7 @@
       <c r="P12" s="31"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="47" t="s">
         <v>100</v>
       </c>
@@ -2202,15 +2225,15 @@
       <c r="Q13" s="46"/>
       <c r="R13" s="17"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="20"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="20"/>
       <c r="P25" s="20"/>
       <c r="S25" s="20"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="20"/>
       <c r="P26" s="20"/>
       <c r="S26" s="20"/>
@@ -2225,25 +2248,26 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="B3:L35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B3:L37"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.453125" customWidth="1"/>
-    <col min="9" max="9" width="52.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.21875" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" customWidth="1"/>
+    <col min="9" max="9" width="43.6640625" customWidth="1"/>
+    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:12" ht="46" x14ac:dyDescent="1">
+    <row r="3" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
       <c r="B5" s="7"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
@@ -2268,7 +2292,7 @@
       </c>
       <c r="L5" s="6"/>
     </row>
-    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B6" s="7" t="s">
         <v>1</v>
       </c>
@@ -2303,7 +2327,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="35" t="s">
         <v>24</v>
       </c>
@@ -2316,7 +2340,7 @@
       <c r="E7" s="11">
         <v>100</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="54" t="s">
         <v>159</v>
       </c>
       <c r="G7" s="21"/>
@@ -2326,7 +2350,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="36" t="s">
         <v>35</v>
       </c>
@@ -2344,7 +2368,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
@@ -2362,7 +2386,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="36" t="s">
         <v>75</v>
       </c>
@@ -2380,7 +2404,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="36" t="s">
         <v>122</v>
       </c>
@@ -2395,7 +2419,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="36" t="s">
         <v>25</v>
       </c>
@@ -2404,13 +2428,16 @@
       </c>
       <c r="D12" s="18"/>
       <c r="F12" s="14"/>
-      <c r="G12" s="18" t="s">
-        <v>89</v>
+      <c r="G12" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H12">
+        <v>100</v>
       </c>
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="36" t="s">
         <v>26</v>
       </c>
@@ -2419,13 +2446,16 @@
       </c>
       <c r="D13" s="18"/>
       <c r="F13" s="14"/>
-      <c r="G13" s="18" t="s">
-        <v>89</v>
+      <c r="G13" s="18">
+        <v>0.15</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
       </c>
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="36" t="s">
         <v>27</v>
       </c>
@@ -2434,13 +2464,16 @@
       </c>
       <c r="D14" s="18"/>
       <c r="F14" s="14"/>
-      <c r="G14" s="18" t="s">
-        <v>89</v>
+      <c r="G14" s="18">
+        <v>0.15</v>
+      </c>
+      <c r="H14">
+        <v>100</v>
       </c>
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="36" t="s">
         <v>29</v>
       </c>
@@ -2449,13 +2482,16 @@
       </c>
       <c r="D15" s="18"/>
       <c r="F15" s="14"/>
-      <c r="G15" s="18" t="s">
-        <v>89</v>
+      <c r="G15" s="18">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>100</v>
       </c>
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
         <v>30</v>
       </c>
@@ -2464,43 +2500,44 @@
       </c>
       <c r="D16" s="18"/>
       <c r="F16" s="14"/>
-      <c r="G16" s="18" t="s">
-        <v>89</v>
+      <c r="G16" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="H16">
+        <v>100</v>
       </c>
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="36" t="s">
-        <v>92</v>
+        <v>162</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D17" s="18"/>
       <c r="F17" s="14"/>
       <c r="G17" s="18">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="H17">
         <v>100</v>
       </c>
-      <c r="I17" s="14" t="s">
-        <v>160</v>
-      </c>
+      <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="36" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D18" s="18"/>
       <c r="F18" s="14"/>
       <c r="G18" s="18">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H18">
         <v>100</v>
@@ -2508,41 +2545,47 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="36" t="s">
-        <v>90</v>
+        <v>164</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D19" s="18"/>
       <c r="F19" s="14"/>
-      <c r="G19" s="18" t="s">
-        <v>89</v>
+      <c r="G19" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="H19">
+        <v>100</v>
       </c>
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="36" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="C20" s="36" t="s">
         <v>107</v>
       </c>
+      <c r="D20" s="18"/>
       <c r="F20" s="14"/>
       <c r="G20" s="18">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H20">
         <v>100</v>
       </c>
-      <c r="I20" s="14"/>
+      <c r="I20" s="55" t="s">
+        <v>160</v>
+      </c>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="36" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="C21" s="36" t="s">
         <v>107</v>
@@ -2550,52 +2593,49 @@
       <c r="D21" s="18"/>
       <c r="F21" s="14"/>
       <c r="G21" s="18">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H21">
         <v>100</v>
       </c>
       <c r="I21" s="14"/>
-      <c r="J21" t="s">
-        <v>89</v>
-      </c>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="36" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C22" s="36" t="s">
         <v>107</v>
       </c>
       <c r="D22" s="18"/>
       <c r="F22" s="14"/>
-      <c r="G22" s="18"/>
+      <c r="G22" s="18" t="s">
+        <v>89</v>
+      </c>
       <c r="I22" s="14"/>
-      <c r="J22" t="s">
-        <v>89</v>
-      </c>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="36" t="s">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="C23" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="D23" s="18"/>
       <c r="F23" s="14"/>
-      <c r="G23" s="18"/>
+      <c r="G23" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H23">
+        <v>100</v>
+      </c>
       <c r="I23" s="14"/>
-      <c r="J23" t="s">
-        <v>89</v>
-      </c>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C24" s="36" t="s">
         <v>107</v>
@@ -2606,19 +2646,14 @@
         <v>0.5</v>
       </c>
       <c r="H24">
-        <v>25</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="J24" t="s">
-        <v>89</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B25" s="18" t="s">
-        <v>76</v>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B25" s="36" t="s">
+        <v>93</v>
       </c>
       <c r="C25" s="36" t="s">
         <v>107</v>
@@ -2627,62 +2662,57 @@
       <c r="F25" s="14"/>
       <c r="G25" s="18"/>
       <c r="I25" s="14"/>
-      <c r="J25" t="s">
-        <v>89</v>
-      </c>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="36" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D26" s="18"/>
       <c r="F26" s="14"/>
       <c r="G26" s="18"/>
       <c r="I26" s="14"/>
-      <c r="J26" t="s">
-        <v>89</v>
-      </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B27" s="18" t="s">
-        <v>44</v>
+    <row r="27" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B27" s="36" t="s">
+        <v>79</v>
       </c>
       <c r="C27" s="36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D27" s="18"/>
       <c r="F27" s="14"/>
-      <c r="G27" s="18"/>
-      <c r="I27" s="14"/>
-      <c r="J27" t="s">
-        <v>89</v>
+      <c r="G27" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="H27">
+        <v>25</v>
+      </c>
+      <c r="I27" s="55" t="s">
+        <v>161</v>
       </c>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B28" s="36" t="s">
-        <v>37</v>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B28" s="18" t="s">
+        <v>76</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D28" s="18"/>
       <c r="F28" s="14"/>
       <c r="G28" s="18"/>
       <c r="I28" s="14"/>
-      <c r="J28" t="s">
-        <v>89</v>
-      </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B29" s="36" t="s">
-        <v>73</v>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B29" s="18" t="s">
+        <v>44</v>
       </c>
       <c r="C29" s="36" t="s">
         <v>106</v>
@@ -2691,14 +2721,11 @@
       <c r="F29" s="14"/>
       <c r="G29" s="18"/>
       <c r="I29" s="14"/>
-      <c r="J29" t="s">
-        <v>89</v>
-      </c>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="36" t="s">
-        <v>38</v>
+        <v>165</v>
       </c>
       <c r="C30" s="36" t="s">
         <v>106</v>
@@ -2707,14 +2734,11 @@
       <c r="F30" s="14"/>
       <c r="G30" s="18"/>
       <c r="I30" s="14"/>
-      <c r="J30" t="s">
-        <v>89</v>
-      </c>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="36" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="C31" s="36" t="s">
         <v>106</v>
@@ -2723,14 +2747,11 @@
       <c r="F31" s="14"/>
       <c r="G31" s="18"/>
       <c r="I31" s="14"/>
-      <c r="J31" t="s">
-        <v>89</v>
-      </c>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="36" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C32" s="36" t="s">
         <v>106</v>
@@ -2739,14 +2760,11 @@
       <c r="F32" s="14"/>
       <c r="G32" s="18"/>
       <c r="I32" s="14"/>
-      <c r="J32" t="s">
-        <v>89</v>
-      </c>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="36" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>106</v>
@@ -2755,14 +2773,11 @@
       <c r="F33" s="14"/>
       <c r="G33" s="18"/>
       <c r="I33" s="14"/>
-      <c r="J33" t="s">
-        <v>89</v>
-      </c>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="36" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="C34" s="36" t="s">
         <v>106</v>
@@ -2771,29 +2786,50 @@
       <c r="F34" s="14"/>
       <c r="G34" s="18"/>
       <c r="I34" s="14"/>
-      <c r="J34" t="s">
-        <v>89</v>
-      </c>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B35" s="37" t="s">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B35" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D35" s="18"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="18"/>
+      <c r="I35" s="14"/>
+      <c r="L35" s="14"/>
+    </row>
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B36" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="18"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="18"/>
+      <c r="I36" s="14"/>
+      <c r="L36" s="14"/>
+    </row>
+    <row r="37" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="37" t="s">
+      <c r="C37" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="D35" s="22"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="17"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="16"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2806,27 +2842,27 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.1796875" customWidth="1"/>
-    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.1796875" customWidth="1"/>
-    <col min="9" max="9" width="19.81640625" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="19.453125" customWidth="1"/>
+    <col min="1" max="1" width="2.21875" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.5546875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="19.77734375" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -2845,7 +2881,7 @@
       <c r="K3" s="4"/>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -2880,7 +2916,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="35"/>
       <c r="C5" s="12"/>
       <c r="D5" s="49"/>
@@ -2893,7 +2929,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="36"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -2902,7 +2938,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="36"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -2911,7 +2947,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="36"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -2920,7 +2956,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="36"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -2929,7 +2965,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="36"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -2938,7 +2974,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="36"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -2947,7 +2983,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="36"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -2956,7 +2992,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="36"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -2965,7 +3001,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="36"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -2974,7 +3010,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="36"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -2983,7 +3019,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="36"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -2992,7 +3028,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="36"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -3001,7 +3037,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="36"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -3010,7 +3046,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="36"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -3019,7 +3055,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="36"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3028,7 +3064,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="36"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3037,7 +3073,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="36"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3046,7 +3082,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="36"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3055,7 +3091,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="36"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3064,7 +3100,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3073,7 +3109,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="36"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3082,7 +3118,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="36"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3091,7 +3127,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="36"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3100,7 +3136,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="36"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3109,7 +3145,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="36"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3118,7 +3154,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="36"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3127,7 +3163,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="36"/>
       <c r="C32" s="14"/>
       <c r="D32" s="50"/>
@@ -3136,7 +3172,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="36"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3145,7 +3181,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="36"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3154,7 +3190,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="36"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3163,7 +3199,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="36"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3172,7 +3208,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="36"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3181,7 +3217,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="36"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3190,7 +3226,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="36"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3199,7 +3235,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="37"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3232,21 +3268,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="70.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="70.77734375" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" customWidth="1"/>
-    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="9" t="s">
         <v>22</v>
       </c>
@@ -3260,151 +3296,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -3420,28 +3456,28 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" customWidth="1"/>
-    <col min="5" max="5" width="21.1796875" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.81640625" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
-    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -3466,7 +3502,7 @@
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -3501,7 +3537,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="51"/>
       <c r="C5" s="12"/>
       <c r="D5" s="21"/>
@@ -3514,7 +3550,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="52"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -3523,7 +3559,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="52"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -3532,7 +3568,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="52"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -3541,7 +3577,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="52"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -3550,7 +3586,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="52"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -3559,7 +3595,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="52"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -3568,7 +3604,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="52"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -3577,7 +3613,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="52"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -3586,7 +3622,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="52"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -3595,7 +3631,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="52"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -3604,7 +3640,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="52"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -3613,7 +3649,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="52"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -3622,7 +3658,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="52"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -3631,7 +3667,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="52"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -3640,7 +3676,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="52"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3649,7 +3685,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="52"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3658,7 +3694,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="52"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3667,7 +3703,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="52"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3676,7 +3712,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="52"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3685,7 +3721,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="52"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3694,7 +3730,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="52"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3703,7 +3739,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="52"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3712,7 +3748,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="52"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3721,7 +3757,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="52"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3730,7 +3766,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="52"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3739,7 +3775,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="52"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3748,7 +3784,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="52"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -3757,7 +3793,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="52"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3766,7 +3802,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="52"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3775,7 +3811,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="52"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3784,7 +3820,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="52"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3793,7 +3829,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="52"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3802,7 +3838,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="52"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3811,7 +3847,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="52"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3820,7 +3856,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="53"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3853,18 +3889,18 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B2:O56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -3888,7 +3924,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -3932,7 +3968,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="10" t="s">
         <v>95</v>
       </c>
@@ -3954,7 +3990,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -3972,7 +4008,7 @@
       <c r="M7" s="18"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
         <v>84</v>
       </c>
@@ -3990,7 +4026,7 @@
       <c r="M8" s="18"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
@@ -4008,7 +4044,7 @@
       <c r="M9" s="18"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="13" t="s">
         <v>83</v>
       </c>
@@ -4026,7 +4062,7 @@
       <c r="M10" s="18"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="13" t="s">
         <v>62</v>
       </c>
@@ -4044,7 +4080,7 @@
       <c r="M11" s="18"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
@@ -4062,7 +4098,7 @@
       <c r="M12" s="18"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="13" t="s">
         <v>86</v>
       </c>
@@ -4080,7 +4116,7 @@
       <c r="M13" s="18"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="13" t="s">
         <v>54</v>
       </c>
@@ -4098,7 +4134,7 @@
       <c r="M14" s="18"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="13" t="s">
         <v>58</v>
       </c>
@@ -4116,7 +4152,7 @@
       <c r="M15" s="18"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="13" t="s">
         <v>59</v>
       </c>
@@ -4134,7 +4170,7 @@
       <c r="M16" s="18"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
         <v>60</v>
       </c>
@@ -4152,7 +4188,7 @@
       <c r="M17" s="18"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="13" t="s">
         <v>63</v>
       </c>
@@ -4170,7 +4206,7 @@
       <c r="M18" s="18"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="13" t="s">
         <v>46</v>
       </c>
@@ -4188,7 +4224,7 @@
       <c r="M19" s="18"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
         <v>45</v>
       </c>
@@ -4206,7 +4242,7 @@
       <c r="M20" s="18"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>82</v>
       </c>
@@ -4224,7 +4260,7 @@
       <c r="M21" s="18"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="13" t="s">
         <v>40</v>
       </c>
@@ -4242,7 +4278,7 @@
       <c r="M22" s="18"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="13" t="s">
         <v>41</v>
       </c>
@@ -4260,7 +4296,7 @@
       <c r="M23" s="18"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="13" t="s">
         <v>57</v>
       </c>
@@ -4278,7 +4314,7 @@
       <c r="M24" s="18"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="13" t="s">
         <v>53</v>
       </c>
@@ -4296,7 +4332,7 @@
       <c r="M25" s="18"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="13" t="s">
         <v>72</v>
       </c>
@@ -4314,7 +4350,7 @@
       <c r="M26" s="18"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
@@ -4332,7 +4368,7 @@
       <c r="M27" s="18"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="13" t="s">
         <v>69</v>
       </c>
@@ -4350,7 +4386,7 @@
       <c r="M28" s="18"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="13" t="s">
         <v>71</v>
       </c>
@@ -4368,7 +4404,7 @@
       <c r="M29" s="18"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="13" t="s">
         <v>67</v>
       </c>
@@ -4386,7 +4422,7 @@
       </c>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="13" t="s">
         <v>65</v>
       </c>
@@ -4404,7 +4440,7 @@
       </c>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B32" s="13" t="s">
         <v>66</v>
       </c>
@@ -4422,7 +4458,7 @@
       </c>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="13" t="s">
         <v>114</v>
       </c>
@@ -4440,7 +4476,7 @@
       </c>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="13" t="s">
         <v>88</v>
       </c>
@@ -4458,7 +4494,7 @@
       </c>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="15" t="s">
         <v>70</v>
       </c>
@@ -4480,47 +4516,47 @@
       <c r="N35" s="16"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="40" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B53" s="36" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4532,29 +4568,29 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="51.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.54296875" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.1796875" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.1796875" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="51.5546875" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
+    <col min="7" max="7" width="20.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -4586,7 +4622,7 @@
       </c>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -4630,7 +4666,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="51"/>
       <c r="C6" s="12"/>
       <c r="D6" s="21"/>
@@ -4646,7 +4682,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="52"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -4656,7 +4692,7 @@
       <c r="L7" s="14"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="52"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -4666,7 +4702,7 @@
       <c r="L8" s="14"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="52"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -4676,7 +4712,7 @@
       <c r="L9" s="14"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="52"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -4686,7 +4722,7 @@
       <c r="L10" s="14"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="52"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -4696,7 +4732,7 @@
       <c r="L11" s="14"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="52"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -4706,7 +4742,7 @@
       <c r="L12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="52"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -4716,7 +4752,7 @@
       <c r="L13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="52"/>
       <c r="C14" s="14"/>
       <c r="D14" s="50"/>
@@ -4726,7 +4762,7 @@
       <c r="L14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="52"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -4736,7 +4772,7 @@
       <c r="L15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="52"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -4746,7 +4782,7 @@
       <c r="L16" s="14"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="52"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -4756,7 +4792,7 @@
       <c r="L17" s="14"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="52"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -4766,7 +4802,7 @@
       <c r="L18" s="14"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="52"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -4776,7 +4812,7 @@
       <c r="L19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="52"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -4786,7 +4822,7 @@
       <c r="L20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="52"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -4796,7 +4832,7 @@
       <c r="L21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="52"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -4806,7 +4842,7 @@
       <c r="L22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="52"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -4816,7 +4852,7 @@
       <c r="L23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="52"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -4826,7 +4862,7 @@
       <c r="L24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="52"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -4836,7 +4872,7 @@
       <c r="L25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="52"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -4846,7 +4882,7 @@
       <c r="L26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="52"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -4856,7 +4892,7 @@
       <c r="L27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="52"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -4866,7 +4902,7 @@
       <c r="L28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="52"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -4876,7 +4912,7 @@
       <c r="L29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="52"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -4886,7 +4922,7 @@
       <c r="L30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="52"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -4896,7 +4932,7 @@
       <c r="L31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B32" s="52"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -4906,7 +4942,7 @@
       <c r="L32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="52"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -4916,7 +4952,7 @@
       <c r="L33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="52"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -4926,7 +4962,7 @@
       <c r="L34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="52"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -4936,7 +4972,7 @@
       <c r="L35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="52"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -4946,7 +4982,7 @@
       <c r="L36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="52"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -4956,7 +4992,7 @@
       <c r="L37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B38" s="52"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -4966,7 +5002,7 @@
       <c r="L38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B39" s="52"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -4976,7 +5012,7 @@
       <c r="L39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B40" s="52"/>
       <c r="C40" s="14"/>
       <c r="D40" s="18"/>
@@ -4986,7 +5022,7 @@
       <c r="L40" s="14"/>
       <c r="O40" s="14"/>
     </row>
-    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="53"/>
       <c r="C41" s="17"/>
       <c r="D41" s="22"/>
@@ -5002,7 +5038,7 @@
       <c r="N41" s="16"/>
       <c r="O41" s="17"/>
     </row>
-    <row r="64" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="64" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" t="s">
@@ -5011,7 +5047,7 @@
       <c r="J64" s="5"/>
       <c r="M64" s="5"/>
     </row>
-    <row r="65" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="65" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" t="s">
@@ -5020,7 +5056,7 @@
       <c r="J65" s="5"/>
       <c r="M65" s="5"/>
     </row>
-    <row r="67" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="67" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" t="s">
@@ -5029,7 +5065,7 @@
       <c r="J67" s="5"/>
       <c r="M67" s="5"/>
     </row>
-    <row r="68" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="68" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D68" s="5"/>
       <c r="G68" s="5"/>
       <c r="J68" s="5"/>
@@ -5038,17 +5074,17 @@
       </c>
       <c r="M68" s="5"/>
     </row>
-    <row r="71" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="71" spans="4:13" x14ac:dyDescent="0.3">
       <c r="H71" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="72" spans="4:13" x14ac:dyDescent="0.3">
       <c r="K72" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="4:13" x14ac:dyDescent="0.35">
+    <row r="73" spans="4:13" x14ac:dyDescent="0.3">
       <c r="D73" s="5"/>
       <c r="G73" s="5"/>
       <c r="J73" s="5"/>
@@ -5076,28 +5112,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
-    <col min="2" max="2" width="93.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="2" max="2" width="93.21875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="42.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.75" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:6" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -5114,7 +5150,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -5127,7 +5163,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -5140,7 +5176,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -5153,7 +5189,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -5166,7 +5202,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -5179,7 +5215,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -5192,7 +5228,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -5205,7 +5241,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -5218,7 +5254,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5231,7 +5267,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -5244,7 +5280,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -5257,7 +5293,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5270,7 +5306,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -5283,7 +5319,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -5296,7 +5332,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -5309,7 +5345,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -5322,7 +5358,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -5335,7 +5371,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -5348,7 +5384,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -5361,7 +5397,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -5374,7 +5410,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5387,7 +5423,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -5400,7 +5436,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -5413,7 +5449,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -5426,7 +5462,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -5439,7 +5475,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -5452,7 +5488,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -5465,7 +5501,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -5478,7 +5514,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -5491,7 +5527,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -5504,7 +5540,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -5517,7 +5553,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -5530,7 +5566,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -5543,7 +5579,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -5556,7 +5592,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -5569,7 +5605,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -5582,7 +5618,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -5595,7 +5631,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -5608,7 +5644,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -5621,7 +5657,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -5634,7 +5670,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -5647,7 +5683,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -5660,7 +5696,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -5673,7 +5709,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -5686,7 +5722,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -5699,7 +5735,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -5712,7 +5748,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -5725,7 +5761,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -5738,7 +5774,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -5751,7 +5787,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -5764,7 +5800,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -5777,7 +5813,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -5790,7 +5826,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -5803,7 +5839,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -5816,7 +5852,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -5829,7 +5865,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -5842,7 +5878,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -5855,7 +5891,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -5868,7 +5904,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -5881,7 +5917,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>96</v>
       </c>
@@ -5892,7 +5928,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>97</v>
       </c>
@@ -5903,7 +5939,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>98</v>
       </c>
@@ -5914,7 +5950,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>99</v>
       </c>
@@ -5925,7 +5961,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>100</v>
       </c>
@@ -5936,7 +5972,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>101</v>
       </c>
@@ -5947,7 +5983,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>102</v>
       </c>
@@ -5958,7 +5994,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>103</v>
       </c>
@@ -5969,7 +6005,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>104</v>
       </c>
@@ -5980,7 +6016,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>120</v>
       </c>
@@ -5991,7 +6027,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>121</v>
       </c>
@@ -6002,182 +6038,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Mise a jour index.jsx:bg,logo,buttons+ debut fonction fetch
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86B1876-8C49-4207-9813-D509DE7E0027}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B23B575-F3C4-4EF7-AD9B-6AC688A0A80F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="168">
   <si>
     <t>Planification globale</t>
   </si>
@@ -541,6 +541,9 @@
 navbar conditionnelle (visible si connecté)
 , fond d'écran dynamique,
  conteneur principal</t>
+  </si>
+  <si>
+    <t>Page index.jsx: ajut : background ,logo,boutons</t>
   </si>
 </sst>
 </file>
@@ -1081,6 +1084,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1107,9 +1113,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2410,7 +2413,7 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="B2:L37"/>
+  <dimension ref="B2:L38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.54296875" customWidth="1"/>
@@ -2429,26 +2432,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="64"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="67" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="57" t="s">
@@ -2457,7 +2460,7 @@
       <c r="E5" s="58">
         <v>46083</v>
       </c>
-      <c r="F5" s="68" t="s">
+      <c r="F5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="60" t="s">
@@ -2466,7 +2469,7 @@
       <c r="H5" s="58">
         <v>46090</v>
       </c>
-      <c r="I5" s="68" t="s">
+      <c r="I5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="60" t="s">
@@ -2475,34 +2478,34 @@
       <c r="K5" s="58">
         <v>46104</v>
       </c>
-      <c r="L5" s="68" t="s">
+      <c r="L5" s="69" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="65"/>
-      <c r="C6" s="67"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="57" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="69"/>
+      <c r="F6" s="70"/>
       <c r="G6" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="69"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="59" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="69"/>
+      <c r="L6" s="70"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
@@ -2756,7 +2759,7 @@
       <c r="L19" s="14"/>
     </row>
     <row r="20" spans="2:12" ht="58" x14ac:dyDescent="0.35">
-      <c r="B20" s="70" t="s">
+      <c r="B20" s="61" t="s">
         <v>166</v>
       </c>
       <c r="C20" s="36" t="s">
@@ -2945,8 +2948,12 @@
       <c r="D30" s="31"/>
       <c r="E30" s="40"/>
       <c r="F30" s="14"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="40"/>
+      <c r="G30" s="31">
+        <v>2</v>
+      </c>
+      <c r="H30" s="40">
+        <v>100</v>
+      </c>
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
@@ -2960,14 +2967,18 @@
       <c r="D31" s="31"/>
       <c r="E31" s="40"/>
       <c r="F31" s="14"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="40"/>
+      <c r="G31" s="31">
+        <v>1.3</v>
+      </c>
+      <c r="H31" s="40">
+        <v>100</v>
+      </c>
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="36" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C32" s="36" t="s">
         <v>106</v>
@@ -2975,14 +2986,18 @@
       <c r="D32" s="31"/>
       <c r="E32" s="40"/>
       <c r="F32" s="14"/>
-      <c r="G32" s="31"/>
-      <c r="H32" s="40"/>
+      <c r="G32" s="31">
+        <v>1.5</v>
+      </c>
+      <c r="H32" s="40">
+        <v>100</v>
+      </c>
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="36" t="s">
-        <v>73</v>
+        <v>164</v>
       </c>
       <c r="C33" s="36" t="s">
         <v>106</v>
@@ -2997,7 +3012,7 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="36" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="C34" s="36" t="s">
         <v>106</v>
@@ -3012,7 +3027,7 @@
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C35" s="36" t="s">
         <v>106</v>
@@ -3027,7 +3042,7 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="36" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C36" s="36" t="s">
         <v>106</v>
@@ -3040,22 +3055,37 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="37" t="s">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B37" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C37" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="31"/>
+      <c r="E37" s="40"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="40"/>
+      <c r="I37" s="14"/>
+      <c r="L37" s="14"/>
+    </row>
+    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B38" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="37" t="s">
+      <c r="C38" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="D37" s="32"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="17"/>
-      <c r="G37" s="32"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="16"/>
-      <c r="K37" s="16"/>
-      <c r="L37" s="17"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="56"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="16"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="B5:L6" xr:uid="{00000000-0009-0000-0000-000002000000}"/>

</xml_diff>

<commit_message>
debut tour, connexion db
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86B1876-8C49-4207-9813-D509DE7E0027}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F84E09F-2AB3-4EF4-9310-5BE65899CF3A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="168">
   <si>
     <t>Planification globale</t>
   </si>
@@ -541,6 +541,9 @@
 navbar conditionnelle (visible si connecté)
 , fond d'écran dynamique,
  conteneur principal</t>
+  </si>
+  <si>
+    <t>Création de toutes les tables</t>
   </si>
 </sst>
 </file>
@@ -1081,6 +1084,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1107,9 +1113,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2429,26 +2432,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="64"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="67" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="57" t="s">
@@ -2457,7 +2460,7 @@
       <c r="E5" s="58">
         <v>46083</v>
       </c>
-      <c r="F5" s="68" t="s">
+      <c r="F5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="60" t="s">
@@ -2466,7 +2469,7 @@
       <c r="H5" s="58">
         <v>46090</v>
       </c>
-      <c r="I5" s="68" t="s">
+      <c r="I5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="60" t="s">
@@ -2475,34 +2478,34 @@
       <c r="K5" s="58">
         <v>46104</v>
       </c>
-      <c r="L5" s="68" t="s">
+      <c r="L5" s="69" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="65"/>
-      <c r="C6" s="67"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="57" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="69"/>
+      <c r="F6" s="70"/>
       <c r="G6" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="69"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="59" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="69"/>
+      <c r="L6" s="70"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
@@ -2756,7 +2759,7 @@
       <c r="L19" s="14"/>
     </row>
     <row r="20" spans="2:12" ht="58" x14ac:dyDescent="0.35">
-      <c r="B20" s="70" t="s">
+      <c r="B20" s="61" t="s">
         <v>166</v>
       </c>
       <c r="C20" s="36" t="s">
@@ -2824,9 +2827,7 @@
       <c r="D23" s="31"/>
       <c r="E23" s="40"/>
       <c r="F23" s="14"/>
-      <c r="G23" s="31" t="s">
-        <v>89</v>
-      </c>
+      <c r="G23" s="31"/>
       <c r="H23" s="40"/>
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
@@ -2879,9 +2880,15 @@
       <c r="D26" s="31"/>
       <c r="E26" s="40"/>
       <c r="F26" s="14"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="14"/>
+      <c r="G26" s="31">
+        <v>1</v>
+      </c>
+      <c r="H26" s="40">
+        <v>100</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>167</v>
+      </c>
       <c r="L26" s="14"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Mise a jour planification
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD9F194-8782-451D-9518-91862A3A7CC4}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773CBCD3-7D1C-471B-A490-96D1864AC313}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,22 +27,17 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planification!$B$5:$E$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="171">
   <si>
     <t>Planification globale</t>
   </si>
@@ -552,6 +547,12 @@
   </si>
   <si>
     <t>Gerer les erreurs dans page index</t>
+  </si>
+  <si>
+    <t>Creation page administration liste les comptes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajouter permettre la supression d un compte </t>
   </si>
 </sst>
 </file>
@@ -1508,26 +1509,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="5" spans="2:5" ht="46.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="21" t="s">
         <v>152</v>
       </c>
@@ -1555,7 +1556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="18" t="s">
         <v>122</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>123</v>
       </c>
@@ -1583,7 +1584,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="18" t="s">
         <v>124</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="18" t="s">
         <v>125</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="18" t="s">
         <v>127</v>
       </c>
@@ -1625,7 +1626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="18" t="s">
         <v>128</v>
       </c>
@@ -1639,7 +1640,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="18" t="s">
         <v>129</v>
       </c>
@@ -1653,7 +1654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>156</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="18" t="s">
         <v>132</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="18" t="s">
         <v>133</v>
       </c>
@@ -1695,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="18" t="s">
         <v>135</v>
       </c>
@@ -1709,7 +1710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="18" t="s">
         <v>141</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="18" t="s">
         <v>130</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
         <v>131</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="18" t="s">
         <v>136</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="18" t="s">
         <v>137</v>
       </c>
@@ -1779,7 +1780,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="18" t="s">
         <v>138</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="18" t="s">
         <v>140</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="18" t="s">
         <v>144</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>145</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="18" t="s">
         <v>146</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="18" t="s">
         <v>139</v>
       </c>
@@ -1863,7 +1864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="18" t="s">
         <v>142</v>
       </c>
@@ -1877,7 +1878,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="18" t="s">
         <v>134</v>
       </c>
@@ -1891,7 +1892,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>143</v>
       </c>
@@ -1905,7 +1906,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>147</v>
       </c>
@@ -1919,7 +1920,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="18" t="s">
         <v>148</v>
       </c>
@@ -1933,7 +1934,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="18" t="s">
         <v>149</v>
       </c>
@@ -1947,7 +1948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="18" t="s">
         <v>150</v>
       </c>
@@ -1961,7 +1962,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="18" t="s">
         <v>151</v>
       </c>
@@ -1975,7 +1976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="22" t="s">
         <v>126</v>
       </c>
@@ -1989,8 +1990,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="41" t="s">
         <v>157</v>
       </c>
@@ -2019,32 +2020,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2074,7 +2075,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2128,7 +2129,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="23" t="s">
         <v>97</v>
       </c>
@@ -2155,7 +2156,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="26" t="s">
         <v>96</v>
       </c>
@@ -2177,7 +2178,7 @@
       <c r="P6" s="31"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="26" t="s">
         <v>98</v>
       </c>
@@ -2204,7 +2205,7 @@
       <c r="P7" s="31"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="26" t="s">
         <v>104</v>
       </c>
@@ -2237,7 +2238,7 @@
       <c r="P8" s="31"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="26" t="s">
         <v>99</v>
       </c>
@@ -2274,7 +2275,7 @@
       </c>
       <c r="R9" s="28"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="26" t="s">
         <v>103</v>
       </c>
@@ -2311,7 +2312,7 @@
       </c>
       <c r="R10" s="28"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="26" t="s">
         <v>101</v>
       </c>
@@ -2343,7 +2344,7 @@
       </c>
       <c r="R11" s="28"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="26" t="s">
         <v>102</v>
       </c>
@@ -2371,7 +2372,7 @@
       <c r="P12" s="31"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="47" t="s">
         <v>100</v>
       </c>
@@ -2398,15 +2399,15 @@
       <c r="Q13" s="46"/>
       <c r="R13" s="17"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="20"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="20"/>
       <c r="P25" s="20"/>
       <c r="S25" s="20"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="20"/>
       <c r="P26" s="20"/>
       <c r="S26" s="20"/>
@@ -2421,25 +2422,25 @@
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
-  <dimension ref="B2:L38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:L40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
-    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="56.21875" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.77734375" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="56.1796875" customWidth="1"/>
+    <col min="10" max="10" width="16.6328125" customWidth="1"/>
+    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B3" s="62" t="s">
         <v>6</v>
       </c>
@@ -2454,8 +2455,8 @@
       <c r="K3" s="63"/>
       <c r="L3" s="64"/>
     </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B5" s="65" t="s">
         <v>1</v>
       </c>
@@ -2490,7 +2491,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="66"/>
       <c r="C6" s="68"/>
       <c r="D6" s="57" t="s">
@@ -2515,7 +2516,7 @@
       </c>
       <c r="L6" s="70"/>
     </row>
-    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
         <v>24</v>
       </c>
@@ -2538,7 +2539,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="36" t="s">
         <v>35</v>
       </c>
@@ -2557,7 +2558,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
@@ -2576,7 +2577,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="36" t="s">
         <v>75</v>
       </c>
@@ -2595,7 +2596,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="36" t="s">
         <v>165</v>
       </c>
@@ -2614,7 +2615,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="36" t="s">
         <v>25</v>
       </c>
@@ -2633,7 +2634,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="36" t="s">
         <v>26</v>
       </c>
@@ -2652,7 +2653,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="36" t="s">
         <v>27</v>
       </c>
@@ -2671,7 +2672,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="36" t="s">
         <v>163</v>
       </c>
@@ -2690,7 +2691,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="36" t="s">
         <v>29</v>
       </c>
@@ -2709,7 +2710,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="36" t="s">
         <v>30</v>
       </c>
@@ -2728,7 +2729,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="36" t="s">
         <v>161</v>
       </c>
@@ -2747,7 +2748,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="36" t="s">
         <v>162</v>
       </c>
@@ -2766,7 +2767,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" ht="58" x14ac:dyDescent="0.35">
       <c r="B20" s="61" t="s">
         <v>166</v>
       </c>
@@ -2785,7 +2786,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="36" t="s">
         <v>92</v>
       </c>
@@ -2806,7 +2807,7 @@
       </c>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="36" t="s">
         <v>51</v>
       </c>
@@ -2825,7 +2826,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="36" t="s">
         <v>90</v>
       </c>
@@ -2840,7 +2841,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="36" t="s">
         <v>74</v>
       </c>
@@ -2859,7 +2860,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="36" t="s">
         <v>80</v>
       </c>
@@ -2878,7 +2879,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="36" t="s">
         <v>93</v>
       </c>
@@ -2899,7 +2900,7 @@
       </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="36" t="s">
         <v>94</v>
       </c>
@@ -2914,7 +2915,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B28" s="36" t="s">
         <v>79</v>
       </c>
@@ -2935,7 +2936,7 @@
       </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="18" t="s">
         <v>76</v>
       </c>
@@ -2950,7 +2951,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="36" t="s">
         <v>42</v>
       </c>
@@ -2969,7 +2970,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="36" t="s">
         <v>43</v>
       </c>
@@ -2988,7 +2989,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="36" t="s">
         <v>164</v>
       </c>
@@ -3003,7 +3004,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="36" t="s">
         <v>168</v>
       </c>
@@ -3020,9 +3021,15 @@
         <v>100</v>
       </c>
       <c r="I33" s="14"/>
+      <c r="J33">
+        <v>1</v>
+      </c>
+      <c r="K33">
+        <v>100</v>
+      </c>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="36" t="s">
         <v>73</v>
       </c>
@@ -3035,9 +3042,15 @@
       <c r="G34" s="31"/>
       <c r="H34" s="40"/>
       <c r="I34" s="14"/>
+      <c r="J34">
+        <v>1.5</v>
+      </c>
+      <c r="K34">
+        <v>100</v>
+      </c>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="36" t="s">
         <v>38</v>
       </c>
@@ -3050,9 +3063,15 @@
       <c r="G35" s="31"/>
       <c r="H35" s="40"/>
       <c r="I35" s="14"/>
+      <c r="J35">
+        <v>1</v>
+      </c>
+      <c r="K35">
+        <v>100</v>
+      </c>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="36" t="s">
         <v>39</v>
       </c>
@@ -3065,9 +3084,15 @@
       <c r="G36" s="31"/>
       <c r="H36" s="40"/>
       <c r="I36" s="14"/>
+      <c r="J36">
+        <v>0.75</v>
+      </c>
+      <c r="K36">
+        <v>100</v>
+      </c>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="36" t="s">
         <v>61</v>
       </c>
@@ -3080,24 +3105,68 @@
       <c r="G37" s="31"/>
       <c r="H37" s="40"/>
       <c r="I37" s="14"/>
+      <c r="J37">
+        <v>1.5</v>
+      </c>
+      <c r="K37">
+        <v>100</v>
+      </c>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="C38" s="37" t="s">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B38" s="36" t="s">
+        <v>169</v>
+      </c>
+      <c r="C38" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="D38" s="32"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="32"/>
-      <c r="H38" s="56"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="16"/>
-      <c r="K38" s="16"/>
-      <c r="L38" s="17"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="40"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="31"/>
+      <c r="H38" s="40"/>
+      <c r="I38" s="14"/>
+      <c r="J38">
+        <v>1.3</v>
+      </c>
+      <c r="K38">
+        <v>100</v>
+      </c>
+      <c r="L38" s="14"/>
+    </row>
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B39" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="C39" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D39" s="31"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="31"/>
+      <c r="H39" s="40"/>
+      <c r="I39" s="14"/>
+      <c r="J39">
+        <v>0.75</v>
+      </c>
+      <c r="K39">
+        <v>100</v>
+      </c>
+      <c r="L39" s="14"/>
+    </row>
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="32"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="56"/>
+      <c r="I40" s="17"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="16"/>
+      <c r="L40" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="B5:L6" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
@@ -3136,21 +3205,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="70.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="70.81640625" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" customWidth="1"/>
+    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="9" t="s">
         <v>22</v>
       </c>
@@ -3164,151 +3233,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -3324,28 +3393,28 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -3370,7 +3439,7 @@
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -3405,7 +3474,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="50"/>
       <c r="C5" s="12"/>
       <c r="D5" s="21"/>
@@ -3418,7 +3487,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="51"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -3427,7 +3496,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="51"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -3436,7 +3505,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="51"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -3445,7 +3514,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="51"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -3454,7 +3523,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="51"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -3463,7 +3532,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="51"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -3472,7 +3541,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="51"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -3481,7 +3550,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="51"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -3490,7 +3559,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="51"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -3499,7 +3568,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="51"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -3508,7 +3577,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="51"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -3517,7 +3586,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="51"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -3526,7 +3595,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="51"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -3535,7 +3604,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="51"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -3544,7 +3613,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="51"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3553,7 +3622,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="51"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3562,7 +3631,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="51"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3571,7 +3640,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="51"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3580,7 +3649,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="51"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3589,7 +3658,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="51"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3598,7 +3667,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="51"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3607,7 +3676,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="51"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3616,7 +3685,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="51"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3625,7 +3694,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="51"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3634,7 +3703,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="51"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3643,7 +3712,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="51"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3652,7 +3721,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="51"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -3661,7 +3730,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="51"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3670,7 +3739,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="51"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3679,7 +3748,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="51"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3688,7 +3757,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="51"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3697,7 +3766,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="51"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3706,7 +3775,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="51"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3715,7 +3784,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="51"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3724,7 +3793,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B40" s="52"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3757,18 +3826,18 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B2:O56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -3792,7 +3861,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -3836,7 +3905,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="10" t="s">
         <v>95</v>
       </c>
@@ -3858,7 +3927,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -3876,7 +3945,7 @@
       <c r="M7" s="18"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="13" t="s">
         <v>84</v>
       </c>
@@ -3894,7 +3963,7 @@
       <c r="M8" s="18"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
@@ -3912,7 +3981,7 @@
       <c r="M9" s="18"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="13" t="s">
         <v>83</v>
       </c>
@@ -3930,7 +3999,7 @@
       <c r="M10" s="18"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="13" t="s">
         <v>62</v>
       </c>
@@ -3948,7 +4017,7 @@
       <c r="M11" s="18"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
@@ -3966,7 +4035,7 @@
       <c r="M12" s="18"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="13" t="s">
         <v>86</v>
       </c>
@@ -3984,7 +4053,7 @@
       <c r="M13" s="18"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="13" t="s">
         <v>54</v>
       </c>
@@ -4002,7 +4071,7 @@
       <c r="M14" s="18"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="13" t="s">
         <v>58</v>
       </c>
@@ -4020,7 +4089,7 @@
       <c r="M15" s="18"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="13" t="s">
         <v>59</v>
       </c>
@@ -4038,7 +4107,7 @@
       <c r="M16" s="18"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="13" t="s">
         <v>60</v>
       </c>
@@ -4056,7 +4125,7 @@
       <c r="M17" s="18"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="13" t="s">
         <v>63</v>
       </c>
@@ -4074,7 +4143,7 @@
       <c r="M18" s="18"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="13" t="s">
         <v>46</v>
       </c>
@@ -4092,7 +4161,7 @@
       <c r="M19" s="18"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="13" t="s">
         <v>45</v>
       </c>
@@ -4110,7 +4179,7 @@
       <c r="M20" s="18"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="13" t="s">
         <v>82</v>
       </c>
@@ -4128,7 +4197,7 @@
       <c r="M21" s="18"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
         <v>40</v>
       </c>
@@ -4146,7 +4215,7 @@
       <c r="M22" s="18"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="13" t="s">
         <v>41</v>
       </c>
@@ -4164,7 +4233,7 @@
       <c r="M23" s="18"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="13" t="s">
         <v>57</v>
       </c>
@@ -4182,7 +4251,7 @@
       <c r="M24" s="18"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="13" t="s">
         <v>53</v>
       </c>
@@ -4200,7 +4269,7 @@
       <c r="M25" s="18"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="13" t="s">
         <v>72</v>
       </c>
@@ -4218,7 +4287,7 @@
       <c r="M26" s="18"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
@@ -4236,7 +4305,7 @@
       <c r="M27" s="18"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="13" t="s">
         <v>69</v>
       </c>
@@ -4254,7 +4323,7 @@
       <c r="M28" s="18"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="13" t="s">
         <v>71</v>
       </c>
@@ -4272,7 +4341,7 @@
       <c r="M29" s="18"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>67</v>
       </c>
@@ -4290,7 +4359,7 @@
       </c>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="13" t="s">
         <v>65</v>
       </c>
@@ -4308,7 +4377,7 @@
       </c>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="13" t="s">
         <v>66</v>
       </c>
@@ -4326,7 +4395,7 @@
       </c>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="13" t="s">
         <v>114</v>
       </c>
@@ -4344,7 +4413,7 @@
       </c>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="13" t="s">
         <v>88</v>
       </c>
@@ -4362,7 +4431,7 @@
       </c>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="15" t="s">
         <v>70</v>
       </c>
@@ -4384,47 +4453,47 @@
       <c r="N35" s="16"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="40" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B48" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" s="36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" s="36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" s="36" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B54" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4436,29 +4505,29 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="51.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.21875" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" customWidth="1"/>
-    <col min="7" max="7" width="20.44140625" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.21875" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.21875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="51.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -4490,7 +4559,7 @@
       </c>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -4534,7 +4603,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="50"/>
       <c r="C6" s="12"/>
       <c r="D6" s="21"/>
@@ -4550,7 +4619,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="51"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -4560,7 +4629,7 @@
       <c r="L7" s="14"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="51"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -4570,7 +4639,7 @@
       <c r="L8" s="14"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="51"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -4580,7 +4649,7 @@
       <c r="L9" s="14"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="51"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -4590,7 +4659,7 @@
       <c r="L10" s="14"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="51"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -4600,7 +4669,7 @@
       <c r="L11" s="14"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="51"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -4610,7 +4679,7 @@
       <c r="L12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="51"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -4620,7 +4689,7 @@
       <c r="L13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="51"/>
       <c r="C14" s="14"/>
       <c r="D14" s="49"/>
@@ -4630,7 +4699,7 @@
       <c r="L14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="51"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -4640,7 +4709,7 @@
       <c r="L15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="51"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -4650,7 +4719,7 @@
       <c r="L16" s="14"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="51"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -4660,7 +4729,7 @@
       <c r="L17" s="14"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="51"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -4670,7 +4739,7 @@
       <c r="L18" s="14"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="51"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -4680,7 +4749,7 @@
       <c r="L19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="51"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -4690,7 +4759,7 @@
       <c r="L20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="51"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -4700,7 +4769,7 @@
       <c r="L21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="51"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -4710,7 +4779,7 @@
       <c r="L22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="51"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -4720,7 +4789,7 @@
       <c r="L23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="51"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -4730,7 +4799,7 @@
       <c r="L24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="51"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -4740,7 +4809,7 @@
       <c r="L25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="51"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -4750,7 +4819,7 @@
       <c r="L26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="51"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -4760,7 +4829,7 @@
       <c r="L27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="51"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -4770,7 +4839,7 @@
       <c r="L28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="51"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -4780,7 +4849,7 @@
       <c r="L29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="51"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -4790,7 +4859,7 @@
       <c r="L30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="51"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -4800,7 +4869,7 @@
       <c r="L31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="51"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -4810,7 +4879,7 @@
       <c r="L32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="51"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -4820,7 +4889,7 @@
       <c r="L33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="51"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -4830,7 +4899,7 @@
       <c r="L34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B35" s="51"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -4840,7 +4909,7 @@
       <c r="L35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B36" s="51"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -4850,7 +4919,7 @@
       <c r="L36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B37" s="51"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -4860,7 +4929,7 @@
       <c r="L37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B38" s="51"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -4870,7 +4939,7 @@
       <c r="L38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B39" s="51"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -4880,7 +4949,7 @@
       <c r="L39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B40" s="51"/>
       <c r="C40" s="14"/>
       <c r="D40" s="18"/>
@@ -4890,7 +4959,7 @@
       <c r="L40" s="14"/>
       <c r="O40" s="14"/>
     </row>
-    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B41" s="52"/>
       <c r="C41" s="17"/>
       <c r="D41" s="22"/>
@@ -4906,7 +4975,7 @@
       <c r="N41" s="16"/>
       <c r="O41" s="17"/>
     </row>
-    <row r="64" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" t="s">
@@ -4915,7 +4984,7 @@
       <c r="J64" s="5"/>
       <c r="M64" s="5"/>
     </row>
-    <row r="65" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" t="s">
@@ -4924,7 +4993,7 @@
       <c r="J65" s="5"/>
       <c r="M65" s="5"/>
     </row>
-    <row r="67" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" t="s">
@@ -4933,7 +5002,7 @@
       <c r="J67" s="5"/>
       <c r="M67" s="5"/>
     </row>
-    <row r="68" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D68" s="5"/>
       <c r="G68" s="5"/>
       <c r="J68" s="5"/>
@@ -4942,17 +5011,17 @@
       </c>
       <c r="M68" s="5"/>
     </row>
-    <row r="71" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:13" x14ac:dyDescent="0.35">
       <c r="H71" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:13" x14ac:dyDescent="0.35">
       <c r="K72" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D73" s="5"/>
       <c r="G73" s="5"/>
       <c r="J73" s="5"/>
@@ -4980,28 +5049,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
-    <col min="2" max="2" width="93.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1796875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:6" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -5018,7 +5087,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -5031,7 +5100,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -5044,7 +5113,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -5057,7 +5126,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -5070,7 +5139,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -5083,7 +5152,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -5096,7 +5165,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -5109,7 +5178,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -5122,7 +5191,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5135,7 +5204,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -5148,7 +5217,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -5161,7 +5230,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5174,7 +5243,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -5187,7 +5256,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -5200,7 +5269,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -5213,7 +5282,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -5226,7 +5295,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -5239,7 +5308,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -5252,7 +5321,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -5265,7 +5334,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -5278,7 +5347,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5291,7 +5360,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -5304,7 +5373,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -5317,7 +5386,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -5330,7 +5399,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -5343,7 +5412,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -5356,7 +5425,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -5369,7 +5438,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -5382,7 +5451,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -5395,7 +5464,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -5408,7 +5477,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -5421,7 +5490,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -5434,7 +5503,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -5447,7 +5516,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -5460,7 +5529,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -5473,7 +5542,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -5486,7 +5555,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -5499,7 +5568,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -5512,7 +5581,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -5525,7 +5594,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -5538,7 +5607,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -5551,7 +5620,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -5564,7 +5633,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -5577,7 +5646,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -5590,7 +5659,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -5603,7 +5672,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -5616,7 +5685,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -5629,7 +5698,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -5642,7 +5711,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -5655,7 +5724,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -5668,7 +5737,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -5681,7 +5750,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -5694,7 +5763,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -5707,7 +5776,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -5720,7 +5789,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -5733,7 +5802,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -5746,7 +5815,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -5759,7 +5828,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -5772,7 +5841,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -5785,7 +5854,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>96</v>
       </c>
@@ -5796,7 +5865,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>97</v>
       </c>
@@ -5807,7 +5876,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>98</v>
       </c>
@@ -5818,7 +5887,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>99</v>
       </c>
@@ -5829,7 +5898,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>100</v>
       </c>
@@ -5840,7 +5909,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>101</v>
       </c>
@@ -5851,7 +5920,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>102</v>
       </c>
@@ -5862,7 +5931,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>103</v>
       </c>
@@ -5873,7 +5942,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>104</v>
       </c>
@@ -5884,7 +5953,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
         <v>120</v>
       </c>
@@ -5895,7 +5964,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
         <v>121</v>
       </c>
@@ -5906,182 +5975,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
modified game for server
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD9F194-8782-451D-9518-91862A3A7CC4}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BEE6A3-0D8D-43F6-9F53-BC93A3B7AF5E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="2" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,22 +27,17 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planification!$B$5:$E$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="171">
   <si>
     <t>Planification globale</t>
   </si>
@@ -552,6 +547,12 @@
   </si>
   <si>
     <t>Gerer les erreurs dans page index</t>
+  </si>
+  <si>
+    <t>À tester avec le jeu, mais devrait marcher</t>
+  </si>
+  <si>
+    <t>Connection avec une session_key unique</t>
   </si>
 </sst>
 </file>
@@ -1508,26 +1509,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="5" spans="2:5" ht="46.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="21" t="s">
         <v>152</v>
       </c>
@@ -1555,7 +1556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="18" t="s">
         <v>122</v>
       </c>
@@ -1569,7 +1570,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="18" t="s">
         <v>123</v>
       </c>
@@ -1583,7 +1584,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="18" t="s">
         <v>124</v>
       </c>
@@ -1597,7 +1598,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="18" t="s">
         <v>125</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="18" t="s">
         <v>127</v>
       </c>
@@ -1625,7 +1626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="18" t="s">
         <v>128</v>
       </c>
@@ -1639,7 +1640,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="18" t="s">
         <v>129</v>
       </c>
@@ -1653,7 +1654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="18" t="s">
         <v>156</v>
       </c>
@@ -1667,7 +1668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="18" t="s">
         <v>132</v>
       </c>
@@ -1681,7 +1682,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="18" t="s">
         <v>133</v>
       </c>
@@ -1695,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="18" t="s">
         <v>135</v>
       </c>
@@ -1709,7 +1710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="18" t="s">
         <v>141</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="18" t="s">
         <v>130</v>
       </c>
@@ -1737,7 +1738,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="18" t="s">
         <v>131</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="18" t="s">
         <v>136</v>
       </c>
@@ -1765,7 +1766,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="18" t="s">
         <v>137</v>
       </c>
@@ -1779,7 +1780,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="18" t="s">
         <v>138</v>
       </c>
@@ -1793,7 +1794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="18" t="s">
         <v>140</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="18" t="s">
         <v>144</v>
       </c>
@@ -1821,7 +1822,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="18" t="s">
         <v>145</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="18" t="s">
         <v>146</v>
       </c>
@@ -1849,7 +1850,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="18" t="s">
         <v>139</v>
       </c>
@@ -1863,7 +1864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="18" t="s">
         <v>142</v>
       </c>
@@ -1877,7 +1878,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="18" t="s">
         <v>134</v>
       </c>
@@ -1891,7 +1892,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="18" t="s">
         <v>143</v>
       </c>
@@ -1905,7 +1906,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="18" t="s">
         <v>147</v>
       </c>
@@ -1919,7 +1920,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="18" t="s">
         <v>148</v>
       </c>
@@ -1933,7 +1934,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="18" t="s">
         <v>149</v>
       </c>
@@ -1947,7 +1948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="18" t="s">
         <v>150</v>
       </c>
@@ -1961,7 +1962,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="18" t="s">
         <v>151</v>
       </c>
@@ -1975,7 +1976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="22" t="s">
         <v>126</v>
       </c>
@@ -1989,8 +1990,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="41" t="s">
         <v>157</v>
       </c>
@@ -2019,32 +2020,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2074,7 +2075,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2128,7 +2129,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="23" t="s">
         <v>97</v>
       </c>
@@ -2155,7 +2156,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="26" t="s">
         <v>96</v>
       </c>
@@ -2177,7 +2178,7 @@
       <c r="P6" s="31"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="26" t="s">
         <v>98</v>
       </c>
@@ -2204,7 +2205,7 @@
       <c r="P7" s="31"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="26" t="s">
         <v>104</v>
       </c>
@@ -2237,7 +2238,7 @@
       <c r="P8" s="31"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="26" t="s">
         <v>99</v>
       </c>
@@ -2274,7 +2275,7 @@
       </c>
       <c r="R9" s="28"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="26" t="s">
         <v>103</v>
       </c>
@@ -2311,7 +2312,7 @@
       </c>
       <c r="R10" s="28"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="26" t="s">
         <v>101</v>
       </c>
@@ -2343,7 +2344,7 @@
       </c>
       <c r="R11" s="28"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="26" t="s">
         <v>102</v>
       </c>
@@ -2371,7 +2372,7 @@
       <c r="P12" s="31"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="47" t="s">
         <v>100</v>
       </c>
@@ -2398,15 +2399,15 @@
       <c r="Q13" s="46"/>
       <c r="R13" s="17"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="20"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="20"/>
       <c r="P25" s="20"/>
       <c r="S25" s="20"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="20"/>
       <c r="P26" s="20"/>
       <c r="S26" s="20"/>
@@ -2422,24 +2423,24 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
-    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="56.21875" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
-    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.77734375" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="56.1796875" customWidth="1"/>
+    <col min="10" max="10" width="16.6328125" customWidth="1"/>
+    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B3" s="62" t="s">
         <v>6</v>
       </c>
@@ -2454,8 +2455,8 @@
       <c r="K3" s="63"/>
       <c r="L3" s="64"/>
     </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B5" s="65" t="s">
         <v>1</v>
       </c>
@@ -2490,7 +2491,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="66"/>
       <c r="C6" s="68"/>
       <c r="D6" s="57" t="s">
@@ -2515,7 +2516,7 @@
       </c>
       <c r="L6" s="70"/>
     </row>
-    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
         <v>24</v>
       </c>
@@ -2538,7 +2539,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="36" t="s">
         <v>35</v>
       </c>
@@ -2557,7 +2558,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
@@ -2576,7 +2577,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="36" t="s">
         <v>75</v>
       </c>
@@ -2595,7 +2596,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="36" t="s">
         <v>165</v>
       </c>
@@ -2614,7 +2615,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="36" t="s">
         <v>25</v>
       </c>
@@ -2633,7 +2634,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="36" t="s">
         <v>26</v>
       </c>
@@ -2652,7 +2653,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="36" t="s">
         <v>27</v>
       </c>
@@ -2671,7 +2672,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="36" t="s">
         <v>163</v>
       </c>
@@ -2690,7 +2691,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="36" t="s">
         <v>29</v>
       </c>
@@ -2709,7 +2710,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="36" t="s">
         <v>30</v>
       </c>
@@ -2728,7 +2729,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="36" t="s">
         <v>161</v>
       </c>
@@ -2747,7 +2748,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="36" t="s">
         <v>162</v>
       </c>
@@ -2766,7 +2767,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" ht="58" x14ac:dyDescent="0.35">
       <c r="B20" s="61" t="s">
         <v>166</v>
       </c>
@@ -2785,7 +2786,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="36" t="s">
         <v>92</v>
       </c>
@@ -2806,7 +2807,7 @@
       </c>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="36" t="s">
         <v>51</v>
       </c>
@@ -2825,7 +2826,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="36" t="s">
         <v>90</v>
       </c>
@@ -2835,12 +2836,18 @@
       <c r="D23" s="31"/>
       <c r="E23" s="40"/>
       <c r="F23" s="14"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="14"/>
+      <c r="G23" s="31">
+        <v>2</v>
+      </c>
+      <c r="H23" s="40">
+        <v>100</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>169</v>
+      </c>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="36" t="s">
         <v>74</v>
       </c>
@@ -2859,7 +2866,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="36" t="s">
         <v>80</v>
       </c>
@@ -2878,7 +2885,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="36" t="s">
         <v>93</v>
       </c>
@@ -2899,7 +2906,7 @@
       </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="36" t="s">
         <v>94</v>
       </c>
@@ -2909,12 +2916,18 @@
       <c r="D27" s="31"/>
       <c r="E27" s="40"/>
       <c r="F27" s="14"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="14"/>
+      <c r="G27" s="31">
+        <v>1</v>
+      </c>
+      <c r="H27" s="40">
+        <v>100</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>170</v>
+      </c>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B28" s="36" t="s">
         <v>79</v>
       </c>
@@ -2928,14 +2941,14 @@
         <v>0.5</v>
       </c>
       <c r="H28" s="40">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="I28" s="54" t="s">
         <v>160</v>
       </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="18" t="s">
         <v>76</v>
       </c>
@@ -2945,12 +2958,16 @@
       <c r="D29" s="31"/>
       <c r="E29" s="40"/>
       <c r="F29" s="14"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="40"/>
+      <c r="G29" s="31">
+        <v>1</v>
+      </c>
+      <c r="H29" s="40">
+        <v>100</v>
+      </c>
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="36" t="s">
         <v>42</v>
       </c>
@@ -2969,7 +2986,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="36" t="s">
         <v>43</v>
       </c>
@@ -2988,7 +3005,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="36" t="s">
         <v>164</v>
       </c>
@@ -3003,7 +3020,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="36" t="s">
         <v>168</v>
       </c>
@@ -3022,7 +3039,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="36" t="s">
         <v>73</v>
       </c>
@@ -3037,7 +3054,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="36" t="s">
         <v>38</v>
       </c>
@@ -3052,7 +3069,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="36" t="s">
         <v>39</v>
       </c>
@@ -3067,7 +3084,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="36" t="s">
         <v>61</v>
       </c>
@@ -3082,7 +3099,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B38" s="37" t="s">
         <v>56</v>
       </c>
@@ -3136,21 +3153,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="70.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="70.81640625" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" customWidth="1"/>
-    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" customWidth="1"/>
+    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="9" t="s">
         <v>22</v>
       </c>
@@ -3164,151 +3181,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -3324,28 +3341,28 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.77734375" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.81640625" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:12" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="7"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
@@ -3370,7 +3387,7 @@
       </c>
       <c r="L3" s="6"/>
     </row>
-    <row r="4" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B4" s="7" t="s">
         <v>1</v>
       </c>
@@ -3405,7 +3422,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B5" s="50"/>
       <c r="C5" s="12"/>
       <c r="D5" s="21"/>
@@ -3418,7 +3435,7 @@
       <c r="K5" s="11"/>
       <c r="L5" s="12"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="51"/>
       <c r="C6" s="14"/>
       <c r="D6" s="18"/>
@@ -3427,7 +3444,7 @@
       <c r="I6" s="14"/>
       <c r="L6" s="14"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="51"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -3436,7 +3453,7 @@
       <c r="I7" s="14"/>
       <c r="L7" s="14"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="51"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -3445,7 +3462,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="51"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -3454,7 +3471,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="51"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -3463,7 +3480,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="51"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -3472,7 +3489,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="51"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -3481,7 +3498,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="51"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -3490,7 +3507,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="51"/>
       <c r="C14" s="14"/>
       <c r="D14" s="18"/>
@@ -3499,7 +3516,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="51"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -3508,7 +3525,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="51"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -3517,7 +3534,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="51"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -3526,7 +3543,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="51"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -3535,7 +3552,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="51"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -3544,7 +3561,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="51"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -3553,7 +3570,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="51"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -3562,7 +3579,7 @@
       <c r="I21" s="14"/>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="51"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -3571,7 +3588,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="51"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -3580,7 +3597,7 @@
       <c r="I23" s="14"/>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="51"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -3589,7 +3606,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="51"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -3598,7 +3615,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="51"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -3607,7 +3624,7 @@
       <c r="I26" s="14"/>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="51"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -3616,7 +3633,7 @@
       <c r="I27" s="14"/>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="51"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -3625,7 +3642,7 @@
       <c r="I28" s="14"/>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="51"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -3634,7 +3651,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="51"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -3643,7 +3660,7 @@
       <c r="I30" s="14"/>
       <c r="L30" s="14"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="51"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -3652,7 +3669,7 @@
       <c r="I31" s="14"/>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="51"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -3661,7 +3678,7 @@
       <c r="I32" s="14"/>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="51"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -3670,7 +3687,7 @@
       <c r="I33" s="14"/>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="51"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -3679,7 +3696,7 @@
       <c r="I34" s="14"/>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="51"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -3688,7 +3705,7 @@
       <c r="I35" s="14"/>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="51"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -3697,7 +3714,7 @@
       <c r="I36" s="14"/>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="51"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -3706,7 +3723,7 @@
       <c r="I37" s="14"/>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="51"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -3715,7 +3732,7 @@
       <c r="I38" s="14"/>
       <c r="L38" s="14"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="51"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -3724,7 +3741,7 @@
       <c r="I39" s="14"/>
       <c r="L39" s="14"/>
     </row>
-    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B40" s="52"/>
       <c r="C40" s="17"/>
       <c r="D40" s="22"/>
@@ -3757,18 +3774,18 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B2:O56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -3792,7 +3809,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -3836,7 +3853,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="10" t="s">
         <v>95</v>
       </c>
@@ -3858,7 +3875,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -3876,7 +3893,7 @@
       <c r="M7" s="18"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="13" t="s">
         <v>84</v>
       </c>
@@ -3894,7 +3911,7 @@
       <c r="M8" s="18"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
@@ -3912,7 +3929,7 @@
       <c r="M9" s="18"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="13" t="s">
         <v>83</v>
       </c>
@@ -3930,7 +3947,7 @@
       <c r="M10" s="18"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="13" t="s">
         <v>62</v>
       </c>
@@ -3948,7 +3965,7 @@
       <c r="M11" s="18"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
@@ -3966,7 +3983,7 @@
       <c r="M12" s="18"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="13" t="s">
         <v>86</v>
       </c>
@@ -3984,7 +4001,7 @@
       <c r="M13" s="18"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="13" t="s">
         <v>54</v>
       </c>
@@ -4002,7 +4019,7 @@
       <c r="M14" s="18"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="13" t="s">
         <v>58</v>
       </c>
@@ -4020,7 +4037,7 @@
       <c r="M15" s="18"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="13" t="s">
         <v>59</v>
       </c>
@@ -4038,7 +4055,7 @@
       <c r="M16" s="18"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="13" t="s">
         <v>60</v>
       </c>
@@ -4056,7 +4073,7 @@
       <c r="M17" s="18"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="13" t="s">
         <v>63</v>
       </c>
@@ -4074,7 +4091,7 @@
       <c r="M18" s="18"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="13" t="s">
         <v>46</v>
       </c>
@@ -4092,7 +4109,7 @@
       <c r="M19" s="18"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="13" t="s">
         <v>45</v>
       </c>
@@ -4110,7 +4127,7 @@
       <c r="M20" s="18"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="13" t="s">
         <v>82</v>
       </c>
@@ -4128,7 +4145,7 @@
       <c r="M21" s="18"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
         <v>40</v>
       </c>
@@ -4146,7 +4163,7 @@
       <c r="M22" s="18"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="13" t="s">
         <v>41</v>
       </c>
@@ -4164,7 +4181,7 @@
       <c r="M23" s="18"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="13" t="s">
         <v>57</v>
       </c>
@@ -4182,7 +4199,7 @@
       <c r="M24" s="18"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="13" t="s">
         <v>53</v>
       </c>
@@ -4200,7 +4217,7 @@
       <c r="M25" s="18"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="13" t="s">
         <v>72</v>
       </c>
@@ -4218,7 +4235,7 @@
       <c r="M26" s="18"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
@@ -4236,7 +4253,7 @@
       <c r="M27" s="18"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="13" t="s">
         <v>69</v>
       </c>
@@ -4254,7 +4271,7 @@
       <c r="M28" s="18"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="13" t="s">
         <v>71</v>
       </c>
@@ -4272,7 +4289,7 @@
       <c r="M29" s="18"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="13" t="s">
         <v>67</v>
       </c>
@@ -4290,7 +4307,7 @@
       </c>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="13" t="s">
         <v>65</v>
       </c>
@@ -4308,7 +4325,7 @@
       </c>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="13" t="s">
         <v>66</v>
       </c>
@@ -4326,7 +4343,7 @@
       </c>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="13" t="s">
         <v>114</v>
       </c>
@@ -4344,7 +4361,7 @@
       </c>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="13" t="s">
         <v>88</v>
       </c>
@@ -4362,7 +4379,7 @@
       </c>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="15" t="s">
         <v>70</v>
       </c>
@@ -4384,47 +4401,47 @@
       <c r="N35" s="16"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B47" s="40" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B48" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B49" s="36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B52" s="36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B53" s="36" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B54" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4436,29 +4453,29 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="51.5546875" customWidth="1"/>
-    <col min="3" max="3" width="15.5546875" customWidth="1"/>
-    <col min="4" max="4" width="20.21875" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" customWidth="1"/>
-    <col min="7" max="7" width="20.44140625" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.21875" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.21875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="51.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" customWidth="1"/>
+    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -4490,7 +4507,7 @@
       </c>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -4534,7 +4551,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" s="50"/>
       <c r="C6" s="12"/>
       <c r="D6" s="21"/>
@@ -4550,7 +4567,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="51"/>
       <c r="C7" s="14"/>
       <c r="D7" s="18"/>
@@ -4560,7 +4577,7 @@
       <c r="L7" s="14"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="51"/>
       <c r="C8" s="14"/>
       <c r="D8" s="18"/>
@@ -4570,7 +4587,7 @@
       <c r="L8" s="14"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="51"/>
       <c r="C9" s="14"/>
       <c r="D9" s="18"/>
@@ -4580,7 +4597,7 @@
       <c r="L9" s="14"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="51"/>
       <c r="C10" s="14"/>
       <c r="D10" s="18"/>
@@ -4590,7 +4607,7 @@
       <c r="L10" s="14"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="51"/>
       <c r="C11" s="14"/>
       <c r="D11" s="18"/>
@@ -4600,7 +4617,7 @@
       <c r="L11" s="14"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="51"/>
       <c r="C12" s="14"/>
       <c r="D12" s="18"/>
@@ -4610,7 +4627,7 @@
       <c r="L12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="51"/>
       <c r="C13" s="14"/>
       <c r="D13" s="18"/>
@@ -4620,7 +4637,7 @@
       <c r="L13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="51"/>
       <c r="C14" s="14"/>
       <c r="D14" s="49"/>
@@ -4630,7 +4647,7 @@
       <c r="L14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="51"/>
       <c r="C15" s="14"/>
       <c r="D15" s="18"/>
@@ -4640,7 +4657,7 @@
       <c r="L15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="51"/>
       <c r="C16" s="14"/>
       <c r="D16" s="18"/>
@@ -4650,7 +4667,7 @@
       <c r="L16" s="14"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="51"/>
       <c r="C17" s="14"/>
       <c r="D17" s="18"/>
@@ -4660,7 +4677,7 @@
       <c r="L17" s="14"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="51"/>
       <c r="C18" s="14"/>
       <c r="D18" s="18"/>
@@ -4670,7 +4687,7 @@
       <c r="L18" s="14"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="51"/>
       <c r="C19" s="14"/>
       <c r="D19" s="18"/>
@@ -4680,7 +4697,7 @@
       <c r="L19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="51"/>
       <c r="C20" s="14"/>
       <c r="D20" s="18"/>
@@ -4690,7 +4707,7 @@
       <c r="L20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="51"/>
       <c r="C21" s="14"/>
       <c r="D21" s="18"/>
@@ -4700,7 +4717,7 @@
       <c r="L21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="51"/>
       <c r="C22" s="14"/>
       <c r="D22" s="18"/>
@@ -4710,7 +4727,7 @@
       <c r="L22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="51"/>
       <c r="C23" s="14"/>
       <c r="D23" s="18"/>
@@ -4720,7 +4737,7 @@
       <c r="L23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="51"/>
       <c r="C24" s="14"/>
       <c r="D24" s="18"/>
@@ -4730,7 +4747,7 @@
       <c r="L24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="51"/>
       <c r="C25" s="14"/>
       <c r="D25" s="18"/>
@@ -4740,7 +4757,7 @@
       <c r="L25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="51"/>
       <c r="C26" s="14"/>
       <c r="D26" s="18"/>
@@ -4750,7 +4767,7 @@
       <c r="L26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="51"/>
       <c r="C27" s="14"/>
       <c r="D27" s="18"/>
@@ -4760,7 +4777,7 @@
       <c r="L27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="51"/>
       <c r="C28" s="14"/>
       <c r="D28" s="18"/>
@@ -4770,7 +4787,7 @@
       <c r="L28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="51"/>
       <c r="C29" s="14"/>
       <c r="D29" s="18"/>
@@ -4780,7 +4797,7 @@
       <c r="L29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="51"/>
       <c r="C30" s="14"/>
       <c r="D30" s="18"/>
@@ -4790,7 +4807,7 @@
       <c r="L30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="51"/>
       <c r="C31" s="14"/>
       <c r="D31" s="18"/>
@@ -4800,7 +4817,7 @@
       <c r="L31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="51"/>
       <c r="C32" s="14"/>
       <c r="D32" s="18"/>
@@ -4810,7 +4827,7 @@
       <c r="L32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="51"/>
       <c r="C33" s="14"/>
       <c r="D33" s="18"/>
@@ -4820,7 +4837,7 @@
       <c r="L33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="51"/>
       <c r="C34" s="14"/>
       <c r="D34" s="18"/>
@@ -4830,7 +4847,7 @@
       <c r="L34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B35" s="51"/>
       <c r="C35" s="14"/>
       <c r="D35" s="18"/>
@@ -4840,7 +4857,7 @@
       <c r="L35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B36" s="51"/>
       <c r="C36" s="14"/>
       <c r="D36" s="18"/>
@@ -4850,7 +4867,7 @@
       <c r="L36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B37" s="51"/>
       <c r="C37" s="14"/>
       <c r="D37" s="18"/>
@@ -4860,7 +4877,7 @@
       <c r="L37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B38" s="51"/>
       <c r="C38" s="14"/>
       <c r="D38" s="18"/>
@@ -4870,7 +4887,7 @@
       <c r="L38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B39" s="51"/>
       <c r="C39" s="14"/>
       <c r="D39" s="18"/>
@@ -4880,7 +4897,7 @@
       <c r="L39" s="14"/>
       <c r="O39" s="14"/>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B40" s="51"/>
       <c r="C40" s="14"/>
       <c r="D40" s="18"/>
@@ -4890,7 +4907,7 @@
       <c r="L40" s="14"/>
       <c r="O40" s="14"/>
     </row>
-    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B41" s="52"/>
       <c r="C41" s="17"/>
       <c r="D41" s="22"/>
@@ -4906,7 +4923,7 @@
       <c r="N41" s="16"/>
       <c r="O41" s="17"/>
     </row>
-    <row r="64" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D64" s="5"/>
       <c r="G64" s="5"/>
       <c r="H64" t="s">
@@ -4915,7 +4932,7 @@
       <c r="J64" s="5"/>
       <c r="M64" s="5"/>
     </row>
-    <row r="65" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D65" s="5"/>
       <c r="G65" s="5"/>
       <c r="H65" t="s">
@@ -4924,7 +4941,7 @@
       <c r="J65" s="5"/>
       <c r="M65" s="5"/>
     </row>
-    <row r="67" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D67" s="5"/>
       <c r="G67" s="5"/>
       <c r="H67" t="s">
@@ -4933,7 +4950,7 @@
       <c r="J67" s="5"/>
       <c r="M67" s="5"/>
     </row>
-    <row r="68" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D68" s="5"/>
       <c r="G68" s="5"/>
       <c r="J68" s="5"/>
@@ -4942,17 +4959,17 @@
       </c>
       <c r="M68" s="5"/>
     </row>
-    <row r="71" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:13" x14ac:dyDescent="0.35">
       <c r="H71" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:13" x14ac:dyDescent="0.35">
       <c r="K72" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="73" spans="4:13" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:13" x14ac:dyDescent="0.35">
       <c r="D73" s="5"/>
       <c r="G73" s="5"/>
       <c r="J73" s="5"/>
@@ -4980,28 +4997,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
-    <col min="2" max="2" width="93.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1796875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:6" ht="44.75" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -5018,7 +5035,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -5031,7 +5048,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -5044,7 +5061,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -5057,7 +5074,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -5070,7 +5087,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -5083,7 +5100,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -5096,7 +5113,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -5109,7 +5126,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -5122,7 +5139,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5135,7 +5152,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -5148,7 +5165,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -5161,7 +5178,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5174,7 +5191,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -5187,7 +5204,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -5200,7 +5217,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -5213,7 +5230,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -5226,7 +5243,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -5239,7 +5256,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -5252,7 +5269,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -5265,7 +5282,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -5278,7 +5295,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5291,7 +5308,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -5304,7 +5321,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -5317,7 +5334,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -5330,7 +5347,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -5343,7 +5360,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -5356,7 +5373,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -5369,7 +5386,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -5382,7 +5399,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -5395,7 +5412,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -5408,7 +5425,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -5421,7 +5438,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -5434,7 +5451,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -5447,7 +5464,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -5460,7 +5477,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -5473,7 +5490,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -5486,7 +5503,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -5499,7 +5516,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -5512,7 +5529,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -5525,7 +5542,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -5538,7 +5555,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -5551,7 +5568,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -5564,7 +5581,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -5577,7 +5594,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -5590,7 +5607,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -5603,7 +5620,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -5616,7 +5633,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -5629,7 +5646,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -5642,7 +5659,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -5655,7 +5672,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -5668,7 +5685,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -5681,7 +5698,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -5694,7 +5711,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -5707,7 +5724,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -5720,7 +5737,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -5733,7 +5750,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -5746,7 +5763,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -5759,7 +5776,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -5772,7 +5789,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -5785,7 +5802,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>96</v>
       </c>
@@ -5796,7 +5813,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>97</v>
       </c>
@@ -5807,7 +5824,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>98</v>
       </c>
@@ -5818,7 +5835,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>99</v>
       </c>
@@ -5829,7 +5846,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>100</v>
       </c>
@@ -5840,7 +5857,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>101</v>
       </c>
@@ -5851,7 +5868,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>102</v>
       </c>
@@ -5862,7 +5879,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>103</v>
       </c>
@@ -5873,7 +5890,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>104</v>
       </c>
@@ -5884,7 +5901,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
         <v>120</v>
       </c>
@@ -5895,7 +5912,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
         <v>121</v>
       </c>
@@ -5906,182 +5923,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Changer aspect pieces du pool avec svg
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA97923-ADCA-40DF-898B-D1D1361BED22}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C656DC3A-7DC7-42ED-992D-71563A94710B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="206">
   <si>
     <t>Planification globale</t>
   </si>
@@ -650,6 +650,12 @@
   </si>
   <si>
     <t>Créer la classe Piece/BeliefPiece</t>
+  </si>
+  <si>
+    <t>Centrage + scale des svg</t>
+  </si>
+  <si>
+    <t>Changer aspect des pieces du pool</t>
   </si>
 </sst>
 </file>
@@ -1213,6 +1219,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1246,48 +1256,11 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="68">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="56">
     <dxf>
       <fill>
         <patternFill>
@@ -1416,79 +1389,8 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -2620,7 +2522,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="67" priority="1">
+    <cfRule type="expression" dxfId="55" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3064,26 +2966,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="86"/>
-      <c r="D3" s="86"/>
-      <c r="E3" s="86"/>
-      <c r="F3" s="86"/>
-      <c r="G3" s="86"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
-      <c r="K3" s="86"/>
-      <c r="L3" s="87"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
+      <c r="K3" s="88"/>
+      <c r="L3" s="89"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="88" t="s">
+      <c r="B5" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="90" t="s">
+      <c r="C5" s="92" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="52" t="s">
@@ -3092,7 +2994,7 @@
       <c r="E5" s="53">
         <v>46083</v>
       </c>
-      <c r="F5" s="92" t="s">
+      <c r="F5" s="94" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="55" t="s">
@@ -3101,7 +3003,7 @@
       <c r="H5" s="53">
         <v>46090</v>
       </c>
-      <c r="I5" s="92" t="s">
+      <c r="I5" s="94" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="55" t="s">
@@ -3110,34 +3012,34 @@
       <c r="K5" s="53">
         <v>46104</v>
       </c>
-      <c r="L5" s="92" t="s">
+      <c r="L5" s="94" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="89"/>
-      <c r="C6" s="91"/>
+      <c r="B6" s="91"/>
+      <c r="C6" s="93"/>
       <c r="D6" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="93"/>
+      <c r="F6" s="95"/>
       <c r="G6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="93"/>
+      <c r="I6" s="95"/>
       <c r="J6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="93"/>
+      <c r="L6" s="95"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="35" t="s">
@@ -3963,81 +3865,81 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B45 B47:B1048576 B1:B42">
-    <cfRule type="expression" dxfId="66" priority="28">
+    <cfRule type="expression" dxfId="54" priority="28">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49:C1048576 C1:C45">
-    <cfRule type="expression" dxfId="65" priority="23">
+    <cfRule type="expression" dxfId="53" priority="23">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="25">
+    <cfRule type="expression" dxfId="52" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="27">
+    <cfRule type="expression" dxfId="51" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="62" priority="19">
+    <cfRule type="expression" dxfId="50" priority="19">
       <formula>$C47="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="20">
+    <cfRule type="expression" dxfId="49" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="21">
+    <cfRule type="expression" dxfId="48" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="59" priority="8">
+    <cfRule type="expression" dxfId="47" priority="8">
       <formula>$C48="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="9">
+    <cfRule type="expression" dxfId="46" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="10">
+    <cfRule type="expression" dxfId="45" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C48">
-    <cfRule type="expression" dxfId="56" priority="12">
+    <cfRule type="expression" dxfId="44" priority="12">
       <formula>$C42="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="13">
+    <cfRule type="expression" dxfId="43" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="14">
+    <cfRule type="expression" dxfId="42" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:B48 B45 B31:B42">
-    <cfRule type="expression" dxfId="53" priority="30">
+    <cfRule type="expression" dxfId="41" priority="30">
       <formula>MAX($E31,$K31,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="expression" dxfId="52" priority="7">
+    <cfRule type="expression" dxfId="40" priority="7">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="51" priority="32">
+    <cfRule type="expression" dxfId="39" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="50" priority="38">
+    <cfRule type="expression" dxfId="38" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="expression" dxfId="49" priority="6">
+    <cfRule type="expression" dxfId="37" priority="6">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="expression" dxfId="48" priority="1">
+    <cfRule type="expression" dxfId="36" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4051,7 +3953,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="B1:M60"/>
+  <dimension ref="B1:M62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
@@ -4069,26 +3971,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="87" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="86"/>
-      <c r="J1" s="86"/>
-      <c r="K1" s="86"/>
-      <c r="L1" s="87"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
+      <c r="K1" s="88"/>
+      <c r="L1" s="89"/>
     </row>
     <row r="3" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="2:13" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="90" t="s">
+      <c r="C4" s="92" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="52" t="s">
@@ -4097,7 +3999,7 @@
       <c r="E4" s="53">
         <v>46111</v>
       </c>
-      <c r="F4" s="92" t="s">
+      <c r="F4" s="94" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="55" t="s">
@@ -4106,7 +4008,7 @@
       <c r="H4" s="53">
         <v>46125</v>
       </c>
-      <c r="I4" s="92" t="s">
+      <c r="I4" s="94" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="55" t="s">
@@ -4115,34 +4017,34 @@
       <c r="K4" s="53">
         <v>46132</v>
       </c>
-      <c r="L4" s="92" t="s">
+      <c r="L4" s="94" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="89"/>
-      <c r="C5" s="91"/>
+      <c r="B5" s="91"/>
+      <c r="C5" s="93"/>
       <c r="D5" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="93"/>
+      <c r="F5" s="95"/>
       <c r="G5" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="93"/>
+      <c r="I5" s="95"/>
       <c r="J5" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="93"/>
+      <c r="L5" s="95"/>
     </row>
     <row r="6" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B6" s="82" t="s">
@@ -4366,23 +4268,31 @@
       <c r="C17" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="D17" s="81"/>
-      <c r="E17" s="83"/>
+      <c r="D17" s="81">
+        <v>2</v>
+      </c>
+      <c r="E17" s="83">
+        <v>100</v>
+      </c>
       <c r="F17" s="80"/>
       <c r="G17" s="81"/>
       <c r="H17" s="83"/>
       <c r="I17" s="80"/>
       <c r="L17" s="80"/>
     </row>
-    <row r="18" spans="2:13" s="79" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="B18" s="84" t="s">
-        <v>191</v>
+    <row r="18" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="82" t="s">
+        <v>204</v>
       </c>
       <c r="C18" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="D18" s="81"/>
-      <c r="E18" s="83"/>
+      <c r="D18" s="81">
+        <v>1</v>
+      </c>
+      <c r="E18" s="83">
+        <v>100</v>
+      </c>
       <c r="F18" s="80"/>
       <c r="G18" s="81"/>
       <c r="H18" s="83"/>
@@ -4391,22 +4301,26 @@
     </row>
     <row r="19" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B19" s="82" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="C19" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="81"/>
-      <c r="E19" s="83"/>
+      <c r="D19" s="81">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="83">
+        <v>100</v>
+      </c>
       <c r="F19" s="80"/>
       <c r="G19" s="81"/>
       <c r="H19" s="83"/>
       <c r="I19" s="80"/>
       <c r="L19" s="80"/>
     </row>
-    <row r="20" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="82" t="s">
-        <v>192</v>
+    <row r="20" spans="2:13" s="79" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="B20" s="84" t="s">
+        <v>191</v>
       </c>
       <c r="C20" s="82" t="s">
         <v>106</v>
@@ -4421,7 +4335,7 @@
     </row>
     <row r="21" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B21" s="82" t="s">
-        <v>54</v>
+        <v>193</v>
       </c>
       <c r="C21" s="82" t="s">
         <v>106</v>
@@ -4436,7 +4350,7 @@
     </row>
     <row r="22" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B22" s="82" t="s">
-        <v>72</v>
+        <v>192</v>
       </c>
       <c r="C22" s="82" t="s">
         <v>106</v>
@@ -4449,9 +4363,9 @@
       <c r="I22" s="80"/>
       <c r="L22" s="80"/>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B23" s="82" t="s">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="C23" s="82" t="s">
         <v>106</v>
@@ -4462,14 +4376,11 @@
       <c r="G23" s="81"/>
       <c r="H23" s="83"/>
       <c r="I23" s="80"/>
-      <c r="J23" s="79"/>
-      <c r="K23" s="79"/>
       <c r="L23" s="80"/>
-      <c r="M23" s="79"/>
     </row>
     <row r="24" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B24" s="82" t="s">
-        <v>194</v>
+        <v>72</v>
       </c>
       <c r="C24" s="82" t="s">
         <v>106</v>
@@ -4484,7 +4395,7 @@
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" s="82" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="C25" s="82" t="s">
         <v>106</v>
@@ -4500,9 +4411,9 @@
       <c r="L25" s="80"/>
       <c r="M25" s="79"/>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B26" s="82" t="s">
-        <v>46</v>
+        <v>194</v>
       </c>
       <c r="C26" s="82" t="s">
         <v>106</v>
@@ -4513,14 +4424,11 @@
       <c r="G26" s="81"/>
       <c r="H26" s="83"/>
       <c r="I26" s="80"/>
-      <c r="J26" s="79"/>
-      <c r="K26" s="79"/>
       <c r="L26" s="80"/>
-      <c r="M26" s="79"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B27" s="82" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C27" s="82" t="s">
         <v>106</v>
@@ -4538,7 +4446,7 @@
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B28" s="82" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C28" s="82" t="s">
         <v>106</v>
@@ -4556,7 +4464,7 @@
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B29" s="82" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C29" s="82" t="s">
         <v>106</v>
@@ -4574,7 +4482,7 @@
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B30" s="82" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="C30" s="82" t="s">
         <v>106</v>
@@ -4592,7 +4500,7 @@
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B31" s="82" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="C31" s="82" t="s">
         <v>106</v>
@@ -4610,7 +4518,7 @@
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B32" s="82" t="s">
-        <v>114</v>
+        <v>57</v>
       </c>
       <c r="C32" s="82" t="s">
         <v>106</v>
@@ -4628,7 +4536,7 @@
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B33" s="82" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="82" t="s">
         <v>106</v>
@@ -4646,7 +4554,7 @@
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B34" s="82" t="s">
-        <v>56</v>
+        <v>114</v>
       </c>
       <c r="C34" s="82" t="s">
         <v>106</v>
@@ -4664,7 +4572,7 @@
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B35" s="82" t="s">
-        <v>198</v>
+        <v>70</v>
       </c>
       <c r="C35" s="82" t="s">
         <v>106</v>
@@ -4681,18 +4589,14 @@
       <c r="M35" s="79"/>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B36" s="74" t="s">
-        <v>203</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D36" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="E36" s="83">
-        <v>100</v>
-      </c>
+      <c r="B36" s="82" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="81"/>
+      <c r="E36" s="83"/>
       <c r="F36" s="80"/>
       <c r="G36" s="81"/>
       <c r="H36" s="83"/>
@@ -4703,18 +4607,14 @@
       <c r="M36" s="79"/>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B37" s="74" t="s">
-        <v>85</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D37" s="81">
-        <v>1</v>
-      </c>
-      <c r="E37" s="83">
-        <v>100</v>
-      </c>
+      <c r="B37" s="82" t="s">
+        <v>198</v>
+      </c>
+      <c r="C37" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="81"/>
+      <c r="E37" s="83"/>
       <c r="F37" s="80"/>
       <c r="G37" s="81"/>
       <c r="H37" s="83"/>
@@ -4726,7 +4626,7 @@
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B38" s="74" t="s">
-        <v>83</v>
+        <v>203</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>107</v>
@@ -4748,13 +4648,13 @@
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B39" s="74" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>107</v>
       </c>
       <c r="D39" s="81">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E39" s="83">
         <v>100</v>
@@ -4768,9 +4668,9 @@
       <c r="L39" s="80"/>
       <c r="M39" s="79"/>
     </row>
-    <row r="40" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B40" s="74" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>107</v>
@@ -4785,17 +4685,24 @@
       <c r="G40" s="81"/>
       <c r="H40" s="83"/>
       <c r="I40" s="80"/>
+      <c r="J40" s="79"/>
+      <c r="K40" s="79"/>
       <c r="L40" s="80"/>
+      <c r="M40" s="79"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B41" s="96" t="s">
-        <v>201</v>
+      <c r="B41" s="74" t="s">
+        <v>62</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D41" s="81"/>
-      <c r="E41" s="83"/>
+      <c r="D41" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="E41" s="83">
+        <v>100</v>
+      </c>
       <c r="F41" s="80"/>
       <c r="G41" s="81"/>
       <c r="H41" s="83"/>
@@ -4805,9 +4712,9 @@
       <c r="L41" s="80"/>
       <c r="M41" s="79"/>
     </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B42" s="74" t="s">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>107</v>
@@ -4822,24 +4729,17 @@
       <c r="G42" s="81"/>
       <c r="H42" s="83"/>
       <c r="I42" s="80"/>
-      <c r="J42" s="79"/>
-      <c r="K42" s="79"/>
       <c r="L42" s="80"/>
-      <c r="M42" s="79"/>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B43" s="74" t="s">
-        <v>59</v>
+      <c r="B43" s="85" t="s">
+        <v>201</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D43" s="81">
-        <v>0.75</v>
-      </c>
-      <c r="E43" s="83">
-        <v>100</v>
-      </c>
+      <c r="D43" s="81"/>
+      <c r="E43" s="83"/>
       <c r="F43" s="80"/>
       <c r="G43" s="81"/>
       <c r="H43" s="83"/>
@@ -4847,10 +4747,11 @@
       <c r="J43" s="79"/>
       <c r="K43" s="79"/>
       <c r="L43" s="80"/>
+      <c r="M43" s="79"/>
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B44" s="74" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>107</v>
@@ -4868,118 +4769,161 @@
       <c r="J44" s="79"/>
       <c r="K44" s="79"/>
       <c r="L44" s="80"/>
+      <c r="M44" s="79"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B45" s="74" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D45" s="97">
-        <v>1</v>
+      <c r="D45" s="81">
+        <v>0.75</v>
       </c>
       <c r="E45" s="83">
         <v>100</v>
       </c>
+      <c r="F45" s="80"/>
+      <c r="G45" s="81"/>
+      <c r="H45" s="83"/>
+      <c r="I45" s="80"/>
+      <c r="J45" s="79"/>
+      <c r="K45" s="79"/>
+      <c r="L45" s="80"/>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B46" s="74" t="s">
-        <v>202</v>
+        <v>60</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D46" s="97">
-        <v>0.25</v>
+      <c r="D46" s="81">
+        <v>0.5</v>
       </c>
       <c r="E46" s="83">
         <v>100</v>
       </c>
-    </row>
-    <row r="47" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F46" s="80"/>
+      <c r="G46" s="81"/>
+      <c r="H46" s="83"/>
+      <c r="I46" s="80"/>
+      <c r="J46" s="79"/>
+      <c r="K46" s="79"/>
+      <c r="L46" s="80"/>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B47" s="74" t="s">
-        <v>200</v>
+        <v>57</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D47" s="97"/>
+      <c r="D47" s="86">
+        <v>1</v>
+      </c>
+      <c r="E47" s="83">
+        <v>100</v>
+      </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B48" s="74" t="s">
-        <v>65</v>
+        <v>202</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="97"/>
-    </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="D48" s="86">
+        <v>0.25</v>
+      </c>
+      <c r="E48" s="83">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" s="79" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B49" s="74" t="s">
-        <v>66</v>
+        <v>200</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D49" s="97"/>
+      <c r="D49" s="86"/>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B50" s="74" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D50" s="97"/>
+      <c r="D50" s="86"/>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B51" s="74"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="97"/>
+      <c r="B51" s="74" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D51" s="86"/>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B52" s="74"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="97"/>
+      <c r="B52" s="74" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D52" s="86"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B53" s="74"/>
       <c r="C53" s="8"/>
-      <c r="D53" s="97"/>
+      <c r="D53" s="86"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B54" s="74"/>
       <c r="C54" s="8"/>
-      <c r="D54" s="97"/>
+      <c r="D54" s="86"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B55" s="74"/>
       <c r="C55" s="8"/>
-      <c r="D55" s="97"/>
+      <c r="D55" s="86"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B56" s="74"/>
       <c r="C56" s="8"/>
-      <c r="D56" s="97"/>
+      <c r="D56" s="86"/>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B57" s="74"/>
       <c r="C57" s="8"/>
-      <c r="D57" s="97"/>
+      <c r="D57" s="86"/>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B58" s="74"/>
       <c r="C58" s="8"/>
-      <c r="D58" s="97"/>
+      <c r="D58" s="86"/>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B59" s="74"/>
-      <c r="D59" s="97"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="86"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B60" s="74"/>
-      <c r="D60" s="97"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="86"/>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B61" s="74"/>
+      <c r="D61" s="86"/>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B62" s="74"/>
+      <c r="D62" s="86"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:L5" xr:uid="{2EE69061-1192-400C-B500-1B4897FD0585}"/>
@@ -4992,108 +4936,108 @@
     <mergeCell ref="L4:L5"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="B4:B18 B25:B39 B41:B44">
-    <cfRule type="expression" dxfId="47" priority="47">
+  <conditionalFormatting sqref="B27:B41 B43:B46 B4:B20">
+    <cfRule type="expression" dxfId="35" priority="47">
       <formula>MAX($E4,$H4,$K4)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C5 C9:C44">
-    <cfRule type="expression" dxfId="46" priority="44">
+  <conditionalFormatting sqref="C4:C5 C9:C46">
+    <cfRule type="expression" dxfId="34" priority="44">
       <formula>$C4="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="45">
+    <cfRule type="expression" dxfId="33" priority="45">
       <formula>$C4="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="46">
+    <cfRule type="expression" dxfId="32" priority="46">
       <formula>$C4="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
-    <cfRule type="expression" dxfId="43" priority="43">
+    <cfRule type="expression" dxfId="31" priority="43">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="expression" dxfId="42" priority="40">
+    <cfRule type="expression" dxfId="30" priority="40">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="41">
+    <cfRule type="expression" dxfId="29" priority="41">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="42">
+    <cfRule type="expression" dxfId="28" priority="42">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="39" priority="36">
+    <cfRule type="expression" dxfId="27" priority="36">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="expression" dxfId="38" priority="30">
+    <cfRule type="expression" dxfId="26" priority="30">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="37" priority="29">
+    <cfRule type="expression" dxfId="25" priority="29">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="36" priority="28">
+    <cfRule type="expression" dxfId="24" priority="28">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
-    <cfRule type="expression" dxfId="35" priority="83">
+  <conditionalFormatting sqref="B36">
+    <cfRule type="expression" dxfId="23" priority="83">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B12">
-    <cfRule type="expression" dxfId="34" priority="25">
+    <cfRule type="expression" dxfId="22" priority="25">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C8">
-    <cfRule type="expression" dxfId="33" priority="22">
+    <cfRule type="expression" dxfId="21" priority="22">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="23">
+    <cfRule type="expression" dxfId="20" priority="23">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="24">
+    <cfRule type="expression" dxfId="19" priority="24">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B19:B24">
-    <cfRule type="expression" dxfId="30" priority="21">
-      <formula>MAX($E19,$H19,$K19)=100</formula>
+  <conditionalFormatting sqref="B21:B26">
+    <cfRule type="expression" dxfId="18" priority="21">
+      <formula>MAX($E21,$H21,$K21)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B19:B24">
-    <cfRule type="expression" dxfId="29" priority="20">
-      <formula>MAX($E19,$H19,$K19)=100</formula>
+  <conditionalFormatting sqref="B21:B26">
+    <cfRule type="expression" dxfId="17" priority="20">
+      <formula>MAX($E21,$H21,$K21)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B40">
-    <cfRule type="expression" dxfId="28" priority="85">
-      <formula>MAX($E41,$H41,$K41)=100</formula>
+  <conditionalFormatting sqref="B42">
+    <cfRule type="expression" dxfId="16" priority="85">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45:B60">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>MAX($E45,$H45,$K45)=100</formula>
+  <conditionalFormatting sqref="B47:B62">
+    <cfRule type="expression" dxfId="15" priority="4">
+      <formula>MAX($E47,$H47,$K47)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C45:C58">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>$C45="Charlotte/Eddy"</formula>
+  <conditionalFormatting sqref="C47:C60">
+    <cfRule type="expression" dxfId="14" priority="1">
+      <formula>$C47="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$C45="Charlotte"</formula>
+    <cfRule type="expression" dxfId="13" priority="2">
+      <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>$C45="Eddy"</formula>
+    <cfRule type="expression" dxfId="12" priority="3">
+      <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5992,29 +5936,29 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="94" t="s">
+      <c r="B2" s="96" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
     </row>
     <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="88" t="s">
+      <c r="B5" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="90" t="s">
+      <c r="C5" s="92" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="52" t="s">
@@ -6023,7 +5967,7 @@
       <c r="E5" s="53">
         <v>46139</v>
       </c>
-      <c r="F5" s="92" t="s">
+      <c r="F5" s="94" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="55" t="s">
@@ -6032,7 +5976,7 @@
       <c r="H5" s="53">
         <v>46146</v>
       </c>
-      <c r="I5" s="92" t="s">
+      <c r="I5" s="94" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="55" t="s">
@@ -6041,7 +5985,7 @@
       <c r="K5" s="53">
         <v>46153</v>
       </c>
-      <c r="L5" s="92" t="s">
+      <c r="L5" s="94" t="s">
         <v>12</v>
       </c>
       <c r="M5" s="55" t="s">
@@ -6050,41 +5994,41 @@
       <c r="N5" s="53">
         <v>46161</v>
       </c>
-      <c r="O5" s="92" t="s">
+      <c r="O5" s="94" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="89"/>
-      <c r="C6" s="91"/>
+      <c r="B6" s="91"/>
+      <c r="C6" s="93"/>
       <c r="D6" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="93"/>
+      <c r="F6" s="95"/>
       <c r="G6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="93"/>
+      <c r="I6" s="95"/>
       <c r="J6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="93"/>
+      <c r="L6" s="95"/>
       <c r="M6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="N6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="O6" s="93"/>
+      <c r="O6" s="95"/>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="35"/>
@@ -6501,39 +6445,39 @@
     <mergeCell ref="O5:O6"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:B36">
-    <cfRule type="expression" dxfId="12" priority="12">
+    <cfRule type="expression" dxfId="8" priority="12">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C36">
-    <cfRule type="expression" dxfId="11" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>$C5="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="10">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>$C5="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="11">
+    <cfRule type="expression" dxfId="5" priority="11">
       <formula>$C5="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2">
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C37:C39">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$C37="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$C37="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$C37="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37:B39">
-    <cfRule type="expression" dxfId="4" priority="4">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Ajout end.jsx :ecran victoire ou defaite + bouton retour au lobby
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C656DC3A-7DC7-42ED-992D-71563A94710B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D705F6C-2928-4869-872A-EF1631713E7F}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -28,17 +28,22 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="219">
   <si>
     <t>Planification globale</t>
   </si>
@@ -613,18 +618,6 @@
     <t>Création d un component piece</t>
   </si>
   <si>
-    <t>Mise à jour  aspect game,jsx en fonction  du getGameStatus( ) : afficher le board avec les pieces des 2 joueurs et du tour de jeu</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Afficher le tour de jeu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Créer le composant PlayerInfo  pour afficher les informations des joueurs (noms, avatars, scores,tour)  </t>
-  </si>
-  <si>
-    <t>Implémentation de la logique  ecran combat des pieces</t>
-  </si>
-  <si>
     <t>Régler l affichage du board selon la phase de jeu suite a mise en place des phases de jeu</t>
   </si>
   <si>
@@ -634,9 +627,6 @@
     <t>Créer une page administration:gestion des utilisateurs</t>
   </si>
   <si>
-    <t>Permettre le drag and drop sur les pieces</t>
-  </si>
-  <si>
     <t>Importation des svg en tant que Composant pour les pieces</t>
   </si>
   <si>
@@ -655,7 +645,61 @@
     <t>Centrage + scale des svg</t>
   </si>
   <si>
-    <t>Changer aspect des pieces du pool</t>
+    <t>Changer aspect des pieces du pool avec des components svg</t>
+  </si>
+  <si>
+    <t>Ajout component Timer non full complete</t>
+  </si>
+  <si>
+    <t>Ajout fonction transformation tableau api vers matrice React pour le Board</t>
+  </si>
+  <si>
+    <t>Modifier makeBoard pour recevoir x,y,rank,player</t>
+  </si>
+  <si>
+    <t>Ajout fonctions de drag drop dans usePlacement.js</t>
+  </si>
+  <si>
+    <t>Ajout drag drop dans useCellClick.js</t>
+  </si>
+  <si>
+    <t>Ajout drag drop dans cell.jsx</t>
+  </si>
+  <si>
+    <t>AJout Drag drop dans game.jsx</t>
+  </si>
+  <si>
+    <t>Ajout pieceCard + debut battle screen</t>
+  </si>
+  <si>
+    <t>Modifier timer avec un timer local pour l affichage et compenser la latence reseau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise a jour affichage suite à combat: ajout  battle.jsx </t>
+  </si>
+  <si>
+    <t>Mise a jour board suite a un deplacement</t>
+  </si>
+  <si>
+    <t>Ajout component TurnIndicator pour signifier le tour</t>
+  </si>
+  <si>
+    <t>Ajout du Timer depuis api  (Compte à rebourd)</t>
+  </si>
+  <si>
+    <t>Afficher le tour de jeu message a u centre de l écran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajouter  end.jsx victoire ou defaite avec bouton recommencer </t>
+  </si>
+  <si>
+    <t>Ajouter le score de chaque joueur</t>
+  </si>
+  <si>
+    <t>Refactoriser game.jsx( redecouapge en differents components)</t>
+  </si>
+  <si>
+    <t>Implémentation du Factory Pattern pour les aspects des pièces(couleur + divers apects,,)</t>
   </si>
 </sst>
 </file>
@@ -1087,7 +1131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1216,9 +1260,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1260,7 +1301,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="56">
+  <dxfs count="51">
     <dxf>
       <fill>
         <patternFill>
@@ -1358,46 +1399,6 @@
             <color rgb="FFCCFFFF"/>
           </stop>
         </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -2028,26 +2029,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" customWidth="1"/>
-    <col min="5" max="5" width="42.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.75" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:5" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2061,7 +2062,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="58" t="s">
         <v>152</v>
       </c>
@@ -2075,7 +2076,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="62" t="s">
         <v>122</v>
       </c>
@@ -2089,7 +2090,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="63" t="s">
         <v>123</v>
       </c>
@@ -2103,7 +2104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="63" t="s">
         <v>124</v>
       </c>
@@ -2117,7 +2118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="63" t="s">
         <v>125</v>
       </c>
@@ -2131,7 +2132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="63" t="s">
         <v>127</v>
       </c>
@@ -2145,7 +2146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="63" t="s">
         <v>128</v>
       </c>
@@ -2159,7 +2160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="63" t="s">
         <v>129</v>
       </c>
@@ -2173,7 +2174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="63" t="s">
         <v>156</v>
       </c>
@@ -2187,7 +2188,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="63" t="s">
         <v>132</v>
       </c>
@@ -2201,7 +2202,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="63" t="s">
         <v>133</v>
       </c>
@@ -2215,7 +2216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="63" t="s">
         <v>135</v>
       </c>
@@ -2229,7 +2230,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="63" t="s">
         <v>141</v>
       </c>
@@ -2243,7 +2244,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="59" t="s">
         <v>130</v>
       </c>
@@ -2257,7 +2258,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="59" t="s">
         <v>131</v>
       </c>
@@ -2271,7 +2272,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="59" t="s">
         <v>136</v>
       </c>
@@ -2285,7 +2286,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="59" t="s">
         <v>137</v>
       </c>
@@ -2299,7 +2300,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="59" t="s">
         <v>138</v>
       </c>
@@ -2313,7 +2314,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="59" t="s">
         <v>140</v>
       </c>
@@ -2327,7 +2328,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="59" t="s">
         <v>144</v>
       </c>
@@ -2341,7 +2342,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="59" t="s">
         <v>145</v>
       </c>
@@ -2355,7 +2356,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="59" t="s">
         <v>146</v>
       </c>
@@ -2369,7 +2370,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="64" t="s">
         <v>139</v>
       </c>
@@ -2383,7 +2384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="64" t="s">
         <v>142</v>
       </c>
@@ -2397,7 +2398,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="64" t="s">
         <v>134</v>
       </c>
@@ -2411,7 +2412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="64" t="s">
         <v>143</v>
       </c>
@@ -2425,7 +2426,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="64" t="s">
         <v>147</v>
       </c>
@@ -2439,7 +2440,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="64" t="s">
         <v>148</v>
       </c>
@@ -2453,7 +2454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="64" t="s">
         <v>149</v>
       </c>
@@ -2467,7 +2468,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="64" t="s">
         <v>150</v>
       </c>
@@ -2481,7 +2482,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="64" t="s">
         <v>151</v>
       </c>
@@ -2495,7 +2496,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="66" t="s">
         <v>126</v>
       </c>
@@ -2509,8 +2510,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="41" t="s">
         <v>157</v>
       </c>
@@ -2522,7 +2523,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="55" priority="1">
+    <cfRule type="expression" dxfId="50" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2545,32 +2546,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" customWidth="1"/>
-    <col min="6" max="6" width="18.81640625" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" customWidth="1"/>
-    <col min="8" max="8" width="16.08984375" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
-    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2600,7 +2601,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2654,7 +2655,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="23" t="s">
         <v>97</v>
       </c>
@@ -2681,7 +2682,7 @@
       <c r="Q5" s="11"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="26" t="s">
         <v>96</v>
       </c>
@@ -2703,7 +2704,7 @@
       <c r="P6" s="31"/>
       <c r="R6" s="14"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="26" t="s">
         <v>98</v>
       </c>
@@ -2730,7 +2731,7 @@
       <c r="P7" s="31"/>
       <c r="R7" s="14"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="26" t="s">
         <v>104</v>
       </c>
@@ -2763,7 +2764,7 @@
       <c r="P8" s="31"/>
       <c r="R8" s="14"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="26" t="s">
         <v>99</v>
       </c>
@@ -2800,7 +2801,7 @@
       </c>
       <c r="R9" s="28"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="26" t="s">
         <v>103</v>
       </c>
@@ -2837,7 +2838,7 @@
       </c>
       <c r="R10" s="28"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="26" t="s">
         <v>101</v>
       </c>
@@ -2869,7 +2870,7 @@
       </c>
       <c r="R11" s="28"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="26" t="s">
         <v>102</v>
       </c>
@@ -2897,7 +2898,7 @@
       <c r="P12" s="31"/>
       <c r="R12" s="14"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="47" t="s">
         <v>100</v>
       </c>
@@ -2924,15 +2925,15 @@
       <c r="Q13" s="46"/>
       <c r="R13" s="17"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="20"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="20"/>
       <c r="P25" s="20"/>
       <c r="S25" s="20"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="20"/>
       <c r="P26" s="20"/>
       <c r="S26" s="20"/>
@@ -2948,44 +2949,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:M48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.6328125" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.81640625" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="87" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B3" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="88"/>
-      <c r="K3" s="88"/>
-      <c r="L3" s="89"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="90" t="s">
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="87"/>
+      <c r="L3" s="88"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="91" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="52" t="s">
@@ -2994,7 +2995,7 @@
       <c r="E5" s="53">
         <v>46083</v>
       </c>
-      <c r="F5" s="94" t="s">
+      <c r="F5" s="93" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="55" t="s">
@@ -3003,7 +3004,7 @@
       <c r="H5" s="53">
         <v>46090</v>
       </c>
-      <c r="I5" s="94" t="s">
+      <c r="I5" s="93" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="55" t="s">
@@ -3012,36 +3013,36 @@
       <c r="K5" s="53">
         <v>46104</v>
       </c>
-      <c r="L5" s="94" t="s">
+      <c r="L5" s="93" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="91"/>
-      <c r="C6" s="93"/>
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="90"/>
+      <c r="C6" s="92"/>
       <c r="D6" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="95"/>
+      <c r="F6" s="94"/>
       <c r="G6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="95"/>
+      <c r="I6" s="94"/>
       <c r="J6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="95"/>
-    </row>
-    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="L6" s="94"/>
+    </row>
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="35" t="s">
         <v>24</v>
       </c>
@@ -3064,7 +3065,7 @@
       <c r="K7" s="11"/>
       <c r="L7" s="12"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="36" t="s">
         <v>35</v>
       </c>
@@ -3083,7 +3084,7 @@
       <c r="I8" s="14"/>
       <c r="L8" s="14"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="36" t="s">
         <v>36</v>
       </c>
@@ -3102,7 +3103,7 @@
       <c r="I9" s="14"/>
       <c r="L9" s="14"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="36" t="s">
         <v>75</v>
       </c>
@@ -3121,7 +3122,7 @@
       <c r="I10" s="14"/>
       <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="36" t="s">
         <v>165</v>
       </c>
@@ -3140,7 +3141,7 @@
       <c r="I11" s="14"/>
       <c r="L11" s="14"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="36" t="s">
         <v>25</v>
       </c>
@@ -3159,7 +3160,7 @@
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="36" t="s">
         <v>26</v>
       </c>
@@ -3178,7 +3179,7 @@
       <c r="I13" s="14"/>
       <c r="L13" s="14"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="36" t="s">
         <v>27</v>
       </c>
@@ -3197,7 +3198,7 @@
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="36" t="s">
         <v>163</v>
       </c>
@@ -3216,7 +3217,7 @@
       <c r="I15" s="14"/>
       <c r="L15" s="14"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
         <v>29</v>
       </c>
@@ -3235,7 +3236,7 @@
       <c r="I16" s="14"/>
       <c r="L16" s="14"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="36" t="s">
         <v>30</v>
       </c>
@@ -3254,7 +3255,7 @@
       <c r="I17" s="14"/>
       <c r="L17" s="14"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="36" t="s">
         <v>161</v>
       </c>
@@ -3273,7 +3274,7 @@
       <c r="I18" s="14"/>
       <c r="L18" s="14"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="36" t="s">
         <v>162</v>
       </c>
@@ -3292,7 +3293,7 @@
       <c r="I19" s="14"/>
       <c r="L19" s="14"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="56" t="s">
         <v>170</v>
       </c>
@@ -3311,7 +3312,7 @@
       <c r="I20" s="14"/>
       <c r="L20" s="14"/>
     </row>
-    <row r="21" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="36" t="s">
         <v>92</v>
       </c>
@@ -3332,7 +3333,7 @@
       </c>
       <c r="L21" s="14"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="36" t="s">
         <v>51</v>
       </c>
@@ -3351,7 +3352,7 @@
       <c r="I22" s="14"/>
       <c r="L22" s="14"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="36" t="s">
         <v>90</v>
       </c>
@@ -3372,7 +3373,7 @@
       </c>
       <c r="L23" s="14"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="36" t="s">
         <v>74</v>
       </c>
@@ -3391,7 +3392,7 @@
       <c r="I24" s="14"/>
       <c r="L24" s="14"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="36" t="s">
         <v>80</v>
       </c>
@@ -3410,7 +3411,7 @@
       <c r="I25" s="14"/>
       <c r="L25" s="14"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="36" t="s">
         <v>93</v>
       </c>
@@ -3431,7 +3432,7 @@
       </c>
       <c r="L26" s="14"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="36" t="s">
         <v>94</v>
       </c>
@@ -3452,7 +3453,7 @@
       </c>
       <c r="L27" s="14"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="77" t="s">
         <v>79</v>
       </c>
@@ -3473,7 +3474,7 @@
       </c>
       <c r="L28" s="14"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="77" t="s">
         <v>76</v>
       </c>
@@ -3492,7 +3493,7 @@
       <c r="I29" s="14"/>
       <c r="L29" s="14"/>
     </row>
-    <row r="30" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="82" t="s">
         <v>185</v>
       </c>
@@ -3511,7 +3512,7 @@
       <c r="I30" s="80"/>
       <c r="L30" s="80"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="77" t="s">
         <v>42</v>
       </c>
@@ -3530,7 +3531,7 @@
       </c>
       <c r="L31" s="14"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="77" t="s">
         <v>43</v>
       </c>
@@ -3549,7 +3550,7 @@
       </c>
       <c r="L32" s="14"/>
     </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B33" s="77" t="s">
         <v>164</v>
       </c>
@@ -3568,7 +3569,7 @@
       </c>
       <c r="L33" s="14"/>
     </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B34" s="77" t="s">
         <v>167</v>
       </c>
@@ -3587,7 +3588,7 @@
       </c>
       <c r="L34" s="14"/>
     </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B35" s="77" t="s">
         <v>73</v>
       </c>
@@ -3606,7 +3607,7 @@
       </c>
       <c r="L35" s="14"/>
     </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B36" s="77" t="s">
         <v>38</v>
       </c>
@@ -3625,7 +3626,7 @@
       </c>
       <c r="L36" s="14"/>
     </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B37" s="77" t="s">
         <v>39</v>
       </c>
@@ -3644,7 +3645,7 @@
       </c>
       <c r="L37" s="14"/>
     </row>
-    <row r="38" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="82" t="s">
         <v>181</v>
       </c>
@@ -3663,7 +3664,7 @@
       </c>
       <c r="L38" s="80"/>
     </row>
-    <row r="39" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B39" s="82" t="s">
         <v>182</v>
       </c>
@@ -3682,7 +3683,7 @@
       </c>
       <c r="L39" s="80"/>
     </row>
-    <row r="40" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B40" s="82" t="s">
         <v>179</v>
       </c>
@@ -3701,7 +3702,7 @@
       </c>
       <c r="L40" s="80"/>
     </row>
-    <row r="41" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B41" s="82" t="s">
         <v>180</v>
       </c>
@@ -3720,7 +3721,7 @@
       </c>
       <c r="L41" s="80"/>
     </row>
-    <row r="42" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B42" s="82" t="s">
         <v>177</v>
       </c>
@@ -3739,7 +3740,7 @@
       </c>
       <c r="L42" s="80"/>
     </row>
-    <row r="43" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B43" s="82" t="s">
         <v>176</v>
       </c>
@@ -3758,7 +3759,7 @@
       </c>
       <c r="L43" s="80"/>
     </row>
-    <row r="44" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B44" s="77" t="s">
         <v>172</v>
       </c>
@@ -3777,7 +3778,7 @@
       </c>
       <c r="L44" s="80"/>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B45" s="77" t="s">
         <v>171</v>
       </c>
@@ -3796,7 +3797,7 @@
       </c>
       <c r="L45" s="14"/>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B46" s="82" t="s">
         <v>175</v>
       </c>
@@ -3815,7 +3816,7 @@
       </c>
       <c r="L46" s="70"/>
     </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B47" s="77" t="s">
         <v>183</v>
       </c>
@@ -3835,7 +3836,7 @@
       <c r="L47" s="70"/>
       <c r="M47" s="69"/>
     </row>
-    <row r="48" spans="2:13" s="73" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:13" s="73" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B48" s="74" t="s">
         <v>174</v>
       </c>
@@ -3865,81 +3866,81 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B45 B47:B1048576 B1:B42">
-    <cfRule type="expression" dxfId="54" priority="28">
+    <cfRule type="expression" dxfId="49" priority="28">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C49:C1048576 C1:C45">
-    <cfRule type="expression" dxfId="53" priority="23">
+    <cfRule type="expression" dxfId="48" priority="23">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="25">
+    <cfRule type="expression" dxfId="47" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="27">
+    <cfRule type="expression" dxfId="46" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="50" priority="19">
+    <cfRule type="expression" dxfId="45" priority="19">
       <formula>$C47="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="49" priority="20">
+    <cfRule type="expression" dxfId="44" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="21">
+    <cfRule type="expression" dxfId="43" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="47" priority="8">
+    <cfRule type="expression" dxfId="42" priority="8">
       <formula>$C48="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="9">
+    <cfRule type="expression" dxfId="41" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="10">
+    <cfRule type="expression" dxfId="40" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C48">
-    <cfRule type="expression" dxfId="44" priority="12">
+    <cfRule type="expression" dxfId="39" priority="12">
       <formula>$C42="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="13">
+    <cfRule type="expression" dxfId="38" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="14">
+    <cfRule type="expression" dxfId="37" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B47:B48 B45 B31:B42">
-    <cfRule type="expression" dxfId="41" priority="30">
+    <cfRule type="expression" dxfId="36" priority="30">
       <formula>MAX($E31,$K31,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="expression" dxfId="40" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="39" priority="32">
+    <cfRule type="expression" dxfId="34" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="38" priority="38">
+    <cfRule type="expression" dxfId="33" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="expression" dxfId="37" priority="6">
+    <cfRule type="expression" dxfId="32" priority="6">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="expression" dxfId="36" priority="1">
+    <cfRule type="expression" dxfId="31" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3953,44 +3954,44 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="B1:M62"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B1:M70"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="21.81640625" customWidth="1"/>
-    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="87" t="s">
+    <row r="1" spans="2:13" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B1" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
-    </row>
-    <row r="3" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:13" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="90" t="s">
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
+      <c r="L1" s="88"/>
+    </row>
+    <row r="3" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:13" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="92" t="s">
+      <c r="C4" s="91" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="52" t="s">
@@ -3999,7 +4000,7 @@
       <c r="E4" s="53">
         <v>46111</v>
       </c>
-      <c r="F4" s="94" t="s">
+      <c r="F4" s="93" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="55" t="s">
@@ -4008,7 +4009,7 @@
       <c r="H4" s="53">
         <v>46125</v>
       </c>
-      <c r="I4" s="94" t="s">
+      <c r="I4" s="93" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="55" t="s">
@@ -4017,36 +4018,36 @@
       <c r="K4" s="53">
         <v>46132</v>
       </c>
-      <c r="L4" s="94" t="s">
+      <c r="L4" s="93" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="91"/>
-      <c r="C5" s="93"/>
+    <row r="5" spans="2:13" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="90"/>
+      <c r="C5" s="92"/>
       <c r="D5" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="95"/>
+      <c r="F5" s="94"/>
       <c r="G5" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="95"/>
+      <c r="I5" s="94"/>
       <c r="J5" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="95"/>
-    </row>
-    <row r="6" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="L5" s="94"/>
+    </row>
+    <row r="6" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B6" s="82" t="s">
         <v>188</v>
       </c>
@@ -4065,7 +4066,7 @@
       <c r="I6" s="80"/>
       <c r="L6" s="80"/>
     </row>
-    <row r="7" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="82" t="s">
         <v>189</v>
       </c>
@@ -4084,7 +4085,7 @@
       <c r="I7" s="80"/>
       <c r="L7" s="80"/>
     </row>
-    <row r="8" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B8" s="82" t="s">
         <v>190</v>
       </c>
@@ -4103,7 +4104,7 @@
       <c r="I8" s="80"/>
       <c r="L8" s="80"/>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B9" s="82" t="s">
         <v>173</v>
       </c>
@@ -4124,7 +4125,7 @@
       <c r="K9" s="79"/>
       <c r="L9" s="80"/>
     </row>
-    <row r="10" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="82" t="s">
         <v>187</v>
       </c>
@@ -4143,7 +4144,7 @@
       <c r="I10" s="80"/>
       <c r="L10" s="80"/>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B11" s="82" t="s">
         <v>186</v>
       </c>
@@ -4165,7 +4166,7 @@
       <c r="L11" s="80"/>
       <c r="M11" s="79"/>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B12" s="82" t="s">
         <v>178</v>
       </c>
@@ -4185,7 +4186,7 @@
       <c r="L12" s="14"/>
       <c r="M12" s="79"/>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B13" s="82" t="s">
         <v>184</v>
       </c>
@@ -4207,9 +4208,9 @@
       <c r="L13" s="80"/>
       <c r="M13" s="79"/>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B14" s="82" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C14" s="82" t="s">
         <v>106</v>
@@ -4227,30 +4228,34 @@
       <c r="L14" s="14"/>
       <c r="M14" s="79"/>
     </row>
-    <row r="15" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="82" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C15" s="82" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="81"/>
-      <c r="E15" s="83"/>
+      <c r="D15" s="81">
+        <v>0.05</v>
+      </c>
+      <c r="E15" s="83">
+        <v>100</v>
+      </c>
       <c r="F15" s="80"/>
       <c r="G15" s="81"/>
       <c r="H15" s="83"/>
       <c r="I15" s="80"/>
       <c r="L15" s="80"/>
     </row>
-    <row r="16" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="82" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C16" s="82" t="s">
         <v>106</v>
       </c>
       <c r="D16" s="81">
-        <v>0.05</v>
+        <v>2</v>
       </c>
       <c r="E16" s="83">
         <v>100</v>
@@ -4261,7 +4266,7 @@
       <c r="I16" s="80"/>
       <c r="L16" s="80"/>
     </row>
-    <row r="17" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="82" t="s">
         <v>199</v>
       </c>
@@ -4269,7 +4274,7 @@
         <v>106</v>
       </c>
       <c r="D17" s="81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="83">
         <v>100</v>
@@ -4280,15 +4285,15 @@
       <c r="I17" s="80"/>
       <c r="L17" s="80"/>
     </row>
-    <row r="18" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="82" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C18" s="82" t="s">
         <v>106</v>
       </c>
       <c r="D18" s="81">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="E18" s="83">
         <v>100</v>
@@ -4299,15 +4304,15 @@
       <c r="I18" s="80"/>
       <c r="L18" s="80"/>
     </row>
-    <row r="19" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="82" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C19" s="82" t="s">
         <v>106</v>
       </c>
       <c r="D19" s="81">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E19" s="83">
         <v>100</v>
@@ -4318,9 +4323,9 @@
       <c r="I19" s="80"/>
       <c r="L19" s="80"/>
     </row>
-    <row r="20" spans="2:13" s="79" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="B20" s="84" t="s">
-        <v>191</v>
+    <row r="20" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="82" t="s">
+        <v>212</v>
       </c>
       <c r="C20" s="82" t="s">
         <v>106</v>
@@ -4328,14 +4333,18 @@
       <c r="D20" s="81"/>
       <c r="E20" s="83"/>
       <c r="F20" s="80"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="83"/>
+      <c r="G20" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="H20" s="83">
+        <v>100</v>
+      </c>
       <c r="I20" s="80"/>
       <c r="L20" s="80"/>
     </row>
-    <row r="21" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B21" s="82" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="C21" s="82" t="s">
         <v>106</v>
@@ -4343,14 +4352,18 @@
       <c r="D21" s="81"/>
       <c r="E21" s="83"/>
       <c r="F21" s="80"/>
-      <c r="G21" s="81"/>
-      <c r="H21" s="83"/>
+      <c r="G21" s="81">
+        <v>0.75</v>
+      </c>
+      <c r="H21" s="83">
+        <v>100</v>
+      </c>
       <c r="I21" s="80"/>
       <c r="L21" s="80"/>
     </row>
-    <row r="22" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B22" s="82" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="C22" s="82" t="s">
         <v>106</v>
@@ -4358,14 +4371,18 @@
       <c r="D22" s="81"/>
       <c r="E22" s="83"/>
       <c r="F22" s="80"/>
-      <c r="G22" s="81"/>
-      <c r="H22" s="83"/>
+      <c r="G22" s="81">
+        <v>1</v>
+      </c>
+      <c r="H22" s="83">
+        <v>100</v>
+      </c>
       <c r="I22" s="80"/>
       <c r="L22" s="80"/>
     </row>
-    <row r="23" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="82" t="s">
-        <v>54</v>
+        <v>209</v>
       </c>
       <c r="C23" s="82" t="s">
         <v>106</v>
@@ -4373,14 +4390,18 @@
       <c r="D23" s="81"/>
       <c r="E23" s="83"/>
       <c r="F23" s="80"/>
-      <c r="G23" s="81"/>
-      <c r="H23" s="83"/>
+      <c r="G23" s="81">
+        <v>1</v>
+      </c>
+      <c r="H23" s="83">
+        <v>100</v>
+      </c>
       <c r="I23" s="80"/>
       <c r="L23" s="80"/>
     </row>
-    <row r="24" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B24" s="82" t="s">
-        <v>72</v>
+        <v>203</v>
       </c>
       <c r="C24" s="82" t="s">
         <v>106</v>
@@ -4388,14 +4409,18 @@
       <c r="D24" s="81"/>
       <c r="E24" s="83"/>
       <c r="F24" s="80"/>
-      <c r="G24" s="81"/>
-      <c r="H24" s="83"/>
+      <c r="G24" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="H24" s="83">
+        <v>100</v>
+      </c>
       <c r="I24" s="80"/>
       <c r="L24" s="80"/>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B25" s="82" t="s">
-        <v>91</v>
+        <v>217</v>
       </c>
       <c r="C25" s="82" t="s">
         <v>106</v>
@@ -4403,17 +4428,18 @@
       <c r="D25" s="81"/>
       <c r="E25" s="83"/>
       <c r="F25" s="80"/>
-      <c r="G25" s="81"/>
-      <c r="H25" s="83"/>
+      <c r="G25" s="81">
+        <v>3</v>
+      </c>
+      <c r="H25" s="83">
+        <v>100</v>
+      </c>
       <c r="I25" s="80"/>
-      <c r="J25" s="79"/>
-      <c r="K25" s="79"/>
       <c r="L25" s="80"/>
-      <c r="M25" s="79"/>
-    </row>
-    <row r="26" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B26" s="82" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="C26" s="82" t="s">
         <v>106</v>
@@ -4421,14 +4447,18 @@
       <c r="D26" s="81"/>
       <c r="E26" s="83"/>
       <c r="F26" s="80"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="83"/>
+      <c r="G26" s="81">
+        <v>0.75</v>
+      </c>
+      <c r="H26" s="83">
+        <v>100</v>
+      </c>
       <c r="I26" s="80"/>
       <c r="L26" s="80"/>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B27" s="82" t="s">
-        <v>54</v>
+        <v>205</v>
       </c>
       <c r="C27" s="82" t="s">
         <v>106</v>
@@ -4436,17 +4466,18 @@
       <c r="D27" s="81"/>
       <c r="E27" s="83"/>
       <c r="F27" s="80"/>
-      <c r="G27" s="81"/>
-      <c r="H27" s="83"/>
+      <c r="G27" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="H27" s="83">
+        <v>100</v>
+      </c>
       <c r="I27" s="80"/>
-      <c r="J27" s="79"/>
-      <c r="K27" s="79"/>
       <c r="L27" s="80"/>
-      <c r="M27" s="79"/>
-    </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B28" s="82" t="s">
-        <v>46</v>
+        <v>206</v>
       </c>
       <c r="C28" s="82" t="s">
         <v>106</v>
@@ -4454,17 +4485,18 @@
       <c r="D28" s="81"/>
       <c r="E28" s="83"/>
       <c r="F28" s="80"/>
-      <c r="G28" s="81"/>
-      <c r="H28" s="83"/>
+      <c r="G28" s="81">
+        <v>0.75</v>
+      </c>
+      <c r="H28" s="83">
+        <v>100</v>
+      </c>
       <c r="I28" s="80"/>
-      <c r="J28" s="79"/>
-      <c r="K28" s="79"/>
       <c r="L28" s="80"/>
-      <c r="M28" s="79"/>
-    </row>
-    <row r="29" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="82" t="s">
-        <v>45</v>
+        <v>207</v>
       </c>
       <c r="C29" s="82" t="s">
         <v>106</v>
@@ -4472,17 +4504,18 @@
       <c r="D29" s="81"/>
       <c r="E29" s="83"/>
       <c r="F29" s="80"/>
-      <c r="G29" s="81"/>
-      <c r="H29" s="83"/>
+      <c r="G29" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="H29" s="83">
+        <v>100</v>
+      </c>
       <c r="I29" s="80"/>
-      <c r="J29" s="79"/>
-      <c r="K29" s="79"/>
       <c r="L29" s="80"/>
-      <c r="M29" s="79"/>
-    </row>
-    <row r="30" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="82" t="s">
-        <v>41</v>
+        <v>211</v>
       </c>
       <c r="C30" s="82" t="s">
         <v>106</v>
@@ -4490,17 +4523,18 @@
       <c r="D30" s="81"/>
       <c r="E30" s="83"/>
       <c r="F30" s="80"/>
-      <c r="G30" s="81"/>
-      <c r="H30" s="83"/>
+      <c r="G30" s="81">
+        <v>1.25</v>
+      </c>
+      <c r="H30" s="83">
+        <v>100</v>
+      </c>
       <c r="I30" s="80"/>
-      <c r="J30" s="79"/>
-      <c r="K30" s="79"/>
       <c r="L30" s="80"/>
-      <c r="M30" s="79"/>
-    </row>
-    <row r="31" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B31" s="82" t="s">
-        <v>53</v>
+        <v>208</v>
       </c>
       <c r="C31" s="82" t="s">
         <v>106</v>
@@ -4508,17 +4542,18 @@
       <c r="D31" s="81"/>
       <c r="E31" s="83"/>
       <c r="F31" s="80"/>
-      <c r="G31" s="81"/>
-      <c r="H31" s="83"/>
+      <c r="G31" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="H31" s="83">
+        <v>100</v>
+      </c>
       <c r="I31" s="80"/>
-      <c r="J31" s="79"/>
-      <c r="K31" s="79"/>
       <c r="L31" s="80"/>
-      <c r="M31" s="79"/>
-    </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="2:12" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B32" s="82" t="s">
-        <v>57</v>
+        <v>210</v>
       </c>
       <c r="C32" s="82" t="s">
         <v>106</v>
@@ -4526,17 +4561,18 @@
       <c r="D32" s="81"/>
       <c r="E32" s="83"/>
       <c r="F32" s="80"/>
-      <c r="G32" s="81"/>
-      <c r="H32" s="83"/>
+      <c r="G32" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="H32" s="83">
+        <v>100</v>
+      </c>
       <c r="I32" s="80"/>
-      <c r="J32" s="79"/>
-      <c r="K32" s="79"/>
       <c r="L32" s="80"/>
-      <c r="M32" s="79"/>
-    </row>
-    <row r="33" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B33" s="82" t="s">
-        <v>71</v>
+        <v>215</v>
       </c>
       <c r="C33" s="82" t="s">
         <v>106</v>
@@ -4544,17 +4580,18 @@
       <c r="D33" s="81"/>
       <c r="E33" s="83"/>
       <c r="F33" s="80"/>
-      <c r="G33" s="81"/>
-      <c r="H33" s="83"/>
+      <c r="G33" s="81">
+        <v>1.25</v>
+      </c>
+      <c r="H33" s="83">
+        <v>100</v>
+      </c>
       <c r="I33" s="80"/>
-      <c r="J33" s="79"/>
-      <c r="K33" s="79"/>
       <c r="L33" s="80"/>
-      <c r="M33" s="79"/>
-    </row>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B34" s="82" t="s">
-        <v>114</v>
+        <v>216</v>
       </c>
       <c r="C34" s="82" t="s">
         <v>106</v>
@@ -4565,14 +4602,11 @@
       <c r="G34" s="81"/>
       <c r="H34" s="83"/>
       <c r="I34" s="80"/>
-      <c r="J34" s="79"/>
-      <c r="K34" s="79"/>
       <c r="L34" s="80"/>
-      <c r="M34" s="79"/>
-    </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B35" s="82" t="s">
-        <v>70</v>
+        <v>193</v>
       </c>
       <c r="C35" s="82" t="s">
         <v>106</v>
@@ -4583,14 +4617,11 @@
       <c r="G35" s="81"/>
       <c r="H35" s="83"/>
       <c r="I35" s="80"/>
-      <c r="J35" s="79"/>
-      <c r="K35" s="79"/>
       <c r="L35" s="80"/>
-      <c r="M35" s="79"/>
-    </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B36" s="82" t="s">
-        <v>56</v>
+        <v>214</v>
       </c>
       <c r="C36" s="82" t="s">
         <v>106</v>
@@ -4601,14 +4632,11 @@
       <c r="G36" s="81"/>
       <c r="H36" s="83"/>
       <c r="I36" s="80"/>
-      <c r="J36" s="79"/>
-      <c r="K36" s="79"/>
       <c r="L36" s="80"/>
-      <c r="M36" s="79"/>
-    </row>
-    <row r="37" spans="2:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B37" s="82" t="s">
-        <v>198</v>
+        <v>54</v>
       </c>
       <c r="C37" s="82" t="s">
         <v>106</v>
@@ -4619,46 +4647,32 @@
       <c r="G37" s="81"/>
       <c r="H37" s="83"/>
       <c r="I37" s="80"/>
-      <c r="J37" s="79"/>
-      <c r="K37" s="79"/>
       <c r="L37" s="80"/>
-      <c r="M37" s="79"/>
-    </row>
-    <row r="38" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B38" s="74" t="s">
-        <v>203</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D38" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="E38" s="83">
-        <v>100</v>
-      </c>
+    </row>
+    <row r="38" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="82" t="s">
+        <v>218</v>
+      </c>
+      <c r="C38" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" s="81"/>
+      <c r="E38" s="83"/>
       <c r="F38" s="80"/>
       <c r="G38" s="81"/>
       <c r="H38" s="83"/>
       <c r="I38" s="80"/>
-      <c r="J38" s="79"/>
-      <c r="K38" s="79"/>
       <c r="L38" s="80"/>
-      <c r="M38" s="79"/>
-    </row>
-    <row r="39" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B39" s="74" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D39" s="81">
-        <v>1</v>
-      </c>
-      <c r="E39" s="83">
-        <v>100</v>
-      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B39" s="82" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D39" s="81"/>
+      <c r="E39" s="83"/>
       <c r="F39" s="80"/>
       <c r="G39" s="81"/>
       <c r="H39" s="83"/>
@@ -4668,19 +4682,15 @@
       <c r="L39" s="80"/>
       <c r="M39" s="79"/>
     </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B40" s="74" t="s">
-        <v>83</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D40" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="E40" s="83">
-        <v>100</v>
-      </c>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B40" s="82" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="81"/>
+      <c r="E40" s="83"/>
       <c r="F40" s="80"/>
       <c r="G40" s="81"/>
       <c r="H40" s="83"/>
@@ -4690,19 +4700,15 @@
       <c r="L40" s="80"/>
       <c r="M40" s="79"/>
     </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B41" s="74" t="s">
-        <v>62</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D41" s="81">
-        <v>1.5</v>
-      </c>
-      <c r="E41" s="83">
-        <v>100</v>
-      </c>
+    <row r="41" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B41" s="82" t="s">
+        <v>41</v>
+      </c>
+      <c r="C41" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D41" s="81"/>
+      <c r="E41" s="83"/>
       <c r="F41" s="80"/>
       <c r="G41" s="81"/>
       <c r="H41" s="83"/>
@@ -4712,31 +4718,30 @@
       <c r="L41" s="80"/>
       <c r="M41" s="79"/>
     </row>
-    <row r="42" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="74" t="s">
-        <v>86</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D42" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="E42" s="83">
-        <v>100</v>
-      </c>
+    <row r="42" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B42" s="82" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D42" s="81"/>
+      <c r="E42" s="83"/>
       <c r="F42" s="80"/>
       <c r="G42" s="81"/>
       <c r="H42" s="83"/>
       <c r="I42" s="80"/>
+      <c r="J42" s="79"/>
+      <c r="K42" s="79"/>
       <c r="L42" s="80"/>
-    </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B43" s="85" t="s">
-        <v>201</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>107</v>
+      <c r="M42" s="79"/>
+    </row>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B43" s="82" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="82" t="s">
+        <v>106</v>
       </c>
       <c r="D43" s="81"/>
       <c r="E43" s="83"/>
@@ -4749,19 +4754,15 @@
       <c r="L43" s="80"/>
       <c r="M43" s="79"/>
     </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B44" s="74" t="s">
-        <v>58</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D44" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="E44" s="83">
-        <v>100</v>
-      </c>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B44" s="82" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D44" s="81"/>
+      <c r="E44" s="83"/>
       <c r="F44" s="80"/>
       <c r="G44" s="81"/>
       <c r="H44" s="83"/>
@@ -4771,19 +4772,15 @@
       <c r="L44" s="80"/>
       <c r="M44" s="79"/>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B45" s="74" t="s">
-        <v>59</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D45" s="81">
-        <v>0.75</v>
-      </c>
-      <c r="E45" s="83">
-        <v>100</v>
-      </c>
+    <row r="45" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B45" s="82" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" s="82" t="s">
+        <v>106</v>
+      </c>
+      <c r="D45" s="81"/>
+      <c r="E45" s="83"/>
       <c r="F45" s="80"/>
       <c r="G45" s="81"/>
       <c r="H45" s="83"/>
@@ -4791,10 +4788,11 @@
       <c r="J45" s="79"/>
       <c r="K45" s="79"/>
       <c r="L45" s="80"/>
-    </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="M45" s="79"/>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B46" s="74" t="s">
-        <v>60</v>
+        <v>198</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>107</v>
@@ -4812,118 +4810,286 @@
       <c r="J46" s="79"/>
       <c r="K46" s="79"/>
       <c r="L46" s="80"/>
-    </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="M46" s="79"/>
+    </row>
+    <row r="47" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B47" s="74" t="s">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D47" s="86">
+      <c r="D47" s="81">
         <v>1</v>
       </c>
       <c r="E47" s="83">
         <v>100</v>
       </c>
-    </row>
-    <row r="48" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="F47" s="80"/>
+      <c r="G47" s="81"/>
+      <c r="H47" s="83"/>
+      <c r="I47" s="80"/>
+      <c r="J47" s="79"/>
+      <c r="K47" s="79"/>
+      <c r="L47" s="80"/>
+      <c r="M47" s="79"/>
+    </row>
+    <row r="48" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B48" s="74" t="s">
-        <v>202</v>
+        <v>83</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D48" s="86">
-        <v>0.25</v>
+      <c r="D48" s="81">
+        <v>0.5</v>
       </c>
       <c r="E48" s="83">
         <v>100</v>
       </c>
-    </row>
-    <row r="49" spans="2:4" s="79" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F48" s="80"/>
+      <c r="G48" s="81"/>
+      <c r="H48" s="83"/>
+      <c r="I48" s="80"/>
+      <c r="J48" s="79"/>
+      <c r="K48" s="79"/>
+      <c r="L48" s="80"/>
+      <c r="M48" s="79"/>
+    </row>
+    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B49" s="74" t="s">
-        <v>200</v>
+        <v>62</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D49" s="86"/>
-    </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="D49" s="81">
+        <v>1.5</v>
+      </c>
+      <c r="E49" s="83">
+        <v>100</v>
+      </c>
+      <c r="F49" s="80"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="83"/>
+      <c r="I49" s="80"/>
+      <c r="J49" s="79"/>
+      <c r="K49" s="79"/>
+      <c r="L49" s="80"/>
+      <c r="M49" s="79"/>
+    </row>
+    <row r="50" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B50" s="74" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D50" s="86"/>
-    </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B51" s="74" t="s">
-        <v>66</v>
+      <c r="D50" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="E50" s="83">
+        <v>100</v>
+      </c>
+      <c r="F50" s="80"/>
+      <c r="G50" s="81"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="80"/>
+      <c r="L50" s="80"/>
+    </row>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B51" s="84" t="s">
+        <v>196</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D51" s="86"/>
-    </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="D51" s="81"/>
+      <c r="E51" s="83"/>
+      <c r="F51" s="80"/>
+      <c r="G51" s="81"/>
+      <c r="H51" s="83"/>
+      <c r="I51" s="80"/>
+      <c r="J51" s="79"/>
+      <c r="K51" s="79"/>
+      <c r="L51" s="80"/>
+      <c r="M51" s="79"/>
+    </row>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B52" s="74" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D52" s="86"/>
-    </row>
-    <row r="53" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B53" s="74"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="86"/>
-    </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B54" s="74"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="86"/>
-    </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B55" s="74"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="86"/>
-    </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B56" s="74"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="86"/>
-    </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B57" s="74"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="86"/>
-    </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B58" s="74"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="86"/>
-    </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B59" s="74"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="86"/>
-    </row>
-    <row r="60" spans="2:4" x14ac:dyDescent="0.35">
-      <c r="B60" s="74"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="86"/>
-    </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="D52" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="E52" s="83">
+        <v>100</v>
+      </c>
+      <c r="F52" s="80"/>
+      <c r="G52" s="81"/>
+      <c r="H52" s="83"/>
+      <c r="I52" s="80"/>
+      <c r="J52" s="79"/>
+      <c r="K52" s="79"/>
+      <c r="L52" s="80"/>
+      <c r="M52" s="79"/>
+    </row>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B53" s="74" t="s">
+        <v>59</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D53" s="81">
+        <v>0.75</v>
+      </c>
+      <c r="E53" s="83">
+        <v>100</v>
+      </c>
+      <c r="F53" s="80"/>
+      <c r="G53" s="81"/>
+      <c r="H53" s="83"/>
+      <c r="I53" s="80"/>
+      <c r="J53" s="79"/>
+      <c r="K53" s="79"/>
+      <c r="L53" s="80"/>
+    </row>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B54" s="74" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D54" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="E54" s="83">
+        <v>100</v>
+      </c>
+      <c r="F54" s="80"/>
+      <c r="G54" s="81"/>
+      <c r="H54" s="83"/>
+      <c r="I54" s="80"/>
+      <c r="J54" s="79"/>
+      <c r="K54" s="79"/>
+      <c r="L54" s="80"/>
+    </row>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B55" s="74" t="s">
+        <v>57</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D55" s="85">
+        <v>1</v>
+      </c>
+      <c r="E55" s="83">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B56" s="74" t="s">
+        <v>197</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D56" s="85">
+        <v>0.25</v>
+      </c>
+      <c r="E56" s="83">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="2:13" s="79" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="74" t="s">
+        <v>195</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D57" s="85"/>
+    </row>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B58" s="74" t="s">
+        <v>65</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D58" s="85"/>
+    </row>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B59" s="74" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D59" s="85"/>
+    </row>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B60" s="74" t="s">
+        <v>88</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="D60" s="85"/>
+    </row>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B61" s="74"/>
-      <c r="D61" s="86"/>
-    </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C61" s="8"/>
+      <c r="D61" s="85"/>
+    </row>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B62" s="74"/>
-      <c r="D62" s="86"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="85"/>
+    </row>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B63" s="74"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="85"/>
+    </row>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B64" s="74"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="85"/>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B65" s="74"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="85"/>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B66" s="74"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="85"/>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B67" s="74"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="85"/>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B68" s="74"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="85"/>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B69" s="74"/>
+      <c r="D69" s="85"/>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B70" s="74"/>
+      <c r="D70" s="85"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:L5" xr:uid="{2EE69061-1192-400C-B500-1B4897FD0585}"/>
@@ -4936,108 +5102,98 @@
     <mergeCell ref="L4:L5"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="B27:B41 B43:B46 B4:B20">
-    <cfRule type="expression" dxfId="35" priority="47">
+  <conditionalFormatting sqref="B51:B54 B4:B49">
+    <cfRule type="expression" dxfId="30" priority="47">
       <formula>MAX($E4,$H4,$K4)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C5 C9:C46">
-    <cfRule type="expression" dxfId="34" priority="44">
+  <conditionalFormatting sqref="C4:C5 C9:C54">
+    <cfRule type="expression" dxfId="29" priority="44">
       <formula>$C4="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="45">
+    <cfRule type="expression" dxfId="28" priority="45">
       <formula>$C4="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="46">
+    <cfRule type="expression" dxfId="27" priority="46">
       <formula>$C4="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1">
-    <cfRule type="expression" dxfId="31" priority="43">
+    <cfRule type="expression" dxfId="26" priority="43">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="expression" dxfId="30" priority="40">
+    <cfRule type="expression" dxfId="25" priority="40">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="41">
+    <cfRule type="expression" dxfId="24" priority="41">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="42">
+    <cfRule type="expression" dxfId="23" priority="42">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="27" priority="36">
+    <cfRule type="expression" dxfId="22" priority="36">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="expression" dxfId="26" priority="30">
+    <cfRule type="expression" dxfId="21" priority="30">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="25" priority="29">
+    <cfRule type="expression" dxfId="20" priority="29">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="24" priority="28">
+    <cfRule type="expression" dxfId="19" priority="28">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B36">
-    <cfRule type="expression" dxfId="23" priority="83">
+  <conditionalFormatting sqref="B45">
+    <cfRule type="expression" dxfId="18" priority="83">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B12">
-    <cfRule type="expression" dxfId="22" priority="25">
+    <cfRule type="expression" dxfId="17" priority="25">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C8">
-    <cfRule type="expression" dxfId="21" priority="22">
+    <cfRule type="expression" dxfId="16" priority="22">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="23">
+    <cfRule type="expression" dxfId="15" priority="23">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="24">
+    <cfRule type="expression" dxfId="14" priority="24">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21:B26">
-    <cfRule type="expression" dxfId="18" priority="21">
-      <formula>MAX($E21,$H21,$K21)=100</formula>
+  <conditionalFormatting sqref="B50">
+    <cfRule type="expression" dxfId="13" priority="85">
+      <formula>MAX($E51,$H51,$K51)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21:B26">
-    <cfRule type="expression" dxfId="17" priority="20">
-      <formula>MAX($E21,$H21,$K21)=100</formula>
+  <conditionalFormatting sqref="B55:B70">
+    <cfRule type="expression" dxfId="12" priority="4">
+      <formula>MAX($E55,$H55,$K55)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="16" priority="85">
-      <formula>MAX($E43,$H43,$K43)=100</formula>
+  <conditionalFormatting sqref="C55:C68">
+    <cfRule type="expression" dxfId="11" priority="1">
+      <formula>$C55="Charlotte/Eddy"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B47:B62">
-    <cfRule type="expression" dxfId="15" priority="4">
-      <formula>MAX($E47,$H47,$K47)=100</formula>
+    <cfRule type="expression" dxfId="10" priority="2">
+      <formula>$C55="Charlotte"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C47:C60">
-    <cfRule type="expression" dxfId="14" priority="1">
-      <formula>$C47="Charlotte/Eddy"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="2">
-      <formula>$C47="Charlotte"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="3">
-      <formula>$C47="Eddy"</formula>
+    <cfRule type="expression" dxfId="9" priority="3">
+      <formula>$C55="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5050,21 +5206,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="70.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="70.77734375" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" customWidth="1"/>
-    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="28.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="9" t="s">
         <v>22</v>
       </c>
@@ -5078,151 +5234,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -5238,18 +5394,18 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B2:O56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:15" ht="21" x14ac:dyDescent="0.4">
       <c r="B4" s="7"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4" t="s">
@@ -5273,7 +5429,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="6"/>
     </row>
-    <row r="5" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
@@ -5317,7 +5473,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B6" s="10" t="s">
         <v>95</v>
       </c>
@@ -5339,7 +5495,7 @@
       <c r="N6" s="11"/>
       <c r="O6" s="12"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="13" t="s">
         <v>55</v>
       </c>
@@ -5357,7 +5513,7 @@
       <c r="M7" s="18"/>
       <c r="O7" s="14"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="13" t="s">
         <v>84</v>
       </c>
@@ -5375,7 +5531,7 @@
       <c r="M8" s="18"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="13" t="s">
         <v>85</v>
       </c>
@@ -5393,7 +5549,7 @@
       <c r="M9" s="18"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="13" t="s">
         <v>83</v>
       </c>
@@ -5411,7 +5567,7 @@
       <c r="M10" s="18"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="13" t="s">
         <v>62</v>
       </c>
@@ -5429,7 +5585,7 @@
       <c r="M11" s="18"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
@@ -5447,7 +5603,7 @@
       <c r="M12" s="18"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="13" t="s">
         <v>86</v>
       </c>
@@ -5465,7 +5621,7 @@
       <c r="M13" s="18"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="13" t="s">
         <v>54</v>
       </c>
@@ -5483,7 +5639,7 @@
       <c r="M14" s="18"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="13" t="s">
         <v>58</v>
       </c>
@@ -5501,7 +5657,7 @@
       <c r="M15" s="18"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="13" t="s">
         <v>59</v>
       </c>
@@ -5519,7 +5675,7 @@
       <c r="M16" s="18"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="13" t="s">
         <v>60</v>
       </c>
@@ -5537,7 +5693,7 @@
       <c r="M17" s="18"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="13" t="s">
         <v>63</v>
       </c>
@@ -5555,7 +5711,7 @@
       <c r="M18" s="18"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="13" t="s">
         <v>46</v>
       </c>
@@ -5573,7 +5729,7 @@
       <c r="M19" s="18"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
         <v>45</v>
       </c>
@@ -5591,7 +5747,7 @@
       <c r="M20" s="18"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="13" t="s">
         <v>82</v>
       </c>
@@ -5609,7 +5765,7 @@
       <c r="M21" s="18"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="13" t="s">
         <v>40</v>
       </c>
@@ -5627,7 +5783,7 @@
       <c r="M22" s="18"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="13" t="s">
         <v>41</v>
       </c>
@@ -5645,7 +5801,7 @@
       <c r="M23" s="18"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="13" t="s">
         <v>57</v>
       </c>
@@ -5663,7 +5819,7 @@
       <c r="M24" s="18"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="13" t="s">
         <v>53</v>
       </c>
@@ -5681,7 +5837,7 @@
       <c r="M25" s="18"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="13" t="s">
         <v>72</v>
       </c>
@@ -5699,7 +5855,7 @@
       <c r="M26" s="18"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="13" t="s">
         <v>57</v>
       </c>
@@ -5717,7 +5873,7 @@
       <c r="M27" s="18"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="13" t="s">
         <v>69</v>
       </c>
@@ -5735,7 +5891,7 @@
       <c r="M28" s="18"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="13" t="s">
         <v>71</v>
       </c>
@@ -5753,9 +5909,9 @@
       <c r="M29" s="18"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="13" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>107</v>
@@ -5771,7 +5927,7 @@
       </c>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="13" t="s">
         <v>65</v>
       </c>
@@ -5789,7 +5945,7 @@
       </c>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B32" s="13" t="s">
         <v>66</v>
       </c>
@@ -5807,7 +5963,7 @@
       </c>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="13" t="s">
         <v>114</v>
       </c>
@@ -5825,7 +5981,7 @@
       </c>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="13" t="s">
         <v>88</v>
       </c>
@@ -5843,7 +5999,7 @@
       </c>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="15" t="s">
         <v>70</v>
       </c>
@@ -5865,47 +6021,47 @@
       <c r="N35" s="16"/>
       <c r="O35" s="17"/>
     </row>
-    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="40" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B48" s="35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="36" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="36" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="36" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="36" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B53" s="36" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="2:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B54" s="37" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="56" spans="2:2" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5917,48 +6073,48 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="51.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" customWidth="1"/>
-    <col min="11" max="11" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="51.5546875" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
+    <col min="7" max="7" width="20.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="96" t="s">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="B2" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="97"/>
-      <c r="L2" s="97"/>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-    </row>
-    <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="90" t="s">
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="96"/>
+      <c r="J2" s="96"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="96"/>
+      <c r="M2" s="96"/>
+      <c r="N2" s="96"/>
+      <c r="O2" s="96"/>
+    </row>
+    <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="91" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="52" t="s">
@@ -5967,7 +6123,7 @@
       <c r="E5" s="53">
         <v>46139</v>
       </c>
-      <c r="F5" s="94" t="s">
+      <c r="F5" s="93" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="55" t="s">
@@ -5976,7 +6132,7 @@
       <c r="H5" s="53">
         <v>46146</v>
       </c>
-      <c r="I5" s="94" t="s">
+      <c r="I5" s="93" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="55" t="s">
@@ -5985,7 +6141,7 @@
       <c r="K5" s="53">
         <v>46153</v>
       </c>
-      <c r="L5" s="94" t="s">
+      <c r="L5" s="93" t="s">
         <v>12</v>
       </c>
       <c r="M5" s="55" t="s">
@@ -5994,43 +6150,43 @@
       <c r="N5" s="53">
         <v>46161</v>
       </c>
-      <c r="O5" s="94" t="s">
+      <c r="O5" s="93" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="91"/>
-      <c r="C6" s="93"/>
+    <row r="6" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="90"/>
+      <c r="C6" s="92"/>
       <c r="D6" s="52" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="95"/>
+      <c r="F6" s="94"/>
       <c r="G6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="95"/>
+      <c r="I6" s="94"/>
       <c r="J6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="95"/>
+      <c r="L6" s="94"/>
       <c r="M6" s="54" t="s">
         <v>10</v>
       </c>
       <c r="N6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="O6" s="95"/>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="O6" s="94"/>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B7" s="35"/>
       <c r="C7" s="35"/>
       <c r="D7" s="33"/>
@@ -6046,7 +6202,7 @@
       <c r="N7" s="11"/>
       <c r="O7" s="12"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="36"/>
       <c r="C8" s="36"/>
       <c r="D8" s="31"/>
@@ -6058,7 +6214,7 @@
       <c r="L8" s="14"/>
       <c r="O8" s="14"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="36"/>
       <c r="C9" s="36"/>
       <c r="D9" s="31"/>
@@ -6070,7 +6226,7 @@
       <c r="L9" s="14"/>
       <c r="O9" s="14"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="36"/>
       <c r="C10" s="36"/>
       <c r="D10" s="31"/>
@@ -6082,7 +6238,7 @@
       <c r="L10" s="14"/>
       <c r="O10" s="14"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="36"/>
       <c r="C11" s="36"/>
       <c r="D11" s="31"/>
@@ -6094,7 +6250,7 @@
       <c r="L11" s="14"/>
       <c r="O11" s="14"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="36"/>
       <c r="C12" s="36"/>
       <c r="D12" s="31"/>
@@ -6106,7 +6262,7 @@
       <c r="L12" s="14"/>
       <c r="O12" s="14"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="36"/>
       <c r="C13" s="36"/>
       <c r="D13" s="31"/>
@@ -6118,7 +6274,7 @@
       <c r="L13" s="14"/>
       <c r="O13" s="14"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="36"/>
       <c r="C14" s="36"/>
       <c r="D14" s="31"/>
@@ -6130,7 +6286,7 @@
       <c r="L14" s="14"/>
       <c r="O14" s="14"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="36"/>
       <c r="C15" s="36"/>
       <c r="D15" s="31"/>
@@ -6142,7 +6298,7 @@
       <c r="L15" s="14"/>
       <c r="O15" s="14"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="36"/>
       <c r="C16" s="36"/>
       <c r="D16" s="31"/>
@@ -6154,7 +6310,7 @@
       <c r="L16" s="14"/>
       <c r="O16" s="14"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="36"/>
       <c r="C17" s="36"/>
       <c r="D17" s="31"/>
@@ -6166,7 +6322,7 @@
       <c r="L17" s="14"/>
       <c r="O17" s="14"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="36"/>
       <c r="C18" s="36"/>
       <c r="D18" s="31"/>
@@ -6178,7 +6334,7 @@
       <c r="L18" s="14"/>
       <c r="O18" s="14"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="36"/>
       <c r="C19" s="36"/>
       <c r="D19" s="31"/>
@@ -6190,7 +6346,7 @@
       <c r="L19" s="14"/>
       <c r="O19" s="14"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="56"/>
       <c r="C20" s="36"/>
       <c r="D20" s="31"/>
@@ -6202,7 +6358,7 @@
       <c r="L20" s="14"/>
       <c r="O20" s="14"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="36"/>
       <c r="C21" s="36"/>
       <c r="D21" s="31"/>
@@ -6214,7 +6370,7 @@
       <c r="L21" s="14"/>
       <c r="O21" s="14"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="36"/>
       <c r="C22" s="36"/>
       <c r="D22" s="31"/>
@@ -6226,7 +6382,7 @@
       <c r="L22" s="14"/>
       <c r="O22" s="14"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B23" s="36"/>
       <c r="C23" s="36"/>
       <c r="D23" s="31"/>
@@ -6238,7 +6394,7 @@
       <c r="L23" s="14"/>
       <c r="O23" s="14"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B24" s="36"/>
       <c r="C24" s="36"/>
       <c r="D24" s="40"/>
@@ -6250,7 +6406,7 @@
       <c r="L24" s="14"/>
       <c r="O24" s="14"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B25" s="36"/>
       <c r="C25" s="36"/>
       <c r="D25" s="31"/>
@@ -6262,7 +6418,7 @@
       <c r="L25" s="14"/>
       <c r="O25" s="14"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B26" s="36"/>
       <c r="C26" s="36"/>
       <c r="D26" s="31"/>
@@ -6274,7 +6430,7 @@
       <c r="L26" s="14"/>
       <c r="O26" s="14"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="36"/>
       <c r="C27" s="36"/>
       <c r="D27" s="31"/>
@@ -6286,7 +6442,7 @@
       <c r="L27" s="14"/>
       <c r="O27" s="14"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B28" s="36"/>
       <c r="C28" s="36"/>
       <c r="D28" s="31"/>
@@ -6298,7 +6454,7 @@
       <c r="L28" s="14"/>
       <c r="O28" s="14"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B29" s="18"/>
       <c r="C29" s="36"/>
       <c r="D29" s="31"/>
@@ -6310,7 +6466,7 @@
       <c r="L29" s="14"/>
       <c r="O29" s="14"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B30" s="36"/>
       <c r="C30" s="36"/>
       <c r="D30" s="31"/>
@@ -6322,7 +6478,7 @@
       <c r="L30" s="14"/>
       <c r="O30" s="14"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B31" s="36"/>
       <c r="C31" s="36"/>
       <c r="D31" s="31"/>
@@ -6334,7 +6490,7 @@
       <c r="L31" s="14"/>
       <c r="O31" s="14"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B32" s="36"/>
       <c r="C32" s="36"/>
       <c r="D32" s="31"/>
@@ -6346,7 +6502,7 @@
       <c r="L32" s="14"/>
       <c r="O32" s="14"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B33" s="36"/>
       <c r="C33" s="36"/>
       <c r="D33" s="31"/>
@@ -6358,7 +6514,7 @@
       <c r="L33" s="14"/>
       <c r="O33" s="14"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B34" s="36"/>
       <c r="C34" s="36"/>
       <c r="D34" s="31"/>
@@ -6370,7 +6526,7 @@
       <c r="L34" s="14"/>
       <c r="O34" s="14"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B35" s="36"/>
       <c r="C35" s="36"/>
       <c r="D35" s="31"/>
@@ -6382,7 +6538,7 @@
       <c r="L35" s="14"/>
       <c r="O35" s="14"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B36" s="36"/>
       <c r="C36" s="36"/>
       <c r="D36" s="31"/>
@@ -6394,7 +6550,7 @@
       <c r="L36" s="14"/>
       <c r="O36" s="14"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B37" s="36"/>
       <c r="C37" s="36"/>
       <c r="D37" s="31"/>
@@ -6406,7 +6562,7 @@
       <c r="L37" s="14"/>
       <c r="O37" s="14"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B38" s="36"/>
       <c r="C38" s="36"/>
       <c r="D38" s="31"/>
@@ -6418,7 +6574,7 @@
       <c r="L38" s="14"/>
       <c r="O38" s="14"/>
     </row>
-    <row r="39" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="37"/>
       <c r="C39" s="37"/>
       <c r="D39" s="32"/>
@@ -6491,28 +6647,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
-    <col min="2" max="2" width="93.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="2" max="2" width="93.21875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="42.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.75" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:6" ht="44.7" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -6529,7 +6685,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -6542,7 +6698,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -6555,7 +6711,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -6568,7 +6724,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -6581,7 +6737,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -6594,7 +6750,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -6607,7 +6763,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -6620,7 +6776,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -6633,7 +6789,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -6646,7 +6802,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -6659,7 +6815,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -6672,7 +6828,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -6685,7 +6841,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -6698,7 +6854,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -6711,7 +6867,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -6724,7 +6880,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -6737,7 +6893,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -6750,7 +6906,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -6763,7 +6919,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -6776,7 +6932,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -6789,7 +6945,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -6802,7 +6958,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -6815,7 +6971,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -6828,7 +6984,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -6841,7 +6997,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -6854,7 +7010,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -6867,7 +7023,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -6880,7 +7036,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -6893,7 +7049,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -6906,7 +7062,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -6919,7 +7075,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -6932,7 +7088,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -6945,7 +7101,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -6958,7 +7114,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -6971,7 +7127,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -6984,7 +7140,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -6997,7 +7153,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -7010,7 +7166,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -7023,7 +7179,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -7036,7 +7192,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -7049,7 +7205,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -7062,7 +7218,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -7075,7 +7231,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -7088,7 +7244,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -7101,7 +7257,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -7114,7 +7270,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -7127,7 +7283,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -7140,7 +7296,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -7153,7 +7309,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -7166,7 +7322,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -7179,7 +7335,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -7192,7 +7348,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -7205,7 +7361,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -7218,7 +7374,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -7231,7 +7387,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -7244,7 +7400,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -7257,7 +7413,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -7270,7 +7426,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -7283,7 +7439,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -7296,7 +7452,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>96</v>
       </c>
@@ -7307,7 +7463,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>97</v>
       </c>
@@ -7318,7 +7474,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>98</v>
       </c>
@@ -7329,7 +7485,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>99</v>
       </c>
@@ -7340,7 +7496,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>100</v>
       </c>
@@ -7351,7 +7507,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>101</v>
       </c>
@@ -7362,7 +7518,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>102</v>
       </c>
@@ -7373,7 +7529,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>103</v>
       </c>
@@ -7384,7 +7540,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>104</v>
       </c>
@@ -7395,7 +7551,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>120</v>
       </c>
@@ -7406,7 +7562,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>121</v>
       </c>
@@ -7417,182 +7573,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Debug Combats, Début de difficulté AI
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C83DF5-DA03-41A5-9BFC-2D0721530902}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4386DCE5-2AD6-4799-9046-B999A47CBBCC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="223">
   <si>
     <t>Planification globale</t>
   </si>
@@ -701,6 +701,12 @@
   </si>
   <si>
     <t>Afficher le tour de jeu message au centre de l écran: Ajouter component YourTurn</t>
+  </si>
+  <si>
+    <t>Implémentation des combats</t>
+  </si>
+  <si>
+    <t>Erreurs d'affichage, problèmes avec la pause pour l'affichage</t>
   </si>
 </sst>
 </file>
@@ -1132,7 +1138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1296,6 +1302,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3964,8 +3976,8 @@
     <col min="4" max="4" width="21.81640625" customWidth="1"/>
     <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.1796875" customWidth="1"/>
-    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="83" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" style="83" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="52.81640625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
@@ -4004,7 +4016,7 @@
       <c r="F4" s="93" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="55" t="s">
+      <c r="G4" s="98" t="s">
         <v>14</v>
       </c>
       <c r="H4" s="53">
@@ -4033,10 +4045,10 @@
         <v>11</v>
       </c>
       <c r="F5" s="94"/>
-      <c r="G5" s="54" t="s">
+      <c r="G5" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="54" t="s">
+      <c r="H5" s="97" t="s">
         <v>11</v>
       </c>
       <c r="I5" s="94"/>
@@ -4120,7 +4132,6 @@
       </c>
       <c r="F9" s="80"/>
       <c r="G9" s="81"/>
-      <c r="H9" s="83"/>
       <c r="I9" s="80"/>
       <c r="J9" s="79"/>
       <c r="K9" s="79"/>
@@ -4160,7 +4171,6 @@
       </c>
       <c r="F11" s="80"/>
       <c r="G11" s="81"/>
-      <c r="H11" s="83"/>
       <c r="I11" s="80"/>
       <c r="J11" s="79"/>
       <c r="K11" s="79"/>
@@ -4181,8 +4191,7 @@
         <v>100</v>
       </c>
       <c r="F12" s="14"/>
-      <c r="G12" s="31"/>
-      <c r="H12" s="40"/>
+      <c r="G12" s="81"/>
       <c r="I12" s="14"/>
       <c r="L12" s="14"/>
       <c r="M12" s="79"/>
@@ -4202,7 +4211,6 @@
       </c>
       <c r="F13" s="80"/>
       <c r="G13" s="81"/>
-      <c r="H13" s="83"/>
       <c r="I13" s="80"/>
       <c r="J13" s="79"/>
       <c r="K13" s="79"/>
@@ -4223,8 +4231,7 @@
         <v>100</v>
       </c>
       <c r="F14" s="14"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="40"/>
+      <c r="G14" s="81"/>
       <c r="I14" s="14"/>
       <c r="L14" s="14"/>
       <c r="M14" s="79"/>
@@ -4697,7 +4704,6 @@
       <c r="E40" s="83"/>
       <c r="F40" s="80"/>
       <c r="G40" s="81"/>
-      <c r="H40" s="83"/>
       <c r="I40" s="80"/>
       <c r="J40" s="79"/>
       <c r="K40" s="79"/>
@@ -4715,7 +4721,6 @@
       <c r="E41" s="83"/>
       <c r="F41" s="80"/>
       <c r="G41" s="81"/>
-      <c r="H41" s="83"/>
       <c r="I41" s="80"/>
       <c r="J41" s="79"/>
       <c r="K41" s="79"/>
@@ -4733,7 +4738,6 @@
       <c r="E42" s="83"/>
       <c r="F42" s="80"/>
       <c r="G42" s="81"/>
-      <c r="H42" s="83"/>
       <c r="I42" s="80"/>
       <c r="J42" s="79"/>
       <c r="K42" s="79"/>
@@ -4751,7 +4755,6 @@
       <c r="E43" s="83"/>
       <c r="F43" s="80"/>
       <c r="G43" s="81"/>
-      <c r="H43" s="83"/>
       <c r="I43" s="80"/>
       <c r="J43" s="79"/>
       <c r="K43" s="79"/>
@@ -4769,7 +4772,6 @@
       <c r="E44" s="83"/>
       <c r="F44" s="80"/>
       <c r="G44" s="81"/>
-      <c r="H44" s="83"/>
       <c r="I44" s="80"/>
       <c r="J44" s="79"/>
       <c r="K44" s="79"/>
@@ -4787,7 +4789,6 @@
       <c r="E45" s="83"/>
       <c r="F45" s="80"/>
       <c r="G45" s="81"/>
-      <c r="H45" s="83"/>
       <c r="I45" s="80"/>
       <c r="J45" s="79"/>
       <c r="K45" s="79"/>
@@ -4805,7 +4806,6 @@
       <c r="E46" s="83"/>
       <c r="F46" s="80"/>
       <c r="G46" s="81"/>
-      <c r="H46" s="83"/>
       <c r="I46" s="80"/>
       <c r="J46" s="79"/>
       <c r="K46" s="79"/>
@@ -4827,7 +4827,6 @@
       </c>
       <c r="F47" s="80"/>
       <c r="G47" s="81"/>
-      <c r="H47" s="83"/>
       <c r="I47" s="80"/>
       <c r="J47" s="79"/>
       <c r="K47" s="79"/>
@@ -4849,7 +4848,6 @@
       </c>
       <c r="F48" s="80"/>
       <c r="G48" s="81"/>
-      <c r="H48" s="83"/>
       <c r="I48" s="80"/>
       <c r="J48" s="79"/>
       <c r="K48" s="79"/>
@@ -4871,7 +4869,6 @@
       </c>
       <c r="F49" s="80"/>
       <c r="G49" s="81"/>
-      <c r="H49" s="83"/>
       <c r="I49" s="80"/>
       <c r="J49" s="79"/>
       <c r="K49" s="79"/>
@@ -4893,7 +4890,6 @@
       </c>
       <c r="F50" s="80"/>
       <c r="G50" s="81"/>
-      <c r="H50" s="83"/>
       <c r="I50" s="80"/>
       <c r="J50" s="79"/>
       <c r="K50" s="79"/>
@@ -4930,7 +4926,6 @@
       <c r="E52" s="83"/>
       <c r="F52" s="80"/>
       <c r="G52" s="81"/>
-      <c r="H52" s="83"/>
       <c r="I52" s="80"/>
       <c r="J52" s="79"/>
       <c r="K52" s="79"/>
@@ -4952,7 +4947,6 @@
       </c>
       <c r="F53" s="80"/>
       <c r="G53" s="81"/>
-      <c r="H53" s="83"/>
       <c r="I53" s="80"/>
       <c r="J53" s="79"/>
       <c r="K53" s="79"/>
@@ -4974,7 +4968,6 @@
       </c>
       <c r="F54" s="80"/>
       <c r="G54" s="81"/>
-      <c r="H54" s="83"/>
       <c r="I54" s="80"/>
       <c r="J54" s="79"/>
       <c r="K54" s="79"/>
@@ -4995,7 +4988,6 @@
       </c>
       <c r="F55" s="80"/>
       <c r="G55" s="81"/>
-      <c r="H55" s="83"/>
       <c r="I55" s="80"/>
       <c r="J55" s="79"/>
       <c r="K55" s="79"/>
@@ -5037,6 +5029,8 @@
         <v>107</v>
       </c>
       <c r="D58" s="85"/>
+      <c r="G58" s="83"/>
+      <c r="H58" s="83"/>
     </row>
     <row r="59" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B59" s="74" t="s">
@@ -5045,7 +5039,12 @@
       <c r="C59" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D59" s="85"/>
+      <c r="D59" s="85">
+        <v>1.5</v>
+      </c>
+      <c r="E59" s="83">
+        <v>75</v>
+      </c>
     </row>
     <row r="60" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B60" s="74" t="s">
@@ -5055,6 +5054,12 @@
         <v>107</v>
       </c>
       <c r="D60" s="85"/>
+      <c r="G60" s="83">
+        <v>2</v>
+      </c>
+      <c r="H60" s="83">
+        <v>25</v>
+      </c>
     </row>
     <row r="61" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B61" s="74" t="s">
@@ -5066,9 +5071,22 @@
       <c r="D61" s="85"/>
     </row>
     <row r="62" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B62" s="74"/>
-      <c r="C62" s="8"/>
+      <c r="B62" s="74" t="s">
+        <v>221</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>107</v>
+      </c>
       <c r="D62" s="85"/>
+      <c r="G62" s="83">
+        <v>1.5</v>
+      </c>
+      <c r="H62" s="83">
+        <v>75</v>
+      </c>
+      <c r="I62" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="63" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B63" s="74"/>

</xml_diff>

<commit_message>
Mise à jour planification
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE37183-6DA6-4031-8F15-03FDB66025D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DA43DA-A901-45B7-B726-4CD5EA7FFAB7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -32,23 +32,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="217">
   <si>
     <t>Planification globale</t>
   </si>
@@ -689,13 +678,16 @@
     <t>Ajout des compteurs de pieces dans les cimetieres en fonction des resultats de combat</t>
   </si>
   <si>
-    <t>en cours</t>
-  </si>
-  <si>
-    <t>Ajouter le score de chaque joueur scores</t>
-  </si>
-  <si>
     <t>Reste à tester, mais semble fonctionner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajouter le score de chaque joueur scores: component panel utilisé et customisé pour les scores </t>
+  </si>
+  <si>
+    <t>Mise a jour useGameSync pour récupérer les scores depuis le serveur</t>
+  </si>
+  <si>
+    <t>Fixer le problème de décalage du plateau pendant le combat</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1206,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="28">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1439,9 +1438,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1479,7 +1478,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1585,7 +1584,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1727,7 +1726,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1739,26 +1738,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="42.85546875" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.7" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:5" ht="46.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1772,7 +1771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="50" t="s">
         <v>141</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="54" t="s">
         <v>111</v>
       </c>
@@ -1800,7 +1799,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="55" t="s">
         <v>112</v>
       </c>
@@ -1814,7 +1813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="55" t="s">
         <v>113</v>
       </c>
@@ -1828,7 +1827,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="55" t="s">
         <v>114</v>
       </c>
@@ -1842,7 +1841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="55" t="s">
         <v>116</v>
       </c>
@@ -1856,7 +1855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="55" t="s">
         <v>117</v>
       </c>
@@ -1870,7 +1869,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="55" t="s">
         <v>118</v>
       </c>
@@ -1884,7 +1883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="55" t="s">
         <v>145</v>
       </c>
@@ -1898,7 +1897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="55" t="s">
         <v>121</v>
       </c>
@@ -1912,7 +1911,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="55" t="s">
         <v>122</v>
       </c>
@@ -1926,7 +1925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="55" t="s">
         <v>124</v>
       </c>
@@ -1940,7 +1939,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="55" t="s">
         <v>130</v>
       </c>
@@ -1954,7 +1953,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="51" t="s">
         <v>119</v>
       </c>
@@ -1968,7 +1967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="51" t="s">
         <v>120</v>
       </c>
@@ -1982,7 +1981,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="51" t="s">
         <v>125</v>
       </c>
@@ -1996,7 +1995,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="51" t="s">
         <v>126</v>
       </c>
@@ -2010,7 +2009,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="51" t="s">
         <v>127</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="51" t="s">
         <v>129</v>
       </c>
@@ -2038,7 +2037,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="51" t="s">
         <v>133</v>
       </c>
@@ -2052,7 +2051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="51" t="s">
         <v>134</v>
       </c>
@@ -2066,7 +2065,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="51" t="s">
         <v>135</v>
       </c>
@@ -2080,7 +2079,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="56" t="s">
         <v>128</v>
       </c>
@@ -2094,7 +2093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="56" t="s">
         <v>131</v>
       </c>
@@ -2108,7 +2107,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="56" t="s">
         <v>123</v>
       </c>
@@ -2122,7 +2121,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="56" t="s">
         <v>132</v>
       </c>
@@ -2136,7 +2135,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="56" t="s">
         <v>136</v>
       </c>
@@ -2150,7 +2149,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="56" t="s">
         <v>137</v>
       </c>
@@ -2164,7 +2163,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="56" t="s">
         <v>138</v>
       </c>
@@ -2178,7 +2177,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="56" t="s">
         <v>139</v>
       </c>
@@ -2192,7 +2191,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="56" t="s">
         <v>140</v>
       </c>
@@ -2206,7 +2205,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="58" t="s">
         <v>115</v>
       </c>
@@ -2220,8 +2219,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="33" t="s">
         <v>146</v>
       </c>
@@ -2233,7 +2232,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="26" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2256,32 +2255,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
-    <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
-    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="16.1796875" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2311,7 +2310,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2365,7 +2364,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="17" t="s">
         <v>95</v>
       </c>
@@ -2392,7 +2391,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="20" t="s">
         <v>94</v>
       </c>
@@ -2414,7 +2413,7 @@
       <c r="P6" s="25"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="20" t="s">
         <v>96</v>
       </c>
@@ -2441,7 +2440,7 @@
       <c r="P7" s="25"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="20" t="s">
         <v>102</v>
       </c>
@@ -2474,7 +2473,7 @@
       <c r="P8" s="25"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="20" t="s">
         <v>97</v>
       </c>
@@ -2511,7 +2510,7 @@
       </c>
       <c r="R9" s="22"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="20" t="s">
         <v>101</v>
       </c>
@@ -2548,7 +2547,7 @@
       </c>
       <c r="R10" s="22"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="20" t="s">
         <v>99</v>
       </c>
@@ -2580,7 +2579,7 @@
       </c>
       <c r="R11" s="22"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="20" t="s">
         <v>100</v>
       </c>
@@ -2608,7 +2607,7 @@
       <c r="P12" s="25"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="39" t="s">
         <v>98</v>
       </c>
@@ -2635,15 +2634,15 @@
       <c r="Q13" s="38"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="16"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="16"/>
       <c r="P25" s="16"/>
       <c r="S25" s="16"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="16"/>
       <c r="P26" s="16"/>
       <c r="S26" s="16"/>
@@ -2659,24 +2658,24 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="77.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.54296875" customWidth="1"/>
+    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B3" s="63" t="s">
         <v>6</v>
       </c>
@@ -2691,8 +2690,8 @@
       <c r="K3" s="64"/>
       <c r="L3" s="65"/>
     </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B5" s="66" t="s">
         <v>1</v>
       </c>
@@ -2727,7 +2726,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="67"/>
       <c r="C6" s="69"/>
       <c r="D6" s="44" t="s">
@@ -2752,7 +2751,7 @@
       </c>
       <c r="L6" s="71"/>
     </row>
-    <row r="7" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="29" t="s">
         <v>24</v>
       </c>
@@ -2775,7 +2774,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="30" t="s">
         <v>35</v>
       </c>
@@ -2794,7 +2793,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="30" t="s">
         <v>36</v>
       </c>
@@ -2813,7 +2812,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="30" t="s">
         <v>75</v>
       </c>
@@ -2832,7 +2831,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="30" t="s">
         <v>154</v>
       </c>
@@ -2851,7 +2850,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="30" t="s">
         <v>25</v>
       </c>
@@ -2870,7 +2869,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="30" t="s">
         <v>26</v>
       </c>
@@ -2889,7 +2888,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="30" t="s">
         <v>27</v>
       </c>
@@ -2908,7 +2907,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="30" t="s">
         <v>152</v>
       </c>
@@ -2927,7 +2926,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="30" t="s">
         <v>29</v>
       </c>
@@ -2946,7 +2945,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="30" t="s">
         <v>30</v>
       </c>
@@ -2965,7 +2964,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="30" t="s">
         <v>150</v>
       </c>
@@ -2984,7 +2983,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="30" t="s">
         <v>151</v>
       </c>
@@ -3003,7 +3002,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="48" t="s">
         <v>159</v>
       </c>
@@ -3022,7 +3021,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="30" t="s">
         <v>91</v>
       </c>
@@ -3043,7 +3042,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="30" t="s">
         <v>51</v>
       </c>
@@ -3062,7 +3061,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="30" t="s">
         <v>90</v>
       </c>
@@ -3083,7 +3082,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="30" t="s">
         <v>74</v>
       </c>
@@ -3102,7 +3101,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="30" t="s">
         <v>80</v>
       </c>
@@ -3121,7 +3120,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="30" t="s">
         <v>92</v>
       </c>
@@ -3142,7 +3141,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="30" t="s">
         <v>93</v>
       </c>
@@ -3163,7 +3162,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="30" t="s">
         <v>79</v>
       </c>
@@ -3184,7 +3183,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="30" t="s">
         <v>76</v>
       </c>
@@ -3203,7 +3202,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="30" t="s">
         <v>174</v>
       </c>
@@ -3222,7 +3221,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="30" t="s">
         <v>42</v>
       </c>
@@ -3241,7 +3240,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="30" t="s">
         <v>43</v>
       </c>
@@ -3260,7 +3259,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="30" t="s">
         <v>153</v>
       </c>
@@ -3279,7 +3278,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="30" t="s">
         <v>156</v>
       </c>
@@ -3298,7 +3297,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="30" t="s">
         <v>73</v>
       </c>
@@ -3317,7 +3316,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="30" t="s">
         <v>38</v>
       </c>
@@ -3336,7 +3335,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="30" t="s">
         <v>39</v>
       </c>
@@ -3355,7 +3354,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="30" t="s">
         <v>170</v>
       </c>
@@ -3374,7 +3373,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="30" t="s">
         <v>171</v>
       </c>
@@ -3393,7 +3392,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="30" t="s">
         <v>168</v>
       </c>
@@ -3412,7 +3411,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="30" t="s">
         <v>169</v>
       </c>
@@ -3431,7 +3430,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="30" t="s">
         <v>166</v>
       </c>
@@ -3450,7 +3449,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="30" t="s">
         <v>165</v>
       </c>
@@ -3469,7 +3468,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="30" t="s">
         <v>161</v>
       </c>
@@ -3488,7 +3487,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="30" t="s">
         <v>160</v>
       </c>
@@ -3507,7 +3506,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="30" t="s">
         <v>164</v>
       </c>
@@ -3526,7 +3525,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="30" t="s">
         <v>172</v>
       </c>
@@ -3545,7 +3544,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="60" t="s">
         <v>163</v>
       </c>
@@ -3575,67 +3574,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="25" priority="7">
+    <cfRule type="expression" dxfId="26" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="24" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="23" priority="32">
+    <cfRule type="expression" dxfId="24" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="38">
+    <cfRule type="expression" dxfId="23" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="21" priority="30">
+    <cfRule type="expression" dxfId="22" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="20" priority="6">
+    <cfRule type="expression" dxfId="21" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="19" priority="25">
+    <cfRule type="expression" dxfId="20" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="27">
+    <cfRule type="expression" dxfId="19" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="17" priority="8">
+    <cfRule type="expression" dxfId="18" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="16" priority="13">
+    <cfRule type="expression" dxfId="17" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="14">
+    <cfRule type="expression" dxfId="16" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="14" priority="20">
+    <cfRule type="expression" dxfId="15" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="21">
+    <cfRule type="expression" dxfId="14" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="12" priority="9">
+    <cfRule type="expression" dxfId="13" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="10">
+    <cfRule type="expression" dxfId="12" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3649,24 +3648,24 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="B1:L71"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:L73"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
     <col min="7" max="7" width="16" style="32" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="32" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" style="32" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.81640625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
       <c r="B1" s="63" t="s">
         <v>16</v>
       </c>
@@ -3681,8 +3680,8 @@
       <c r="K1" s="64"/>
       <c r="L1" s="65"/>
     </row>
-    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
       <c r="B4" s="66" t="s">
         <v>1</v>
       </c>
@@ -3717,7 +3716,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="67"/>
       <c r="C5" s="69"/>
       <c r="D5" s="44" t="s">
@@ -3742,7 +3741,7 @@
       </c>
       <c r="L5" s="71"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="30" t="s">
         <v>177</v>
       </c>
@@ -3760,7 +3759,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="30" t="s">
         <v>178</v>
       </c>
@@ -3778,7 +3777,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="30" t="s">
         <v>179</v>
       </c>
@@ -3796,7 +3795,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="30" t="s">
         <v>162</v>
       </c>
@@ -3814,7 +3813,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="30" t="s">
         <v>176</v>
       </c>
@@ -3832,7 +3831,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="30" t="s">
         <v>175</v>
       </c>
@@ -3850,7 +3849,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="30" t="s">
         <v>167</v>
       </c>
@@ -3868,7 +3867,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="30" t="s">
         <v>173</v>
       </c>
@@ -3886,7 +3885,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="30" t="s">
         <v>180</v>
       </c>
@@ -3904,7 +3903,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="30" t="s">
         <v>181</v>
       </c>
@@ -3922,7 +3921,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="30" t="s">
         <v>183</v>
       </c>
@@ -3940,7 +3939,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="30" t="s">
         <v>187</v>
       </c>
@@ -3958,7 +3957,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="30" t="s">
         <v>188</v>
       </c>
@@ -3976,7 +3975,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="30" t="s">
         <v>189</v>
       </c>
@@ -3994,7 +3993,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="30" t="s">
         <v>200</v>
       </c>
@@ -4013,7 +4012,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="30" t="s">
         <v>190</v>
       </c>
@@ -4032,7 +4031,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="30" t="s">
         <v>201</v>
       </c>
@@ -4051,7 +4050,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="30" t="s">
         <v>197</v>
       </c>
@@ -4070,7 +4069,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="30" t="s">
         <v>191</v>
       </c>
@@ -4089,7 +4088,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="30" t="s">
         <v>203</v>
       </c>
@@ -4108,7 +4107,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="30" t="s">
         <v>192</v>
       </c>
@@ -4127,7 +4126,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="30" t="s">
         <v>193</v>
       </c>
@@ -4146,7 +4145,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="30" t="s">
         <v>194</v>
       </c>
@@ -4165,7 +4164,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="30" t="s">
         <v>195</v>
       </c>
@@ -4184,7 +4183,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="30" t="s">
         <v>199</v>
       </c>
@@ -4203,7 +4202,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="30" t="s">
         <v>196</v>
       </c>
@@ -4222,7 +4221,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="30" t="s">
         <v>198</v>
       </c>
@@ -4241,7 +4240,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="30" t="s">
         <v>202</v>
       </c>
@@ -4260,7 +4259,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="30" t="s">
         <v>205</v>
       </c>
@@ -4281,7 +4280,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="30" t="s">
         <v>210</v>
       </c>
@@ -4301,7 +4300,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="30" t="s">
         <v>209</v>
       </c>
@@ -4321,7 +4320,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="30" t="s">
         <v>211</v>
       </c>
@@ -4341,7 +4340,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="30" t="s">
         <v>212</v>
       </c>
@@ -4361,7 +4360,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="30" t="s">
         <v>214</v>
       </c>
@@ -4373,14 +4372,17 @@
       <c r="F39" s="11"/>
       <c r="G39" s="25"/>
       <c r="I39" s="11"/>
-      <c r="K39" t="s">
-        <v>213</v>
+      <c r="J39">
+        <v>2</v>
+      </c>
+      <c r="K39">
+        <v>100</v>
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="30" t="s">
-        <v>182</v>
+        <v>215</v>
       </c>
       <c r="C40" s="30" t="s">
         <v>104</v>
@@ -4390,11 +4392,17 @@
       <c r="F40" s="11"/>
       <c r="G40" s="25"/>
       <c r="I40" s="11"/>
+      <c r="J40">
+        <v>0.75</v>
+      </c>
+      <c r="K40">
+        <v>100</v>
+      </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="30" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="C41" s="30" t="s">
         <v>104</v>
@@ -4404,11 +4412,17 @@
       <c r="F41" s="11"/>
       <c r="G41" s="25"/>
       <c r="I41" s="11"/>
+      <c r="J41">
+        <v>0.3</v>
+      </c>
+      <c r="K41">
+        <v>100</v>
+      </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="30" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="C42" s="30" t="s">
         <v>104</v>
@@ -4418,11 +4432,17 @@
       <c r="F42" s="11"/>
       <c r="G42" s="25"/>
       <c r="I42" s="11"/>
+      <c r="J42">
+        <v>0.5</v>
+      </c>
+      <c r="K42">
+        <v>100</v>
+      </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="30" t="s">
-        <v>45</v>
+        <v>182</v>
       </c>
       <c r="C43" s="30" t="s">
         <v>104</v>
@@ -4434,9 +4454,9 @@
       <c r="I43" s="11"/>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="30" t="s">
-        <v>41</v>
+        <v>204</v>
       </c>
       <c r="C44" s="30" t="s">
         <v>104</v>
@@ -4448,9 +4468,9 @@
       <c r="I44" s="11"/>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="30" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C45" s="30" t="s">
         <v>104</v>
@@ -4462,9 +4482,9 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="30" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="C46" s="30" t="s">
         <v>104</v>
@@ -4476,9 +4496,9 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="30" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="C47" s="30" t="s">
         <v>104</v>
@@ -4490,9 +4510,9 @@
       <c r="I47" s="11"/>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="30" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C48" s="30" t="s">
         <v>104</v>
@@ -4504,45 +4524,37 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B49" s="60" t="s">
-        <v>186</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D49" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="E49" s="32">
-        <v>100</v>
-      </c>
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B49" s="30" t="s">
+        <v>108</v>
+      </c>
+      <c r="C49" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D49" s="25"/>
+      <c r="E49" s="32"/>
       <c r="F49" s="11"/>
       <c r="G49" s="25"/>
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B50" s="60" t="s">
-        <v>85</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D50" s="25">
-        <v>1</v>
-      </c>
-      <c r="E50" s="32">
-        <v>100</v>
-      </c>
+    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B50" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="25"/>
+      <c r="E50" s="32"/>
       <c r="F50" s="11"/>
       <c r="G50" s="25"/>
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B51" s="60" t="s">
-        <v>83</v>
+        <v>186</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>105</v>
@@ -4558,15 +4570,15 @@
       <c r="I51" s="11"/>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B52" s="60" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>105</v>
       </c>
       <c r="D52" s="25">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E52" s="32">
         <v>100</v>
@@ -4576,9 +4588,9 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B53" s="60" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C53" s="7" t="s">
         <v>105</v>
@@ -4594,28 +4606,27 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B54" s="60" t="s">
-        <v>184</v>
+        <v>62</v>
       </c>
       <c r="C54" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D54" s="25"/>
-      <c r="E54" s="32"/>
+      <c r="D54" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="E54" s="32">
+        <v>100</v>
+      </c>
       <c r="F54" s="11"/>
-      <c r="G54" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="H54" s="32">
-        <v>25</v>
-      </c>
+      <c r="G54" s="25"/>
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B55" s="60" t="s">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="C55" s="7" t="s">
         <v>105</v>
@@ -4631,27 +4642,28 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B56" s="60" t="s">
-        <v>59</v>
+        <v>184</v>
       </c>
       <c r="C56" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D56" s="25">
-        <v>0.75</v>
-      </c>
-      <c r="E56" s="32">
-        <v>100</v>
-      </c>
+      <c r="D56" s="25"/>
+      <c r="E56" s="32"/>
       <c r="F56" s="11"/>
-      <c r="G56" s="25"/>
+      <c r="G56" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="H56" s="32">
+        <v>25</v>
+      </c>
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B57" s="60" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>105</v>
@@ -4667,135 +4679,171 @@
       <c r="I57" s="11"/>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B58" s="60" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>105</v>
       </c>
       <c r="D58" s="25">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E58" s="32">
         <v>100</v>
       </c>
-    </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F58" s="11"/>
+      <c r="G58" s="25"/>
+      <c r="I58" s="11"/>
+      <c r="L58" s="11"/>
+    </row>
+    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B59" s="60" t="s">
-        <v>185</v>
+        <v>60</v>
       </c>
       <c r="C59" s="7" t="s">
         <v>105</v>
       </c>
       <c r="D59" s="25">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="E59" s="32">
         <v>100</v>
       </c>
-    </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="F59" s="11"/>
+      <c r="G59" s="25"/>
+      <c r="I59" s="11"/>
+      <c r="L59" s="11"/>
+    </row>
+    <row r="60" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B60" s="60" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C60" s="7" t="s">
         <v>105</v>
       </c>
       <c r="D60" s="25">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E60" s="32">
-        <v>75</v>
-      </c>
-      <c r="J60">
-        <v>1</v>
-      </c>
-      <c r="K60">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B61" s="60" t="s">
-        <v>66</v>
+        <v>185</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D61" s="25"/>
-      <c r="G61" s="32">
-        <v>2</v>
-      </c>
-      <c r="H61" s="32">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D61" s="25">
+        <v>0.25</v>
+      </c>
+      <c r="E61" s="32">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B62" s="60" t="s">
-        <v>206</v>
+        <v>65</v>
       </c>
       <c r="C62" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D62" s="25"/>
-      <c r="G62" s="32">
+      <c r="D62" s="25">
         <v>1.5</v>
       </c>
-      <c r="H62" s="32">
+      <c r="E62" s="32">
         <v>75</v>
       </c>
-      <c r="I62" t="s">
+      <c r="J62">
+        <v>1</v>
+      </c>
+      <c r="K62">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B63" s="60" t="s">
+        <v>66</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D63" s="25"/>
+      <c r="G63" s="32">
+        <v>2</v>
+      </c>
+      <c r="H63" s="32">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B64" s="60" t="s">
+        <v>206</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D64" s="25"/>
+      <c r="G64" s="32">
+        <v>1.5</v>
+      </c>
+      <c r="H64" s="32">
+        <v>75</v>
+      </c>
+      <c r="I64" t="s">
         <v>207</v>
       </c>
-      <c r="K62">
-        <v>100</v>
-      </c>
-      <c r="L62" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="63" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B63" s="60"/>
-      <c r="C63" s="7"/>
-      <c r="D63" s="25"/>
-    </row>
-    <row r="64" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B64" s="60"/>
-      <c r="C64" s="7"/>
-      <c r="D64" s="25"/>
-    </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="K64">
+        <v>100</v>
+      </c>
+      <c r="L64" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B65" s="60"/>
       <c r="C65" s="7"/>
       <c r="D65" s="25"/>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B66" s="60"/>
       <c r="C66" s="7"/>
       <c r="D66" s="25"/>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B67" s="60"/>
       <c r="C67" s="7"/>
       <c r="D67" s="25"/>
     </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B68" s="60"/>
       <c r="C68" s="7"/>
       <c r="D68" s="25"/>
     </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B69" s="60"/>
       <c r="C69" s="7"/>
       <c r="D69" s="25"/>
     </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B70" s="60"/>
+      <c r="C70" s="7"/>
       <c r="D70" s="25"/>
     </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B71" s="60"/>
+      <c r="C71" s="7"/>
       <c r="D71" s="25"/>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B72" s="60"/>
+      <c r="D72" s="25"/>
+    </row>
+    <row r="73" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="B73" s="60"/>
+      <c r="D73" s="25"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:L5" xr:uid="{2EE69061-1192-400C-B500-1B4897FD0585}"/>
@@ -4808,30 +4856,35 @@
     <mergeCell ref="L4:L5"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="B1 B4:B64">
-    <cfRule type="expression" dxfId="10" priority="45">
+  <conditionalFormatting sqref="B1 B4:B66">
+    <cfRule type="expression" dxfId="11" priority="45">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
-    <cfRule type="expression" dxfId="9" priority="85">
+  <conditionalFormatting sqref="B42">
+    <cfRule type="expression" dxfId="10" priority="85">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B65:B71">
-    <cfRule type="expression" dxfId="8" priority="6">
-      <formula>MAX($E65,$H65,$K65)=100</formula>
+  <conditionalFormatting sqref="B67:B73">
+    <cfRule type="expression" dxfId="9" priority="6">
+      <formula>MAX($E67,$H67,$K67)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1 C4:C69">
-    <cfRule type="expression" dxfId="7" priority="42">
+  <conditionalFormatting sqref="C1 C4:C71">
+    <cfRule type="expression" dxfId="8" priority="42">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="43">
+    <cfRule type="expression" dxfId="7" priority="43">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="44">
+    <cfRule type="expression" dxfId="6" priority="44">
       <formula>$C1="Eddy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B42">
+    <cfRule type="expression" dxfId="0" priority="94">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4845,21 +4898,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E40"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
-    <col min="2" max="2" width="70.85546875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="70.81640625" customWidth="1"/>
     <col min="3" max="3" width="81" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" customWidth="1"/>
+    <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="8" t="s">
         <v>22</v>
       </c>
@@ -4873,151 +4926,151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
@@ -5033,25 +5086,25 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
-    <col min="2" max="2" width="51.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.140625" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="51.54296875" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.81640625" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="72" t="s">
         <v>17</v>
       </c>
@@ -5069,8 +5122,8 @@
       <c r="N2" s="73"/>
       <c r="O2" s="73"/>
     </row>
-    <row r="4" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:15" ht="21" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:15" ht="21" x14ac:dyDescent="0.5">
       <c r="B5" s="66" t="s">
         <v>1</v>
       </c>
@@ -5114,7 +5167,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B6" s="67"/>
       <c r="C6" s="69"/>
       <c r="D6" s="44" t="s">
@@ -5146,7 +5199,7 @@
       </c>
       <c r="O6" s="71"/>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="29"/>
       <c r="C7" s="29"/>
       <c r="D7" s="27"/>
@@ -5162,7 +5215,7 @@
       <c r="N7" s="9"/>
       <c r="O7" s="10"/>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="30"/>
       <c r="C8" s="30"/>
       <c r="D8" s="25"/>
@@ -5174,7 +5227,7 @@
       <c r="L8" s="11"/>
       <c r="O8" s="11"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="30"/>
       <c r="C9" s="30"/>
       <c r="D9" s="25"/>
@@ -5186,7 +5239,7 @@
       <c r="L9" s="11"/>
       <c r="O9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="30"/>
       <c r="C10" s="30"/>
       <c r="D10" s="25"/>
@@ -5198,7 +5251,7 @@
       <c r="L10" s="11"/>
       <c r="O10" s="11"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="30"/>
       <c r="C11" s="30"/>
       <c r="D11" s="25"/>
@@ -5210,7 +5263,7 @@
       <c r="L11" s="11"/>
       <c r="O11" s="11"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="30"/>
       <c r="C12" s="30"/>
       <c r="D12" s="25"/>
@@ -5222,7 +5275,7 @@
       <c r="L12" s="11"/>
       <c r="O12" s="11"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="30"/>
       <c r="C13" s="30"/>
       <c r="D13" s="25"/>
@@ -5234,7 +5287,7 @@
       <c r="L13" s="11"/>
       <c r="O13" s="11"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="30"/>
       <c r="C14" s="30"/>
       <c r="D14" s="25"/>
@@ -5246,7 +5299,7 @@
       <c r="L14" s="11"/>
       <c r="O14" s="11"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="30"/>
       <c r="C15" s="30"/>
       <c r="D15" s="25"/>
@@ -5258,7 +5311,7 @@
       <c r="L15" s="11"/>
       <c r="O15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="30"/>
       <c r="C16" s="30"/>
       <c r="D16" s="25"/>
@@ -5270,7 +5323,7 @@
       <c r="L16" s="11"/>
       <c r="O16" s="11"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="30"/>
       <c r="C17" s="30"/>
       <c r="D17" s="25"/>
@@ -5282,7 +5335,7 @@
       <c r="L17" s="11"/>
       <c r="O17" s="11"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="30"/>
       <c r="C18" s="30"/>
       <c r="D18" s="25"/>
@@ -5294,7 +5347,7 @@
       <c r="L18" s="11"/>
       <c r="O18" s="11"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="30"/>
       <c r="C19" s="30"/>
       <c r="D19" s="25"/>
@@ -5306,7 +5359,7 @@
       <c r="L19" s="11"/>
       <c r="O19" s="11"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="48"/>
       <c r="C20" s="30"/>
       <c r="D20" s="25"/>
@@ -5318,7 +5371,7 @@
       <c r="L20" s="11"/>
       <c r="O20" s="11"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="30"/>
       <c r="C21" s="30"/>
       <c r="D21" s="25"/>
@@ -5330,7 +5383,7 @@
       <c r="L21" s="11"/>
       <c r="O21" s="11"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="30"/>
       <c r="C22" s="30"/>
       <c r="D22" s="25"/>
@@ -5342,7 +5395,7 @@
       <c r="L22" s="11"/>
       <c r="O22" s="11"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="30"/>
       <c r="C23" s="30"/>
       <c r="D23" s="25"/>
@@ -5354,7 +5407,7 @@
       <c r="L23" s="11"/>
       <c r="O23" s="11"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="30"/>
       <c r="C24" s="30"/>
       <c r="D24" s="32"/>
@@ -5366,7 +5419,7 @@
       <c r="L24" s="11"/>
       <c r="O24" s="11"/>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B25" s="30"/>
       <c r="C25" s="30"/>
       <c r="D25" s="25"/>
@@ -5378,7 +5431,7 @@
       <c r="L25" s="11"/>
       <c r="O25" s="11"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="30"/>
       <c r="C26" s="30"/>
       <c r="D26" s="25"/>
@@ -5390,7 +5443,7 @@
       <c r="L26" s="11"/>
       <c r="O26" s="11"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="30"/>
       <c r="C27" s="30"/>
       <c r="D27" s="25"/>
@@ -5402,7 +5455,7 @@
       <c r="L27" s="11"/>
       <c r="O27" s="11"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="30"/>
       <c r="C28" s="30"/>
       <c r="D28" s="25"/>
@@ -5414,7 +5467,7 @@
       <c r="L28" s="11"/>
       <c r="O28" s="11"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="14"/>
       <c r="C29" s="30"/>
       <c r="D29" s="25"/>
@@ -5426,7 +5479,7 @@
       <c r="L29" s="11"/>
       <c r="O29" s="11"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="30"/>
       <c r="C30" s="30"/>
       <c r="D30" s="25"/>
@@ -5438,7 +5491,7 @@
       <c r="L30" s="11"/>
       <c r="O30" s="11"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="30"/>
       <c r="C31" s="30"/>
       <c r="D31" s="25"/>
@@ -5450,7 +5503,7 @@
       <c r="L31" s="11"/>
       <c r="O31" s="11"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="30"/>
       <c r="C32" s="30"/>
       <c r="D32" s="25"/>
@@ -5462,7 +5515,7 @@
       <c r="L32" s="11"/>
       <c r="O32" s="11"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="30"/>
       <c r="C33" s="30"/>
       <c r="D33" s="25"/>
@@ -5474,7 +5527,7 @@
       <c r="L33" s="11"/>
       <c r="O33" s="11"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="30"/>
       <c r="C34" s="30"/>
       <c r="D34" s="25"/>
@@ -5486,7 +5539,7 @@
       <c r="L34" s="11"/>
       <c r="O34" s="11"/>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B35" s="30"/>
       <c r="C35" s="30"/>
       <c r="D35" s="25"/>
@@ -5498,7 +5551,7 @@
       <c r="L35" s="11"/>
       <c r="O35" s="11"/>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B36" s="30"/>
       <c r="C36" s="30"/>
       <c r="D36" s="25"/>
@@ -5510,7 +5563,7 @@
       <c r="L36" s="11"/>
       <c r="O36" s="11"/>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B37" s="30"/>
       <c r="C37" s="30"/>
       <c r="D37" s="25"/>
@@ -5522,7 +5575,7 @@
       <c r="L37" s="11"/>
       <c r="O37" s="11"/>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B38" s="30"/>
       <c r="C38" s="30"/>
       <c r="D38" s="25"/>
@@ -5534,7 +5587,7 @@
       <c r="L38" s="11"/>
       <c r="O38" s="11"/>
     </row>
-    <row r="39" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B39" s="31"/>
       <c r="C39" s="31"/>
       <c r="D39" s="26"/>
@@ -5561,23 +5614,23 @@
     <mergeCell ref="O5:O6"/>
   </mergeCells>
   <conditionalFormatting sqref="B2">
-    <cfRule type="expression" dxfId="4" priority="8">
+    <cfRule type="expression" dxfId="5" priority="8">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:B39">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="4" priority="4">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C39">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$C5="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$C5="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>$C5="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5591,28 +5644,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.140625" customWidth="1"/>
-    <col min="2" max="2" width="93.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1796875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" customWidth="1"/>
-    <col min="6" max="6" width="42.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.7" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>64</v>
       </c>
@@ -5629,7 +5682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -5642,7 +5695,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>23</v>
       </c>
@@ -5655,7 +5708,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
@@ -5668,7 +5721,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>26</v>
       </c>
@@ -5681,7 +5734,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -5694,7 +5747,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -5707,7 +5760,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -5720,7 +5773,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -5733,7 +5786,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5746,7 +5799,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
@@ -5759,7 +5812,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
@@ -5772,7 +5825,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>73</v>
       </c>
@@ -5785,7 +5838,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
@@ -5798,7 +5851,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>39</v>
       </c>
@@ -5811,7 +5864,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>42</v>
       </c>
@@ -5824,7 +5877,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -5837,7 +5890,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>44</v>
       </c>
@@ -5850,7 +5903,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>40</v>
       </c>
@@ -5863,7 +5916,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>41</v>
       </c>
@@ -5876,7 +5929,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
@@ -5889,7 +5942,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
@@ -5902,7 +5955,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -5915,7 +5968,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>82</v>
       </c>
@@ -5928,7 +5981,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>48</v>
       </c>
@@ -5941,7 +5994,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>49</v>
       </c>
@@ -5954,7 +6007,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
@@ -5967,7 +6020,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>50</v>
       </c>
@@ -5980,7 +6033,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>51</v>
       </c>
@@ -5993,7 +6046,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>62</v>
       </c>
@@ -6006,7 +6059,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>53</v>
       </c>
@@ -6019,7 +6072,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>55</v>
       </c>
@@ -6032,7 +6085,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -6045,7 +6098,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>56</v>
       </c>
@@ -6058,7 +6111,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>57</v>
       </c>
@@ -6071,7 +6124,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>58</v>
       </c>
@@ -6084,7 +6137,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>59</v>
       </c>
@@ -6097,7 +6150,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>60</v>
       </c>
@@ -6110,7 +6163,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>61</v>
       </c>
@@ -6123,7 +6176,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>63</v>
       </c>
@@ -6136,7 +6189,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>65</v>
       </c>
@@ -6149,7 +6202,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>66</v>
       </c>
@@ -6162,7 +6215,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>67</v>
       </c>
@@ -6175,7 +6228,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>88</v>
       </c>
@@ -6188,7 +6241,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>69</v>
       </c>
@@ -6201,7 +6254,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>70</v>
       </c>
@@ -6214,7 +6267,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>71</v>
       </c>
@@ -6227,7 +6280,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>74</v>
       </c>
@@ -6240,7 +6293,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>75</v>
       </c>
@@ -6253,7 +6306,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>76</v>
       </c>
@@ -6266,7 +6319,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>87</v>
       </c>
@@ -6279,7 +6332,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>78</v>
       </c>
@@ -6292,7 +6345,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>79</v>
       </c>
@@ -6305,7 +6358,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>80</v>
       </c>
@@ -6318,7 +6371,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>81</v>
       </c>
@@ -6331,7 +6384,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>83</v>
       </c>
@@ -6344,7 +6397,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>84</v>
       </c>
@@ -6357,7 +6410,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>85</v>
       </c>
@@ -6370,7 +6423,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>86</v>
       </c>
@@ -6383,7 +6436,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>77</v>
       </c>
@@ -6396,7 +6449,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>94</v>
       </c>
@@ -6407,7 +6460,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>95</v>
       </c>
@@ -6418,7 +6471,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>96</v>
       </c>
@@ -6429,7 +6482,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>97</v>
       </c>
@@ -6440,7 +6493,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>98</v>
       </c>
@@ -6451,7 +6504,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>99</v>
       </c>
@@ -6462,7 +6515,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>100</v>
       </c>
@@ -6473,7 +6526,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>101</v>
       </c>
@@ -6484,7 +6537,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>102</v>
       </c>
@@ -6495,7 +6548,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
         <v>109</v>
       </c>
@@ -6506,7 +6559,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
         <v>110</v>
       </c>
@@ -6517,182 +6570,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
planification après rencontre prof
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44B76CC-FC9F-4170-8010-8310BB854698}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC3A9F7F-AF37-4BED-AEDD-FF941FCAF237}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" activeTab="3" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" activeTab="4" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="238">
   <si>
     <t>Planification globale</t>
   </si>
@@ -102,12 +102,6 @@
     <t>Mi-mandat</t>
   </si>
   <si>
-    <t>Ce qui doit être fait…</t>
-  </si>
-  <si>
-    <t>Ce qui est problématique…</t>
-  </si>
-  <si>
     <t>Création de la base de données MySQL et des tables</t>
   </si>
   <si>
@@ -730,6 +724,33 @@
   </si>
   <si>
     <t>Implémenter le MCTS de base</t>
+  </si>
+  <si>
+    <t>À Faire</t>
+  </si>
+  <si>
+    <t>Comment Faire</t>
+  </si>
+  <si>
+    <t>Jouer contre un joueur</t>
+  </si>
+  <si>
+    <t>Raffiner modèle AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajouter l'option dans le front end quand on commence une partie. Valider avec le back-end si ça fonctionne toujours </t>
+  </si>
+  <si>
+    <t>Ajouter les priors, modifier les fonctions heuristiques d'évaluation et de simulation, ajouter les fonctions de setup de pièces</t>
+  </si>
+  <si>
+    <t>Tutoriel</t>
+  </si>
+  <si>
+    <t>Enregistrer le vidéo de tutoriel, ajouter les commentaires, ajouter le vidéo dans le front end</t>
+  </si>
+  <si>
+    <t>Tout le monde</t>
   </si>
 </sst>
 </file>
@@ -1113,7 +1134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1207,6 +1228,9 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1240,38 +1264,22 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="36">
+  <dxfs count="38">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -1340,6 +1348,39 @@
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -1875,13 +1916,13 @@
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="48" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C6" s="51" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E6" s="10">
         <v>10</v>
@@ -1889,13 +1930,13 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="52" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E7" s="11">
         <v>4</v>
@@ -1903,13 +1944,13 @@
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="53" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E8" s="11">
         <v>4</v>
@@ -1917,13 +1958,13 @@
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="53" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E9" s="11">
         <v>2</v>
@@ -1931,13 +1972,13 @@
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="53" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E10" s="11">
         <v>1</v>
@@ -1945,13 +1986,13 @@
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="53" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C11" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E11" s="11">
         <v>1</v>
@@ -1959,13 +2000,13 @@
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="53" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E12" s="11">
         <v>3</v>
@@ -1973,13 +2014,13 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="53" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E13" s="11">
         <v>3</v>
@@ -1987,13 +2028,13 @@
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="53" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E14" s="11">
         <v>2</v>
@@ -2001,13 +2042,13 @@
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="53" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E15" s="11">
         <v>4</v>
@@ -2015,13 +2056,13 @@
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="53" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E16" s="11">
         <v>1</v>
@@ -2029,13 +2070,13 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="53" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E17" s="11">
         <v>2</v>
@@ -2043,13 +2084,13 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="53" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E18" s="11">
         <v>1.5</v>
@@ -2057,13 +2098,13 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="49" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C19" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E19" s="11">
         <v>3</v>
@@ -2071,13 +2112,13 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="49" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C20" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E20" s="11">
         <v>4</v>
@@ -2085,13 +2126,13 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="49" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C21" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E21" s="11">
         <v>3</v>
@@ -2099,13 +2140,13 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="49" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C22" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E22" s="11">
         <v>2</v>
@@ -2113,13 +2154,13 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="49" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E23" s="11">
         <v>4</v>
@@ -2127,13 +2168,13 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="49" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C24" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E24" s="11">
         <v>1.5</v>
@@ -2141,13 +2182,13 @@
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="49" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C25" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E25" s="11">
         <v>5</v>
@@ -2155,13 +2196,13 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="49" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C26" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E26" s="11">
         <v>3</v>
@@ -2169,13 +2210,13 @@
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="49" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C27" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E27" s="11">
         <v>7</v>
@@ -2183,13 +2224,13 @@
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="54" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C28" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E28" s="11">
         <v>1</v>
@@ -2197,13 +2238,13 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="54" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C29" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E29" s="11">
         <v>3.5</v>
@@ -2211,13 +2252,13 @@
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C30" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E30" s="11">
         <v>4</v>
@@ -2225,13 +2266,13 @@
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="54" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C31" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E31" s="11">
         <v>3</v>
@@ -2239,13 +2280,13 @@
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="54" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C32" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E32" s="11">
         <v>2</v>
@@ -2253,13 +2294,13 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="54" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C33" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E33" s="11">
         <v>4</v>
@@ -2267,13 +2308,13 @@
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="54" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C34" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E34" s="11">
         <v>4</v>
@@ -2281,13 +2322,13 @@
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="54" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C35" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E35" s="11">
         <v>4</v>
@@ -2295,13 +2336,13 @@
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="54" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C36" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E36" s="11">
         <v>3</v>
@@ -2309,13 +2350,13 @@
     </row>
     <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="56" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C37" s="57" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E37" s="13">
         <v>2</v>
@@ -2324,7 +2365,7 @@
     <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="32" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E39" s="33">
         <f>SUM(E6:E37)</f>
@@ -2334,7 +2375,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="35" priority="1">
+    <cfRule type="expression" dxfId="37" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2407,7 +2448,7 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
@@ -2468,13 +2509,13 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="16" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E5" s="17">
         <v>1</v>
@@ -2495,15 +2536,15 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D6" s="24"/>
       <c r="F6" s="11"/>
       <c r="G6" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H6" s="20">
         <v>1</v>
@@ -2517,22 +2558,22 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="19" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D7" s="24"/>
       <c r="F7" s="11"/>
       <c r="G7" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H7" s="15">
         <v>0.6</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K7" s="20">
         <v>1</v>
@@ -2544,29 +2585,29 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" s="24"/>
       <c r="F8" s="11"/>
       <c r="G8" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H8" s="15">
         <v>0.6</v>
       </c>
       <c r="I8" s="11"/>
       <c r="J8" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K8" s="15">
         <v>0.9</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N8" s="20">
         <v>1</v>
@@ -2577,35 +2618,35 @@
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="19" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D9" s="24"/>
       <c r="F9" s="11"/>
       <c r="G9" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H9" s="15">
         <v>0.3</v>
       </c>
       <c r="I9" s="11"/>
       <c r="J9" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K9" s="15">
         <v>0.7</v>
       </c>
       <c r="L9" s="11"/>
       <c r="M9" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N9" s="15">
         <v>0.9</v>
       </c>
       <c r="P9" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="Q9" s="20">
         <v>1</v>
@@ -2614,35 +2655,35 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D10" s="24"/>
       <c r="F10" s="11"/>
       <c r="G10" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H10" s="15">
         <v>0.2</v>
       </c>
       <c r="I10" s="11"/>
       <c r="J10" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K10" s="15">
         <v>0.6</v>
       </c>
       <c r="L10" s="11"/>
       <c r="M10" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N10" s="15">
         <v>0.9</v>
       </c>
       <c r="P10" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="Q10" s="20">
         <v>1</v>
@@ -2651,30 +2692,30 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="19" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D11" s="24"/>
       <c r="F11" s="11"/>
       <c r="G11" s="24"/>
       <c r="I11" s="11"/>
       <c r="J11" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K11" s="15">
         <v>0.3</v>
       </c>
       <c r="L11" s="11"/>
       <c r="M11" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N11" s="15">
         <v>0.9</v>
       </c>
       <c r="P11" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="Q11" s="20">
         <v>1</v>
@@ -2683,24 +2724,24 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="19" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D12" s="24"/>
       <c r="F12" s="11"/>
       <c r="G12" s="24"/>
       <c r="I12" s="11"/>
       <c r="J12" s="24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K12" s="15">
         <v>0.5</v>
       </c>
       <c r="L12" s="11"/>
       <c r="M12" s="27" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N12" s="20">
         <v>1</v>
@@ -2711,10 +2752,10 @@
     </row>
     <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="38" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D13" s="25"/>
       <c r="E13" s="12"/>
@@ -2726,7 +2767,7 @@
       <c r="K13" s="12"/>
       <c r="L13" s="13"/>
       <c r="M13" s="34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N13" s="35">
         <v>1</v>
@@ -2778,26 +2819,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="64"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="64" t="s">
+      <c r="B5" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="66" t="s">
+      <c r="C5" s="67" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -2806,7 +2847,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="68" t="s">
+      <c r="F5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -2815,7 +2856,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="68" t="s">
+      <c r="I5" s="69" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -2824,41 +2865,41 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="68" t="s">
+      <c r="L5" s="69" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="65"/>
-      <c r="C6" s="67"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="69"/>
+      <c r="F6" s="70"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="69"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="69"/>
+      <c r="L6" s="70"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D7" s="26">
         <v>3.5</v>
@@ -2867,7 +2908,7 @@
         <v>100</v>
       </c>
       <c r="F7" s="39" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="41"/>
@@ -2878,10 +2919,10 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" s="24">
         <v>1.5</v>
@@ -2897,10 +2938,10 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" s="24">
         <v>0.1</v>
@@ -2916,10 +2957,10 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D10" s="24">
         <v>0.5</v>
@@ -2935,10 +2976,10 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D11" s="24">
         <v>0.2</v>
@@ -2954,10 +2995,10 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D12" s="24"/>
       <c r="E12" s="31"/>
@@ -2973,10 +3014,10 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="31"/>
@@ -2992,10 +3033,10 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="31"/>
@@ -3011,10 +3052,10 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="31"/>
@@ -3030,10 +3071,10 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D16" s="24"/>
       <c r="E16" s="31"/>
@@ -3049,10 +3090,10 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D17" s="24"/>
       <c r="E17" s="31"/>
@@ -3068,10 +3109,10 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D18" s="24"/>
       <c r="E18" s="31"/>
@@ -3087,10 +3128,10 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D19" s="24"/>
       <c r="E19" s="31"/>
@@ -3106,10 +3147,10 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="46" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C20" s="47" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D20" s="24"/>
       <c r="E20" s="31"/>
@@ -3125,10 +3166,10 @@
     </row>
     <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D21" s="24"/>
       <c r="E21" s="31"/>
@@ -3140,16 +3181,16 @@
         <v>100</v>
       </c>
       <c r="I21" s="40" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="L21" s="11"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D22" s="24"/>
       <c r="E22" s="31"/>
@@ -3165,10 +3206,10 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D23" s="24"/>
       <c r="E23" s="31"/>
@@ -3180,16 +3221,16 @@
         <v>100</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="L23" s="11"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D24" s="31"/>
       <c r="E24" s="31"/>
@@ -3205,10 +3246,10 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D25" s="24"/>
       <c r="E25" s="31"/>
@@ -3224,10 +3265,10 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="31"/>
@@ -3239,16 +3280,16 @@
         <v>100</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="L26" s="11"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="31"/>
@@ -3260,16 +3301,16 @@
         <v>100</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="L27" s="11"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="31"/>
@@ -3281,16 +3322,16 @@
         <v>100</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L28" s="11"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D29" s="24"/>
       <c r="E29" s="31"/>
@@ -3306,10 +3347,10 @@
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D30" s="24"/>
       <c r="E30" s="31"/>
@@ -3325,10 +3366,10 @@
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C31" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D31" s="24"/>
       <c r="E31" s="31"/>
@@ -3344,10 +3385,10 @@
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D32" s="24"/>
       <c r="E32" s="31"/>
@@ -3363,10 +3404,10 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D33" s="24"/>
       <c r="E33" s="31"/>
@@ -3382,10 +3423,10 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D34" s="24"/>
       <c r="E34" s="31"/>
@@ -3401,10 +3442,10 @@
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D35" s="24"/>
       <c r="E35" s="31"/>
@@ -3420,10 +3461,10 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D36" s="24"/>
       <c r="E36" s="31"/>
@@ -3439,10 +3480,10 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D37" s="24"/>
       <c r="E37" s="31"/>
@@ -3458,10 +3499,10 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D38" s="24"/>
       <c r="E38" s="31"/>
@@ -3477,10 +3518,10 @@
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D39" s="24"/>
       <c r="E39" s="31"/>
@@ -3496,10 +3537,10 @@
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D40" s="24"/>
       <c r="E40" s="31"/>
@@ -3515,10 +3556,10 @@
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D41" s="24"/>
       <c r="E41" s="31"/>
@@ -3534,10 +3575,10 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D42" s="24"/>
       <c r="E42" s="31"/>
@@ -3553,10 +3594,10 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C43" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D43" s="24"/>
       <c r="E43" s="31"/>
@@ -3572,10 +3613,10 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C44" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D44" s="24"/>
       <c r="E44" s="31"/>
@@ -3591,10 +3632,10 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="29" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C45" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D45" s="24"/>
       <c r="E45" s="31"/>
@@ -3610,10 +3651,10 @@
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="29" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C46" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D46" s="24"/>
       <c r="E46" s="31"/>
@@ -3629,10 +3670,10 @@
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="29" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C47" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D47" s="24"/>
       <c r="E47" s="31"/>
@@ -3648,10 +3689,10 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C48" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D48" s="24"/>
       <c r="E48" s="31"/>
@@ -3676,67 +3717,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="34" priority="7">
+    <cfRule type="expression" dxfId="36" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="33" priority="1">
+    <cfRule type="expression" dxfId="35" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="32" priority="32">
+    <cfRule type="expression" dxfId="34" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="38">
+    <cfRule type="expression" dxfId="33" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="30" priority="30">
+    <cfRule type="expression" dxfId="32" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="29" priority="6">
+    <cfRule type="expression" dxfId="31" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="28" priority="25">
+    <cfRule type="expression" dxfId="30" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="27">
+    <cfRule type="expression" dxfId="29" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="26" priority="8">
+    <cfRule type="expression" dxfId="28" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="25" priority="13">
+    <cfRule type="expression" dxfId="27" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="14">
+    <cfRule type="expression" dxfId="26" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="23" priority="20">
+    <cfRule type="expression" dxfId="25" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="21">
+    <cfRule type="expression" dxfId="24" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="21" priority="9">
+    <cfRule type="expression" dxfId="23" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="10">
+    <cfRule type="expression" dxfId="22" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3768,26 +3809,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="64"/>
     </row>
     <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="67" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -3796,7 +3837,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="68" t="s">
+      <c r="F4" s="69" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -3805,7 +3846,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="68" t="s">
+      <c r="I4" s="69" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -3814,41 +3855,41 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="68" t="s">
+      <c r="L4" s="69" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="65"/>
-      <c r="C5" s="67"/>
+      <c r="B5" s="66"/>
+      <c r="C5" s="68"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="69"/>
+      <c r="F5" s="70"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="69"/>
+      <c r="I5" s="70"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="69"/>
+      <c r="L5" s="70"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="29" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D6" s="24">
         <v>0.5</v>
@@ -3863,10 +3904,10 @@
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D7" s="24">
         <v>0.5</v>
@@ -3881,10 +3922,10 @@
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" s="24">
         <v>0.75</v>
@@ -3899,10 +3940,10 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" s="24">
         <v>0.5</v>
@@ -3917,10 +3958,10 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D10" s="24">
         <v>0.75</v>
@@ -3935,10 +3976,10 @@
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D11" s="24">
         <v>1.5</v>
@@ -3953,10 +3994,10 @@
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D12" s="24">
         <v>1</v>
@@ -3971,10 +4012,10 @@
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D13" s="24">
         <v>0.75</v>
@@ -3989,10 +4030,10 @@
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D14" s="24">
         <v>1</v>
@@ -4007,10 +4048,10 @@
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D15" s="24">
         <v>0.05</v>
@@ -4025,10 +4066,10 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D16" s="24">
         <v>2</v>
@@ -4043,10 +4084,10 @@
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D17" s="24">
         <v>1</v>
@@ -4061,10 +4102,10 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D18" s="24">
         <v>0.25</v>
@@ -4079,10 +4120,10 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D19" s="24">
         <v>1</v>
@@ -4097,10 +4138,10 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D20" s="24"/>
       <c r="E20" s="31"/>
@@ -4116,10 +4157,10 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D21" s="24"/>
       <c r="E21" s="31"/>
@@ -4135,10 +4176,10 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D22" s="24"/>
       <c r="E22" s="31"/>
@@ -4154,10 +4195,10 @@
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C23" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D23" s="24"/>
       <c r="E23" s="31"/>
@@ -4173,10 +4214,10 @@
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D24" s="24"/>
       <c r="E24" s="31"/>
@@ -4192,10 +4233,10 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C25" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D25" s="24"/>
       <c r="E25" s="31"/>
@@ -4211,10 +4252,10 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D26" s="24"/>
       <c r="E26" s="31"/>
@@ -4230,10 +4271,10 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C27" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D27" s="24"/>
       <c r="E27" s="31"/>
@@ -4249,10 +4290,10 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D28" s="24"/>
       <c r="E28" s="31"/>
@@ -4268,10 +4309,10 @@
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D29" s="24"/>
       <c r="E29" s="31"/>
@@ -4287,10 +4328,10 @@
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D30" s="24"/>
       <c r="E30" s="31"/>
@@ -4306,10 +4347,10 @@
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C31" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D31" s="24"/>
       <c r="E31" s="31"/>
@@ -4325,10 +4366,10 @@
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D32" s="24"/>
       <c r="E32" s="31"/>
@@ -4344,10 +4385,10 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D33" s="24"/>
       <c r="E33" s="31"/>
@@ -4363,10 +4404,10 @@
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D34" s="24"/>
       <c r="E34" s="31"/>
@@ -4378,16 +4419,16 @@
         <v>100</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="L34" s="11"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D35" s="24"/>
       <c r="E35" s="31"/>
@@ -4404,10 +4445,10 @@
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D36" s="24"/>
       <c r="E36" s="31"/>
@@ -4424,10 +4465,10 @@
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D37" s="24"/>
       <c r="E37" s="31"/>
@@ -4444,10 +4485,10 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D38" s="24"/>
       <c r="E38" s="31"/>
@@ -4464,10 +4505,10 @@
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D39" s="24"/>
       <c r="E39" s="31"/>
@@ -4484,10 +4525,10 @@
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D40" s="24"/>
       <c r="E40" s="31"/>
@@ -4504,10 +4545,10 @@
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D41" s="24"/>
       <c r="E41" s="31"/>
@@ -4524,10 +4565,10 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D42" s="24"/>
       <c r="E42" s="31"/>
@@ -4544,10 +4585,10 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C43" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D43" s="24"/>
       <c r="E43" s="31"/>
@@ -4564,10 +4605,10 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C44" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D44" s="24"/>
       <c r="E44" s="31"/>
@@ -4584,10 +4625,10 @@
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="58" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D45" s="24">
         <v>0.5</v>
@@ -4602,10 +4643,10 @@
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="58" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D46" s="24">
         <v>1</v>
@@ -4620,10 +4661,10 @@
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="58" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D47" s="24">
         <v>0.5</v>
@@ -4638,10 +4679,10 @@
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D48" s="24">
         <v>1.5</v>
@@ -4656,10 +4697,10 @@
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B49" s="58" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D49" s="24">
         <v>0.5</v>
@@ -4674,10 +4715,10 @@
     </row>
     <row r="50" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B50" s="58" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D50" s="24">
         <v>2</v>
@@ -4697,10 +4738,10 @@
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B51" s="58" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D51" s="24">
         <v>0.5</v>
@@ -4715,10 +4756,10 @@
     </row>
     <row r="52" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B52" s="58" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D52" s="24">
         <v>0.75</v>
@@ -4733,10 +4774,10 @@
     </row>
     <row r="53" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B53" s="58" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D53" s="24">
         <v>0.5</v>
@@ -4751,10 +4792,10 @@
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B54" s="58" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D54" s="24">
         <v>1</v>
@@ -4768,10 +4809,10 @@
     </row>
     <row r="55" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B55" s="58" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D55" s="24">
         <v>0.25</v>
@@ -4785,10 +4826,10 @@
     </row>
     <row r="56" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B56" s="58" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D56" s="24">
         <v>1.5</v>
@@ -4808,10 +4849,10 @@
     </row>
     <row r="57" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B57" s="58" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D57" s="24"/>
       <c r="G57" s="24">
@@ -4831,10 +4872,10 @@
     </row>
     <row r="58" spans="2:12" ht="58" x14ac:dyDescent="0.35">
       <c r="B58" s="58" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D58" s="24"/>
       <c r="G58" s="24">
@@ -4843,8 +4884,8 @@
       <c r="H58" s="31">
         <v>75</v>
       </c>
-      <c r="I58" s="72" t="s">
-        <v>219</v>
+      <c r="I58" s="61" t="s">
+        <v>217</v>
       </c>
       <c r="J58">
         <v>2</v>
@@ -4853,15 +4894,15 @@
         <v>100</v>
       </c>
       <c r="L58" s="40" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="59" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B59" s="58" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D59" s="24"/>
       <c r="J59">
@@ -4871,15 +4912,15 @@
         <v>100</v>
       </c>
       <c r="L59" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="60" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B60" s="58" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D60" s="24"/>
       <c r="J60">
@@ -4889,7 +4930,7 @@
         <v>100</v>
       </c>
       <c r="L60" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="61" spans="2:12" x14ac:dyDescent="0.35">
@@ -4937,49 +4978,49 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B58">
-    <cfRule type="expression" dxfId="19" priority="49">
+    <cfRule type="expression" dxfId="21" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="18" priority="89">
+    <cfRule type="expression" dxfId="20" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61:B67">
-    <cfRule type="expression" dxfId="17" priority="10">
+    <cfRule type="expression" dxfId="19" priority="10">
       <formula>MAX($E61,$H61,$K61)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C58 C61:C65">
-    <cfRule type="expression" dxfId="16" priority="46">
+    <cfRule type="expression" dxfId="18" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="47">
+    <cfRule type="expression" dxfId="17" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="48">
+    <cfRule type="expression" dxfId="16" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="13" priority="98">
+    <cfRule type="expression" dxfId="15" priority="98">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59:B60">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>MAX($E59,$H59,$K59)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C59:C60">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="13" priority="1">
       <formula>$C59="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="12" priority="2">
       <formula>$C59="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>$C59="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4993,12 +5034,12 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="B1:E40"/>
+  <dimension ref="B1:E39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="70.81640625" customWidth="1"/>
-    <col min="3" max="3" width="81" customWidth="1"/>
+    <col min="3" max="3" width="81" style="61" customWidth="1"/>
     <col min="4" max="4" width="19.81640625" customWidth="1"/>
     <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
   </cols>
@@ -5010,10 +5051,10 @@
     </row>
     <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
       <c r="B3" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>21</v>
+        <v>229</v>
+      </c>
+      <c r="C3" s="74" t="s">
+        <v>230</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>7</v>
@@ -5022,153 +5063,173 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="73" t="s">
+        <v>233</v>
+      </c>
+      <c r="D4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="C5" s="73" t="s">
+        <v>234</v>
+      </c>
+      <c r="D5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C6" s="73" t="s">
+        <v>236</v>
+      </c>
+      <c r="D6" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="C7" s="73"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="C8" s="73"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="C9" s="73"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+      <c r="C10" s="73"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="C11" s="73"/>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="73"/>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="C13" s="73"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
+      <c r="C14" s="73"/>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+      <c r="C15" s="73"/>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+      <c r="C16" s="73"/>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="C17" s="73"/>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="C18" s="73"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="C19" s="73"/>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
+      <c r="C20" s="73"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
+      <c r="C21" s="73"/>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
+      <c r="C22" s="73"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+      <c r="C23" s="73"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
+      <c r="C24" s="73"/>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
+      <c r="C25" s="73"/>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
+      <c r="C26" s="73"/>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
+      <c r="C27" s="73"/>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="C28" s="73"/>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
+      <c r="C29" s="73"/>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+      <c r="C30" s="73"/>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="C31" s="73"/>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
+      <c r="C32" s="73"/>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+      <c r="C33" s="73"/>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="C34" s="73"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+      <c r="C35" s="73"/>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
+      <c r="C36" s="73"/>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+      <c r="C37" s="73"/>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="C38" s="73"/>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="C39" s="73"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5181,7 +5242,7 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:O24"/>
+  <dimension ref="B2:O23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
@@ -5202,29 +5263,29 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="70" t="s">
+      <c r="B2" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
     </row>
     <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="67" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="42" t="s">
@@ -5233,7 +5294,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="68" t="s">
+      <c r="F6" s="69" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5242,7 +5303,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="68" t="s">
+      <c r="I6" s="69" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="45" t="s">
@@ -5251,7 +5312,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="68" t="s">
+      <c r="L6" s="69" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="45" t="s">
@@ -5260,48 +5321,48 @@
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="68" t="s">
+      <c r="O6" s="69" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="65"/>
-      <c r="C7" s="67"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="68"/>
       <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="69"/>
+      <c r="F7" s="70"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="69"/>
+      <c r="I7" s="70"/>
       <c r="J7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="69"/>
+      <c r="L7" s="70"/>
       <c r="M7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="N7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="69"/>
+      <c r="O7" s="70"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" s="24"/>
       <c r="E8" s="31"/>
@@ -5316,10 +5377,10 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D9" s="24"/>
       <c r="E9" s="31"/>
@@ -5332,10 +5393,10 @@
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D10" s="24"/>
       <c r="E10" s="31"/>
@@ -5348,10 +5409,10 @@
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C11" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D11" s="24"/>
       <c r="E11" s="31"/>
@@ -5364,10 +5425,10 @@
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D12" s="24"/>
       <c r="E12" s="31"/>
@@ -5380,10 +5441,10 @@
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="31"/>
@@ -5396,10 +5457,10 @@
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="31"/>
@@ -5412,10 +5473,10 @@
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="31"/>
@@ -5427,10 +5488,10 @@
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D16" s="24"/>
       <c r="E16" s="31"/>
@@ -5441,9 +5502,11 @@
       <c r="L16" s="11"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B17" s="29"/>
+      <c r="B17" s="29" t="s">
+        <v>219</v>
+      </c>
       <c r="C17" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D17" s="24"/>
       <c r="E17" s="31"/>
@@ -5455,10 +5518,10 @@
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D18" s="24"/>
       <c r="E18" s="31"/>
@@ -5470,10 +5533,10 @@
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C19" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D19" s="24"/>
       <c r="E19" s="31"/>
@@ -5485,10 +5548,10 @@
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D20" s="24"/>
       <c r="E20" s="31"/>
@@ -5500,10 +5563,10 @@
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D21" s="24"/>
       <c r="E21" s="31"/>
@@ -5515,10 +5578,10 @@
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D22" s="24"/>
       <c r="E22" s="31"/>
@@ -5529,12 +5592,8 @@
       <c r="L22" s="11"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B23" s="29" t="s">
-        <v>228</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>105</v>
-      </c>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
       <c r="D23" s="24"/>
       <c r="E23" s="31"/>
       <c r="F23" s="11"/>
@@ -5542,17 +5601,6 @@
       <c r="H23" s="31"/>
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="11"/>
-      <c r="L24" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5564,45 +5612,55 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B9:B15 B17:B24">
-    <cfRule type="expression" dxfId="12" priority="17">
+  <conditionalFormatting sqref="B2 B9:B15 B17:B23">
+    <cfRule type="expression" dxfId="10" priority="17">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="11" priority="9">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C24">
-    <cfRule type="expression" dxfId="10" priority="6">
+  <conditionalFormatting sqref="C6:C23">
+    <cfRule type="expression" dxfId="8" priority="6">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="7">
+    <cfRule type="expression" dxfId="7" priority="7">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="expression" dxfId="7" priority="101">
+    <cfRule type="expression" dxfId="5" priority="101">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="6" priority="103">
+    <cfRule type="expression" dxfId="4" priority="103">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="5" priority="105">
+    <cfRule type="expression" dxfId="3" priority="105">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B9:B16">
-    <cfRule type="expression" dxfId="4" priority="107">
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" dxfId="2" priority="107">
       <formula>MAX($E16,$H16,$K16)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11:B16">
+    <cfRule type="expression" dxfId="1" priority="116">
+      <formula>MAX($E17,$H17,$K17)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" dxfId="0" priority="117">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5638,10 +5696,10 @@
     </row>
     <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>2</v>
@@ -5655,10 +5713,10 @@
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>6</v>
@@ -5668,10 +5726,10 @@
     </row>
     <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>16</v>
@@ -5681,10 +5739,10 @@
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>6</v>
@@ -5694,10 +5752,10 @@
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>6</v>
@@ -5707,10 +5765,10 @@
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>6</v>
@@ -5720,10 +5778,10 @@
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>6</v>
@@ -5733,10 +5791,10 @@
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>6</v>
@@ -5746,10 +5804,10 @@
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>6</v>
@@ -5759,10 +5817,10 @@
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>6</v>
@@ -5772,10 +5830,10 @@
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>6</v>
@@ -5785,10 +5843,10 @@
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>6</v>
@@ -5798,10 +5856,10 @@
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>6</v>
@@ -5811,10 +5869,10 @@
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>6</v>
@@ -5824,10 +5882,10 @@
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>6</v>
@@ -5837,10 +5895,10 @@
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>6</v>
@@ -5850,10 +5908,10 @@
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>6</v>
@@ -5863,10 +5921,10 @@
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>6</v>
@@ -5876,10 +5934,10 @@
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>6</v>
@@ -5889,10 +5947,10 @@
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>6</v>
@@ -5902,10 +5960,10 @@
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>6</v>
@@ -5915,10 +5973,10 @@
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>6</v>
@@ -5928,10 +5986,10 @@
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>6</v>
@@ -5941,10 +5999,10 @@
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>6</v>
@@ -5954,10 +6012,10 @@
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>6</v>
@@ -5967,10 +6025,10 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>6</v>
@@ -5980,10 +6038,10 @@
     </row>
     <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>16</v>
@@ -5993,10 +6051,10 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>6</v>
@@ -6006,10 +6064,10 @@
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>6</v>
@@ -6019,10 +6077,10 @@
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>6</v>
@@ -6032,10 +6090,10 @@
     </row>
     <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>16</v>
@@ -6045,10 +6103,10 @@
     </row>
     <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>16</v>
@@ -6058,10 +6116,10 @@
     </row>
     <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>16</v>
@@ -6071,10 +6129,10 @@
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>6</v>
@@ -6084,10 +6142,10 @@
     </row>
     <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>16</v>
@@ -6097,10 +6155,10 @@
     </row>
     <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>16</v>
@@ -6110,10 +6168,10 @@
     </row>
     <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>16</v>
@@ -6123,10 +6181,10 @@
     </row>
     <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>16</v>
@@ -6136,10 +6194,10 @@
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>6</v>
@@ -6149,10 +6207,10 @@
     </row>
     <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>16</v>
@@ -6162,10 +6220,10 @@
     </row>
     <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>16</v>
@@ -6175,10 +6233,10 @@
     </row>
     <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>17</v>
@@ -6188,10 +6246,10 @@
     </row>
     <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D47" s="3" t="s">
         <v>16</v>
@@ -6201,10 +6259,10 @@
     </row>
     <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>16</v>
@@ -6214,10 +6272,10 @@
     </row>
     <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>16</v>
@@ -6227,10 +6285,10 @@
     </row>
     <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>16</v>
@@ -6240,10 +6298,10 @@
     </row>
     <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>16</v>
@@ -6253,10 +6311,10 @@
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>6</v>
@@ -6266,10 +6324,10 @@
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>6</v>
@@ -6279,10 +6337,10 @@
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>6</v>
@@ -6292,10 +6350,10 @@
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>6</v>
@@ -6305,10 +6363,10 @@
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>6</v>
@@ -6318,10 +6376,10 @@
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>6</v>
@@ -6331,10 +6389,10 @@
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>6</v>
@@ -6344,10 +6402,10 @@
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>6</v>
@@ -6357,10 +6415,10 @@
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>6</v>
@@ -6370,10 +6428,10 @@
     </row>
     <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>16</v>
@@ -6383,10 +6441,10 @@
     </row>
     <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>16</v>
@@ -6396,10 +6454,10 @@
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>6</v>
@@ -6409,10 +6467,10 @@
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>6</v>
@@ -6422,7 +6480,7 @@
     </row>
     <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C65" s="3"/>
       <c r="D65" s="3" t="s">
@@ -6433,7 +6491,7 @@
     </row>
     <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C66" s="3"/>
       <c r="D66" s="3" t="s">
@@ -6444,7 +6502,7 @@
     </row>
     <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C67" s="3"/>
       <c r="D67" s="3" t="s">
@@ -6455,7 +6513,7 @@
     </row>
     <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="3" t="s">
@@ -6466,7 +6524,7 @@
     </row>
     <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C69" s="3"/>
       <c r="D69" s="3" t="s">
@@ -6477,7 +6535,7 @@
     </row>
     <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C70" s="3"/>
       <c r="D70" s="3" t="s">
@@ -6488,7 +6546,7 @@
     </row>
     <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C71" s="3"/>
       <c r="D71" s="3" t="s">
@@ -6499,7 +6557,7 @@
     </row>
     <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C72" s="3"/>
       <c r="D72" s="3" t="s">
@@ -6510,7 +6568,7 @@
     </row>
     <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C73" s="3"/>
       <c r="D73" s="3" t="s">
@@ -6521,7 +6579,7 @@
     </row>
     <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C74" s="3"/>
       <c r="D74" s="3" t="s">
@@ -6532,7 +6590,7 @@
     </row>
     <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C75" s="3"/>
       <c r="D75" s="3" t="s">

</xml_diff>

<commit_message>
Mise a jour planif
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC3A9F7F-AF37-4BED-AEDD-FF941FCAF237}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D6FFD4-C6DC-40E1-B979-FF542F2E08C9}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17730" activeTab="4" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,17 +27,22 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="246">
   <si>
     <t>Planification globale</t>
   </si>
@@ -747,10 +752,35 @@
     <t>Tutoriel</t>
   </si>
   <si>
-    <t>Enregistrer le vidéo de tutoriel, ajouter les commentaires, ajouter le vidéo dans le front end</t>
-  </si>
-  <si>
     <t>Tout le monde</t>
+  </si>
+  <si>
+    <t>Idée abandonnée  à la vue de l'aspect du jeu</t>
+  </si>
+  <si>
+    <t>Mise a jour de la page classement depuis le serveur</t>
+  </si>
+  <si>
+    <t>Fetch  des données  de la base de donnée du serveur depuis le client</t>
+  </si>
+  <si>
+    <t>Enregistrer différentes  vidéos  de tutoriel, ajouter des commentaires , ajouter le tout dans une page dédiée sur le frontend client, permettre des options de controles de la video eventuellement</t>
+  </si>
+  <si>
+    <t>Développement du système de sauvegarde et restauration des parties contre IA</t>
+  </si>
+  <si>
+    <t>Sérialisation du Board, l'état AIPlayer (MCTS) et l'historique en JSON  dans la base de donnée MySQL. React : boutons Save/Load + composant liste des parties sauvegardées, restauration via useGameSync.</t>
+  </si>
+  <si>
+    <t>Idée abandonnée:  le plateau  avec 40 pièces par joueur est trop dense pour être jouable sur un petit écran</t>
+  </si>
+  <si>
+    <t>Cacher les composants non essentiels pour régler l'affichage de la page.</t>
+  </si>
+  <si>
+    <t>Créer une page accessible uniquement aux admins qui affiche la liste des utilisateurs avec leurs infos. Ajouter des boutons pour bannir, promouvoir en admin ou supprimer un compte. 
+Le serveur donne des droits aux comptes utilisateurs,ajouter un système de log.</t>
   </si>
 </sst>
 </file>
@@ -801,7 +831,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -853,6 +883,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1134,7 +1170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1231,6 +1267,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1264,17 +1306,54 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="53">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1341,6 +1420,69 @@
             <color rgb="FFCCFFFF"/>
           </stop>
         </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -1881,26 +2023,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" customWidth="1"/>
-    <col min="5" max="5" width="42.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:5" ht="46.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -1914,7 +2056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="48" t="s">
         <v>139</v>
       </c>
@@ -1928,7 +2070,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="52" t="s">
         <v>109</v>
       </c>
@@ -1942,7 +2084,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="53" t="s">
         <v>110</v>
       </c>
@@ -1956,7 +2098,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="53" t="s">
         <v>111</v>
       </c>
@@ -1970,7 +2112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="53" t="s">
         <v>112</v>
       </c>
@@ -1984,7 +2126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="53" t="s">
         <v>114</v>
       </c>
@@ -1998,7 +2140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="53" t="s">
         <v>115</v>
       </c>
@@ -2012,7 +2154,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="53" t="s">
         <v>116</v>
       </c>
@@ -2026,7 +2168,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="53" t="s">
         <v>143</v>
       </c>
@@ -2040,7 +2182,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>119</v>
       </c>
@@ -2054,7 +2196,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="53" t="s">
         <v>120</v>
       </c>
@@ -2068,7 +2210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="53" t="s">
         <v>122</v>
       </c>
@@ -2082,7 +2224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="53" t="s">
         <v>128</v>
       </c>
@@ -2096,7 +2238,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="49" t="s">
         <v>117</v>
       </c>
@@ -2110,7 +2252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="49" t="s">
         <v>118</v>
       </c>
@@ -2124,7 +2266,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="49" t="s">
         <v>123</v>
       </c>
@@ -2138,7 +2280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="49" t="s">
         <v>124</v>
       </c>
@@ -2152,7 +2294,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="49" t="s">
         <v>125</v>
       </c>
@@ -2166,7 +2308,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="49" t="s">
         <v>127</v>
       </c>
@@ -2180,7 +2322,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="49" t="s">
         <v>131</v>
       </c>
@@ -2194,7 +2336,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="49" t="s">
         <v>132</v>
       </c>
@@ -2208,7 +2350,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="49" t="s">
         <v>133</v>
       </c>
@@ -2222,7 +2364,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="54" t="s">
         <v>126</v>
       </c>
@@ -2236,7 +2378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="54" t="s">
         <v>129</v>
       </c>
@@ -2250,7 +2392,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="54" t="s">
         <v>121</v>
       </c>
@@ -2264,7 +2406,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="54" t="s">
         <v>130</v>
       </c>
@@ -2278,7 +2420,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="54" t="s">
         <v>134</v>
       </c>
@@ -2292,7 +2434,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="54" t="s">
         <v>135</v>
       </c>
@@ -2306,7 +2448,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="54" t="s">
         <v>136</v>
       </c>
@@ -2320,7 +2462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
         <v>137</v>
       </c>
@@ -2334,7 +2476,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="54" t="s">
         <v>138</v>
       </c>
@@ -2348,7 +2490,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="56" t="s">
         <v>113</v>
       </c>
@@ -2362,8 +2504,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="32" t="s">
         <v>144</v>
       </c>
@@ -2375,7 +2517,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="37" priority="1">
+    <cfRule type="expression" dxfId="52" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2398,32 +2540,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" customWidth="1"/>
-    <col min="6" max="6" width="18.81640625" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" customWidth="1"/>
-    <col min="8" max="8" width="16.1796875" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
-    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2453,7 +2595,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2507,7 +2649,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -2534,7 +2676,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -2556,7 +2698,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -2583,7 +2725,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -2616,7 +2758,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -2653,7 +2795,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -2690,7 +2832,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -2722,7 +2864,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -2750,7 +2892,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -2777,15 +2919,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -2801,44 +2943,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.54296875" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.81640625" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="62" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B3" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-      <c r="L3" s="64"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="65" t="s">
+      <c r="C3" s="65"/>
+      <c r="D3" s="65"/>
+      <c r="E3" s="65"/>
+      <c r="F3" s="65"/>
+      <c r="G3" s="65"/>
+      <c r="H3" s="65"/>
+      <c r="I3" s="65"/>
+      <c r="J3" s="65"/>
+      <c r="K3" s="65"/>
+      <c r="L3" s="66"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="69" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -2847,7 +2989,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="69" t="s">
+      <c r="F5" s="71" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -2856,7 +2998,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="69" t="s">
+      <c r="I5" s="71" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -2865,36 +3007,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="69" t="s">
+      <c r="L5" s="71" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="66"/>
-      <c r="C6" s="68"/>
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="68"/>
+      <c r="C6" s="70"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="70"/>
+      <c r="F6" s="72"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="70"/>
+      <c r="I6" s="72"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="70"/>
-    </row>
-    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="L6" s="72"/>
+    </row>
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -2917,7 +3059,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -2936,7 +3078,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -2955,7 +3097,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -2974,7 +3116,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>152</v>
       </c>
@@ -2993,7 +3135,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3012,7 +3154,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3031,7 +3173,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3050,7 +3192,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>150</v>
       </c>
@@ -3069,7 +3211,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3088,7 +3230,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3107,7 +3249,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>148</v>
       </c>
@@ -3126,7 +3268,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>149</v>
       </c>
@@ -3145,7 +3287,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="46" t="s">
         <v>157</v>
       </c>
@@ -3164,7 +3306,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3185,7 +3327,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3204,7 +3346,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3225,7 +3367,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3244,7 +3386,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3263,7 +3405,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3284,7 +3426,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3305,7 +3447,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3326,7 +3468,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3345,7 +3487,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>172</v>
       </c>
@@ -3364,7 +3506,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3383,7 +3525,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -3402,7 +3544,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>151</v>
       </c>
@@ -3421,7 +3563,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>154</v>
       </c>
@@ -3440,7 +3582,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -3459,7 +3601,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -3478,7 +3620,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -3497,7 +3639,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>168</v>
       </c>
@@ -3516,7 +3658,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>169</v>
       </c>
@@ -3535,7 +3677,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>166</v>
       </c>
@@ -3554,7 +3696,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>167</v>
       </c>
@@ -3573,7 +3715,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>164</v>
       </c>
@@ -3592,7 +3734,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>163</v>
       </c>
@@ -3611,7 +3753,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>159</v>
       </c>
@@ -3630,7 +3772,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="29" t="s">
         <v>158</v>
       </c>
@@ -3649,7 +3791,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
         <v>162</v>
       </c>
@@ -3668,7 +3810,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="29" t="s">
         <v>170</v>
       </c>
@@ -3687,7 +3829,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>161</v>
       </c>
@@ -3717,67 +3859,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="36" priority="7">
+    <cfRule type="expression" dxfId="51" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="35" priority="1">
+    <cfRule type="expression" dxfId="50" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="34" priority="32">
+    <cfRule type="expression" dxfId="49" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="38">
+    <cfRule type="expression" dxfId="48" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="32" priority="30">
+    <cfRule type="expression" dxfId="47" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="31" priority="6">
+    <cfRule type="expression" dxfId="46" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="30" priority="25">
+    <cfRule type="expression" dxfId="45" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="27">
+    <cfRule type="expression" dxfId="44" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="28" priority="8">
+    <cfRule type="expression" dxfId="43" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="27" priority="13">
+    <cfRule type="expression" dxfId="42" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="14">
+    <cfRule type="expression" dxfId="41" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="25" priority="20">
+    <cfRule type="expression" dxfId="40" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="21">
+    <cfRule type="expression" dxfId="39" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="23" priority="9">
+    <cfRule type="expression" dxfId="38" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="10">
+    <cfRule type="expression" dxfId="37" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3792,43 +3934,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L67"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="21.81640625" customWidth="1"/>
-    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.81640625" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.77734375" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="51.54296875" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="62" t="s">
+    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B1" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="64"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="65" t="s">
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="66"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="67" t="s">
+      <c r="C4" s="69" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -3837,7 +3979,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="69" t="s">
+      <c r="F4" s="71" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -3846,7 +3988,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="69" t="s">
+      <c r="I4" s="71" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -3855,36 +3997,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="69" t="s">
+      <c r="L4" s="71" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="66"/>
-      <c r="C5" s="68"/>
+    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="68"/>
+      <c r="C5" s="70"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="70"/>
+      <c r="F5" s="72"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="70"/>
+      <c r="I5" s="72"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="70"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L5" s="72"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>175</v>
       </c>
@@ -3902,7 +4044,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>176</v>
       </c>
@@ -3920,7 +4062,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>177</v>
       </c>
@@ -3938,7 +4080,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>160</v>
       </c>
@@ -3956,7 +4098,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>174</v>
       </c>
@@ -3974,7 +4116,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>173</v>
       </c>
@@ -3992,7 +4134,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>165</v>
       </c>
@@ -4010,7 +4152,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>171</v>
       </c>
@@ -4028,7 +4170,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>178</v>
       </c>
@@ -4046,7 +4188,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>179</v>
       </c>
@@ -4064,7 +4206,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>181</v>
       </c>
@@ -4082,7 +4224,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>184</v>
       </c>
@@ -4100,7 +4242,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>185</v>
       </c>
@@ -4118,7 +4260,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>186</v>
       </c>
@@ -4136,7 +4278,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>197</v>
       </c>
@@ -4155,7 +4297,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>187</v>
       </c>
@@ -4174,7 +4316,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>198</v>
       </c>
@@ -4193,7 +4335,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>194</v>
       </c>
@@ -4212,7 +4354,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>188</v>
       </c>
@@ -4231,7 +4373,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>200</v>
       </c>
@@ -4250,7 +4392,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>189</v>
       </c>
@@ -4269,7 +4411,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>190</v>
       </c>
@@ -4288,7 +4430,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>191</v>
       </c>
@@ -4307,7 +4449,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>192</v>
       </c>
@@ -4326,7 +4468,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>196</v>
       </c>
@@ -4345,7 +4487,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>193</v>
       </c>
@@ -4364,7 +4506,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>195</v>
       </c>
@@ -4383,7 +4525,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>199</v>
       </c>
@@ -4402,7 +4544,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>202</v>
       </c>
@@ -4423,7 +4565,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>206</v>
       </c>
@@ -4443,7 +4585,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>205</v>
       </c>
@@ -4463,7 +4605,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>207</v>
       </c>
@@ -4483,7 +4625,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>208</v>
       </c>
@@ -4503,7 +4645,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>209</v>
       </c>
@@ -4523,7 +4665,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>210</v>
       </c>
@@ -4543,7 +4685,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>211</v>
       </c>
@@ -4561,9 +4703,11 @@
       <c r="K41">
         <v>100</v>
       </c>
-      <c r="L41" s="11"/>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L41" s="11" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -4583,7 +4727,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>213</v>
       </c>
@@ -4603,7 +4747,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>212</v>
       </c>
@@ -4623,7 +4767,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="58" t="s">
         <v>183</v>
       </c>
@@ -4641,7 +4785,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="58" t="s">
         <v>83</v>
       </c>
@@ -4659,7 +4803,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="58" t="s">
         <v>81</v>
       </c>
@@ -4677,7 +4821,7 @@
       <c r="I47" s="11"/>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>60</v>
       </c>
@@ -4695,7 +4839,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="58" t="s">
         <v>84</v>
       </c>
@@ -4713,7 +4857,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="58" t="s">
         <v>228</v>
       </c>
@@ -4736,7 +4880,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="58" t="s">
         <v>56</v>
       </c>
@@ -4754,7 +4898,7 @@
       <c r="I51" s="11"/>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="58" t="s">
         <v>57</v>
       </c>
@@ -4772,7 +4916,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="58" t="s">
         <v>58</v>
       </c>
@@ -4790,7 +4934,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -4807,7 +4951,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="58" t="s">
         <v>182</v>
       </c>
@@ -4824,7 +4968,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="58" t="s">
         <v>223</v>
       </c>
@@ -4847,7 +4991,7 @@
       </c>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="58" t="s">
         <v>224</v>
       </c>
@@ -4870,7 +5014,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B58" s="58" t="s">
         <v>203</v>
       </c>
@@ -4897,7 +5041,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="58" t="s">
         <v>215</v>
       </c>
@@ -4915,7 +5059,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B60" s="58" t="s">
         <v>216</v>
       </c>
@@ -4933,36 +5077,36 @@
         <v>227</v>
       </c>
     </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B61" s="58"/>
       <c r="C61" s="7"/>
       <c r="D61" s="24"/>
     </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B62" s="58"/>
       <c r="C62" s="7"/>
       <c r="D62" s="24"/>
     </row>
-    <row r="63" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B63" s="58"/>
       <c r="C63" s="7"/>
       <c r="D63" s="24"/>
     </row>
-    <row r="64" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B64" s="58"/>
       <c r="C64" s="7"/>
       <c r="D64" s="24"/>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B65" s="58"/>
       <c r="C65" s="7"/>
       <c r="D65" s="24"/>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B66" s="58"/>
       <c r="D66" s="24"/>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B67" s="58"/>
       <c r="D67" s="24"/>
     </row>
@@ -4978,49 +5122,49 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B58">
-    <cfRule type="expression" dxfId="21" priority="49">
+    <cfRule type="expression" dxfId="36" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="20" priority="89">
+    <cfRule type="expression" dxfId="35" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B61:B67">
-    <cfRule type="expression" dxfId="19" priority="10">
+    <cfRule type="expression" dxfId="34" priority="10">
       <formula>MAX($E61,$H61,$K61)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C58 C61:C65">
-    <cfRule type="expression" dxfId="18" priority="46">
+    <cfRule type="expression" dxfId="33" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="47">
+    <cfRule type="expression" dxfId="32" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="16" priority="48">
+    <cfRule type="expression" dxfId="31" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="15" priority="98">
+    <cfRule type="expression" dxfId="30" priority="98">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59:B60">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="29" priority="4">
       <formula>MAX($E59,$H59,$K59)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C59:C60">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="28" priority="1">
       <formula>$C59="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="27" priority="2">
       <formula>$C59="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="26" priority="3">
       <formula>$C59="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5035,25 +5179,25 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="70.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="70.77734375" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" customWidth="1"/>
-    <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="28.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:5" ht="21" x14ac:dyDescent="0.4">
       <c r="B3" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="C3" s="74" t="s">
+      <c r="C3" s="63" t="s">
         <v>230</v>
       </c>
       <c r="D3" s="8" t="s">
@@ -5063,22 +5207,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C4" s="73" t="s">
+      <c r="C4" s="62" t="s">
         <v>233</v>
       </c>
       <c r="D4" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+        <v>236</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="C5" s="73" t="s">
+      <c r="C5" s="62" t="s">
         <v>234</v>
       </c>
       <c r="D5" t="s">
@@ -5088,150 +5235,217 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="C6" s="73" t="s">
+      <c r="C6" s="62" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C7" s="62" t="s">
+        <v>239</v>
+      </c>
+      <c r="D7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C8" s="62" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" t="s">
         <v>236</v>
       </c>
-      <c r="D6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B7" s="3"/>
-      <c r="C7" s="73"/>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B8" s="3"/>
-      <c r="C8" s="73"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B9" s="3"/>
-      <c r="C9" s="73"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B10" s="3"/>
-      <c r="C10" s="73"/>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B11" s="3"/>
-      <c r="C11" s="73"/>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B12" s="3"/>
-      <c r="C12" s="73"/>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B13" s="3"/>
-      <c r="C13" s="73"/>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B14" s="3"/>
-      <c r="C14" s="73"/>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="E8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C9" s="62" t="s">
+        <v>245</v>
+      </c>
+      <c r="D9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="62" t="s">
+        <v>243</v>
+      </c>
+      <c r="D10" s="75"/>
+      <c r="E10" s="75"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="62"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C12" s="62"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C13" s="62"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C14" s="62"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="3"/>
-      <c r="C15" s="73"/>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="C15" s="62"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
-      <c r="C16" s="73"/>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C16" s="62"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
-      <c r="C17" s="73"/>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C17" s="62"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B18" s="3"/>
-      <c r="C18" s="73"/>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C18" s="62"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B19" s="3"/>
-      <c r="C19" s="73"/>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C19" s="62"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
-      <c r="C20" s="73"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C20" s="62"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
-      <c r="C21" s="73"/>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C21" s="62"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B22" s="3"/>
-      <c r="C22" s="73"/>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C22" s="62"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
-      <c r="C23" s="73"/>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C23" s="62"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" s="3"/>
-      <c r="C24" s="73"/>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C24" s="62"/>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
-      <c r="C25" s="73"/>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C25" s="62"/>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
-      <c r="C26" s="73"/>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C26" s="62"/>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
-      <c r="C27" s="73"/>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C27" s="62"/>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
-      <c r="C28" s="73"/>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C28" s="62"/>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B29" s="3"/>
-      <c r="C29" s="73"/>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C29" s="62"/>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
-      <c r="C30" s="73"/>
-    </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C30" s="62"/>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
-      <c r="C31" s="73"/>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C31" s="62"/>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B32" s="3"/>
-      <c r="C32" s="73"/>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C32" s="62"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B33" s="3"/>
-      <c r="C33" s="73"/>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C33" s="62"/>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B34" s="3"/>
-      <c r="C34" s="73"/>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C34" s="62"/>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B35" s="3"/>
-      <c r="C35" s="73"/>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C35" s="62"/>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B36" s="3"/>
-      <c r="C36" s="73"/>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C36" s="62"/>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B37" s="3"/>
-      <c r="C37" s="73"/>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C37" s="62"/>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B38" s="3"/>
-      <c r="C38" s="73"/>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="C38" s="62"/>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B39" s="3"/>
-      <c r="C39" s="73"/>
+      <c r="C39" s="62"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" dxfId="20" priority="10">
+      <formula>MAX($E20,$H20,$K20)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" dxfId="19" priority="11">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -5242,50 +5456,50 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:O23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:O20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.81640625" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.6328125" customWidth="1"/>
-    <col min="15" max="15" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.44140625" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.6640625" customWidth="1"/>
+    <col min="15" max="15" width="19.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="71" t="s">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="B2" s="73" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="72"/>
-      <c r="D2" s="72"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="72"/>
-      <c r="G2" s="72"/>
-      <c r="H2" s="72"/>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-    </row>
-    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B6" s="65" t="s">
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="74"/>
+      <c r="M2" s="74"/>
+      <c r="N2" s="74"/>
+      <c r="O2" s="74"/>
+    </row>
+    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="67" t="s">
+      <c r="C6" s="69" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="42" t="s">
@@ -5294,7 +5508,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="69" t="s">
+      <c r="F6" s="71" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5303,7 +5517,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="69" t="s">
+      <c r="I6" s="71" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="45" t="s">
@@ -5312,7 +5526,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="69" t="s">
+      <c r="L6" s="71" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="45" t="s">
@@ -5321,43 +5535,43 @@
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="69" t="s">
+      <c r="O6" s="71" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="66"/>
-      <c r="C7" s="68"/>
+    <row r="7" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="68"/>
+      <c r="C7" s="70"/>
       <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="70"/>
+      <c r="F7" s="72"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="70"/>
+      <c r="I7" s="72"/>
       <c r="J7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="70"/>
+      <c r="L7" s="72"/>
       <c r="M7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="N7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="70"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="O7" s="72"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>214</v>
       </c>
@@ -5375,7 +5589,7 @@
       <c r="N8" s="9"/>
       <c r="O8" s="10"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>201</v>
       </c>
@@ -5391,9 +5605,9 @@
       <c r="L9" s="11"/>
       <c r="O9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>102</v>
@@ -5407,25 +5621,18 @@
       <c r="L10" s="11"/>
       <c r="O10" s="11"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="11"/>
       <c r="G11" s="24"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="O11" s="11"/>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>102</v>
@@ -5439,28 +5646,30 @@
       <c r="L12" s="11"/>
       <c r="O12" s="11"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="31"/>
-      <c r="F13" s="11"/>
+      <c r="F13" s="11" t="s">
+        <v>237</v>
+      </c>
       <c r="G13" s="24"/>
       <c r="H13" s="31"/>
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
       <c r="O13" s="11"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
-        <v>106</v>
+        <v>219</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="31"/>
@@ -5469,14 +5678,13 @@
       <c r="H14" s="31"/>
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
-      <c r="O14" s="11"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
-        <v>68</v>
+        <v>220</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="31"/>
@@ -5486,12 +5694,12 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D16" s="24"/>
       <c r="E16" s="31"/>
@@ -5501,9 +5709,9 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>103</v>
@@ -5516,9 +5724,9 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C18" s="29" t="s">
         <v>103</v>
@@ -5531,9 +5739,9 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C19" s="29" t="s">
         <v>103</v>
@@ -5546,13 +5754,9 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B20" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="C20" s="29" t="s">
-        <v>103</v>
-      </c>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
       <c r="D20" s="24"/>
       <c r="E20" s="31"/>
       <c r="F20" s="11"/>
@@ -5560,47 +5764,6 @@
       <c r="H20" s="31"/>
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B21" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D21" s="24"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="11"/>
-      <c r="L21" s="11"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B22" s="29" t="s">
-        <v>226</v>
-      </c>
-      <c r="C22" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D22" s="24"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="11"/>
-      <c r="L22" s="11"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="11"/>
-      <c r="L23" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5612,55 +5775,75 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B9:B15 B17:B23">
-    <cfRule type="expression" dxfId="10" priority="17">
+  <conditionalFormatting sqref="B2 B14:B20 B9:B10">
+    <cfRule type="expression" dxfId="16" priority="20">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="15" priority="12">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C23">
-    <cfRule type="expression" dxfId="8" priority="6">
+  <conditionalFormatting sqref="C6:C20">
+    <cfRule type="expression" dxfId="14" priority="9">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="7">
+    <cfRule type="expression" dxfId="13" priority="10">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="8">
+    <cfRule type="expression" dxfId="12" priority="11">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16">
-    <cfRule type="expression" dxfId="5" priority="101">
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" dxfId="11" priority="104">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="4" priority="103">
+    <cfRule type="expression" dxfId="10" priority="106">
+      <formula>MAX($E13,$H13,$K13)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="expression" dxfId="9" priority="108">
+      <formula>MAX($E5,$H5,$K5)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" dxfId="8" priority="131">
+      <formula>MAX($E18,$H18,$K18)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" dxfId="7" priority="138">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" dxfId="6" priority="141">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11:B12">
+    <cfRule type="expression" dxfId="5" priority="143">
+      <formula>MAX($E17,$H17,$K17)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" dxfId="4" priority="153">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="3" priority="105">
-      <formula>MAX($E5,$H5,$K5)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="2" priority="107">
-      <formula>MAX($E16,$H16,$K16)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B16">
-    <cfRule type="expression" dxfId="1" priority="116">
-      <formula>MAX($E17,$H17,$K17)=100</formula>
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" dxfId="3" priority="155">
+      <formula>MAX($E19,$H19,$K19)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="0" priority="117">
-      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    <cfRule type="expression" dxfId="2" priority="156">
+      <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5673,28 +5856,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
-    <col min="2" max="2" width="93.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="2" max="2" width="93.21875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="42.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.75" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -5711,7 +5894,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -5724,7 +5907,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -5737,7 +5920,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -5750,7 +5933,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -5763,7 +5946,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -5776,7 +5959,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -5789,7 +5972,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -5802,7 +5985,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -5815,7 +5998,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -5828,7 +6011,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -5841,7 +6024,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -5854,7 +6037,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -5867,7 +6050,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -5880,7 +6063,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -5893,7 +6076,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -5906,7 +6089,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -5919,7 +6102,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -5932,7 +6115,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -5945,7 +6128,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -5958,7 +6141,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -5971,7 +6154,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -5984,7 +6167,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -5997,7 +6180,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -6010,7 +6193,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -6023,7 +6206,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -6036,7 +6219,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -6049,7 +6232,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -6062,7 +6245,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -6075,7 +6258,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -6088,7 +6271,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -6101,7 +6284,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -6114,7 +6297,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -6127,7 +6310,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -6140,7 +6323,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -6153,7 +6336,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -6166,7 +6349,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -6179,7 +6362,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -6192,7 +6375,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -6205,7 +6388,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -6218,7 +6401,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -6231,7 +6414,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -6244,7 +6427,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -6257,7 +6440,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -6270,7 +6453,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -6283,7 +6466,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -6296,7 +6479,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -6309,7 +6492,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -6322,7 +6505,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -6335,7 +6518,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -6348,7 +6531,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -6361,7 +6544,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -6374,7 +6557,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -6387,7 +6570,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -6400,7 +6583,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -6413,7 +6596,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -6426,7 +6609,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -6439,7 +6622,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -6452,7 +6635,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -6465,7 +6648,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -6478,7 +6661,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -6489,7 +6672,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -6500,7 +6683,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -6511,7 +6694,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -6522,7 +6705,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -6533,7 +6716,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -6544,7 +6727,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -6555,7 +6738,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -6566,7 +6749,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -6577,7 +6760,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>107</v>
       </c>
@@ -6588,7 +6771,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>108</v>
       </c>
@@ -6599,182 +6782,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
ajout bouton surrender + fonction end game+ ajout noms des joueurs / adversaire hardcodé
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01BE244B-50B9-4789-A2C1-997F4F8DE96B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B0504C-4D3D-4E41-937F-16CC6C24B8FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -32,23 +32,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="249">
   <si>
     <t>Planification globale</t>
   </si>
@@ -368,9 +357,6 @@
     <t>Charlotte/Eddy</t>
   </si>
   <si>
-    <t>Instructions de jeu</t>
-  </si>
-  <si>
     <t>Gestion des droits des usagers</t>
   </si>
   <si>
@@ -650,9 +636,6 @@
     <t>Refactoriser game.jsx( redecouapge en differents components)</t>
   </si>
   <si>
-    <t>Implémentation du Factory Pattern pour les aspects des pièces(couleur + divers apects,,)</t>
-  </si>
-  <si>
     <t>Afficher le tour de jeu message au centre de l écran: Ajouter component YourTurn</t>
   </si>
   <si>
@@ -687,9 +670,6 @@
   </si>
   <si>
     <t>Modifier frontend pour recuperer ordre du joueur (plus hardcodé dans le code)</t>
-  </si>
-  <si>
-    <t>Leaderboard fetch données depuis le serveur</t>
   </si>
   <si>
     <t>Sauvegarde de scores dans bd</t>
@@ -790,6 +770,21 @@
   </si>
   <si>
     <t>Créer table pour les chats entre joueurs dans la base de données</t>
+  </si>
+  <si>
+    <t>Créer une fonction abandonner et set la partie à perdue</t>
+  </si>
+  <si>
+    <t>Ajouter bouton  capituler en phase "playing"</t>
+  </si>
+  <si>
+    <t>Leaderboard fetch données depuis le serveur classe les résultats</t>
+  </si>
+  <si>
+    <t>Implémentation du Factory Pattern pour les aspects des pièces(couleur + divers apects)</t>
+  </si>
+  <si>
+    <t>Tutoriel de jeu</t>
   </si>
 </sst>
 </file>
@@ -1337,7 +1332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1440,6 +1435,31 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1473,36 +1493,84 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="44">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1541,34 +1609,6 @@
             <color rgb="FFCCFFFF"/>
           </stop>
         </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -1804,9 +1844,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1844,7 +1884,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1950,7 +1990,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2092,7 +2132,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2104,26 +2144,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
+    <col min="1" max="1" width="3.26953125" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="42.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.7265625" customWidth="1"/>
+    <col min="5" max="5" width="42.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2137,458 +2177,458 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="48" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C6" s="51" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="28" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E6" s="10">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="52" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E7" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C8" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E8" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C9" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E9" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="53" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C10" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E10" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="53" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C11" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E11" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="53" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C12" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E12" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="53" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C13" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E13" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="53" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C14" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E14" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="53" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C15" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E15" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="53" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C16" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E16" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="53" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C17" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E17" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C18" s="52" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E18" s="11">
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="49" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C19" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E19" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="49" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C20" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E20" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C21" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D21" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E21" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C22" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E22" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C23" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D23" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E23" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C24" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D24" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E24" s="11">
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="49" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C25" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D25" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E25" s="11">
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="49" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C26" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D26" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E26" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="49" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C27" s="50" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E27" s="11">
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="54" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C28" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E28" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C29" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D29" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E29" s="11">
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="54" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C30" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E30" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="54" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C31" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D31" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E31" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="54" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C32" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D32" s="29" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E32" s="11">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="54" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C33" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E33" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C34" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D34" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E34" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="54" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C35" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D35" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E35" s="11">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C36" s="55" t="s">
         <v>17</v>
       </c>
       <c r="D36" s="29" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E36" s="11">
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C37" s="57" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E37" s="13">
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="32" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E39" s="33">
         <f>SUM(E6:E37)</f>
@@ -2598,7 +2638,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="37" priority="1">
+    <cfRule type="expression" dxfId="43" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2621,32 +2661,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
-    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" customWidth="1"/>
+    <col min="2" max="2" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" customWidth="1"/>
+    <col min="7" max="7" width="9.7265625" customWidth="1"/>
+    <col min="8" max="8" width="16.26953125" customWidth="1"/>
+    <col min="9" max="9" width="18.7265625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2676,7 +2716,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2730,7 +2770,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -2757,7 +2797,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -2779,7 +2819,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -2806,7 +2846,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -2839,7 +2879,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -2876,7 +2916,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -2913,7 +2953,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -2945,7 +2985,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -2973,7 +3013,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3000,15 +3040,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3024,44 +3064,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="77.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="77.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.54296875" customWidth="1"/>
+    <col min="11" max="11" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B3" s="64" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+      <c r="B3" s="81" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="65"/>
-      <c r="L3" s="66"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B5" s="67" t="s">
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
+      <c r="L3" s="83"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+      <c r="B5" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="C5" s="86" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3070,7 +3110,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="88" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3079,7 +3119,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="71" t="s">
+      <c r="I5" s="88" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3088,36 +3128,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="71" t="s">
+      <c r="L5" s="88" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="68"/>
-      <c r="C6" s="70"/>
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="85"/>
+      <c r="C6" s="87"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="72"/>
+      <c r="F6" s="89"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="72"/>
+      <c r="I6" s="89"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="72"/>
-    </row>
-    <row r="7" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L6" s="89"/>
+    </row>
+    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3131,7 +3171,7 @@
         <v>100</v>
       </c>
       <c r="F7" s="39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G7" s="26"/>
       <c r="H7" s="41"/>
@@ -3140,7 +3180,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3159,7 +3199,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3178,7 +3218,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3197,9 +3237,9 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>105</v>
@@ -3216,7 +3256,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3235,7 +3275,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3254,7 +3294,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3273,9 +3313,9 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C15" s="29" t="s">
         <v>102</v>
@@ -3292,7 +3332,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3311,7 +3351,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3330,9 +3370,9 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C18" s="29" t="s">
         <v>102</v>
@@ -3349,9 +3389,9 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C19" s="29" t="s">
         <v>102</v>
@@ -3368,9 +3408,9 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="46" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C20" s="47" t="s">
         <v>102</v>
@@ -3387,7 +3427,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3404,11 +3444,11 @@
         <v>100</v>
       </c>
       <c r="I21" s="40" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3427,7 +3467,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3444,11 +3484,11 @@
         <v>100</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3467,7 +3507,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3486,7 +3526,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3503,11 +3543,11 @@
         <v>100</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3524,11 +3564,11 @@
         <v>100</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3545,11 +3585,11 @@
         <v>100</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3568,9 +3608,9 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>102</v>
@@ -3587,7 +3627,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3606,7 +3646,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -3625,9 +3665,9 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C33" s="29" t="s">
         <v>102</v>
@@ -3644,9 +3684,9 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C34" s="29" t="s">
         <v>102</v>
@@ -3663,7 +3703,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -3682,7 +3722,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -3701,7 +3741,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -3720,9 +3760,9 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C38" s="29" t="s">
         <v>102</v>
@@ -3739,9 +3779,9 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C39" s="29" t="s">
         <v>102</v>
@@ -3758,9 +3798,9 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C40" s="29" t="s">
         <v>102</v>
@@ -3777,9 +3817,9 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C41" s="29" t="s">
         <v>102</v>
@@ -3796,9 +3836,9 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C42" s="29" t="s">
         <v>102</v>
@@ -3815,9 +3855,9 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C43" s="29" t="s">
         <v>102</v>
@@ -3834,9 +3874,9 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C44" s="29" t="s">
         <v>102</v>
@@ -3853,9 +3893,9 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C45" s="29" t="s">
         <v>102</v>
@@ -3872,9 +3912,9 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="29" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C46" s="29" t="s">
         <v>102</v>
@@ -3891,9 +3931,9 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="29" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C47" s="29" t="s">
         <v>102</v>
@@ -3910,9 +3950,9 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C48" s="29" t="s">
         <v>102</v>
@@ -3940,67 +3980,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="36" priority="7">
+    <cfRule type="expression" dxfId="42" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="35" priority="1">
+    <cfRule type="expression" dxfId="41" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="34" priority="32">
+    <cfRule type="expression" dxfId="40" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="38">
+    <cfRule type="expression" dxfId="39" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="32" priority="30">
+    <cfRule type="expression" dxfId="38" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="31" priority="6">
+    <cfRule type="expression" dxfId="37" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="30" priority="25">
+    <cfRule type="expression" dxfId="36" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="27">
+    <cfRule type="expression" dxfId="35" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="28" priority="8">
+    <cfRule type="expression" dxfId="34" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="27" priority="13">
+    <cfRule type="expression" dxfId="33" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="14">
+    <cfRule type="expression" dxfId="32" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="25" priority="20">
+    <cfRule type="expression" dxfId="31" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="21">
+    <cfRule type="expression" dxfId="30" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="23" priority="9">
+    <cfRule type="expression" dxfId="29" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="10">
+    <cfRule type="expression" dxfId="28" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4015,43 +4055,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" customWidth="1"/>
+    <col min="4" max="4" width="21.7265625" customWidth="1"/>
+    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.26953125" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.7265625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B1" s="64" t="s">
+    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+      <c r="B1" s="81" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="66"/>
-    </row>
-    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B4" s="67" t="s">
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="83"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+      <c r="B4" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="86" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4060,7 +4100,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="71" t="s">
+      <c r="F4" s="88" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4069,7 +4109,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="71" t="s">
+      <c r="I4" s="88" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4078,38 +4118,38 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="71" t="s">
+      <c r="L4" s="88" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="68"/>
-      <c r="C5" s="70"/>
+    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B5" s="85"/>
+      <c r="C5" s="87"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="72"/>
+      <c r="F5" s="89"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="72"/>
+      <c r="I5" s="89"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="72"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="89"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="29" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C6" s="29" t="s">
         <v>102</v>
@@ -4125,9 +4165,9 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C7" s="29" t="s">
         <v>102</v>
@@ -4143,9 +4183,9 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C8" s="29" t="s">
         <v>102</v>
@@ -4161,9 +4201,9 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>102</v>
@@ -4179,9 +4219,9 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>102</v>
@@ -4197,9 +4237,9 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>102</v>
@@ -4215,9 +4255,9 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>102</v>
@@ -4233,9 +4273,9 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>102</v>
@@ -4251,9 +4291,9 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C14" s="29" t="s">
         <v>102</v>
@@ -4269,9 +4309,9 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C15" s="29" t="s">
         <v>102</v>
@@ -4287,9 +4327,9 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C16" s="29" t="s">
         <v>102</v>
@@ -4305,9 +4345,9 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>102</v>
@@ -4323,9 +4363,9 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C18" s="29" t="s">
         <v>102</v>
@@ -4341,9 +4381,9 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C19" s="29" t="s">
         <v>102</v>
@@ -4359,9 +4399,9 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C20" s="29" t="s">
         <v>102</v>
@@ -4378,9 +4418,9 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C21" s="29" t="s">
         <v>102</v>
@@ -4397,9 +4437,9 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C22" s="29" t="s">
         <v>102</v>
@@ -4416,9 +4456,9 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C23" s="29" t="s">
         <v>102</v>
@@ -4435,9 +4475,9 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C24" s="29" t="s">
         <v>102</v>
@@ -4454,9 +4494,9 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C25" s="29" t="s">
         <v>102</v>
@@ -4473,9 +4513,9 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C26" s="29" t="s">
         <v>102</v>
@@ -4492,9 +4532,9 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C27" s="29" t="s">
         <v>102</v>
@@ -4511,9 +4551,9 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C28" s="29" t="s">
         <v>102</v>
@@ -4530,9 +4570,9 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C29" s="29" t="s">
         <v>102</v>
@@ -4549,9 +4589,9 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C30" s="29" t="s">
         <v>102</v>
@@ -4568,9 +4608,9 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C31" s="29" t="s">
         <v>102</v>
@@ -4587,9 +4627,9 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C32" s="29" t="s">
         <v>102</v>
@@ -4606,9 +4646,9 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C33" s="29" t="s">
         <v>102</v>
@@ -4625,9 +4665,9 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C34" s="29" t="s">
         <v>102</v>
@@ -4642,13 +4682,13 @@
         <v>100</v>
       </c>
       <c r="I34" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="L34" s="11"/>
+    </row>
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B35" s="29" t="s">
         <v>203</v>
-      </c>
-      <c r="L34" s="11"/>
-    </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B35" s="29" t="s">
-        <v>205</v>
       </c>
       <c r="C35" s="29" t="s">
         <v>102</v>
@@ -4666,9 +4706,9 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C36" s="29" t="s">
         <v>102</v>
@@ -4686,9 +4726,9 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C37" s="29" t="s">
         <v>102</v>
@@ -4706,9 +4746,9 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C38" s="29" t="s">
         <v>102</v>
@@ -4726,9 +4766,9 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C39" s="29" t="s">
         <v>102</v>
@@ -4746,9 +4786,9 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C40" s="29" t="s">
         <v>102</v>
@@ -4766,9 +4806,9 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C41" s="29" t="s">
         <v>102</v>
@@ -4785,10 +4825,10 @@
         <v>100</v>
       </c>
       <c r="L41" s="11" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -4808,9 +4848,9 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C43" s="29" t="s">
         <v>102</v>
@@ -4828,9 +4868,9 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C44" s="29" t="s">
         <v>102</v>
@@ -4848,9 +4888,9 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="58" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>103</v>
@@ -4866,7 +4906,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -4884,7 +4924,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" ht="58" x14ac:dyDescent="0.35">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -4905,11 +4945,11 @@
         <v>100</v>
       </c>
       <c r="I47" s="40" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -4927,7 +4967,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -4945,9 +4985,9 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B50" s="58" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C50" s="7" t="s">
         <v>103</v>
@@ -4968,9 +5008,9 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B51" s="58" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>103</v>
@@ -4991,7 +5031,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5009,7 +5049,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5027,7 +5067,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5044,7 +5084,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5062,9 +5102,9 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B56" s="58" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C56" s="7" t="s">
         <v>103</v>
@@ -5079,9 +5119,9 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B57" s="58" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>103</v>
@@ -5102,9 +5142,9 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B58" s="58" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>103</v>
@@ -5117,7 +5157,7 @@
         <v>75</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="J58">
         <v>2</v>
@@ -5126,12 +5166,12 @@
         <v>100</v>
       </c>
       <c r="L58" s="40" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B59" s="58" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C59" s="7" t="s">
         <v>103</v>
@@ -5147,26 +5187,26 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="75" t="s">
-        <v>215</v>
-      </c>
-      <c r="C60" s="76" t="s">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B60" s="64" t="s">
+        <v>212</v>
+      </c>
+      <c r="C60" s="65" t="s">
         <v>103</v>
       </c>
-      <c r="D60" s="77"/>
-      <c r="E60" s="78"/>
-      <c r="F60" s="78"/>
-      <c r="G60" s="77"/>
-      <c r="H60" s="79"/>
-      <c r="I60" s="80"/>
-      <c r="J60" s="78">
+      <c r="D60" s="66"/>
+      <c r="E60" s="67"/>
+      <c r="F60" s="67"/>
+      <c r="G60" s="66"/>
+      <c r="H60" s="68"/>
+      <c r="I60" s="69"/>
+      <c r="J60" s="67">
         <v>0.5</v>
       </c>
-      <c r="K60" s="78">
-        <v>100</v>
-      </c>
-      <c r="L60" s="80"/>
+      <c r="K60" s="67">
+        <v>100</v>
+      </c>
+      <c r="L60" s="69"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:L5" xr:uid="{2EE69061-1192-400C-B500-1B4897FD0585}"/>
@@ -5180,23 +5220,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="21" priority="49">
+    <cfRule type="expression" dxfId="27" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="20" priority="89">
+    <cfRule type="expression" dxfId="26" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="19" priority="46">
+    <cfRule type="expression" dxfId="25" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="47">
+    <cfRule type="expression" dxfId="24" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="48">
+    <cfRule type="expression" dxfId="23" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5211,26 +5251,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="81.5703125" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" customWidth="1"/>
+    <col min="2" max="2" width="81.54296875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" customWidth="1"/>
+    <col min="5" max="5" width="28.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B3" s="8" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C3" s="63" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>7</v>
@@ -5239,106 +5279,106 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="B4" s="81" t="s">
-        <v>229</v>
-      </c>
-      <c r="C4" s="82" t="s">
+    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B4" s="70" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" s="71" t="s">
+        <v>227</v>
+      </c>
+      <c r="D4" s="72" t="s">
+        <v>228</v>
+      </c>
+      <c r="E4" s="73">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="B5" s="74" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="62" t="s">
+        <v>238</v>
+      </c>
+      <c r="D5" s="75" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="76">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C6" s="62" t="s">
+        <v>232</v>
+      </c>
+      <c r="D6" s="75" t="s">
+        <v>102</v>
+      </c>
+      <c r="E6" s="76">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B7" s="74" t="s">
         <v>230</v>
       </c>
-      <c r="D4" s="83" t="s">
+      <c r="C7" s="62" t="s">
         <v>231</v>
       </c>
-      <c r="E4" s="84">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="B5" s="85" t="s">
-        <v>243</v>
-      </c>
-      <c r="C5" s="62" t="s">
-        <v>241</v>
-      </c>
-      <c r="D5" s="86" t="s">
-        <v>103</v>
-      </c>
-      <c r="E5" s="87">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="B6" s="85" t="s">
-        <v>244</v>
-      </c>
-      <c r="C6" s="62" t="s">
+      <c r="D7" s="75" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="76">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B8" s="74" t="s">
+        <v>233</v>
+      </c>
+      <c r="C8" s="62" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" s="75" t="s">
+        <v>228</v>
+      </c>
+      <c r="E8" s="76">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B9" s="74" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="62" t="s">
+        <v>237</v>
+      </c>
+      <c r="D9" s="75" t="s">
+        <v>228</v>
+      </c>
+      <c r="E9" s="76">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="77" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="78" t="s">
         <v>235</v>
       </c>
-      <c r="D6" s="86" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="87">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="85" t="s">
-        <v>233</v>
-      </c>
-      <c r="C7" s="62" t="s">
-        <v>234</v>
-      </c>
-      <c r="D7" s="86" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="87">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="B8" s="85" t="s">
-        <v>236</v>
-      </c>
-      <c r="C8" s="62" t="s">
-        <v>237</v>
-      </c>
-      <c r="D8" s="86" t="s">
-        <v>231</v>
-      </c>
-      <c r="E8" s="87">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="B9" s="85" t="s">
-        <v>180</v>
-      </c>
-      <c r="C9" s="62" t="s">
-        <v>240</v>
-      </c>
-      <c r="D9" s="86" t="s">
-        <v>231</v>
-      </c>
-      <c r="E9" s="87">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="88" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="89" t="s">
-        <v>238</v>
-      </c>
-      <c r="D10" s="90"/>
-      <c r="E10" s="91"/>
+      <c r="D10" s="79"/>
+      <c r="E10" s="80"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="1" priority="157">
+    <cfRule type="expression" dxfId="22" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="158">
+    <cfRule type="expression" dxfId="21" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5352,50 +5392,50 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:O20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:O22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.7265625" customWidth="1"/>
     <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.28515625" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" customWidth="1"/>
-    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.26953125" customWidth="1"/>
+    <col min="5" max="5" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.26953125" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.7265625" customWidth="1"/>
+    <col min="15" max="15" width="19.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="B2" s="73" t="s">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+      <c r="B2" s="90" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="74"/>
-      <c r="J2" s="74"/>
-      <c r="K2" s="74"/>
-      <c r="L2" s="74"/>
-      <c r="M2" s="74"/>
-      <c r="N2" s="74"/>
-      <c r="O2" s="74"/>
-    </row>
-    <row r="5" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.35">
-      <c r="B6" s="67" t="s">
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="91"/>
+      <c r="J2" s="91"/>
+      <c r="K2" s="91"/>
+      <c r="L2" s="91"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="91"/>
+      <c r="O2" s="91"/>
+    </row>
+    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+      <c r="B6" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="86" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="42" t="s">
@@ -5404,7 +5444,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="71" t="s">
+      <c r="F6" s="88" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5413,7 +5453,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="71" t="s">
+      <c r="I6" s="88" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="45" t="s">
@@ -5422,7 +5462,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="71" t="s">
+      <c r="L6" s="88" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="45" t="s">
@@ -5431,142 +5471,154 @@
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="71" t="s">
+      <c r="O6" s="88" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="68"/>
-      <c r="C7" s="70"/>
+    <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="85"/>
+      <c r="C7" s="87"/>
       <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="72"/>
+      <c r="F7" s="89"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="72"/>
+      <c r="I7" s="89"/>
       <c r="J7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="72"/>
+      <c r="L7" s="89"/>
       <c r="M7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="N7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="72"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O7" s="89"/>
+    </row>
+    <row r="8" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="29" t="s">
-        <v>213</v>
+        <v>68</v>
       </c>
       <c r="C8" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D8" s="24"/>
-      <c r="E8" s="31"/>
-      <c r="F8" s="11"/>
+      <c r="E8" s="92">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>229</v>
+      </c>
       <c r="G8" s="24"/>
       <c r="H8" s="31"/>
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="10"/>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O8" s="11"/>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D9" s="24"/>
-      <c r="E9" s="31"/>
+      <c r="E9" s="31">
+        <v>100</v>
+      </c>
       <c r="F9" s="11"/>
       <c r="G9" s="24"/>
       <c r="H9" s="31"/>
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
-      <c r="O9" s="11"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="10"/>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
-        <v>43</v>
+        <v>245</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D10" s="24"/>
-      <c r="E10" s="31"/>
+      <c r="E10" s="31">
+        <v>100</v>
+      </c>
       <c r="F10" s="11"/>
       <c r="G10" s="24"/>
       <c r="H10" s="31"/>
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
+      <c r="M10" s="75"/>
+      <c r="N10" s="75"/>
       <c r="O10" s="11"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
-        <v>106</v>
+        <v>244</v>
       </c>
       <c r="C11" s="29" t="s">
         <v>102</v>
       </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="31">
+        <v>100</v>
+      </c>
+      <c r="F11" s="11"/>
       <c r="G11" s="24"/>
+      <c r="H11" s="31"/>
       <c r="I11" s="11"/>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="L11" s="11"/>
+      <c r="M11" s="75"/>
+      <c r="N11" s="75"/>
+      <c r="O11" s="11"/>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D12" s="24"/>
-      <c r="E12" s="31"/>
-      <c r="F12" s="11"/>
       <c r="G12" s="24"/>
-      <c r="H12" s="31"/>
       <c r="I12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="O12" s="11"/>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
-        <v>68</v>
+        <v>247</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D13" s="24"/>
       <c r="E13" s="31"/>
-      <c r="F13" s="11" t="s">
-        <v>232</v>
-      </c>
+      <c r="F13" s="11"/>
       <c r="G13" s="24"/>
       <c r="H13" s="31"/>
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
       <c r="O13" s="11"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
-        <v>218</v>
+        <v>43</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D14" s="24"/>
       <c r="E14" s="31"/>
@@ -5575,13 +5627,14 @@
       <c r="H14" s="31"/>
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O14" s="11"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
-        <v>219</v>
+        <v>179</v>
       </c>
       <c r="C15" s="29" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D15" s="24"/>
       <c r="E15" s="31"/>
@@ -5590,10 +5643,11 @@
       <c r="H15" s="31"/>
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="O15" s="11"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C16" s="29" t="s">
         <v>103</v>
@@ -5606,9 +5660,9 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>103</v>
@@ -5621,7 +5675,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>221</v>
       </c>
@@ -5636,9 +5690,9 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="C19" s="29" t="s">
         <v>103</v>
@@ -5651,9 +5705,9 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
-        <v>242</v>
+        <v>218</v>
       </c>
       <c r="C20" s="29" t="s">
         <v>103</v>
@@ -5665,6 +5719,36 @@
       <c r="H20" s="31"/>
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B21" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="C21" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="24"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="11"/>
+      <c r="L21" s="11"/>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B22" s="29" t="s">
+        <v>239</v>
+      </c>
+      <c r="C22" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="24"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="11"/>
+      <c r="L22" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5676,69 +5760,92 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B9:B10 B14:B20">
-    <cfRule type="expression" dxfId="16" priority="20">
+  <conditionalFormatting sqref="B2 B6:B7 B13:B22">
+    <cfRule type="expression" dxfId="20" priority="22">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="15" priority="12">
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" dxfId="19" priority="140">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" dxfId="18" priority="158">
+      <formula>MAX($E16,$H16,$K16)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15">
+    <cfRule type="expression" dxfId="2" priority="145">
+      <formula>MAX($E20,$H20,$K20)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="expression" dxfId="16" priority="133">
+      <formula>MAX($E20,$H20,$K20)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="143">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:C22">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>$C6="Charlotte/Eddy"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="12">
+      <formula>$C6="Charlotte"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="13">
+      <formula>$C6="Eddy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B11">
+    <cfRule type="expression" dxfId="11" priority="164">
+      <formula>MAX($E17,$H17,$K17)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" dxfId="10" priority="175">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="expression" dxfId="9" priority="192">
+      <formula>MAX($E8,$H8,$K8)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="193">
+      <formula>MAX($E5,$H5,$K5)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" dxfId="7" priority="208">
+      <formula>MAX($E12,$H12,$K12)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15">
+    <cfRule type="expression" dxfId="1" priority="209">
+      <formula>MAX($E9,$H9,$K9)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="210">
+      <formula>MAX($E21,$H21,$K21)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B11">
+    <cfRule type="expression" dxfId="6" priority="211">
+      <formula>MAX($E16,$H16,$K16)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="212">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="14" priority="106">
-      <formula>MAX($E13,$H13,$K13)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="108">
-      <formula>MAX($E5,$H5,$K5)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="12" priority="138">
-      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="11" priority="156">
-      <formula>MAX($E14,$H14,$K14)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="10" priority="153">
+  <conditionalFormatting sqref="B12">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B12">
-    <cfRule type="expression" dxfId="9" priority="143">
-      <formula>MAX($E17,$H17,$K17)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="expression" dxfId="8" priority="104">
-      <formula>MAX($E8,$H8,$K8)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="155">
-      <formula>MAX($E19,$H19,$K19)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="6" priority="131">
-      <formula>MAX($E18,$H18,$K18)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="141">
-      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C20">
-    <cfRule type="expression" dxfId="4" priority="9">
-      <formula>$C6="Charlotte/Eddy"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="10">
-      <formula>$C6="Charlotte"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="11">
-      <formula>$C6="Eddy"</formula>
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5751,28 +5858,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
-    <col min="2" max="2" width="93.28515625" customWidth="1"/>
+    <col min="1" max="1" width="3.26953125" customWidth="1"/>
+    <col min="2" max="2" width="93.26953125" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.7265625" customWidth="1"/>
+    <col min="6" max="6" width="42.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -5789,7 +5896,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -5802,7 +5909,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -5815,7 +5922,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -5828,7 +5935,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -5841,7 +5948,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -5854,7 +5961,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -5867,7 +5974,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -5880,7 +5987,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -5893,7 +6000,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -5906,7 +6013,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -5919,7 +6026,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -5932,7 +6039,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -5945,7 +6052,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -5958,7 +6065,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -5971,7 +6078,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -5984,7 +6091,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -5997,7 +6104,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -6010,7 +6117,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -6023,7 +6130,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -6036,7 +6143,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -6049,7 +6156,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -6062,7 +6169,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -6075,7 +6182,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -6088,7 +6195,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -6101,7 +6208,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -6114,7 +6221,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -6127,7 +6234,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -6140,7 +6247,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -6153,7 +6260,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -6166,7 +6273,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -6179,7 +6286,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -6192,7 +6299,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -6205,7 +6312,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -6218,7 +6325,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -6231,7 +6338,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -6244,7 +6351,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -6257,7 +6364,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -6270,7 +6377,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -6283,7 +6390,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -6296,7 +6403,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -6309,7 +6416,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -6322,7 +6429,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -6335,7 +6442,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -6348,7 +6455,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -6361,7 +6468,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -6374,7 +6481,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -6387,7 +6494,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -6400,7 +6507,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -6413,7 +6520,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -6426,7 +6533,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -6439,7 +6546,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -6452,7 +6559,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -6465,7 +6572,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -6478,7 +6585,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -6491,7 +6598,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -6504,7 +6611,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -6517,7 +6624,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -6530,7 +6637,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -6543,7 +6650,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -6556,7 +6663,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -6567,7 +6674,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -6578,7 +6685,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -6589,7 +6696,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -6600,7 +6707,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -6611,7 +6718,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -6622,7 +6729,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -6633,7 +6740,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -6644,7 +6751,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -6655,9 +6762,9 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C74" s="3"/>
       <c r="D74" s="3" t="s">
@@ -6666,9 +6773,9 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C75" s="3"/>
       <c r="D75" s="3" t="s">
@@ -6677,182 +6784,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
AJout phase waiting apres placement réussi. Mise a jour tutoriel avec onglets +texte+video ou image
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6B0504C-4D3D-4E41-937F-16CC6C24B8FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8DA629-6DB2-48B3-89FF-E5B185F42D68}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,10 +27,15 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1460,6 +1465,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1493,21 +1501,11 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="44">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="43">
     <dxf>
       <fill>
         <patternFill>
@@ -2144,26 +2142,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.26953125" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="42.7265625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2177,7 +2175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2191,7 +2189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2205,7 +2203,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2219,7 +2217,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2233,7 +2231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2247,7 +2245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2261,7 +2259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2275,7 +2273,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2289,7 +2287,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2303,7 +2301,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2317,7 +2315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2331,7 +2329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2345,7 +2343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2359,7 +2357,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2373,7 +2371,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2387,7 +2385,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2401,7 +2399,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2415,7 +2413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2429,7 +2427,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2443,7 +2441,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2457,7 +2455,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -2471,7 +2469,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -2485,7 +2483,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -2499,7 +2497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -2513,7 +2511,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -2527,7 +2525,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -2541,7 +2539,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -2555,7 +2553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -2569,7 +2567,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -2583,7 +2581,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -2597,7 +2595,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -2611,7 +2609,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -2625,8 +2623,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -2638,7 +2636,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="43" priority="1">
+    <cfRule type="expression" dxfId="42" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2661,32 +2659,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7265625" customWidth="1"/>
-    <col min="2" max="2" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.26953125" customWidth="1"/>
-    <col min="5" max="5" width="19.7265625" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" customWidth="1"/>
-    <col min="7" max="7" width="9.7265625" customWidth="1"/>
-    <col min="8" max="8" width="16.26953125" customWidth="1"/>
-    <col min="9" max="9" width="18.7265625" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" customWidth="1"/>
-    <col min="11" max="11" width="16.26953125" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
-    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2716,7 +2714,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2770,7 +2768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -2797,7 +2795,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -2819,7 +2817,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -2846,7 +2844,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -2879,7 +2877,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -2916,7 +2914,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -2953,7 +2951,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -2985,7 +2983,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3013,7 +3011,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3040,15 +3038,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3064,44 +3062,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="77.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.54296875" customWidth="1"/>
-    <col min="11" max="11" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7265625" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="81" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B3" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="82"/>
-      <c r="D3" s="82"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="82"/>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82"/>
-      <c r="K3" s="82"/>
-      <c r="L3" s="83"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="84" t="s">
+      <c r="C3" s="83"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
+      <c r="K3" s="83"/>
+      <c r="L3" s="84"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="86" t="s">
+      <c r="C5" s="87" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3110,7 +3108,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="88" t="s">
+      <c r="F5" s="89" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3119,7 +3117,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="88" t="s">
+      <c r="I5" s="89" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3128,36 +3126,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="88" t="s">
+      <c r="L5" s="89" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="85"/>
-      <c r="C6" s="87"/>
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="86"/>
+      <c r="C6" s="88"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="89"/>
+      <c r="F6" s="90"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="89"/>
+      <c r="I6" s="90"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="89"/>
-    </row>
-    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
+      <c r="L6" s="90"/>
+    </row>
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3180,7 +3178,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3199,7 +3197,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3218,7 +3216,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3237,7 +3235,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3256,7 +3254,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3275,7 +3273,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3294,7 +3292,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3313,7 +3311,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3332,7 +3330,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3351,7 +3349,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3370,7 +3368,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3389,7 +3387,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3408,7 +3406,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3427,7 +3425,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3448,7 +3446,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3467,7 +3465,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3488,7 +3486,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3507,7 +3505,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3526,7 +3524,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3547,7 +3545,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3568,7 +3566,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3589,7 +3587,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3608,7 +3606,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -3627,7 +3625,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3646,7 +3644,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -3665,7 +3663,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -3684,7 +3682,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -3703,7 +3701,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -3722,7 +3720,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -3741,7 +3739,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -3760,7 +3758,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -3779,7 +3777,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -3798,7 +3796,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -3817,7 +3815,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -3836,7 +3834,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -3855,7 +3853,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -3874,7 +3872,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -3893,7 +3891,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -3912,7 +3910,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -3931,7 +3929,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -3950,7 +3948,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -3980,67 +3978,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="42" priority="7">
+    <cfRule type="expression" dxfId="41" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="41" priority="1">
+    <cfRule type="expression" dxfId="40" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="40" priority="32">
+    <cfRule type="expression" dxfId="39" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="38">
+    <cfRule type="expression" dxfId="38" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="38" priority="30">
+    <cfRule type="expression" dxfId="37" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="37" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="36" priority="25">
+    <cfRule type="expression" dxfId="35" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="27">
+    <cfRule type="expression" dxfId="34" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="34" priority="8">
+    <cfRule type="expression" dxfId="33" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="33" priority="13">
+    <cfRule type="expression" dxfId="32" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="14">
+    <cfRule type="expression" dxfId="31" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="31" priority="20">
+    <cfRule type="expression" dxfId="30" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="21">
+    <cfRule type="expression" dxfId="29" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="29" priority="9">
+    <cfRule type="expression" dxfId="28" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="10">
+    <cfRule type="expression" dxfId="27" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4055,43 +4053,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7265625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.26953125" customWidth="1"/>
-    <col min="4" max="4" width="21.7265625" customWidth="1"/>
-    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.7265625" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.77734375" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.453125" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="81" t="s">
+    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B1" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-      <c r="F1" s="82"/>
-      <c r="G1" s="82"/>
-      <c r="H1" s="82"/>
-      <c r="I1" s="82"/>
-      <c r="J1" s="82"/>
-      <c r="K1" s="82"/>
-      <c r="L1" s="83"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="84" t="s">
+      <c r="C1" s="83"/>
+      <c r="D1" s="83"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="84"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="86" t="s">
+      <c r="C4" s="87" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4100,7 +4098,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="88" t="s">
+      <c r="F4" s="89" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4109,7 +4107,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="88" t="s">
+      <c r="I4" s="89" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4118,36 +4116,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="88" t="s">
+      <c r="L4" s="89" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="85"/>
-      <c r="C5" s="87"/>
+    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="86"/>
+      <c r="C5" s="88"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="89"/>
+      <c r="F5" s="90"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="89"/>
+      <c r="I5" s="90"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="89"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L5" s="90"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4165,7 +4163,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4183,7 +4181,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4201,7 +4199,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4219,7 +4217,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4237,7 +4235,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4255,7 +4253,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4273,7 +4271,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4291,7 +4289,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4309,7 +4307,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4327,7 +4325,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4345,7 +4343,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4363,7 +4361,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4381,7 +4379,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4399,7 +4397,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4418,7 +4416,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4437,7 +4435,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4456,7 +4454,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -4475,7 +4473,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -4494,7 +4492,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -4513,7 +4511,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -4532,7 +4530,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -4551,7 +4549,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -4570,7 +4568,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -4589,7 +4587,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -4608,7 +4606,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -4627,7 +4625,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -4646,7 +4644,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -4665,7 +4663,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -4686,7 +4684,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -4706,7 +4704,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -4726,7 +4724,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -4746,7 +4744,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -4766,7 +4764,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -4786,7 +4784,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -4806,7 +4804,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -4828,7 +4826,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -4848,7 +4846,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -4868,7 +4866,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -4888,7 +4886,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -4906,7 +4904,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -4924,7 +4922,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -4949,7 +4947,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -4967,7 +4965,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -4985,7 +4983,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5008,7 +5006,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5031,7 +5029,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5049,7 +5047,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5067,7 +5065,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5084,7 +5082,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5102,7 +5100,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5119,7 +5117,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5142,7 +5140,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5169,7 +5167,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5187,7 +5185,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5220,23 +5218,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="27" priority="49">
+    <cfRule type="expression" dxfId="26" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="26" priority="89">
+    <cfRule type="expression" dxfId="25" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="25" priority="46">
+    <cfRule type="expression" dxfId="24" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="47">
+    <cfRule type="expression" dxfId="23" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="48">
+    <cfRule type="expression" dxfId="22" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5251,21 +5249,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7265625" customWidth="1"/>
-    <col min="2" max="2" width="81.54296875" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="81.5546875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" customWidth="1"/>
-    <col min="5" max="5" width="28.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="28.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5279,7 +5277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="70" t="s">
         <v>226</v>
       </c>
@@ -5293,7 +5291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="74" t="s">
         <v>240</v>
       </c>
@@ -5307,7 +5305,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="74" t="s">
         <v>241</v>
       </c>
@@ -5321,7 +5319,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="74" t="s">
         <v>230</v>
       </c>
@@ -5335,7 +5333,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="74" t="s">
         <v>233</v>
       </c>
@@ -5349,7 +5347,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="74" t="s">
         <v>179</v>
       </c>
@@ -5363,7 +5361,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="77" t="s">
         <v>68</v>
       </c>
@@ -5375,10 +5373,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="22" priority="157">
+    <cfRule type="expression" dxfId="21" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="158">
+    <cfRule type="expression" dxfId="20" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5393,49 +5391,49 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7265625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.26953125" customWidth="1"/>
-    <col min="5" max="5" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.26953125" customWidth="1"/>
-    <col min="11" max="11" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.7265625" customWidth="1"/>
-    <col min="15" max="15" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.44140625" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="90" t="s">
+    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="B2" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="91"/>
-      <c r="I2" s="91"/>
-      <c r="J2" s="91"/>
-      <c r="K2" s="91"/>
-      <c r="L2" s="91"/>
-      <c r="M2" s="91"/>
-      <c r="N2" s="91"/>
-      <c r="O2" s="91"/>
-    </row>
-    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B6" s="84" t="s">
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
+      <c r="I2" s="92"/>
+      <c r="J2" s="92"/>
+      <c r="K2" s="92"/>
+      <c r="L2" s="92"/>
+      <c r="M2" s="92"/>
+      <c r="N2" s="92"/>
+      <c r="O2" s="92"/>
+    </row>
+    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="86" t="s">
+      <c r="C6" s="87" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="42" t="s">
@@ -5444,7 +5442,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="88" t="s">
+      <c r="F6" s="89" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5453,7 +5451,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="88" t="s">
+      <c r="I6" s="89" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="45" t="s">
@@ -5462,7 +5460,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="88" t="s">
+      <c r="L6" s="89" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="45" t="s">
@@ -5471,43 +5469,43 @@
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="88" t="s">
+      <c r="O6" s="89" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="85"/>
-      <c r="C7" s="87"/>
+    <row r="7" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="86"/>
+      <c r="C7" s="88"/>
       <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="89"/>
+      <c r="F7" s="90"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="89"/>
+      <c r="I7" s="90"/>
       <c r="J7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="89"/>
+      <c r="L7" s="90"/>
       <c r="M7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="N7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="89"/>
-    </row>
-    <row r="8" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="O7" s="90"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>68</v>
       </c>
@@ -5515,7 +5513,7 @@
         <v>102</v>
       </c>
       <c r="D8" s="24"/>
-      <c r="E8" s="92">
+      <c r="E8" s="81">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
@@ -5524,10 +5522,14 @@
       <c r="G8" s="24"/>
       <c r="H8" s="31"/>
       <c r="I8" s="11"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="31"/>
       <c r="L8" s="11"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="31"/>
       <c r="O8" s="11"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>246</v>
       </c>
@@ -5542,12 +5544,14 @@
       <c r="G9" s="24"/>
       <c r="H9" s="31"/>
       <c r="I9" s="11"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="31"/>
       <c r="L9" s="11"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="10"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="M9" s="24"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>245</v>
       </c>
@@ -5562,12 +5566,14 @@
       <c r="G10" s="24"/>
       <c r="H10" s="31"/>
       <c r="I10" s="11"/>
+      <c r="J10" s="24"/>
+      <c r="K10" s="31"/>
       <c r="L10" s="11"/>
-      <c r="M10" s="75"/>
-      <c r="N10" s="75"/>
+      <c r="M10" s="24"/>
+      <c r="N10" s="31"/>
       <c r="O10" s="11"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>244</v>
       </c>
@@ -5582,12 +5588,14 @@
       <c r="G11" s="24"/>
       <c r="H11" s="31"/>
       <c r="I11" s="11"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="31"/>
       <c r="L11" s="11"/>
-      <c r="M11" s="75"/>
-      <c r="N11" s="75"/>
+      <c r="M11" s="24"/>
+      <c r="N11" s="31"/>
       <c r="O11" s="11"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>248</v>
       </c>
@@ -5596,8 +5604,12 @@
       </c>
       <c r="G12" s="24"/>
       <c r="I12" s="11"/>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="J12" s="24"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="24"/>
+      <c r="O12" s="11"/>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>247</v>
       </c>
@@ -5610,10 +5622,14 @@
       <c r="G13" s="24"/>
       <c r="H13" s="31"/>
       <c r="I13" s="11"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="31"/>
       <c r="L13" s="11"/>
+      <c r="M13" s="24"/>
+      <c r="N13" s="31"/>
       <c r="O13" s="11"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>43</v>
       </c>
@@ -5626,10 +5642,14 @@
       <c r="G14" s="24"/>
       <c r="H14" s="31"/>
       <c r="I14" s="11"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="31"/>
       <c r="L14" s="11"/>
+      <c r="M14" s="24"/>
+      <c r="N14" s="31"/>
       <c r="O14" s="11"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>179</v>
       </c>
@@ -5642,10 +5662,14 @@
       <c r="G15" s="24"/>
       <c r="H15" s="31"/>
       <c r="I15" s="11"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="31"/>
       <c r="L15" s="11"/>
+      <c r="M15" s="24"/>
+      <c r="N15" s="31"/>
       <c r="O15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>215</v>
       </c>
@@ -5658,9 +5682,14 @@
       <c r="G16" s="24"/>
       <c r="H16" s="31"/>
       <c r="I16" s="11"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="31"/>
       <c r="L16" s="11"/>
-    </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M16" s="24"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="11"/>
+    </row>
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>216</v>
       </c>
@@ -5673,9 +5702,14 @@
       <c r="G17" s="24"/>
       <c r="H17" s="31"/>
       <c r="I17" s="11"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="31"/>
       <c r="L17" s="11"/>
-    </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M17" s="24"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="11"/>
+    </row>
+    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>221</v>
       </c>
@@ -5688,9 +5722,14 @@
       <c r="G18" s="24"/>
       <c r="H18" s="31"/>
       <c r="I18" s="11"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="31"/>
       <c r="L18" s="11"/>
-    </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M18" s="24"/>
+      <c r="N18" s="31"/>
+      <c r="O18" s="11"/>
+    </row>
+    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>217</v>
       </c>
@@ -5703,9 +5742,14 @@
       <c r="G19" s="24"/>
       <c r="H19" s="31"/>
       <c r="I19" s="11"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="31"/>
       <c r="L19" s="11"/>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M19" s="24"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="11"/>
+    </row>
+    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>218</v>
       </c>
@@ -5718,9 +5762,14 @@
       <c r="G20" s="24"/>
       <c r="H20" s="31"/>
       <c r="I20" s="11"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="31"/>
       <c r="L20" s="11"/>
-    </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M20" s="24"/>
+      <c r="N20" s="31"/>
+      <c r="O20" s="11"/>
+    </row>
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>222</v>
       </c>
@@ -5733,9 +5782,14 @@
       <c r="G21" s="24"/>
       <c r="H21" s="31"/>
       <c r="I21" s="11"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="31"/>
       <c r="L21" s="11"/>
-    </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="M21" s="24"/>
+      <c r="N21" s="31"/>
+      <c r="O21" s="11"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>239</v>
       </c>
@@ -5748,7 +5802,12 @@
       <c r="G22" s="24"/>
       <c r="H22" s="31"/>
       <c r="I22" s="11"/>
+      <c r="J22" s="24"/>
+      <c r="K22" s="31"/>
       <c r="L22" s="11"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="31"/>
+      <c r="O22" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -5761,90 +5820,90 @@
     <mergeCell ref="L6:L7"/>
   </mergeCells>
   <conditionalFormatting sqref="B2 B6:B7 B13:B22">
-    <cfRule type="expression" dxfId="20" priority="22">
+    <cfRule type="expression" dxfId="19" priority="22">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="19" priority="140">
+    <cfRule type="expression" dxfId="18" priority="140">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14">
-    <cfRule type="expression" dxfId="18" priority="158">
+    <cfRule type="expression" dxfId="17" priority="158">
       <formula>MAX($E16,$H16,$K16)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="2" priority="145">
+    <cfRule type="expression" dxfId="16" priority="145">
       <formula>MAX($E20,$H20,$K20)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="16" priority="133">
+    <cfRule type="expression" dxfId="15" priority="133">
       <formula>MAX($E20,$H20,$K20)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="143">
+    <cfRule type="expression" dxfId="14" priority="143">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C22">
-    <cfRule type="expression" dxfId="14" priority="11">
+    <cfRule type="expression" dxfId="13" priority="11">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="12">
+    <cfRule type="expression" dxfId="12" priority="12">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="13">
+    <cfRule type="expression" dxfId="11" priority="13">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:B11">
-    <cfRule type="expression" dxfId="11" priority="164">
+    <cfRule type="expression" dxfId="10" priority="164">
       <formula>MAX($E17,$H17,$K17)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="10" priority="175">
+    <cfRule type="expression" dxfId="9" priority="175">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="9" priority="192">
+    <cfRule type="expression" dxfId="8" priority="192">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="193">
+    <cfRule type="expression" dxfId="7" priority="193">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="7" priority="208">
+    <cfRule type="expression" dxfId="6" priority="208">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="1" priority="209">
+    <cfRule type="expression" dxfId="5" priority="209">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="210">
+    <cfRule type="expression" dxfId="4" priority="210">
       <formula>MAX($E21,$H21,$K21)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:B11">
-    <cfRule type="expression" dxfId="6" priority="211">
+    <cfRule type="expression" dxfId="3" priority="211">
       <formula>MAX($E16,$H16,$K16)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="212">
+    <cfRule type="expression" dxfId="2" priority="212">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>MAX($E12,$H12,$K12)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5858,28 +5917,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.26953125" customWidth="1"/>
-    <col min="2" max="2" width="93.26953125" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="2" max="2" width="93.21875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.7265625" customWidth="1"/>
-    <col min="6" max="6" width="42.7265625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -5896,7 +5955,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -5909,7 +5968,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -5922,7 +5981,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -5935,7 +5994,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -5948,7 +6007,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -5961,7 +6020,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -5974,7 +6033,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -5987,7 +6046,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -6000,7 +6059,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -6013,7 +6072,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -6026,7 +6085,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -6039,7 +6098,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -6052,7 +6111,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -6065,7 +6124,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -6078,7 +6137,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -6091,7 +6150,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -6104,7 +6163,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -6117,7 +6176,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -6130,7 +6189,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -6143,7 +6202,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -6156,7 +6215,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -6169,7 +6228,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -6182,7 +6241,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -6195,7 +6254,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -6208,7 +6267,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -6221,7 +6280,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -6234,7 +6293,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -6247,7 +6306,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -6260,7 +6319,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -6273,7 +6332,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -6286,7 +6345,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -6299,7 +6358,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -6312,7 +6371,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -6325,7 +6384,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -6338,7 +6397,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -6351,7 +6410,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -6364,7 +6423,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -6377,7 +6436,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -6390,7 +6449,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -6403,7 +6462,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -6416,7 +6475,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -6429,7 +6488,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -6442,7 +6501,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -6455,7 +6514,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -6468,7 +6527,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -6481,7 +6540,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -6494,7 +6553,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -6507,7 +6566,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -6520,7 +6579,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -6533,7 +6592,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -6546,7 +6605,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -6559,7 +6618,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -6572,7 +6631,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -6585,7 +6644,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -6598,7 +6657,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -6611,7 +6670,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -6624,7 +6683,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -6637,7 +6696,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -6650,7 +6709,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -6663,7 +6722,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -6674,7 +6733,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -6685,7 +6744,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -6696,7 +6755,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -6707,7 +6766,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -6718,7 +6777,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -6729,7 +6788,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -6740,7 +6799,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -6751,7 +6810,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -6762,7 +6821,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>106</v>
       </c>
@@ -6773,7 +6832,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>107</v>
       </c>
@@ -6784,182 +6843,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Mise a jour tutoriel : résolutions de bug
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE6D18F-50D5-419C-86C3-7D25399D39BA}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A83DB2F-7F5F-49AA-89F5-A4F402B11817}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="4" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,15 +27,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -822,9 +817,6 @@
     <t>Ajout du bouton pause qui toogle avec resume</t>
   </si>
   <si>
-    <t>Créer une page administration:gestion des utilisateurs: mettre des droits  , ajouter suprimer des utilisateurs</t>
-  </si>
-  <si>
     <t>Répartir le classement en 2 sections : vs AI et vs humain</t>
   </si>
   <si>
@@ -832,6 +824,10 @@
   </si>
   <si>
     <t>Ajout action sauvegarder</t>
+  </si>
+  <si>
+    <t>Créer une page administration:gestion des utilisateurs: 
+mettre des droits, ajouter suprimer des utilisateurs</t>
   </si>
 </sst>
 </file>
@@ -882,7 +878,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -964,6 +960,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1403,7 +1405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1525,7 +1527,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1580,6 +1581,9 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2284,26 +2288,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" customWidth="1"/>
-    <col min="5" max="5" width="42.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" customWidth="1"/>
+    <col min="5" max="5" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="5" spans="2:5" ht="47" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2317,7 +2321,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2327,11 +2331,11 @@
       <c r="D6" s="28" t="s">
         <v>139</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="100">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2341,11 +2345,11 @@
       <c r="D7" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2355,11 +2359,11 @@
       <c r="D8" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2369,11 +2373,11 @@
       <c r="D9" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="101">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2383,11 +2387,11 @@
       <c r="D10" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="101">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2397,11 +2401,11 @@
       <c r="D11" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="101">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2411,11 +2415,11 @@
       <c r="D12" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="101">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2425,11 +2429,11 @@
       <c r="D13" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="101">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2439,11 +2443,11 @@
       <c r="D14" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="101">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2453,11 +2457,11 @@
       <c r="D15" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2467,11 +2471,11 @@
       <c r="D16" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E16" s="11">
+      <c r="E16" s="101">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2481,11 +2485,11 @@
       <c r="D17" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="101">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2495,11 +2499,11 @@
       <c r="D18" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="101">
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2509,11 +2513,11 @@
       <c r="D19" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="101">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2523,11 +2527,11 @@
       <c r="D20" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2537,11 +2541,11 @@
       <c r="D21" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="101">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2551,11 +2555,11 @@
       <c r="D22" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="101">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2565,11 +2569,11 @@
       <c r="D23" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2579,11 +2583,11 @@
       <c r="D24" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="101">
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2593,11 +2597,11 @@
       <c r="D25" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="101">
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -2611,7 +2615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -2625,7 +2629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -2635,11 +2639,11 @@
       <c r="D28" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28" s="101">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -2653,7 +2657,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -2663,11 +2667,11 @@
       <c r="D30" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -2677,11 +2681,11 @@
       <c r="D31" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="101">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -2695,7 +2699,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -2705,11 +2709,11 @@
       <c r="D33" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -2723,7 +2727,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -2733,11 +2737,11 @@
       <c r="D35" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E35" s="11">
+      <c r="E35" s="101">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -2751,7 +2755,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -2765,8 +2769,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -2801,32 +2805,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" customWidth="1"/>
-    <col min="7" max="7" width="9.77734375" customWidth="1"/>
-    <col min="8" max="8" width="16.21875" customWidth="1"/>
-    <col min="9" max="9" width="18.77734375" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" customWidth="1"/>
+    <col min="8" max="8" width="16.1796875" customWidth="1"/>
+    <col min="9" max="9" width="18.81640625" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" customWidth="1"/>
+    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2856,7 +2860,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -2910,7 +2914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -2937,7 +2941,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -2959,7 +2963,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -2986,7 +2990,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -3019,7 +3023,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -3056,7 +3060,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -3093,7 +3097,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -3125,7 +3129,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3153,7 +3157,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3180,15 +3184,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3204,44 +3208,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
-    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" customWidth="1"/>
+    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" customWidth="1"/>
-    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.77734375" customWidth="1"/>
+    <col min="10" max="10" width="16.54296875" customWidth="1"/>
+    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B3" s="89" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+      <c r="B3" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="90"/>
-      <c r="I3" s="90"/>
-      <c r="J3" s="90"/>
-      <c r="K3" s="90"/>
-      <c r="L3" s="91"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="B5" s="92" t="s">
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="89"/>
+      <c r="L3" s="90"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+      <c r="B5" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="94" t="s">
+      <c r="C5" s="93" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3250,7 +3254,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="96" t="s">
+      <c r="F5" s="95" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3259,7 +3263,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="96" t="s">
+      <c r="I5" s="95" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3268,36 +3272,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="96" t="s">
+      <c r="L5" s="95" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="93"/>
-      <c r="C6" s="95"/>
+    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B6" s="92"/>
+      <c r="C6" s="94"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="97"/>
+      <c r="F6" s="96"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="97"/>
+      <c r="I6" s="96"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="97"/>
-    </row>
-    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L6" s="96"/>
+    </row>
+    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3320,7 +3324,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3339,7 +3343,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3358,7 +3362,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3377,7 +3381,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3396,7 +3400,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3415,7 +3419,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3434,7 +3438,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3453,7 +3457,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3472,7 +3476,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3491,7 +3495,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3510,7 +3514,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3529,7 +3533,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3548,7 +3552,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3567,7 +3571,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3588,7 +3592,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3607,7 +3611,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3628,7 +3632,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3647,7 +3651,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3666,7 +3670,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3687,7 +3691,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3708,7 +3712,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3729,7 +3733,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3748,7 +3752,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -3767,7 +3771,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3786,7 +3790,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -3805,7 +3809,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -3824,7 +3828,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -3843,7 +3847,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -3862,7 +3866,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -3881,7 +3885,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -3900,7 +3904,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -3919,7 +3923,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -3938,7 +3942,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -3957,7 +3961,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -3976,7 +3980,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -3995,7 +3999,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -4014,7 +4018,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -4033,7 +4037,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -4052,7 +4056,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -4071,7 +4075,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -4090,7 +4094,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -4195,43 +4199,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
-    <col min="4" max="4" width="21.77734375" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.21875" customWidth="1"/>
+    <col min="3" max="3" width="17.1796875" customWidth="1"/>
+    <col min="4" max="4" width="21.81640625" customWidth="1"/>
+    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.77734375" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.81640625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.44140625" customWidth="1"/>
+    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B1" s="89" t="s">
+    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+      <c r="B1" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="91"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="B4" s="92" t="s">
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="90"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+      <c r="B4" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="94" t="s">
+      <c r="C4" s="93" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4240,7 +4244,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="96" t="s">
+      <c r="F4" s="95" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4249,7 +4253,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="96" t="s">
+      <c r="I4" s="95" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4258,36 +4262,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="96" t="s">
+      <c r="L4" s="95" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="93"/>
-      <c r="C5" s="95"/>
+    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B5" s="92"/>
+      <c r="C5" s="94"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="97"/>
+      <c r="F5" s="96"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="97"/>
+      <c r="I5" s="96"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="97"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="L5" s="96"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4305,7 +4309,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4323,7 +4327,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4341,7 +4345,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4359,7 +4363,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4377,7 +4381,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4395,7 +4399,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4413,7 +4417,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4431,7 +4435,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4449,7 +4453,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4467,7 +4471,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4485,7 +4489,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4503,7 +4507,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4521,7 +4525,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4539,7 +4543,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4558,7 +4562,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4577,7 +4581,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4596,7 +4600,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -4615,7 +4619,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -4634,7 +4638,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -4653,7 +4657,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -4672,7 +4676,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -4691,7 +4695,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -4710,7 +4714,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -4729,7 +4733,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -4748,7 +4752,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -4767,7 +4771,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -4786,7 +4790,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -4805,7 +4809,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -4826,7 +4830,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -4846,7 +4850,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -4866,7 +4870,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -4886,7 +4890,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -4906,7 +4910,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -4926,7 +4930,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -4946,7 +4950,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -4968,7 +4972,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -4988,7 +4992,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -5008,7 +5012,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -5028,7 +5032,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -5046,7 +5050,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -5064,7 +5068,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:12" ht="58" x14ac:dyDescent="0.35">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -5089,7 +5093,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -5107,7 +5111,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -5125,7 +5129,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5148,7 +5152,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5171,7 +5175,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5189,7 +5193,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5207,7 +5211,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5224,7 +5228,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5242,7 +5246,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5259,7 +5263,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5282,7 +5286,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5309,7 +5313,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5327,7 +5331,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5391,21 +5395,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
-    <col min="2" max="2" width="81.5546875" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="2" max="2" width="81.54296875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" customWidth="1"/>
-    <col min="5" max="5" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.81640625" customWidth="1"/>
+    <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:5" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5419,7 +5423,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B4" s="70" t="s">
         <v>226</v>
       </c>
@@ -5433,7 +5437,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" s="74" t="s">
         <v>240</v>
       </c>
@@ -5447,11 +5451,11 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B6" s="84" t="s">
+    <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="83" t="s">
         <v>241</v>
       </c>
-      <c r="C6" s="85" t="s">
+      <c r="C6" s="84" t="s">
         <v>232</v>
       </c>
       <c r="D6" s="75" t="s">
@@ -5461,11 +5465,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="84" t="s">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B7" s="83" t="s">
         <v>230</v>
       </c>
-      <c r="C7" s="85" t="s">
+      <c r="C7" s="84" t="s">
         <v>231</v>
       </c>
       <c r="D7" s="75" t="s">
@@ -5475,7 +5479,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B8" s="74" t="s">
         <v>233</v>
       </c>
@@ -5489,7 +5493,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B9" s="74" t="s">
         <v>179</v>
       </c>
@@ -5503,15 +5507,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="77" t="s">
+    <row r="10" spans="2:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="99" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="78" t="s">
+      <c r="C10" s="77" t="s">
         <v>235</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="80"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="79"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
@@ -5533,49 +5537,49 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:O34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.21875" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.44140625" customWidth="1"/>
-    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.21875" customWidth="1"/>
-    <col min="11" max="11" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46.2" x14ac:dyDescent="0.85">
-      <c r="B2" s="98" t="s">
+    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+      <c r="B2" s="97" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="99"/>
-      <c r="D2" s="99"/>
-      <c r="E2" s="99"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-    </row>
-    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.4">
-      <c r="B6" s="92" t="s">
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="98"/>
+      <c r="O2" s="98"/>
+    </row>
+    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+      <c r="B6" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="94" t="s">
+      <c r="C6" s="93" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="42" t="s">
@@ -5584,7 +5588,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="96" t="s">
+      <c r="F6" s="95" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5593,7 +5597,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="96" t="s">
+      <c r="I6" s="95" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="45" t="s">
@@ -5602,7 +5606,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="96" t="s">
+      <c r="L6" s="95" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="45" t="s">
@@ -5611,51 +5615,51 @@
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="96" t="s">
+      <c r="O6" s="95" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="93"/>
-      <c r="C7" s="95"/>
+    <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B7" s="92"/>
+      <c r="C7" s="94"/>
       <c r="D7" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="97"/>
+      <c r="F7" s="96"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="97"/>
+      <c r="I7" s="96"/>
       <c r="J7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="97"/>
+      <c r="L7" s="96"/>
       <c r="M7" s="44" t="s">
         <v>10</v>
       </c>
       <c r="N7" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="97"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B8" s="83" t="s">
+      <c r="O7" s="96"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B8" s="82" t="s">
         <v>68</v>
       </c>
       <c r="C8" s="29" t="s">
         <v>102</v>
       </c>
       <c r="D8" s="24"/>
-      <c r="E8" s="81">
+      <c r="E8" s="80">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
@@ -5671,8 +5675,8 @@
       <c r="N8" s="31"/>
       <c r="O8" s="11"/>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B9" s="83" t="s">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B9" s="82" t="s">
         <v>257</v>
       </c>
       <c r="C9" s="29" t="s">
@@ -5695,8 +5699,8 @@
       <c r="N9" s="31"/>
       <c r="O9" s="11"/>
     </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B10" s="83" t="s">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B10" s="82" t="s">
         <v>246</v>
       </c>
       <c r="C10" s="29" t="s">
@@ -5719,8 +5723,8 @@
       <c r="N10" s="31"/>
       <c r="O10" s="11"/>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B11" s="83" t="s">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B11" s="82" t="s">
         <v>244</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -5743,14 +5747,14 @@
       <c r="N11" s="31"/>
       <c r="O11" s="11"/>
     </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B12" s="83" t="s">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B12" s="82" t="s">
         <v>258</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D12" s="82">
+      <c r="D12" s="81">
         <v>1</v>
       </c>
       <c r="E12" s="31">
@@ -5767,14 +5771,14 @@
       <c r="N12" s="31"/>
       <c r="O12" s="11"/>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>247</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D13" s="82">
+      <c r="D13" s="81">
         <v>0.5</v>
       </c>
       <c r="E13" s="31">
@@ -5791,14 +5795,14 @@
       <c r="N13" s="31"/>
       <c r="O13" s="11"/>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>248</v>
       </c>
       <c r="C14" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D14" s="82">
+      <c r="D14" s="81">
         <v>0.15</v>
       </c>
       <c r="E14" s="31">
@@ -5815,14 +5819,14 @@
       <c r="N14" s="31"/>
       <c r="O14" s="11"/>
     </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
         <v>255</v>
       </c>
       <c r="C15" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D15" s="82">
+      <c r="D15" s="81">
         <v>0.5</v>
       </c>
       <c r="E15" s="31">
@@ -5839,14 +5843,14 @@
       <c r="N15" s="31"/>
       <c r="O15" s="11"/>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>249</v>
       </c>
       <c r="C16" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="82">
+      <c r="D16" s="81">
         <v>0.3</v>
       </c>
       <c r="E16" s="31">
@@ -5863,14 +5867,14 @@
       <c r="N16" s="31"/>
       <c r="O16" s="11"/>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>250</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="82"/>
+      <c r="D17" s="81"/>
       <c r="E17" s="31"/>
       <c r="F17" s="75"/>
       <c r="G17" s="24">
@@ -5885,14 +5889,14 @@
       <c r="N17" s="31"/>
       <c r="O17" s="11"/>
     </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>251</v>
       </c>
       <c r="C18" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D18" s="82"/>
+      <c r="D18" s="81"/>
       <c r="E18" s="31"/>
       <c r="F18" s="75"/>
       <c r="G18" s="24">
@@ -5907,14 +5911,14 @@
       <c r="N18" s="31"/>
       <c r="O18" s="11"/>
     </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>252</v>
       </c>
       <c r="C19" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D19" s="82"/>
+      <c r="D19" s="81"/>
       <c r="E19" s="31"/>
       <c r="F19" s="75"/>
       <c r="G19" s="24">
@@ -5929,14 +5933,14 @@
       <c r="N19" s="31"/>
       <c r="O19" s="11"/>
     </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>253</v>
       </c>
       <c r="C20" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D20" s="82"/>
+      <c r="D20" s="81"/>
       <c r="E20" s="31"/>
       <c r="F20" s="75"/>
       <c r="G20" s="24">
@@ -5951,14 +5955,14 @@
       <c r="N20" s="31"/>
       <c r="O20" s="11"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>254</v>
       </c>
       <c r="C21" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D21" s="82"/>
+      <c r="D21" s="81"/>
       <c r="E21" s="31"/>
       <c r="F21" s="75"/>
       <c r="G21" s="24">
@@ -5973,14 +5977,14 @@
       <c r="N21" s="31"/>
       <c r="O21" s="11"/>
     </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B22" s="83" t="s">
+    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B22" s="82" t="s">
         <v>256</v>
       </c>
       <c r="C22" s="29" t="s">
         <v>102</v>
       </c>
-      <c r="D22" s="82"/>
+      <c r="D22" s="81"/>
       <c r="E22" s="31"/>
       <c r="F22" s="75"/>
       <c r="G22" s="24">
@@ -5995,9 +5999,9 @@
       <c r="N22" s="31"/>
       <c r="O22" s="11"/>
     </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B23" s="87" t="s">
-        <v>261</v>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B23" s="86" t="s">
+        <v>260</v>
       </c>
       <c r="C23" s="29" t="s">
         <v>102</v>
@@ -6017,9 +6021,9 @@
       <c r="N23" s="31"/>
       <c r="O23" s="11"/>
     </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B24" s="87" t="s">
-        <v>262</v>
+    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B24" s="86" t="s">
+        <v>261</v>
       </c>
       <c r="C24" s="29" t="s">
         <v>102</v>
@@ -6037,9 +6041,9 @@
       <c r="N24" s="31"/>
       <c r="O24" s="11"/>
     </row>
-    <row r="25" spans="2:15" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="88" t="s">
-        <v>259</v>
+    <row r="25" spans="2:15" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="87" t="s">
+        <v>262</v>
       </c>
       <c r="C25" s="29" t="s">
         <v>102</v>
@@ -6057,9 +6061,9 @@
       <c r="N25" s="31"/>
       <c r="O25" s="11"/>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B26" s="86" t="s">
-        <v>260</v>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B26" s="85" t="s">
+        <v>259</v>
       </c>
       <c r="C26" s="29" t="s">
         <v>102</v>
@@ -6077,7 +6081,7 @@
       <c r="N26" s="31"/>
       <c r="O26" s="11"/>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
         <v>245</v>
       </c>
@@ -6097,7 +6101,7 @@
       <c r="N27" s="31"/>
       <c r="O27" s="11"/>
     </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
         <v>215</v>
       </c>
@@ -6117,7 +6121,7 @@
       <c r="N28" s="31"/>
       <c r="O28" s="11"/>
     </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
         <v>216</v>
       </c>
@@ -6137,7 +6141,7 @@
       <c r="N29" s="31"/>
       <c r="O29" s="11"/>
     </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
         <v>221</v>
       </c>
@@ -6157,7 +6161,7 @@
       <c r="N30" s="31"/>
       <c r="O30" s="11"/>
     </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>217</v>
       </c>
@@ -6177,7 +6181,7 @@
       <c r="N31" s="31"/>
       <c r="O31" s="11"/>
     </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>218</v>
       </c>
@@ -6197,7 +6201,7 @@
       <c r="N32" s="31"/>
       <c r="O32" s="11"/>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
         <v>222</v>
       </c>
@@ -6217,7 +6221,7 @@
       <c r="N33" s="31"/>
       <c r="O33" s="11"/>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
         <v>239</v>
       </c>
@@ -6387,28 +6391,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.21875" customWidth="1"/>
-    <col min="2" max="2" width="93.21875" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="2" max="2" width="93.1796875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" customWidth="1"/>
+    <col min="5" max="5" width="15.81640625" customWidth="1"/>
+    <col min="6" max="6" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:6" ht="47" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -6425,7 +6429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -6438,7 +6442,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -6451,7 +6455,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -6464,7 +6468,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -6477,7 +6481,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -6490,7 +6494,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -6503,7 +6507,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -6516,7 +6520,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -6529,7 +6533,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -6542,7 +6546,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -6555,7 +6559,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -6568,7 +6572,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -6581,7 +6585,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -6594,7 +6598,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -6607,7 +6611,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -6620,7 +6624,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -6633,7 +6637,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -6646,7 +6650,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -6659,7 +6663,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -6672,7 +6676,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -6685,7 +6689,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -6698,7 +6702,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -6711,7 +6715,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -6724,7 +6728,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -6737,7 +6741,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -6750,7 +6754,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -6763,7 +6767,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -6776,7 +6780,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -6789,7 +6793,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -6802,7 +6806,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -6815,7 +6819,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -6828,7 +6832,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -6841,7 +6845,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -6854,7 +6858,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -6867,7 +6871,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -6880,7 +6884,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -6893,7 +6897,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -6906,7 +6910,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -6919,7 +6923,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -6932,7 +6936,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -6945,7 +6949,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -6958,7 +6962,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -6971,7 +6975,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -6984,7 +6988,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -6997,7 +7001,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -7010,7 +7014,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -7023,7 +7027,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -7036,7 +7040,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -7049,7 +7053,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -7062,7 +7066,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -7075,7 +7079,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -7088,7 +7092,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -7101,7 +7105,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -7114,7 +7118,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -7127,7 +7131,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -7140,7 +7144,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -7153,7 +7157,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -7166,7 +7170,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -7179,7 +7183,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -7192,7 +7196,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -7203,7 +7207,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -7214,7 +7218,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -7225,7 +7229,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -7236,7 +7240,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -7247,7 +7251,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -7258,7 +7262,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -7269,7 +7273,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -7280,7 +7284,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -7291,7 +7295,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B74" s="3" t="s">
         <v>106</v>
       </c>
@@ -7302,7 +7306,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B75" s="3" t="s">
         <v>107</v>
       </c>
@@ -7313,182 +7317,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
fonctions save + load
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2772CD-BF3B-4E75-A011-CFE5F5B3BFE9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8890C9ED-D0A2-4F54-8E98-2982EB5C6F57}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="277">
   <si>
     <t>Planification globale</t>
   </si>
@@ -837,6 +837,39 @@
   </si>
   <si>
     <t>Ajouter un timer sur écran end de surrender pour permettre de recréer une partie</t>
+  </si>
+  <si>
+    <t>Debugger combats</t>
+  </si>
+  <si>
+    <t>Fonction de sauvegarde</t>
+  </si>
+  <si>
+    <t>Fonction de load</t>
+  </si>
+  <si>
+    <t>Problèmes sur le plateau de jeu du perdant quand la pièce de l'attaquant gagne. Ajout d'une fonction qui passe le plateau de jeu et retire tous les doublons de piece.id</t>
+  </si>
+  <si>
+    <t>Terminé l'implémentation de priors</t>
+  </si>
+  <si>
+    <t>Terminé les différents setups</t>
+  </si>
+  <si>
+    <t>Plus long que prévu, création de nouvelles classes dans AIPlayer pour setup et les stratégies</t>
+  </si>
+  <si>
+    <t>Fonctions de bases implémentés. AI facile terminé</t>
+  </si>
+  <si>
+    <t>Fonctions optimizées pour permettre plus d'itérations du MCTS à l'AI</t>
+  </si>
+  <si>
+    <t>Plus long que prévu. Erreurs dans la fonction save qui n'avaient pas été repérés tant que le load n'était pas implémenté. Fonctionne en théorie, mais voir avec frontend si tout est beau</t>
+  </si>
+  <si>
+    <t>Optimizer l'algorithme</t>
   </si>
 </sst>
 </file>
@@ -1415,7 +1448,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1555,6 +1588,9 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="35" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1588,14 +1624,157 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
+  <dxfs count="69">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2716,7 +2895,7 @@
       <c r="D34" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E34" s="100">
+      <c r="E34" s="89">
         <v>4</v>
       </c>
     </row>
@@ -2744,7 +2923,7 @@
       <c r="D36" s="29" t="s">
         <v>140</v>
       </c>
-      <c r="E36" s="100">
+      <c r="E36" s="89">
         <v>3</v>
       </c>
     </row>
@@ -2775,7 +2954,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="49" priority="1">
+    <cfRule type="expression" dxfId="68" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3219,26 +3398,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="87" t="s">
+      <c r="B3" s="90" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
-      <c r="J3" s="88"/>
-      <c r="K3" s="88"/>
-      <c r="L3" s="89"/>
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="91"/>
+      <c r="I3" s="91"/>
+      <c r="J3" s="91"/>
+      <c r="K3" s="91"/>
+      <c r="L3" s="92"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="92" t="s">
+      <c r="C5" s="95" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3247,7 +3426,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="94" t="s">
+      <c r="F5" s="97" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3256,7 +3435,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="94" t="s">
+      <c r="I5" s="97" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3265,34 +3444,34 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="94" t="s">
+      <c r="L5" s="97" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="91"/>
-      <c r="C6" s="93"/>
+      <c r="B6" s="94"/>
+      <c r="C6" s="96"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="95"/>
+      <c r="F6" s="98"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="95"/>
+      <c r="I6" s="98"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="95"/>
+      <c r="L6" s="98"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="28" t="s">
@@ -4117,67 +4296,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="48" priority="7">
+    <cfRule type="expression" dxfId="67" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="47" priority="1">
+    <cfRule type="expression" dxfId="66" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="46" priority="32">
+    <cfRule type="expression" dxfId="65" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="38">
+    <cfRule type="expression" dxfId="64" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="44" priority="30">
+    <cfRule type="expression" dxfId="63" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="43" priority="6">
+    <cfRule type="expression" dxfId="62" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="42" priority="25">
+    <cfRule type="expression" dxfId="61" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="27">
+    <cfRule type="expression" dxfId="60" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="40" priority="8">
+    <cfRule type="expression" dxfId="59" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="39" priority="13">
+    <cfRule type="expression" dxfId="58" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="14">
+    <cfRule type="expression" dxfId="57" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="37" priority="20">
+    <cfRule type="expression" dxfId="56" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="21">
+    <cfRule type="expression" dxfId="55" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="35" priority="9">
+    <cfRule type="expression" dxfId="54" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="10">
+    <cfRule type="expression" dxfId="53" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4209,26 +4388,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="87" t="s">
+      <c r="B1" s="90" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="92"/>
     </row>
     <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="90" t="s">
+      <c r="B4" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="92" t="s">
+      <c r="C4" s="95" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4237,7 +4416,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="94" t="s">
+      <c r="F4" s="97" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4246,7 +4425,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="94" t="s">
+      <c r="I4" s="97" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4255,34 +4434,34 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="94" t="s">
+      <c r="L4" s="97" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="91"/>
-      <c r="C5" s="93"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="96"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="95"/>
+      <c r="F5" s="98"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="95"/>
+      <c r="I5" s="98"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="95"/>
+      <c r="L5" s="98"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="29" t="s">
@@ -5357,23 +5536,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="33" priority="49">
+    <cfRule type="expression" dxfId="52" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="32" priority="89">
+    <cfRule type="expression" dxfId="51" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="31" priority="46">
+    <cfRule type="expression" dxfId="50" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="47">
+    <cfRule type="expression" dxfId="49" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="29" priority="48">
+    <cfRule type="expression" dxfId="48" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5417,7 +5596,7 @@
       </c>
     </row>
     <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="B4" s="98" t="s">
+      <c r="B4" s="87" t="s">
         <v>226</v>
       </c>
       <c r="C4" s="70" t="s">
@@ -5445,7 +5624,7 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B6" s="99" t="s">
+      <c r="B6" s="88" t="s">
         <v>241</v>
       </c>
       <c r="C6" s="62" t="s">
@@ -5459,7 +5638,7 @@
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B7" s="99" t="s">
+      <c r="B7" s="88" t="s">
         <v>230</v>
       </c>
       <c r="C7" s="62" t="s">
@@ -5487,7 +5666,7 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B9" s="99" t="s">
+      <c r="B9" s="88" t="s">
         <v>179</v>
       </c>
       <c r="C9" s="62" t="s">
@@ -5512,10 +5691,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="28" priority="157">
+    <cfRule type="expression" dxfId="47" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="158">
+    <cfRule type="expression" dxfId="46" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5529,59 +5708,59 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:O37"/>
+  <dimension ref="B2:O41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
     <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" style="31" customWidth="1"/>
+    <col min="5" max="5" width="20.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.453125" style="31" customWidth="1"/>
+    <col min="8" max="8" width="20.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.54296875" style="31" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" style="31" customWidth="1"/>
+    <col min="11" max="11" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.08984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.81640625" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="96" t="s">
+      <c r="B2" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="97"/>
-      <c r="D2" s="97"/>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="97"/>
-      <c r="L2" s="97"/>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
+      <c r="C2" s="100"/>
+      <c r="D2" s="100"/>
+      <c r="E2" s="100"/>
+      <c r="F2" s="100"/>
+      <c r="G2" s="100"/>
+      <c r="H2" s="100"/>
+      <c r="I2" s="100"/>
+      <c r="J2" s="100"/>
+      <c r="K2" s="100"/>
+      <c r="L2" s="100"/>
+      <c r="M2" s="100"/>
+      <c r="N2" s="100"/>
+      <c r="O2" s="100"/>
     </row>
     <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
-      <c r="B6" s="90" t="s">
+      <c r="B6" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="92" t="s">
+      <c r="C6" s="95" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="42" t="s">
+      <c r="D6" s="102" t="s">
         <v>13</v>
       </c>
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="94" t="s">
+      <c r="F6" s="97" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5590,59 +5769,59 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="94" t="s">
+      <c r="I6" s="97" t="s">
         <v>12</v>
       </c>
-      <c r="J6" s="45" t="s">
+      <c r="J6" s="60" t="s">
         <v>15</v>
       </c>
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="94" t="s">
+      <c r="L6" s="97" t="s">
         <v>12</v>
       </c>
-      <c r="M6" s="45" t="s">
+      <c r="M6" s="60" t="s">
         <v>19</v>
       </c>
       <c r="N6" s="43">
         <v>46160</v>
       </c>
-      <c r="O6" s="94" t="s">
+      <c r="O6" s="97" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="91"/>
-      <c r="C7" s="93"/>
-      <c r="D7" s="42" t="s">
+      <c r="B7" s="94"/>
+      <c r="C7" s="96"/>
+      <c r="D7" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="44" t="s">
+      <c r="E7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="95"/>
+      <c r="F7" s="98"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="95"/>
-      <c r="J7" s="44" t="s">
+      <c r="I7" s="98"/>
+      <c r="J7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="44" t="s">
+      <c r="K7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="95"/>
-      <c r="M7" s="44" t="s">
+      <c r="L7" s="98"/>
+      <c r="M7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="N7" s="44" t="s">
+      <c r="N7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="95"/>
+      <c r="O7" s="98"/>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="81" t="s">
@@ -5655,18 +5834,15 @@
       <c r="E8" s="79">
         <v>0</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="103" t="s">
         <v>229</v>
       </c>
       <c r="G8" s="24"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="11"/>
+      <c r="I8" s="103"/>
       <c r="J8" s="24"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="11"/>
+      <c r="L8" s="103"/>
       <c r="M8" s="24"/>
-      <c r="N8" s="31"/>
-      <c r="O8" s="11"/>
+      <c r="O8" s="103"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="81" t="s">
@@ -5681,16 +5857,13 @@
       <c r="E9" s="31">
         <v>100</v>
       </c>
-      <c r="F9" s="11"/>
+      <c r="F9" s="103"/>
       <c r="G9" s="24"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="11"/>
+      <c r="I9" s="103"/>
       <c r="J9" s="24"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="11"/>
+      <c r="L9" s="103"/>
       <c r="M9" s="24"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="11"/>
+      <c r="O9" s="103"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="81" t="s">
@@ -5705,16 +5878,13 @@
       <c r="E10" s="31">
         <v>100</v>
       </c>
-      <c r="F10" s="11"/>
+      <c r="F10" s="103"/>
       <c r="G10" s="24"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="11"/>
+      <c r="I10" s="103"/>
       <c r="J10" s="24"/>
-      <c r="K10" s="31"/>
-      <c r="L10" s="11"/>
+      <c r="L10" s="103"/>
       <c r="M10" s="24"/>
-      <c r="N10" s="31"/>
-      <c r="O10" s="11"/>
+      <c r="O10" s="103"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="81" t="s">
@@ -5729,16 +5899,13 @@
       <c r="E11" s="31">
         <v>100</v>
       </c>
-      <c r="F11" s="11"/>
+      <c r="F11" s="103"/>
       <c r="G11" s="24"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="11"/>
+      <c r="I11" s="103"/>
       <c r="J11" s="24"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="11"/>
+      <c r="L11" s="103"/>
       <c r="M11" s="24"/>
-      <c r="N11" s="31"/>
-      <c r="O11" s="11"/>
+      <c r="O11" s="103"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B12" s="81" t="s">
@@ -5753,16 +5920,13 @@
       <c r="E12" s="31">
         <v>100</v>
       </c>
-      <c r="F12" s="74"/>
+      <c r="F12" s="80"/>
       <c r="G12" s="24"/>
-      <c r="H12" s="31"/>
-      <c r="I12" s="11"/>
+      <c r="I12" s="103"/>
       <c r="J12" s="24"/>
-      <c r="K12" s="31"/>
-      <c r="L12" s="11"/>
+      <c r="L12" s="103"/>
       <c r="M12" s="24"/>
-      <c r="N12" s="31"/>
-      <c r="O12" s="11"/>
+      <c r="O12" s="103"/>
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
@@ -5777,16 +5941,13 @@
       <c r="E13" s="31">
         <v>100</v>
       </c>
-      <c r="F13" s="74"/>
+      <c r="F13" s="80"/>
       <c r="G13" s="24"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="11"/>
+      <c r="I13" s="103"/>
       <c r="J13" s="24"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="11"/>
+      <c r="L13" s="103"/>
       <c r="M13" s="24"/>
-      <c r="N13" s="31"/>
-      <c r="O13" s="11"/>
+      <c r="O13" s="103"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
@@ -5801,16 +5962,13 @@
       <c r="E14" s="31">
         <v>100</v>
       </c>
-      <c r="F14" s="74"/>
+      <c r="F14" s="80"/>
       <c r="G14" s="24"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="11"/>
+      <c r="I14" s="103"/>
       <c r="J14" s="24"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="11"/>
+      <c r="L14" s="103"/>
       <c r="M14" s="24"/>
-      <c r="N14" s="31"/>
-      <c r="O14" s="11"/>
+      <c r="O14" s="103"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
@@ -5825,16 +5983,13 @@
       <c r="E15" s="31">
         <v>100</v>
       </c>
-      <c r="F15" s="74"/>
+      <c r="F15" s="80"/>
       <c r="G15" s="24"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="11"/>
+      <c r="I15" s="103"/>
       <c r="J15" s="24"/>
-      <c r="K15" s="31"/>
-      <c r="L15" s="11"/>
+      <c r="L15" s="103"/>
       <c r="M15" s="24"/>
-      <c r="N15" s="31"/>
-      <c r="O15" s="11"/>
+      <c r="O15" s="103"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
@@ -5849,16 +6004,13 @@
       <c r="E16" s="31">
         <v>100</v>
       </c>
-      <c r="F16" s="74"/>
+      <c r="F16" s="80"/>
       <c r="G16" s="24"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="11"/>
+      <c r="I16" s="103"/>
       <c r="J16" s="24"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="11"/>
+      <c r="L16" s="103"/>
       <c r="M16" s="24"/>
-      <c r="N16" s="31"/>
-      <c r="O16" s="11"/>
+      <c r="O16" s="103"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
@@ -5868,19 +6020,15 @@
         <v>102</v>
       </c>
       <c r="D17" s="80"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="74"/>
+      <c r="F17" s="80"/>
       <c r="G17" s="24">
         <v>3</v>
       </c>
-      <c r="H17" s="31"/>
-      <c r="I17" s="11"/>
+      <c r="I17" s="103"/>
       <c r="J17" s="24"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="11"/>
+      <c r="L17" s="103"/>
       <c r="M17" s="24"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="11"/>
+      <c r="O17" s="103"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
@@ -5890,19 +6038,15 @@
         <v>102</v>
       </c>
       <c r="D18" s="80"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="74"/>
+      <c r="F18" s="80"/>
       <c r="G18" s="24">
         <v>0.75</v>
       </c>
-      <c r="H18" s="31"/>
-      <c r="I18" s="11"/>
+      <c r="I18" s="103"/>
       <c r="J18" s="24"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="11"/>
+      <c r="L18" s="103"/>
       <c r="M18" s="24"/>
-      <c r="N18" s="31"/>
-      <c r="O18" s="11"/>
+      <c r="O18" s="103"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
@@ -5912,19 +6056,15 @@
         <v>102</v>
       </c>
       <c r="D19" s="80"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="74"/>
+      <c r="F19" s="80"/>
       <c r="G19" s="24">
         <v>1.25</v>
       </c>
-      <c r="H19" s="31"/>
-      <c r="I19" s="11"/>
+      <c r="I19" s="103"/>
       <c r="J19" s="24"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="11"/>
+      <c r="L19" s="103"/>
       <c r="M19" s="24"/>
-      <c r="N19" s="31"/>
-      <c r="O19" s="11"/>
+      <c r="O19" s="103"/>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
@@ -5934,19 +6074,15 @@
         <v>102</v>
       </c>
       <c r="D20" s="80"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="74"/>
+      <c r="F20" s="80"/>
       <c r="G20" s="24">
         <v>0.15</v>
       </c>
-      <c r="H20" s="31"/>
-      <c r="I20" s="11"/>
+      <c r="I20" s="103"/>
       <c r="J20" s="24"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="11"/>
+      <c r="L20" s="103"/>
       <c r="M20" s="24"/>
-      <c r="N20" s="31"/>
-      <c r="O20" s="11"/>
+      <c r="O20" s="103"/>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
@@ -5956,19 +6092,15 @@
         <v>102</v>
       </c>
       <c r="D21" s="80"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="74"/>
+      <c r="F21" s="80"/>
       <c r="G21" s="24">
         <v>0.5</v>
       </c>
-      <c r="H21" s="31"/>
-      <c r="I21" s="11"/>
+      <c r="I21" s="103"/>
       <c r="J21" s="24"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="11"/>
+      <c r="L21" s="103"/>
       <c r="M21" s="24"/>
-      <c r="N21" s="31"/>
-      <c r="O21" s="11"/>
+      <c r="O21" s="103"/>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B22" s="81" t="s">
@@ -5978,19 +6110,15 @@
         <v>102</v>
       </c>
       <c r="D22" s="80"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="74"/>
+      <c r="F22" s="80"/>
       <c r="G22" s="24">
         <v>0.15</v>
       </c>
-      <c r="H22" s="31"/>
-      <c r="I22" s="11"/>
+      <c r="I22" s="103"/>
       <c r="J22" s="24"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="11"/>
+      <c r="L22" s="103"/>
       <c r="M22" s="24"/>
-      <c r="N22" s="31"/>
-      <c r="O22" s="11"/>
+      <c r="O22" s="103"/>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B23" s="82" t="s">
@@ -6000,19 +6128,15 @@
         <v>102</v>
       </c>
       <c r="D23" s="24"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="11"/>
+      <c r="F23" s="103"/>
       <c r="G23" s="24">
         <v>0.15</v>
       </c>
-      <c r="H23" s="31"/>
-      <c r="I23" s="11"/>
+      <c r="I23" s="103"/>
       <c r="J23" s="24"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="11"/>
+      <c r="L23" s="103"/>
       <c r="M23" s="24"/>
-      <c r="N23" s="31"/>
-      <c r="O23" s="11"/>
+      <c r="O23" s="103"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B24" s="82" t="s">
@@ -6022,17 +6146,13 @@
         <v>102</v>
       </c>
       <c r="D24" s="24"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="11"/>
+      <c r="F24" s="103"/>
       <c r="G24" s="24"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="11"/>
+      <c r="I24" s="103"/>
       <c r="J24" s="24"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="11"/>
+      <c r="L24" s="103"/>
       <c r="M24" s="24"/>
-      <c r="N24" s="31"/>
-      <c r="O24" s="11"/>
+      <c r="O24" s="103"/>
     </row>
     <row r="25" spans="2:15" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="83" t="s">
@@ -6042,19 +6162,15 @@
         <v>102</v>
       </c>
       <c r="D25" s="24"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="11"/>
+      <c r="F25" s="103"/>
       <c r="G25" s="24"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="11"/>
+      <c r="I25" s="103"/>
       <c r="J25" s="24">
         <v>3</v>
       </c>
-      <c r="K25" s="31"/>
-      <c r="L25" s="11"/>
+      <c r="L25" s="103"/>
       <c r="M25" s="24"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="11"/>
+      <c r="O25" s="103"/>
     </row>
     <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B26" s="83" t="s">
@@ -6064,19 +6180,15 @@
         <v>102</v>
       </c>
       <c r="D26" s="24"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="11"/>
+      <c r="F26" s="103"/>
       <c r="G26" s="24"/>
-      <c r="H26" s="31"/>
-      <c r="I26" s="11"/>
+      <c r="I26" s="103"/>
       <c r="J26" s="24">
         <v>1</v>
       </c>
-      <c r="K26" s="31"/>
-      <c r="L26" s="11"/>
+      <c r="L26" s="103"/>
       <c r="M26" s="24"/>
-      <c r="N26" s="31"/>
-      <c r="O26" s="11"/>
+      <c r="O26" s="103"/>
     </row>
     <row r="27" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B27" s="83" t="s">
@@ -6086,19 +6198,15 @@
         <v>102</v>
       </c>
       <c r="D27" s="24"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="11"/>
+      <c r="F27" s="103"/>
       <c r="G27" s="24"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="11"/>
+      <c r="I27" s="103"/>
       <c r="J27" s="24">
         <v>1</v>
       </c>
-      <c r="K27" s="31"/>
-      <c r="L27" s="11"/>
+      <c r="L27" s="103"/>
       <c r="M27" s="24"/>
-      <c r="N27" s="31"/>
-      <c r="O27" s="11"/>
+      <c r="O27" s="103"/>
     </row>
     <row r="28" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B28" s="83" t="s">
@@ -6108,19 +6216,15 @@
         <v>102</v>
       </c>
       <c r="D28" s="24"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="11"/>
+      <c r="F28" s="103"/>
       <c r="G28" s="24"/>
-      <c r="H28" s="31"/>
-      <c r="I28" s="11"/>
+      <c r="I28" s="103"/>
       <c r="J28" s="24">
         <v>0.75</v>
       </c>
-      <c r="K28" s="31"/>
-      <c r="L28" s="11"/>
+      <c r="L28" s="103"/>
       <c r="M28" s="24"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="11"/>
+      <c r="O28" s="103"/>
     </row>
     <row r="29" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B29" s="83" t="s">
@@ -6130,19 +6234,15 @@
         <v>102</v>
       </c>
       <c r="D29" s="24"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="11"/>
+      <c r="F29" s="103"/>
       <c r="G29" s="24"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="11"/>
+      <c r="I29" s="103"/>
       <c r="J29" s="24">
         <v>1</v>
       </c>
-      <c r="K29" s="31"/>
-      <c r="L29" s="11"/>
+      <c r="L29" s="103"/>
       <c r="M29" s="24"/>
-      <c r="N29" s="31"/>
-      <c r="O29" s="11"/>
+      <c r="O29" s="103"/>
     </row>
     <row r="30" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B30" s="83" t="s">
@@ -6152,159 +6252,267 @@
         <v>102</v>
       </c>
       <c r="D30" s="24"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="11"/>
+      <c r="F30" s="103"/>
       <c r="G30" s="24"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="11"/>
+      <c r="I30" s="103"/>
       <c r="J30" s="24">
         <v>0.5</v>
       </c>
-      <c r="K30" s="31"/>
-      <c r="L30" s="11"/>
+      <c r="L30" s="103"/>
       <c r="M30" s="24"/>
-      <c r="N30" s="31"/>
-      <c r="O30" s="11"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="O30" s="103"/>
+    </row>
+    <row r="31" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>215</v>
       </c>
       <c r="C31" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="24"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="11"/>
+      <c r="D31" s="24">
+        <v>2</v>
+      </c>
+      <c r="E31" s="31">
+        <v>50</v>
+      </c>
+      <c r="F31" s="105" t="s">
+        <v>272</v>
+      </c>
+      <c r="G31" s="24">
+        <v>2</v>
+      </c>
+      <c r="H31" s="31">
+        <v>100</v>
+      </c>
+      <c r="I31" s="103"/>
       <c r="J31" s="24"/>
-      <c r="K31" s="31"/>
-      <c r="L31" s="11"/>
+      <c r="L31" s="103"/>
       <c r="M31" s="24"/>
-      <c r="N31" s="31"/>
-      <c r="O31" s="11"/>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="O31" s="103"/>
+    </row>
+    <row r="32" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>216</v>
       </c>
       <c r="C32" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D32" s="24"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="11"/>
+      <c r="D32" s="24">
+        <v>1</v>
+      </c>
+      <c r="E32" s="31">
+        <v>25</v>
+      </c>
+      <c r="F32" s="105" t="s">
+        <v>273</v>
+      </c>
       <c r="G32" s="24"/>
-      <c r="H32" s="31"/>
-      <c r="I32" s="11"/>
+      <c r="I32" s="103"/>
       <c r="J32" s="24"/>
-      <c r="K32" s="31"/>
-      <c r="L32" s="11"/>
+      <c r="L32" s="103"/>
       <c r="M32" s="24"/>
-      <c r="N32" s="31"/>
-      <c r="O32" s="11"/>
+      <c r="O32" s="103"/>
     </row>
     <row r="33" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C33" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D33" s="24"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="11"/>
+      <c r="D33" s="24">
+        <v>5</v>
+      </c>
+      <c r="E33" s="31">
+        <v>100</v>
+      </c>
+      <c r="F33" s="103"/>
       <c r="G33" s="24"/>
-      <c r="H33" s="31"/>
-      <c r="I33" s="11"/>
+      <c r="I33" s="103"/>
       <c r="J33" s="24"/>
-      <c r="K33" s="31"/>
-      <c r="L33" s="11"/>
+      <c r="L33" s="103"/>
       <c r="M33" s="24"/>
-      <c r="N33" s="31"/>
-      <c r="O33" s="11"/>
+      <c r="O33" s="103"/>
     </row>
     <row r="34" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C34" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D34" s="24"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="11"/>
+      <c r="D34" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="E34" s="31">
+        <v>100</v>
+      </c>
+      <c r="F34" s="103"/>
       <c r="G34" s="24"/>
-      <c r="H34" s="31"/>
-      <c r="I34" s="11"/>
+      <c r="I34" s="103"/>
       <c r="J34" s="24"/>
-      <c r="K34" s="31"/>
-      <c r="L34" s="11"/>
+      <c r="L34" s="103"/>
       <c r="M34" s="24"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="11"/>
+      <c r="O34" s="103"/>
     </row>
     <row r="35" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C35" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D35" s="24"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="24"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="11"/>
+      <c r="D35" s="24">
+        <v>1</v>
+      </c>
+      <c r="E35" s="31">
+        <v>25</v>
+      </c>
+      <c r="F35" s="103" t="s">
+        <v>271</v>
+      </c>
+      <c r="G35" s="24">
+        <v>2</v>
+      </c>
+      <c r="H35" s="31">
+        <v>75</v>
+      </c>
+      <c r="I35" s="105" t="s">
+        <v>270</v>
+      </c>
       <c r="J35" s="24"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="11"/>
+      <c r="L35" s="103"/>
       <c r="M35" s="24"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="11"/>
+      <c r="O35" s="103"/>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C36" s="29" t="s">
         <v>103</v>
       </c>
       <c r="D36" s="24"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="24"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="11"/>
+      <c r="F36" s="103"/>
+      <c r="G36" s="24">
+        <v>3</v>
+      </c>
+      <c r="H36" s="31">
+        <v>100</v>
+      </c>
+      <c r="I36" s="103"/>
       <c r="J36" s="24"/>
-      <c r="K36" s="31"/>
-      <c r="L36" s="11"/>
+      <c r="L36" s="103"/>
       <c r="M36" s="24"/>
-      <c r="N36" s="31"/>
-      <c r="O36" s="11"/>
-    </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B37" s="29" t="s">
+      <c r="O36" s="103"/>
+    </row>
+    <row r="37" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B37" s="101" t="s">
+        <v>266</v>
+      </c>
+      <c r="C37" s="101" t="s">
+        <v>103</v>
+      </c>
+      <c r="G37" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="31">
+        <v>100</v>
+      </c>
+      <c r="I37" s="104" t="s">
+        <v>269</v>
+      </c>
+      <c r="J37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="O37" s="103"/>
+    </row>
+    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B38" s="101" t="s">
+        <v>267</v>
+      </c>
+      <c r="C38" s="101" t="s">
+        <v>103</v>
+      </c>
+      <c r="G38" s="24"/>
+      <c r="J38" s="24">
+        <v>2</v>
+      </c>
+      <c r="K38" s="31">
+        <v>100</v>
+      </c>
+      <c r="M38" s="24"/>
+      <c r="O38" s="103"/>
+    </row>
+    <row r="39" spans="2:15" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="B39" s="101" t="s">
+        <v>268</v>
+      </c>
+      <c r="C39" s="101" t="s">
+        <v>103</v>
+      </c>
+      <c r="G39" s="24"/>
+      <c r="J39" s="24">
+        <v>4</v>
+      </c>
+      <c r="K39" s="31">
+        <v>90</v>
+      </c>
+      <c r="L39" s="104" t="s">
+        <v>275</v>
+      </c>
+      <c r="M39" s="24"/>
+      <c r="O39" s="103"/>
+    </row>
+    <row r="40" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+      <c r="B40" s="29" t="s">
         <v>239</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="C40" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="D37" s="24"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="24"/>
-      <c r="H37" s="31"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="24"/>
-      <c r="K37" s="31"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="24"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="11"/>
+      <c r="D40" s="24"/>
+      <c r="F40" s="103"/>
+      <c r="G40" s="24"/>
+      <c r="I40" s="103"/>
+      <c r="J40" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="K40" s="31">
+        <v>100</v>
+      </c>
+      <c r="L40" s="105" t="s">
+        <v>274</v>
+      </c>
+      <c r="M40" s="24"/>
+      <c r="O40" s="103"/>
+    </row>
+    <row r="41" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B41" s="101" t="s">
+        <v>276</v>
+      </c>
+      <c r="C41" s="101" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" s="31">
+        <v>1</v>
+      </c>
+      <c r="E41" s="31">
+        <v>10</v>
+      </c>
+      <c r="G41" s="24">
+        <v>2</v>
+      </c>
+      <c r="H41" s="31">
+        <v>30</v>
+      </c>
+      <c r="J41" s="24">
+        <v>2</v>
+      </c>
+      <c r="K41" s="31">
+        <v>50</v>
+      </c>
+      <c r="M41" s="24"/>
+      <c r="O41" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -6316,123 +6524,208 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B6:B7 B23:B37">
-    <cfRule type="expression" dxfId="26" priority="27">
+  <conditionalFormatting sqref="B2 B6:B7 B23:B41">
+    <cfRule type="expression" dxfId="45" priority="27">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C37">
-    <cfRule type="expression" dxfId="25" priority="16">
+  <conditionalFormatting sqref="C6:C41">
+    <cfRule type="expression" dxfId="44" priority="16">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="17">
+    <cfRule type="expression" dxfId="43" priority="17">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="23" priority="18">
+    <cfRule type="expression" dxfId="42" priority="18">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="22" priority="230">
+    <cfRule type="expression" dxfId="41" priority="230">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14">
-    <cfRule type="expression" dxfId="21" priority="232">
+    <cfRule type="expression" dxfId="40" priority="232">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B9:B19">
-    <cfRule type="expression" dxfId="20" priority="248">
+  <conditionalFormatting sqref="B9:B10">
+    <cfRule type="expression" dxfId="39" priority="248">
       <formula>MAX($E31,$H31,$K31)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="19" priority="269">
+    <cfRule type="expression" dxfId="38" priority="269">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:B12">
-    <cfRule type="expression" dxfId="18" priority="3">
+  <conditionalFormatting sqref="B8:B12 B25:B26">
+    <cfRule type="expression" dxfId="37" priority="3">
       <formula>MAX($E17,$H17,$K17)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B30">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="36" priority="1">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15:B19">
-    <cfRule type="expression" dxfId="16" priority="318">
+  <conditionalFormatting sqref="B15:B16">
+    <cfRule type="expression" dxfId="35" priority="318">
       <formula>MAX($E31,$H31,$K31)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="15" priority="349">
+    <cfRule type="expression" dxfId="34" priority="349">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="14" priority="350">
+    <cfRule type="expression" dxfId="33" priority="350">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B25:B30">
-    <cfRule type="expression" dxfId="13" priority="353">
+  <conditionalFormatting sqref="B28:B30">
+    <cfRule type="expression" dxfId="32" priority="353">
+      <formula>MAX($E37,$H37,$K37)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12:B14 B16:B18">
+    <cfRule type="expression" dxfId="31" priority="355">
+      <formula>MAX($E33,$H33,$K33)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:B19">
+    <cfRule type="expression" dxfId="30" priority="356">
+      <formula>MAX($E33,$H33,$K33)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20:B21 B23:B24">
+    <cfRule type="expression" dxfId="29" priority="388">
+      <formula>MAX($E34,$H34,$K34)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B8">
+    <cfRule type="expression" dxfId="28" priority="437">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="438">
+      <formula>MAX($E4,$H4,$K4)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B11">
+    <cfRule type="expression" dxfId="26" priority="481">
+      <formula>MAX($E31,$H31,$K31)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="25" priority="482">
+      <formula>MAX($E6,$H6,$K6)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
+    <cfRule type="expression" dxfId="24" priority="497">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20">
+    <cfRule type="expression" dxfId="23" priority="502">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30">
+    <cfRule type="expression" dxfId="22" priority="510">
+      <formula>MAX($E14,$H14,$K14)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="511">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21">
+    <cfRule type="expression" dxfId="20" priority="520">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="521">
+      <formula>MAX($E16,$H16,$K16)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="expression" dxfId="18" priority="531">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17">
+    <cfRule type="expression" dxfId="17" priority="533">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12 B16">
+    <cfRule type="expression" dxfId="16" priority="538">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="539">
+      <formula>MAX($E8,$H8,$K8)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13:B15 B17:B19">
+    <cfRule type="expression" dxfId="14" priority="558">
+      <formula>MAX($E33,$H33,$K33)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="559">
+      <formula>MAX($E9,$H9,$K9)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25 B27:B29">
+    <cfRule type="expression" dxfId="12" priority="581">
+      <formula>MAX($E9,$H9,$K9)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="582">
       <formula>MAX($E35,$H35,$K35)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B24">
-    <cfRule type="expression" dxfId="12" priority="355">
+  <conditionalFormatting sqref="B15">
+    <cfRule type="expression" dxfId="10" priority="592">
+      <formula>MAX($E40,$H40,$K40)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B23">
+    <cfRule type="expression" dxfId="9" priority="598">
+      <formula>MAX($E40,$H40,$K40)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21:B24">
+    <cfRule type="expression" dxfId="8" priority="608">
       <formula>MAX($E41,$H41,$K41)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B24">
-    <cfRule type="expression" dxfId="11" priority="356">
-      <formula>MAX($E35,$H35,$K35)=100</formula>
+  <conditionalFormatting sqref="B24 B27">
+    <cfRule type="expression" dxfId="7" priority="610">
+      <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B24">
-    <cfRule type="expression" dxfId="10" priority="388">
+    <cfRule type="expression" dxfId="6" priority="616">
+      <formula>MAX($E11,$H11,$K11)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="617">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="9" priority="437">
-      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+  <conditionalFormatting sqref="B20 B22">
+    <cfRule type="expression" dxfId="4" priority="618">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="438">
-      <formula>MAX($E4,$H4,$K4)=100</formula>
+    <cfRule type="expression" dxfId="3" priority="619">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B25:B30">
-    <cfRule type="expression" dxfId="7" priority="479">
-      <formula>MAX($E9,$H9,$K9)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="480">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+  <conditionalFormatting sqref="B22">
+    <cfRule type="expression" dxfId="2" priority="622">
+      <formula>MAX($E40,$H40,$K40)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10:B19">
-    <cfRule type="expression" dxfId="5" priority="481">
-      <formula>MAX($E31,$H31,$K31)=100</formula>
+  <conditionalFormatting sqref="B26">
+    <cfRule type="expression" dxfId="1" priority="623">
+      <formula>MAX($E10,$H10,$K10)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="482">
-      <formula>MAX($E6,$H6,$K6)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B24">
-    <cfRule type="expression" dxfId="3" priority="483">
-      <formula>MAX($E11,$H11,$K11)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="484">
-      <formula>MAX($E38,$H38,$K38)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B22">
-    <cfRule type="expression" dxfId="1" priority="485">
+    <cfRule type="expression" dxfId="0" priority="624">
       <formula>MAX($E40,$H40,$K40)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="486">
-      <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ajout des critères de mot de passes +  retour à l'utilisateur
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01FAD18-D035-4AD4-B8F0-10A755A63F12}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379C55A0-EC36-487F-A08D-E532E791D9D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="283">
   <si>
     <t>Planification globale</t>
   </si>
@@ -876,13 +876,25 @@
   </si>
   <si>
     <t>Front end affiche quand même erreur de mot de passe + logout jamais appelé</t>
+  </si>
+  <si>
+    <t>Journée nationale des Patriotes</t>
+  </si>
+  <si>
+    <t>Redéfinir la page index en plus grand caractères</t>
+  </si>
+  <si>
+    <t>Optimisation des formulaires: Création d' un component auth.js</t>
+  </si>
+  <si>
+    <t>Ajout des critères de mot de passes + faire un retour à l'utilisateur</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -928,6 +940,20 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="48"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1019,7 +1045,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="38">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -1450,11 +1476,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1643,11 +1717,49 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="69">
+  <dxfs count="71">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -2960,7 +3072,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="68" priority="1">
+    <cfRule type="expression" dxfId="70" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4302,67 +4414,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="67" priority="7">
+    <cfRule type="expression" dxfId="69" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="66" priority="1">
+    <cfRule type="expression" dxfId="68" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="65" priority="32">
+    <cfRule type="expression" dxfId="67" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="38">
+    <cfRule type="expression" dxfId="66" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="63" priority="30">
+    <cfRule type="expression" dxfId="65" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="62" priority="6">
+    <cfRule type="expression" dxfId="64" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="61" priority="25">
+    <cfRule type="expression" dxfId="63" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="27">
+    <cfRule type="expression" dxfId="62" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="59" priority="8">
+    <cfRule type="expression" dxfId="61" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="58" priority="13">
+    <cfRule type="expression" dxfId="60" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="14">
+    <cfRule type="expression" dxfId="59" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="56" priority="20">
+    <cfRule type="expression" dxfId="58" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="21">
+    <cfRule type="expression" dxfId="57" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="54" priority="9">
+    <cfRule type="expression" dxfId="56" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="10">
+    <cfRule type="expression" dxfId="55" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5542,23 +5654,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="52" priority="49">
+    <cfRule type="expression" dxfId="54" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="51" priority="89">
+    <cfRule type="expression" dxfId="53" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="50" priority="46">
+    <cfRule type="expression" dxfId="52" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="49" priority="47">
+    <cfRule type="expression" dxfId="51" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="48">
+    <cfRule type="expression" dxfId="50" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5697,10 +5809,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="47" priority="157">
+    <cfRule type="expression" dxfId="49" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="46" priority="158">
+    <cfRule type="expression" dxfId="48" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5714,27 +5826,28 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:O42"/>
+  <dimension ref="B2:P45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="67.7265625" customWidth="1"/>
+    <col min="3" max="3" width="17.6328125" style="31" customWidth="1"/>
     <col min="4" max="4" width="20.1796875" style="31" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40.81640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.453125" style="31" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.54296875" style="31" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" style="31" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.81640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.08984375" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7265625" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.08984375" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.81640625" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" ht="46" x14ac:dyDescent="1">
+    <row r="2" spans="2:16" ht="46" x14ac:dyDescent="1">
       <c r="B2" s="104" t="s">
         <v>17</v>
       </c>
@@ -5751,9 +5864,10 @@
       <c r="M2" s="105"/>
       <c r="N2" s="105"/>
       <c r="O2" s="105"/>
-    </row>
-    <row r="5" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:15" ht="21" x14ac:dyDescent="0.5">
+      <c r="P2" s="105"/>
+    </row>
+    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.5">
       <c r="B6" s="98" t="s">
         <v>1</v>
       </c>
@@ -5787,53 +5901,59 @@
       <c r="L6" s="102" t="s">
         <v>12</v>
       </c>
-      <c r="M6" s="60" t="s">
+      <c r="M6" s="43">
+        <v>46160</v>
+      </c>
+      <c r="N6" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="N6" s="43">
-        <v>46160</v>
-      </c>
-      <c r="O6" s="102" t="s">
+      <c r="O6" s="43">
+        <v>46167</v>
+      </c>
+      <c r="P6" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="2:16" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B7" s="99"/>
       <c r="C7" s="101"/>
       <c r="D7" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="59" t="s">
+      <c r="E7" s="108" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="103"/>
       <c r="G7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="59" t="s">
+      <c r="H7" s="108" t="s">
         <v>11</v>
       </c>
       <c r="I7" s="103"/>
       <c r="J7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="59" t="s">
+      <c r="K7" s="108" t="s">
         <v>11</v>
       </c>
       <c r="L7" s="103"/>
-      <c r="M7" s="59" t="s">
+      <c r="M7" s="110" t="s">
+        <v>201</v>
+      </c>
+      <c r="N7" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="N7" s="59" t="s">
+      <c r="O7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="O7" s="103"/>
-    </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="P7" s="103"/>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B8" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D8" s="24"/>
@@ -5846,15 +5966,18 @@
       <c r="G8" s="24"/>
       <c r="I8" s="92"/>
       <c r="J8" s="24"/>
-      <c r="L8" s="92"/>
-      <c r="M8" s="24"/>
-      <c r="O8" s="92"/>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L8" s="80"/>
+      <c r="M8" s="111" t="s">
+        <v>279</v>
+      </c>
+      <c r="N8" s="80"/>
+      <c r="P8" s="92"/>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B9" s="81" t="s">
         <v>256</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D9" s="24">
@@ -5867,15 +5990,16 @@
       <c r="G9" s="24"/>
       <c r="I9" s="92"/>
       <c r="J9" s="24"/>
-      <c r="L9" s="92"/>
-      <c r="M9" s="24"/>
-      <c r="O9" s="92"/>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L9" s="80"/>
+      <c r="M9" s="112"/>
+      <c r="N9" s="80"/>
+      <c r="P9" s="92"/>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B10" s="81" t="s">
         <v>245</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D10" s="24">
@@ -5888,15 +6012,16 @@
       <c r="G10" s="24"/>
       <c r="I10" s="92"/>
       <c r="J10" s="24"/>
-      <c r="L10" s="92"/>
-      <c r="M10" s="24"/>
-      <c r="O10" s="92"/>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L10" s="80"/>
+      <c r="M10" s="112"/>
+      <c r="N10" s="80"/>
+      <c r="P10" s="92"/>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="81" t="s">
         <v>244</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D11" s="24">
@@ -5909,15 +6034,16 @@
       <c r="G11" s="24"/>
       <c r="I11" s="92"/>
       <c r="J11" s="24"/>
-      <c r="L11" s="92"/>
-      <c r="M11" s="24"/>
-      <c r="O11" s="92"/>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L11" s="80"/>
+      <c r="M11" s="112"/>
+      <c r="N11" s="80"/>
+      <c r="P11" s="92"/>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="81" t="s">
         <v>257</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D12" s="80">
@@ -5930,15 +6056,16 @@
       <c r="G12" s="24"/>
       <c r="I12" s="92"/>
       <c r="J12" s="24"/>
-      <c r="L12" s="92"/>
-      <c r="M12" s="24"/>
-      <c r="O12" s="92"/>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L12" s="80"/>
+      <c r="M12" s="112"/>
+      <c r="N12" s="80"/>
+      <c r="P12" s="92"/>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D13" s="80">
@@ -5951,15 +6078,16 @@
       <c r="G13" s="24"/>
       <c r="I13" s="92"/>
       <c r="J13" s="24"/>
-      <c r="L13" s="92"/>
-      <c r="M13" s="24"/>
-      <c r="O13" s="92"/>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L13" s="80"/>
+      <c r="M13" s="112"/>
+      <c r="N13" s="80"/>
+      <c r="P13" s="92"/>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D14" s="80">
@@ -5972,15 +6100,16 @@
       <c r="G14" s="24"/>
       <c r="I14" s="92"/>
       <c r="J14" s="24"/>
-      <c r="L14" s="92"/>
-      <c r="M14" s="24"/>
-      <c r="O14" s="92"/>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L14" s="80"/>
+      <c r="M14" s="112"/>
+      <c r="N14" s="80"/>
+      <c r="P14" s="92"/>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D15" s="80">
@@ -5993,15 +6122,16 @@
       <c r="G15" s="24"/>
       <c r="I15" s="92"/>
       <c r="J15" s="24"/>
-      <c r="L15" s="92"/>
-      <c r="M15" s="24"/>
-      <c r="O15" s="92"/>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L15" s="80"/>
+      <c r="M15" s="112"/>
+      <c r="N15" s="80"/>
+      <c r="P15" s="92"/>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D16" s="80">
@@ -6014,15 +6144,16 @@
       <c r="G16" s="24"/>
       <c r="I16" s="92"/>
       <c r="J16" s="24"/>
-      <c r="L16" s="92"/>
-      <c r="M16" s="24"/>
-      <c r="O16" s="92"/>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L16" s="80"/>
+      <c r="M16" s="112"/>
+      <c r="N16" s="80"/>
+      <c r="P16" s="92"/>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D17" s="80"/>
@@ -6030,17 +6161,21 @@
       <c r="G17" s="24">
         <v>3</v>
       </c>
+      <c r="H17" s="31">
+        <v>100</v>
+      </c>
       <c r="I17" s="92"/>
       <c r="J17" s="24"/>
-      <c r="L17" s="92"/>
-      <c r="M17" s="24"/>
-      <c r="O17" s="92"/>
-    </row>
-    <row r="18" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L17" s="80"/>
+      <c r="M17" s="112"/>
+      <c r="N17" s="80"/>
+      <c r="P17" s="92"/>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D18" s="80"/>
@@ -6048,17 +6183,21 @@
       <c r="G18" s="24">
         <v>0.75</v>
       </c>
+      <c r="H18" s="31">
+        <v>100</v>
+      </c>
       <c r="I18" s="92"/>
       <c r="J18" s="24"/>
-      <c r="L18" s="92"/>
-      <c r="M18" s="24"/>
-      <c r="O18" s="92"/>
-    </row>
-    <row r="19" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L18" s="80"/>
+      <c r="M18" s="112"/>
+      <c r="N18" s="80"/>
+      <c r="P18" s="92"/>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D19" s="80"/>
@@ -6066,17 +6205,21 @@
       <c r="G19" s="24">
         <v>1.25</v>
       </c>
+      <c r="H19" s="31">
+        <v>100</v>
+      </c>
       <c r="I19" s="92"/>
       <c r="J19" s="24"/>
-      <c r="L19" s="92"/>
-      <c r="M19" s="24"/>
-      <c r="O19" s="92"/>
-    </row>
-    <row r="20" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L19" s="80"/>
+      <c r="M19" s="112"/>
+      <c r="N19" s="80"/>
+      <c r="P19" s="92"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="C20" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D20" s="80"/>
@@ -6084,17 +6227,21 @@
       <c r="G20" s="24">
         <v>0.15</v>
       </c>
+      <c r="H20" s="31">
+        <v>100</v>
+      </c>
       <c r="I20" s="92"/>
       <c r="J20" s="24"/>
-      <c r="L20" s="92"/>
-      <c r="M20" s="24"/>
-      <c r="O20" s="92"/>
-    </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L20" s="80"/>
+      <c r="M20" s="112"/>
+      <c r="N20" s="80"/>
+      <c r="P20" s="92"/>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D21" s="80"/>
@@ -6102,17 +6249,21 @@
       <c r="G21" s="24">
         <v>0.5</v>
       </c>
+      <c r="H21" s="31">
+        <v>100</v>
+      </c>
       <c r="I21" s="92"/>
       <c r="J21" s="24"/>
-      <c r="L21" s="92"/>
-      <c r="M21" s="24"/>
-      <c r="O21" s="92"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L21" s="80"/>
+      <c r="M21" s="112"/>
+      <c r="N21" s="80"/>
+      <c r="P21" s="92"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="81" t="s">
         <v>255</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D22" s="80"/>
@@ -6120,17 +6271,21 @@
       <c r="G22" s="24">
         <v>0.15</v>
       </c>
+      <c r="H22" s="31">
+        <v>100</v>
+      </c>
       <c r="I22" s="92"/>
       <c r="J22" s="24"/>
-      <c r="L22" s="92"/>
-      <c r="M22" s="24"/>
-      <c r="O22" s="92"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L22" s="80"/>
+      <c r="M22" s="112"/>
+      <c r="N22" s="80"/>
+      <c r="P22" s="92"/>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B23" s="82" t="s">
         <v>258</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D23" s="24"/>
@@ -6138,17 +6293,21 @@
       <c r="G23" s="24">
         <v>0.15</v>
       </c>
+      <c r="H23" s="31">
+        <v>100</v>
+      </c>
       <c r="I23" s="92"/>
       <c r="J23" s="24"/>
-      <c r="L23" s="92"/>
-      <c r="M23" s="24"/>
-      <c r="O23" s="92"/>
-    </row>
-    <row r="24" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L23" s="80"/>
+      <c r="M23" s="112"/>
+      <c r="N23" s="80"/>
+      <c r="P23" s="92"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B24" s="82" t="s">
         <v>259</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D24" s="24"/>
@@ -6156,15 +6315,16 @@
       <c r="G24" s="24"/>
       <c r="I24" s="92"/>
       <c r="J24" s="24"/>
-      <c r="L24" s="92"/>
-      <c r="M24" s="24"/>
-      <c r="O24" s="92"/>
-    </row>
-    <row r="25" spans="2:15" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L24" s="80"/>
+      <c r="M24" s="112"/>
+      <c r="N24" s="80"/>
+      <c r="P24" s="92"/>
+    </row>
+    <row r="25" spans="2:16" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="83" t="s">
         <v>260</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D25" s="24"/>
@@ -6174,15 +6334,19 @@
       <c r="J25" s="24">
         <v>3</v>
       </c>
-      <c r="L25" s="92"/>
-      <c r="M25" s="24"/>
-      <c r="O25" s="92"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K25" s="31">
+        <v>100</v>
+      </c>
+      <c r="L25" s="80"/>
+      <c r="M25" s="112"/>
+      <c r="N25" s="80"/>
+      <c r="P25" s="92"/>
+    </row>
+    <row r="26" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B26" s="83" t="s">
         <v>261</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="C26" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D26" s="24"/>
@@ -6192,15 +6356,19 @@
       <c r="J26" s="24">
         <v>1</v>
       </c>
-      <c r="L26" s="92"/>
-      <c r="M26" s="24"/>
-      <c r="O26" s="92"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K26" s="31">
+        <v>100</v>
+      </c>
+      <c r="L26" s="80"/>
+      <c r="M26" s="112"/>
+      <c r="N26" s="80"/>
+      <c r="P26" s="92"/>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="83" t="s">
         <v>262</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D27" s="24"/>
@@ -6210,15 +6378,19 @@
       <c r="J27" s="24">
         <v>1</v>
       </c>
-      <c r="L27" s="92"/>
-      <c r="M27" s="24"/>
-      <c r="O27" s="92"/>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K27" s="31">
+        <v>100</v>
+      </c>
+      <c r="L27" s="80"/>
+      <c r="M27" s="112"/>
+      <c r="N27" s="80"/>
+      <c r="P27" s="92"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="83" t="s">
         <v>263</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="C28" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D28" s="24"/>
@@ -6228,15 +6400,19 @@
       <c r="J28" s="24">
         <v>0.75</v>
       </c>
-      <c r="L28" s="92"/>
-      <c r="M28" s="24"/>
-      <c r="O28" s="92"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K28" s="31">
+        <v>100</v>
+      </c>
+      <c r="L28" s="80"/>
+      <c r="M28" s="112"/>
+      <c r="N28" s="80"/>
+      <c r="P28" s="92"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="83" t="s">
         <v>264</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="C29" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D29" s="24"/>
@@ -6246,15 +6422,19 @@
       <c r="J29" s="24">
         <v>1</v>
       </c>
-      <c r="L29" s="92"/>
-      <c r="M29" s="24"/>
-      <c r="O29" s="92"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="K29" s="31">
+        <v>100</v>
+      </c>
+      <c r="L29" s="80"/>
+      <c r="M29" s="112"/>
+      <c r="N29" s="80"/>
+      <c r="P29" s="92"/>
+    </row>
+    <row r="30" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B30" s="83" t="s">
         <v>265</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="106" t="s">
         <v>102</v>
       </c>
       <c r="D30" s="24"/>
@@ -6264,108 +6444,114 @@
       <c r="J30" s="24">
         <v>0.5</v>
       </c>
-      <c r="L30" s="92"/>
-      <c r="M30" s="24"/>
-      <c r="O30" s="92"/>
-    </row>
-    <row r="31" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B31" s="29" t="s">
-        <v>215</v>
-      </c>
-      <c r="C31" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D31" s="24">
-        <v>2</v>
-      </c>
-      <c r="E31" s="31">
-        <v>50</v>
-      </c>
-      <c r="F31" s="94" t="s">
-        <v>272</v>
-      </c>
-      <c r="G31" s="24">
-        <v>2</v>
-      </c>
-      <c r="H31" s="31">
-        <v>100</v>
-      </c>
+      <c r="K30" s="31">
+        <v>100</v>
+      </c>
+      <c r="L30" s="80"/>
+      <c r="M30" s="112"/>
+      <c r="N30" s="80"/>
+      <c r="P30" s="92"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B31" s="83" t="s">
+        <v>281</v>
+      </c>
+      <c r="C31" s="106" t="s">
+        <v>102</v>
+      </c>
+      <c r="D31" s="24"/>
+      <c r="F31" s="92"/>
+      <c r="G31" s="24"/>
       <c r="I31" s="92"/>
       <c r="J31" s="24"/>
-      <c r="L31" s="92"/>
-      <c r="M31" s="24"/>
-      <c r="O31" s="92"/>
-    </row>
-    <row r="32" spans="2:15" ht="29" x14ac:dyDescent="0.35">
-      <c r="B32" s="29" t="s">
-        <v>216</v>
-      </c>
-      <c r="C32" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D32" s="24">
-        <v>1</v>
-      </c>
-      <c r="E32" s="31">
-        <v>25</v>
-      </c>
-      <c r="F32" s="94" t="s">
-        <v>273</v>
-      </c>
+      <c r="L31" s="80"/>
+      <c r="M31" s="112"/>
+      <c r="N31" s="80">
+        <v>2</v>
+      </c>
+      <c r="O31" s="31">
+        <v>100</v>
+      </c>
+      <c r="P31" s="92"/>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B32" s="83" t="s">
+        <v>280</v>
+      </c>
+      <c r="C32" s="106" t="s">
+        <v>102</v>
+      </c>
+      <c r="D32" s="24"/>
+      <c r="F32" s="92"/>
       <c r="G32" s="24"/>
       <c r="I32" s="92"/>
       <c r="J32" s="24"/>
-      <c r="L32" s="92"/>
-      <c r="M32" s="24"/>
-      <c r="O32" s="92"/>
-    </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B33" s="29" t="s">
-        <v>217</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D33" s="24">
-        <v>5</v>
-      </c>
-      <c r="E33" s="31">
-        <v>100</v>
-      </c>
+      <c r="L32" s="80"/>
+      <c r="M32" s="112"/>
+      <c r="N32" s="80">
+        <v>1</v>
+      </c>
+      <c r="O32" s="31">
+        <v>100</v>
+      </c>
+      <c r="P32" s="92"/>
+    </row>
+    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B33" s="83" t="s">
+        <v>282</v>
+      </c>
+      <c r="C33" s="106" t="s">
+        <v>102</v>
+      </c>
+      <c r="D33" s="24"/>
       <c r="F33" s="92"/>
       <c r="G33" s="24"/>
       <c r="I33" s="92"/>
       <c r="J33" s="24"/>
-      <c r="L33" s="92"/>
-      <c r="M33" s="24"/>
-      <c r="O33" s="92"/>
-    </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L33" s="80"/>
+      <c r="M33" s="112"/>
+      <c r="N33" s="80">
+        <v>2</v>
+      </c>
+      <c r="O33" s="31">
+        <v>100</v>
+      </c>
+      <c r="P33" s="92"/>
+    </row>
+    <row r="34" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
-        <v>218</v>
-      </c>
-      <c r="C34" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="C34" s="106" t="s">
         <v>103</v>
       </c>
       <c r="D34" s="24">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E34" s="31">
-        <v>100</v>
-      </c>
-      <c r="F34" s="92"/>
-      <c r="G34" s="24"/>
+        <v>50</v>
+      </c>
+      <c r="F34" s="94" t="s">
+        <v>272</v>
+      </c>
+      <c r="G34" s="24">
+        <v>2</v>
+      </c>
+      <c r="H34" s="31">
+        <v>100</v>
+      </c>
       <c r="I34" s="92"/>
       <c r="J34" s="24"/>
-      <c r="L34" s="92"/>
-      <c r="M34" s="24"/>
-      <c r="O34" s="92"/>
-    </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L34" s="80"/>
+      <c r="M34" s="112"/>
+      <c r="N34" s="80"/>
+      <c r="P34" s="92"/>
+    </row>
+    <row r="35" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="C35" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="C35" s="106" t="s">
         <v>103</v>
       </c>
       <c r="D35" s="24">
@@ -6374,374 +6560,459 @@
       <c r="E35" s="31">
         <v>25</v>
       </c>
-      <c r="F35" s="92" t="s">
-        <v>271</v>
-      </c>
-      <c r="G35" s="24">
-        <v>2</v>
-      </c>
-      <c r="H35" s="31">
-        <v>75</v>
-      </c>
-      <c r="I35" s="94" t="s">
-        <v>270</v>
-      </c>
+      <c r="F35" s="94" t="s">
+        <v>273</v>
+      </c>
+      <c r="G35" s="24"/>
+      <c r="I35" s="92"/>
       <c r="J35" s="24"/>
-      <c r="L35" s="92"/>
-      <c r="M35" s="24"/>
-      <c r="O35" s="92"/>
-    </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="L35" s="80"/>
+      <c r="M35" s="112"/>
+      <c r="N35" s="80"/>
+      <c r="P35" s="92"/>
+    </row>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="C36" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="C36" s="106" t="s">
         <v>103</v>
       </c>
-      <c r="D36" s="24"/>
+      <c r="D36" s="24">
+        <v>5</v>
+      </c>
+      <c r="E36" s="31">
+        <v>100</v>
+      </c>
       <c r="F36" s="92"/>
-      <c r="G36" s="24">
-        <v>3</v>
-      </c>
-      <c r="H36" s="31">
-        <v>100</v>
-      </c>
+      <c r="G36" s="24"/>
       <c r="I36" s="92"/>
       <c r="J36" s="24"/>
-      <c r="L36" s="92"/>
-      <c r="M36" s="24"/>
-      <c r="O36" s="92"/>
-    </row>
-    <row r="37" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B37" s="90" t="s">
+      <c r="L36" s="80"/>
+      <c r="M36" s="112"/>
+      <c r="N36" s="80"/>
+      <c r="P36" s="92"/>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B37" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="C37" s="106" t="s">
+        <v>103</v>
+      </c>
+      <c r="D37" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="E37" s="31">
+        <v>100</v>
+      </c>
+      <c r="F37" s="92"/>
+      <c r="G37" s="24"/>
+      <c r="I37" s="92"/>
+      <c r="J37" s="24"/>
+      <c r="L37" s="80"/>
+      <c r="M37" s="112"/>
+      <c r="N37" s="80"/>
+      <c r="P37" s="92"/>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B38" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="C38" s="106" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="24">
+        <v>1</v>
+      </c>
+      <c r="E38" s="31">
+        <v>25</v>
+      </c>
+      <c r="F38" s="92" t="s">
+        <v>271</v>
+      </c>
+      <c r="G38" s="24">
+        <v>2</v>
+      </c>
+      <c r="H38" s="31">
+        <v>75</v>
+      </c>
+      <c r="I38" s="94" t="s">
+        <v>270</v>
+      </c>
+      <c r="J38" s="24"/>
+      <c r="L38" s="80"/>
+      <c r="M38" s="112"/>
+      <c r="N38" s="80"/>
+      <c r="P38" s="92"/>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B39" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="C39" s="106" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="24"/>
+      <c r="F39" s="92"/>
+      <c r="G39" s="24">
+        <v>3</v>
+      </c>
+      <c r="H39" s="31">
+        <v>100</v>
+      </c>
+      <c r="I39" s="92"/>
+      <c r="J39" s="24"/>
+      <c r="L39" s="80"/>
+      <c r="M39" s="112"/>
+      <c r="N39" s="80"/>
+      <c r="P39" s="92"/>
+    </row>
+    <row r="40" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B40" s="90" t="s">
         <v>266</v>
       </c>
-      <c r="C37" s="90" t="s">
+      <c r="C40" s="107" t="s">
         <v>103</v>
       </c>
-      <c r="G37" s="24">
+      <c r="G40" s="24">
         <v>1.5</v>
       </c>
-      <c r="H37" s="31">
-        <v>100</v>
-      </c>
-      <c r="I37" s="93" t="s">
+      <c r="H40" s="31">
+        <v>100</v>
+      </c>
+      <c r="I40" s="93" t="s">
         <v>269</v>
       </c>
-      <c r="J37" s="24"/>
-      <c r="M37" s="24"/>
-      <c r="O37" s="92"/>
-    </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B38" s="90" t="s">
+      <c r="J40" s="24"/>
+      <c r="M40" s="112"/>
+      <c r="N40" s="80"/>
+      <c r="P40" s="92"/>
+    </row>
+    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B41" s="90" t="s">
         <v>267</v>
       </c>
-      <c r="C38" s="90" t="s">
+      <c r="C41" s="107" t="s">
         <v>103</v>
       </c>
-      <c r="G38" s="24"/>
-      <c r="J38" s="24">
-        <v>2</v>
-      </c>
-      <c r="K38" s="31">
-        <v>100</v>
-      </c>
-      <c r="M38" s="24"/>
-      <c r="O38" s="92"/>
-    </row>
-    <row r="39" spans="2:15" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="B39" s="90" t="s">
-        <v>268</v>
-      </c>
-      <c r="C39" s="90" t="s">
-        <v>103</v>
-      </c>
-      <c r="G39" s="24"/>
-      <c r="J39" s="24">
-        <v>4</v>
-      </c>
-      <c r="K39" s="31">
-        <v>90</v>
-      </c>
-      <c r="L39" s="93" t="s">
-        <v>275</v>
-      </c>
-      <c r="M39" s="24"/>
-      <c r="O39" s="92"/>
-    </row>
-    <row r="40" spans="2:15" ht="58" x14ac:dyDescent="0.35">
-      <c r="B40" s="29" t="s">
-        <v>239</v>
-      </c>
-      <c r="C40" s="29" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40" s="24"/>
-      <c r="F40" s="92"/>
-      <c r="G40" s="24"/>
-      <c r="I40" s="92"/>
-      <c r="J40" s="24">
-        <v>1.5</v>
-      </c>
-      <c r="K40" s="31">
-        <v>100</v>
-      </c>
-      <c r="L40" s="94" t="s">
-        <v>274</v>
-      </c>
-      <c r="M40" s="24"/>
-      <c r="O40" s="92"/>
-    </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B41" s="90" t="s">
-        <v>276</v>
-      </c>
-      <c r="C41" s="90" t="s">
-        <v>103</v>
-      </c>
-      <c r="D41" s="31">
-        <v>1</v>
-      </c>
-      <c r="E41" s="31">
-        <v>10</v>
-      </c>
-      <c r="G41" s="24">
-        <v>2</v>
-      </c>
-      <c r="H41" s="31">
-        <v>30</v>
-      </c>
+      <c r="G41" s="24"/>
       <c r="J41" s="24">
         <v>2</v>
       </c>
       <c r="K41" s="31">
+        <v>100</v>
+      </c>
+      <c r="M41" s="112"/>
+      <c r="N41" s="80"/>
+      <c r="P41" s="92"/>
+    </row>
+    <row r="42" spans="2:16" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="B42" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="C42" s="107" t="s">
+        <v>103</v>
+      </c>
+      <c r="G42" s="24"/>
+      <c r="J42" s="24">
+        <v>4</v>
+      </c>
+      <c r="K42" s="31">
+        <v>90</v>
+      </c>
+      <c r="L42" s="93" t="s">
+        <v>275</v>
+      </c>
+      <c r="M42" s="112"/>
+      <c r="N42" s="80"/>
+      <c r="P42" s="92"/>
+    </row>
+    <row r="43" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="B43" s="29" t="s">
+        <v>239</v>
+      </c>
+      <c r="C43" s="106" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="24"/>
+      <c r="F43" s="92"/>
+      <c r="G43" s="24"/>
+      <c r="I43" s="92"/>
+      <c r="J43" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="K43" s="31">
+        <v>100</v>
+      </c>
+      <c r="L43" s="109" t="s">
+        <v>274</v>
+      </c>
+      <c r="M43" s="112"/>
+      <c r="N43" s="80"/>
+      <c r="P43" s="92"/>
+    </row>
+    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B44" s="90" t="s">
+        <v>276</v>
+      </c>
+      <c r="C44" s="107" t="s">
+        <v>103</v>
+      </c>
+      <c r="D44" s="31">
+        <v>1</v>
+      </c>
+      <c r="E44" s="31">
+        <v>10</v>
+      </c>
+      <c r="G44" s="24">
+        <v>2</v>
+      </c>
+      <c r="H44" s="31">
+        <v>30</v>
+      </c>
+      <c r="J44" s="24">
+        <v>2</v>
+      </c>
+      <c r="K44" s="31">
         <v>50</v>
       </c>
-      <c r="M41" s="24"/>
-      <c r="O41" s="92"/>
-    </row>
-    <row r="42" spans="2:15" ht="58" x14ac:dyDescent="0.35">
-      <c r="B42" s="90" t="s">
+      <c r="M44" s="112"/>
+      <c r="N44" s="80"/>
+      <c r="P44" s="92"/>
+    </row>
+    <row r="45" spans="2:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B45" s="90" t="s">
         <v>277</v>
       </c>
-      <c r="J42" s="31">
+      <c r="J45" s="31">
         <v>1</v>
       </c>
-      <c r="L42" s="93" t="s">
+      <c r="L45" s="93" t="s">
         <v>278</v>
       </c>
+      <c r="M45" s="113"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="O6:O7"/>
+  <mergeCells count="8">
+    <mergeCell ref="M8:M45"/>
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="P6:P7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B6:B7 B23:B42">
-    <cfRule type="expression" dxfId="45" priority="27">
+  <conditionalFormatting sqref="B2 B6:B7 B23:B45">
+    <cfRule type="expression" dxfId="47" priority="27">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C41">
-    <cfRule type="expression" dxfId="44" priority="16">
+  <conditionalFormatting sqref="C6:C44">
+    <cfRule type="expression" dxfId="46" priority="16">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="17">
+    <cfRule type="expression" dxfId="45" priority="17">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="18">
+    <cfRule type="expression" dxfId="44" priority="18">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="41" priority="230">
+  <conditionalFormatting sqref="B8 B23:B24">
+    <cfRule type="expression" dxfId="43" priority="230">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14">
-    <cfRule type="expression" dxfId="40" priority="232">
+  <conditionalFormatting sqref="B14 B32:B33">
+    <cfRule type="expression" dxfId="42" priority="232">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="39" priority="248">
-      <formula>MAX($E31,$H31,$K31)=100</formula>
+    <cfRule type="expression" dxfId="41" priority="248">
+      <formula>MAX($E34,$H34,$K34)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="38" priority="269">
+    <cfRule type="expression" dxfId="40" priority="269">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8:B12 B25:B26">
-    <cfRule type="expression" dxfId="37" priority="3">
+  <conditionalFormatting sqref="B8:B12">
+    <cfRule type="expression" dxfId="39" priority="3">
       <formula>MAX($E17,$H17,$K17)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B30">
-    <cfRule type="expression" dxfId="36" priority="1">
+  <conditionalFormatting sqref="B23:B33">
+    <cfRule type="expression" dxfId="38" priority="1">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:B16">
-    <cfRule type="expression" dxfId="35" priority="318">
-      <formula>MAX($E31,$H31,$K31)=100</formula>
+    <cfRule type="expression" dxfId="37" priority="318">
+      <formula>MAX($E34,$H34,$K34)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="34" priority="349">
+    <cfRule type="expression" dxfId="36" priority="349">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="350">
+    <cfRule type="expression" dxfId="35" priority="350">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28:B30">
-    <cfRule type="expression" dxfId="32" priority="353">
+  <conditionalFormatting sqref="B12:B14 B16:B18">
+    <cfRule type="expression" dxfId="34" priority="355">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:B19">
+    <cfRule type="expression" dxfId="33" priority="356">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20:B21">
+    <cfRule type="expression" dxfId="32" priority="388">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12:B14 B16:B18">
-    <cfRule type="expression" dxfId="31" priority="355">
-      <formula>MAX($E33,$H33,$K33)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18:B19">
-    <cfRule type="expression" dxfId="30" priority="356">
-      <formula>MAX($E33,$H33,$K33)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B21 B23:B24">
-    <cfRule type="expression" dxfId="29" priority="388">
-      <formula>MAX($E34,$H34,$K34)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="28" priority="437">
+    <cfRule type="expression" dxfId="31" priority="437">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="27" priority="438">
+    <cfRule type="expression" dxfId="30" priority="438">
       <formula>MAX($E4,$H4,$K4)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10:B11">
-    <cfRule type="expression" dxfId="26" priority="481">
-      <formula>MAX($E31,$H31,$K31)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="25" priority="482">
-      <formula>MAX($E6,$H6,$K6)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="expression" dxfId="24" priority="497">
+    <cfRule type="expression" dxfId="29" priority="497">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="expression" dxfId="23" priority="502">
+    <cfRule type="expression" dxfId="28" priority="502">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30">
-    <cfRule type="expression" dxfId="22" priority="510">
+  <conditionalFormatting sqref="B30:B31">
+    <cfRule type="expression" dxfId="27" priority="510">
       <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="511">
+    <cfRule type="expression" dxfId="26" priority="511">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="expression" dxfId="20" priority="520">
+    <cfRule type="expression" dxfId="25" priority="520">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="521">
+    <cfRule type="expression" dxfId="24" priority="521">
       <formula>MAX($E16,$H16,$K16)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="18" priority="531">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="23" priority="531">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="expression" dxfId="17" priority="533">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="22" priority="533">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12 B16">
-    <cfRule type="expression" dxfId="16" priority="538">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="21" priority="538">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="539">
+    <cfRule type="expression" dxfId="20" priority="539">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B13:B15 B17:B19">
-    <cfRule type="expression" dxfId="14" priority="558">
-      <formula>MAX($E33,$H33,$K33)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="559">
+  <conditionalFormatting sqref="B25 B27:B29">
+    <cfRule type="expression" dxfId="19" priority="581">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25 B27:B29">
-    <cfRule type="expression" dxfId="12" priority="581">
-      <formula>MAX($E9,$H9,$K9)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="11" priority="582">
-      <formula>MAX($E35,$H35,$K35)=100</formula>
+    <cfRule type="expression" dxfId="18" priority="582">
+      <formula>MAX($E38,$H38,$K38)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="10" priority="592">
+    <cfRule type="expression" dxfId="17" priority="592">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B23">
+    <cfRule type="expression" dxfId="16" priority="598">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21:B24">
+    <cfRule type="expression" dxfId="15" priority="608">
+      <formula>MAX($E44,$H44,$K44)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B24 B27">
+    <cfRule type="expression" dxfId="14" priority="610">
       <formula>MAX($E40,$H40,$K40)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23">
-    <cfRule type="expression" dxfId="9" priority="598">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
+  <conditionalFormatting sqref="B20 B22">
+    <cfRule type="expression" dxfId="13" priority="618">
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21:B24">
-    <cfRule type="expression" dxfId="8" priority="608">
-      <formula>MAX($E41,$H41,$K41)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B24 B27">
-    <cfRule type="expression" dxfId="7" priority="610">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B24">
-    <cfRule type="expression" dxfId="6" priority="616">
-      <formula>MAX($E11,$H11,$K11)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="5" priority="617">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20 B22">
-    <cfRule type="expression" dxfId="4" priority="618">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="619">
+    <cfRule type="expression" dxfId="12" priority="619">
       <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="expression" dxfId="2" priority="622">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
+    <cfRule type="expression" dxfId="11" priority="622">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26">
-    <cfRule type="expression" dxfId="1" priority="623">
+    <cfRule type="expression" dxfId="10" priority="623">
       <formula>MAX($E10,$H10,$K10)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="624">
+    <cfRule type="expression" dxfId="9" priority="624">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13:B15 B17:B19">
+    <cfRule type="expression" dxfId="8" priority="655">
+      <formula>MAX($E36,$H36,$K36)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="656">
+      <formula>MAX($E9,$H9,$K9)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:B26 B28:B31">
+    <cfRule type="expression" dxfId="6" priority="659">
+      <formula>MAX($E37,$H37,$K37)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:B33">
+    <cfRule type="expression" dxfId="5" priority="666">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="667">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B10:B11">
+    <cfRule type="expression" dxfId="3" priority="679">
+      <formula>MAX($E34,$H34,$K34)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="680">
+      <formula>MAX($E6,$H6,$K6)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B23:B24">
+    <cfRule type="expression" dxfId="1" priority="681">
+      <formula>MAX($E11,$H11,$K11)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="682">
       <formula>MAX($E40,$H40,$K40)=100</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
debug load + ajout modification de difficulté
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrateur.UTILISA-LQC2BC3\Downloads\__Projet_Projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{379C55A0-EC36-487F-A08D-E532E791D9D4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82D00F7-D4AB-41A5-AAF9-EA7341C98BD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="289">
   <si>
     <t>Planification globale</t>
   </si>
@@ -875,9 +875,6 @@
     <t>Empêcher un joueur d'être connecté plus d'une fois</t>
   </si>
   <si>
-    <t>Front end affiche quand même erreur de mot de passe + logout jamais appelé</t>
-  </si>
-  <si>
     <t>Journée nationale des Patriotes</t>
   </si>
   <si>
@@ -888,6 +885,27 @@
   </si>
   <si>
     <t>Ajout des critères de mot de passes + faire un retour à l'utilisateur</t>
+  </si>
+  <si>
+    <t>Terminé les heuristiques, refonte des priors et des fonctions de setup</t>
+  </si>
+  <si>
+    <t>Comme on n'a pas de disconnect, apparaît comme mauvais mot de passe</t>
+  </si>
+  <si>
+    <t>Debug load</t>
+  </si>
+  <si>
+    <t>Erreur quand on delete une game et qu'on en reccomence une autre trop rapidement - 2e game est deleted</t>
+  </si>
+  <si>
+    <t>Ajouté colonne dans db. Voir si ça fonctionne avec le front end</t>
+  </si>
+  <si>
+    <t>Ajouter option difficulté AI dans le jeu</t>
+  </si>
+  <si>
+    <t>Debug reccomencer un jeu quand on vient d'en finir un</t>
   </si>
 </sst>
 </file>
@@ -1045,7 +1063,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1487,43 +1505,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1684,6 +1665,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1717,35 +1710,148 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="71">
+  <dxfs count="86">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3072,7 +3178,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="70" priority="1">
+    <cfRule type="expression" dxfId="85" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3516,26 +3622,26 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B3" s="95" t="s">
+      <c r="B3" s="99" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="97"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="100"/>
+      <c r="H3" s="100"/>
+      <c r="I3" s="100"/>
+      <c r="J3" s="100"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="101"/>
     </row>
     <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B5" s="98" t="s">
+      <c r="B5" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="100" t="s">
+      <c r="C5" s="104" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3544,7 +3650,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="102" t="s">
+      <c r="F5" s="106" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3553,7 +3659,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="102" t="s">
+      <c r="I5" s="106" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3562,34 +3668,34 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="102" t="s">
+      <c r="L5" s="106" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B6" s="99"/>
-      <c r="C6" s="101"/>
+      <c r="B6" s="103"/>
+      <c r="C6" s="105"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="103"/>
+      <c r="F6" s="107"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="103"/>
+      <c r="I6" s="107"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="103"/>
+      <c r="L6" s="107"/>
     </row>
     <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="28" t="s">
@@ -4414,67 +4520,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="69" priority="7">
+    <cfRule type="expression" dxfId="84" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="68" priority="1">
+    <cfRule type="expression" dxfId="83" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="67" priority="32">
+    <cfRule type="expression" dxfId="82" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="38">
+    <cfRule type="expression" dxfId="81" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="65" priority="30">
+    <cfRule type="expression" dxfId="80" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="64" priority="6">
+    <cfRule type="expression" dxfId="79" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="63" priority="25">
+    <cfRule type="expression" dxfId="78" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="27">
+    <cfRule type="expression" dxfId="77" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="61" priority="8">
+    <cfRule type="expression" dxfId="76" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="60" priority="13">
+    <cfRule type="expression" dxfId="75" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="14">
+    <cfRule type="expression" dxfId="74" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="58" priority="20">
+    <cfRule type="expression" dxfId="73" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="21">
+    <cfRule type="expression" dxfId="72" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="56" priority="9">
+    <cfRule type="expression" dxfId="71" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="10">
+    <cfRule type="expression" dxfId="70" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4506,26 +4612,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
-      <c r="B1" s="95" t="s">
+      <c r="B1" s="99" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="97"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="101"/>
     </row>
     <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="B4" s="98" t="s">
+      <c r="B4" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="100" t="s">
+      <c r="C4" s="104" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4534,7 +4640,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="102" t="s">
+      <c r="F4" s="106" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4543,7 +4649,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="102" t="s">
+      <c r="I4" s="106" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4552,34 +4658,34 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="102" t="s">
+      <c r="L4" s="106" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B5" s="99"/>
-      <c r="C5" s="101"/>
+      <c r="B5" s="103"/>
+      <c r="C5" s="105"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="103"/>
+      <c r="F5" s="107"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="103"/>
+      <c r="I5" s="107"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="103"/>
+      <c r="L5" s="107"/>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B6" s="29" t="s">
@@ -5654,23 +5760,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="54" priority="49">
+    <cfRule type="expression" dxfId="69" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="53" priority="89">
+    <cfRule type="expression" dxfId="68" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="52" priority="46">
+    <cfRule type="expression" dxfId="67" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="47">
+    <cfRule type="expression" dxfId="66" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="48">
+    <cfRule type="expression" dxfId="65" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5809,10 +5915,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="49" priority="157">
+    <cfRule type="expression" dxfId="64" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="158">
+    <cfRule type="expression" dxfId="63" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5826,7 +5932,7 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:P45"/>
+  <dimension ref="B2:P48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
@@ -5840,38 +5946,38 @@
     <col min="9" max="9" width="35.1796875" style="31" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.1796875" style="31" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.54296875" style="93" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.7265625" style="31" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="21.08984375" style="31" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.81640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.54296875" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" ht="46" x14ac:dyDescent="1">
-      <c r="B2" s="104" t="s">
+      <c r="B2" s="108" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="105"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="105"/>
-      <c r="J2" s="105"/>
-      <c r="K2" s="105"/>
-      <c r="L2" s="105"/>
-      <c r="M2" s="105"/>
-      <c r="N2" s="105"/>
-      <c r="O2" s="105"/>
-      <c r="P2" s="105"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="109"/>
+      <c r="M2" s="109"/>
+      <c r="N2" s="109"/>
+      <c r="O2" s="109"/>
+      <c r="P2" s="109"/>
     </row>
     <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.5">
-      <c r="B6" s="98" t="s">
+      <c r="B6" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="C6" s="104" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="91" t="s">
@@ -5880,7 +5986,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="102" t="s">
+      <c r="F6" s="106" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5889,7 +5995,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="102" t="s">
+      <c r="I6" s="106" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="60" t="s">
@@ -5898,7 +6004,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="102" t="s">
+      <c r="L6" s="112" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="43">
@@ -5910,50 +6016,50 @@
       <c r="O6" s="43">
         <v>46167</v>
       </c>
-      <c r="P6" s="102" t="s">
+      <c r="P6" s="106" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B7" s="99"/>
-      <c r="C7" s="101"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="105"/>
       <c r="D7" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="108" t="s">
+      <c r="E7" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="103"/>
-      <c r="G7" s="59" t="s">
+      <c r="F7" s="107"/>
+      <c r="G7" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="108" t="s">
+      <c r="H7" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="103"/>
-      <c r="J7" s="59" t="s">
+      <c r="I7" s="107"/>
+      <c r="J7" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="108" t="s">
+      <c r="K7" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="103"/>
-      <c r="M7" s="110" t="s">
+      <c r="L7" s="113"/>
+      <c r="M7" s="98" t="s">
         <v>201</v>
       </c>
-      <c r="N7" s="59" t="s">
+      <c r="N7" s="91" t="s">
         <v>10</v>
       </c>
       <c r="O7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="103"/>
-    </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="P7" s="107"/>
+    </row>
+    <row r="8" spans="2:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="81" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="106" t="s">
+      <c r="C8" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D8" s="24"/>
@@ -5966,18 +6072,18 @@
       <c r="G8" s="24"/>
       <c r="I8" s="92"/>
       <c r="J8" s="24"/>
-      <c r="L8" s="80"/>
-      <c r="M8" s="111" t="s">
-        <v>279</v>
-      </c>
-      <c r="N8" s="80"/>
+      <c r="L8" s="94"/>
+      <c r="M8" s="110" t="s">
+        <v>278</v>
+      </c>
+      <c r="N8"/>
       <c r="P8" s="92"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B9" s="81" t="s">
         <v>256</v>
       </c>
-      <c r="C9" s="106" t="s">
+      <c r="C9" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D9" s="24">
@@ -5990,16 +6096,16 @@
       <c r="G9" s="24"/>
       <c r="I9" s="92"/>
       <c r="J9" s="24"/>
-      <c r="L9" s="80"/>
-      <c r="M9" s="112"/>
-      <c r="N9" s="80"/>
+      <c r="L9" s="94"/>
+      <c r="M9" s="111"/>
+      <c r="N9"/>
       <c r="P9" s="92"/>
     </row>
     <row r="10" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B10" s="81" t="s">
         <v>245</v>
       </c>
-      <c r="C10" s="106" t="s">
+      <c r="C10" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D10" s="24">
@@ -6012,16 +6118,16 @@
       <c r="G10" s="24"/>
       <c r="I10" s="92"/>
       <c r="J10" s="24"/>
-      <c r="L10" s="80"/>
-      <c r="M10" s="112"/>
-      <c r="N10" s="80"/>
+      <c r="L10" s="94"/>
+      <c r="M10" s="111"/>
+      <c r="N10"/>
       <c r="P10" s="92"/>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B11" s="81" t="s">
         <v>244</v>
       </c>
-      <c r="C11" s="106" t="s">
+      <c r="C11" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D11" s="24">
@@ -6034,16 +6140,16 @@
       <c r="G11" s="24"/>
       <c r="I11" s="92"/>
       <c r="J11" s="24"/>
-      <c r="L11" s="80"/>
-      <c r="M11" s="112"/>
-      <c r="N11" s="80"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="111"/>
+      <c r="N11"/>
       <c r="P11" s="92"/>
     </row>
     <row r="12" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B12" s="81" t="s">
         <v>257</v>
       </c>
-      <c r="C12" s="106" t="s">
+      <c r="C12" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D12" s="80">
@@ -6056,16 +6162,16 @@
       <c r="G12" s="24"/>
       <c r="I12" s="92"/>
       <c r="J12" s="24"/>
-      <c r="L12" s="80"/>
-      <c r="M12" s="112"/>
-      <c r="N12" s="80"/>
+      <c r="L12" s="94"/>
+      <c r="M12" s="111"/>
+      <c r="N12"/>
       <c r="P12" s="92"/>
     </row>
     <row r="13" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
-      <c r="C13" s="106" t="s">
+      <c r="C13" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D13" s="80">
@@ -6078,16 +6184,16 @@
       <c r="G13" s="24"/>
       <c r="I13" s="92"/>
       <c r="J13" s="24"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="112"/>
-      <c r="N13" s="80"/>
+      <c r="L13" s="94"/>
+      <c r="M13" s="111"/>
+      <c r="N13"/>
       <c r="P13" s="92"/>
     </row>
     <row r="14" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
-      <c r="C14" s="106" t="s">
+      <c r="C14" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D14" s="80">
@@ -6100,16 +6206,16 @@
       <c r="G14" s="24"/>
       <c r="I14" s="92"/>
       <c r="J14" s="24"/>
-      <c r="L14" s="80"/>
-      <c r="M14" s="112"/>
-      <c r="N14" s="80"/>
+      <c r="L14" s="94"/>
+      <c r="M14" s="111"/>
+      <c r="N14"/>
       <c r="P14" s="92"/>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
-      <c r="C15" s="106" t="s">
+      <c r="C15" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D15" s="80">
@@ -6122,16 +6228,16 @@
       <c r="G15" s="24"/>
       <c r="I15" s="92"/>
       <c r="J15" s="24"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="112"/>
-      <c r="N15" s="80"/>
+      <c r="L15" s="94"/>
+      <c r="M15" s="111"/>
+      <c r="N15"/>
       <c r="P15" s="92"/>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
-      <c r="C16" s="106" t="s">
+      <c r="C16" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D16" s="80">
@@ -6144,16 +6250,16 @@
       <c r="G16" s="24"/>
       <c r="I16" s="92"/>
       <c r="J16" s="24"/>
-      <c r="L16" s="80"/>
-      <c r="M16" s="112"/>
-      <c r="N16" s="80"/>
+      <c r="L16" s="94"/>
+      <c r="M16" s="111"/>
+      <c r="N16"/>
       <c r="P16" s="92"/>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
-      <c r="C17" s="106" t="s">
+      <c r="C17" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D17" s="80"/>
@@ -6166,16 +6272,16 @@
       </c>
       <c r="I17" s="92"/>
       <c r="J17" s="24"/>
-      <c r="L17" s="80"/>
-      <c r="M17" s="112"/>
-      <c r="N17" s="80"/>
+      <c r="L17" s="94"/>
+      <c r="M17" s="111"/>
+      <c r="N17"/>
       <c r="P17" s="92"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
-      <c r="C18" s="106" t="s">
+      <c r="C18" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D18" s="80"/>
@@ -6188,16 +6294,16 @@
       </c>
       <c r="I18" s="92"/>
       <c r="J18" s="24"/>
-      <c r="L18" s="80"/>
-      <c r="M18" s="112"/>
-      <c r="N18" s="80"/>
+      <c r="L18" s="94"/>
+      <c r="M18" s="111"/>
+      <c r="N18"/>
       <c r="P18" s="92"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
-      <c r="C19" s="106" t="s">
+      <c r="C19" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D19" s="80"/>
@@ -6210,16 +6316,16 @@
       </c>
       <c r="I19" s="92"/>
       <c r="J19" s="24"/>
-      <c r="L19" s="80"/>
-      <c r="M19" s="112"/>
-      <c r="N19" s="80"/>
+      <c r="L19" s="94"/>
+      <c r="M19" s="111"/>
+      <c r="N19"/>
       <c r="P19" s="92"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
-      <c r="C20" s="106" t="s">
+      <c r="C20" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D20" s="80"/>
@@ -6232,16 +6338,16 @@
       </c>
       <c r="I20" s="92"/>
       <c r="J20" s="24"/>
-      <c r="L20" s="80"/>
-      <c r="M20" s="112"/>
-      <c r="N20" s="80"/>
+      <c r="L20" s="94"/>
+      <c r="M20" s="111"/>
+      <c r="N20"/>
       <c r="P20" s="92"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
-      <c r="C21" s="106" t="s">
+      <c r="C21" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D21" s="80"/>
@@ -6254,16 +6360,16 @@
       </c>
       <c r="I21" s="92"/>
       <c r="J21" s="24"/>
-      <c r="L21" s="80"/>
-      <c r="M21" s="112"/>
-      <c r="N21" s="80"/>
+      <c r="L21" s="94"/>
+      <c r="M21" s="111"/>
+      <c r="N21"/>
       <c r="P21" s="92"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B22" s="81" t="s">
         <v>255</v>
       </c>
-      <c r="C22" s="106" t="s">
+      <c r="C22" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D22" s="80"/>
@@ -6276,16 +6382,16 @@
       </c>
       <c r="I22" s="92"/>
       <c r="J22" s="24"/>
-      <c r="L22" s="80"/>
-      <c r="M22" s="112"/>
-      <c r="N22" s="80"/>
+      <c r="L22" s="94"/>
+      <c r="M22" s="111"/>
+      <c r="N22"/>
       <c r="P22" s="92"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B23" s="82" t="s">
         <v>258</v>
       </c>
-      <c r="C23" s="106" t="s">
+      <c r="C23" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D23" s="24"/>
@@ -6298,16 +6404,16 @@
       </c>
       <c r="I23" s="92"/>
       <c r="J23" s="24"/>
-      <c r="L23" s="80"/>
-      <c r="M23" s="112"/>
-      <c r="N23" s="80"/>
+      <c r="L23" s="94"/>
+      <c r="M23" s="111"/>
+      <c r="N23"/>
       <c r="P23" s="92"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B24" s="82" t="s">
         <v>259</v>
       </c>
-      <c r="C24" s="106" t="s">
+      <c r="C24" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D24" s="24"/>
@@ -6315,16 +6421,16 @@
       <c r="G24" s="24"/>
       <c r="I24" s="92"/>
       <c r="J24" s="24"/>
-      <c r="L24" s="80"/>
-      <c r="M24" s="112"/>
-      <c r="N24" s="80"/>
+      <c r="L24" s="94"/>
+      <c r="M24" s="111"/>
+      <c r="N24"/>
       <c r="P24" s="92"/>
     </row>
     <row r="25" spans="2:16" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="83" t="s">
         <v>260</v>
       </c>
-      <c r="C25" s="106" t="s">
+      <c r="C25" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D25" s="24"/>
@@ -6337,16 +6443,16 @@
       <c r="K25" s="31">
         <v>100</v>
       </c>
-      <c r="L25" s="80"/>
-      <c r="M25" s="112"/>
-      <c r="N25" s="80"/>
+      <c r="L25" s="94"/>
+      <c r="M25" s="111"/>
+      <c r="N25"/>
       <c r="P25" s="92"/>
     </row>
     <row r="26" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B26" s="83" t="s">
         <v>261</v>
       </c>
-      <c r="C26" s="106" t="s">
+      <c r="C26" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D26" s="24"/>
@@ -6359,16 +6465,16 @@
       <c r="K26" s="31">
         <v>100</v>
       </c>
-      <c r="L26" s="80"/>
-      <c r="M26" s="112"/>
-      <c r="N26" s="80"/>
+      <c r="L26" s="94"/>
+      <c r="M26" s="111"/>
+      <c r="N26"/>
       <c r="P26" s="92"/>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B27" s="83" t="s">
         <v>262</v>
       </c>
-      <c r="C27" s="106" t="s">
+      <c r="C27" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D27" s="24"/>
@@ -6381,16 +6487,16 @@
       <c r="K27" s="31">
         <v>100</v>
       </c>
-      <c r="L27" s="80"/>
-      <c r="M27" s="112"/>
-      <c r="N27" s="80"/>
+      <c r="L27" s="94"/>
+      <c r="M27" s="111"/>
+      <c r="N27"/>
       <c r="P27" s="92"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B28" s="83" t="s">
         <v>263</v>
       </c>
-      <c r="C28" s="106" t="s">
+      <c r="C28" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D28" s="24"/>
@@ -6403,16 +6509,16 @@
       <c r="K28" s="31">
         <v>100</v>
       </c>
-      <c r="L28" s="80"/>
-      <c r="M28" s="112"/>
-      <c r="N28" s="80"/>
+      <c r="L28" s="94"/>
+      <c r="M28" s="111"/>
+      <c r="N28"/>
       <c r="P28" s="92"/>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B29" s="83" t="s">
         <v>264</v>
       </c>
-      <c r="C29" s="106" t="s">
+      <c r="C29" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D29" s="24"/>
@@ -6425,16 +6531,16 @@
       <c r="K29" s="31">
         <v>100</v>
       </c>
-      <c r="L29" s="80"/>
-      <c r="M29" s="112"/>
-      <c r="N29" s="80"/>
+      <c r="L29" s="94"/>
+      <c r="M29" s="111"/>
+      <c r="N29"/>
       <c r="P29" s="92"/>
     </row>
     <row r="30" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B30" s="83" t="s">
         <v>265</v>
       </c>
-      <c r="C30" s="106" t="s">
+      <c r="C30" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D30" s="24"/>
@@ -6447,16 +6553,16 @@
       <c r="K30" s="31">
         <v>100</v>
       </c>
-      <c r="L30" s="80"/>
-      <c r="M30" s="112"/>
-      <c r="N30" s="80"/>
+      <c r="L30" s="94"/>
+      <c r="M30" s="111"/>
+      <c r="N30"/>
       <c r="P30" s="92"/>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B31" s="83" t="s">
-        <v>281</v>
-      </c>
-      <c r="C31" s="106" t="s">
+        <v>280</v>
+      </c>
+      <c r="C31" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D31" s="24"/>
@@ -6464,9 +6570,9 @@
       <c r="G31" s="24"/>
       <c r="I31" s="92"/>
       <c r="J31" s="24"/>
-      <c r="L31" s="80"/>
-      <c r="M31" s="112"/>
-      <c r="N31" s="80">
+      <c r="L31" s="94"/>
+      <c r="M31" s="111"/>
+      <c r="N31">
         <v>2</v>
       </c>
       <c r="O31" s="31">
@@ -6476,9 +6582,9 @@
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B32" s="83" t="s">
-        <v>280</v>
-      </c>
-      <c r="C32" s="106" t="s">
+        <v>279</v>
+      </c>
+      <c r="C32" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D32" s="24"/>
@@ -6486,9 +6592,9 @@
       <c r="G32" s="24"/>
       <c r="I32" s="92"/>
       <c r="J32" s="24"/>
-      <c r="L32" s="80"/>
-      <c r="M32" s="112"/>
-      <c r="N32" s="80">
+      <c r="L32" s="94"/>
+      <c r="M32" s="111"/>
+      <c r="N32">
         <v>1</v>
       </c>
       <c r="O32" s="31">
@@ -6498,9 +6604,9 @@
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B33" s="83" t="s">
-        <v>282</v>
-      </c>
-      <c r="C33" s="106" t="s">
+        <v>281</v>
+      </c>
+      <c r="C33" s="95" t="s">
         <v>102</v>
       </c>
       <c r="D33" s="24"/>
@@ -6508,9 +6614,9 @@
       <c r="G33" s="24"/>
       <c r="I33" s="92"/>
       <c r="J33" s="24"/>
-      <c r="L33" s="80"/>
-      <c r="M33" s="112"/>
-      <c r="N33" s="80">
+      <c r="L33" s="94"/>
+      <c r="M33" s="111"/>
+      <c r="N33">
         <v>2</v>
       </c>
       <c r="O33" s="31">
@@ -6522,7 +6628,7 @@
       <c r="B34" s="29" t="s">
         <v>215</v>
       </c>
-      <c r="C34" s="106" t="s">
+      <c r="C34" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D34" s="24">
@@ -6542,16 +6648,16 @@
       </c>
       <c r="I34" s="92"/>
       <c r="J34" s="24"/>
-      <c r="L34" s="80"/>
-      <c r="M34" s="112"/>
-      <c r="N34" s="80"/>
+      <c r="L34" s="94"/>
+      <c r="M34" s="111"/>
+      <c r="N34"/>
       <c r="P34" s="92"/>
     </row>
     <row r="35" spans="2:16" ht="29" x14ac:dyDescent="0.35">
       <c r="B35" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="C35" s="106" t="s">
+      <c r="C35" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D35" s="24">
@@ -6565,17 +6671,22 @@
       </c>
       <c r="G35" s="24"/>
       <c r="I35" s="92"/>
-      <c r="J35" s="24"/>
-      <c r="L35" s="80"/>
-      <c r="M35" s="112"/>
-      <c r="N35" s="80"/>
+      <c r="J35" s="24">
+        <v>4</v>
+      </c>
+      <c r="K35" s="31">
+        <v>100</v>
+      </c>
+      <c r="L35" s="94"/>
+      <c r="M35" s="111"/>
+      <c r="N35"/>
       <c r="P35" s="92"/>
     </row>
     <row r="36" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
         <v>217</v>
       </c>
-      <c r="C36" s="106" t="s">
+      <c r="C36" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D36" s="24">
@@ -6588,16 +6699,16 @@
       <c r="G36" s="24"/>
       <c r="I36" s="92"/>
       <c r="J36" s="24"/>
-      <c r="L36" s="80"/>
-      <c r="M36" s="112"/>
-      <c r="N36" s="80"/>
+      <c r="L36" s="94"/>
+      <c r="M36" s="111"/>
+      <c r="N36"/>
       <c r="P36" s="92"/>
     </row>
     <row r="37" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
         <v>218</v>
       </c>
-      <c r="C37" s="106" t="s">
+      <c r="C37" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D37" s="24">
@@ -6610,16 +6721,16 @@
       <c r="G37" s="24"/>
       <c r="I37" s="92"/>
       <c r="J37" s="24"/>
-      <c r="L37" s="80"/>
-      <c r="M37" s="112"/>
-      <c r="N37" s="80"/>
+      <c r="L37" s="94"/>
+      <c r="M37" s="111"/>
+      <c r="N37"/>
       <c r="P37" s="92"/>
     </row>
-    <row r="38" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" ht="58" x14ac:dyDescent="0.35">
       <c r="B38" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="C38" s="106" t="s">
+      <c r="C38" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D38" s="24">
@@ -6640,17 +6751,24 @@
       <c r="I38" s="94" t="s">
         <v>270</v>
       </c>
-      <c r="J38" s="24"/>
-      <c r="L38" s="80"/>
-      <c r="M38" s="112"/>
-      <c r="N38" s="80"/>
+      <c r="J38" s="24">
+        <v>1</v>
+      </c>
+      <c r="K38" s="31">
+        <v>100</v>
+      </c>
+      <c r="L38" s="94" t="s">
+        <v>282</v>
+      </c>
+      <c r="M38" s="111"/>
+      <c r="N38"/>
       <c r="P38" s="92"/>
     </row>
     <row r="39" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B39" s="29" t="s">
         <v>221</v>
       </c>
-      <c r="C39" s="106" t="s">
+      <c r="C39" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D39" s="24"/>
@@ -6663,16 +6781,16 @@
       </c>
       <c r="I39" s="92"/>
       <c r="J39" s="24"/>
-      <c r="L39" s="80"/>
-      <c r="M39" s="112"/>
-      <c r="N39" s="80"/>
+      <c r="L39" s="94"/>
+      <c r="M39" s="111"/>
+      <c r="N39"/>
       <c r="P39" s="92"/>
     </row>
     <row r="40" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B40" s="90" t="s">
         <v>266</v>
       </c>
-      <c r="C40" s="107" t="s">
+      <c r="C40" s="96" t="s">
         <v>103</v>
       </c>
       <c r="G40" s="24">
@@ -6685,15 +6803,16 @@
         <v>269</v>
       </c>
       <c r="J40" s="24"/>
-      <c r="M40" s="112"/>
-      <c r="N40" s="80"/>
+      <c r="L40" s="94"/>
+      <c r="M40" s="111"/>
+      <c r="N40"/>
       <c r="P40" s="92"/>
     </row>
     <row r="41" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B41" s="90" t="s">
         <v>267</v>
       </c>
-      <c r="C41" s="107" t="s">
+      <c r="C41" s="96" t="s">
         <v>103</v>
       </c>
       <c r="G41" s="24"/>
@@ -6703,15 +6822,16 @@
       <c r="K41" s="31">
         <v>100</v>
       </c>
-      <c r="M41" s="112"/>
-      <c r="N41" s="80"/>
+      <c r="L41" s="94"/>
+      <c r="M41" s="111"/>
+      <c r="N41"/>
       <c r="P41" s="92"/>
     </row>
     <row r="42" spans="2:16" ht="159.5" x14ac:dyDescent="0.35">
       <c r="B42" s="90" t="s">
         <v>268</v>
       </c>
-      <c r="C42" s="107" t="s">
+      <c r="C42" s="96" t="s">
         <v>103</v>
       </c>
       <c r="G42" s="24"/>
@@ -6721,18 +6841,18 @@
       <c r="K42" s="31">
         <v>90</v>
       </c>
-      <c r="L42" s="93" t="s">
+      <c r="L42" s="94" t="s">
         <v>275</v>
       </c>
-      <c r="M42" s="112"/>
-      <c r="N42" s="80"/>
+      <c r="M42" s="111"/>
+      <c r="N42"/>
       <c r="P42" s="92"/>
     </row>
     <row r="43" spans="2:16" ht="58" x14ac:dyDescent="0.35">
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="90" t="s">
         <v>239</v>
       </c>
-      <c r="C43" s="106" t="s">
+      <c r="C43" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D43" s="24"/>
@@ -6745,18 +6865,18 @@
       <c r="K43" s="31">
         <v>100</v>
       </c>
-      <c r="L43" s="109" t="s">
+      <c r="L43" s="94" t="s">
         <v>274</v>
       </c>
-      <c r="M43" s="112"/>
-      <c r="N43" s="80"/>
+      <c r="M43" s="111"/>
+      <c r="N43"/>
       <c r="P43" s="92"/>
     </row>
     <row r="44" spans="2:16" x14ac:dyDescent="0.35">
       <c r="B44" s="90" t="s">
         <v>276</v>
       </c>
-      <c r="C44" s="107" t="s">
+      <c r="C44" s="96" t="s">
         <v>103</v>
       </c>
       <c r="D44" s="31">
@@ -6777,25 +6897,104 @@
       <c r="K44" s="31">
         <v>50</v>
       </c>
-      <c r="M44" s="112"/>
-      <c r="N44" s="80"/>
+      <c r="L44" s="94"/>
+      <c r="M44" s="111"/>
+      <c r="N44">
+        <v>4</v>
+      </c>
+      <c r="O44" s="31">
+        <v>75</v>
+      </c>
       <c r="P44" s="92"/>
     </row>
-    <row r="45" spans="2:16" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B45" s="90" t="s">
         <v>277</v>
       </c>
-      <c r="J45" s="31">
+      <c r="C45" s="95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D45" s="24"/>
+      <c r="F45" s="92"/>
+      <c r="G45" s="24"/>
+      <c r="I45" s="92"/>
+      <c r="J45" s="24">
         <v>1</v>
       </c>
-      <c r="L45" s="93" t="s">
-        <v>278</v>
-      </c>
-      <c r="M45" s="113"/>
+      <c r="K45" s="31">
+        <v>75</v>
+      </c>
+      <c r="L45" s="94" t="s">
+        <v>283</v>
+      </c>
+      <c r="M45" s="111"/>
+      <c r="N45"/>
+      <c r="P45" s="92"/>
+    </row>
+    <row r="46" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="B46" s="90" t="s">
+        <v>287</v>
+      </c>
+      <c r="C46" s="95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D46" s="24"/>
+      <c r="F46" s="92"/>
+      <c r="G46" s="24"/>
+      <c r="I46" s="92"/>
+      <c r="J46" s="24"/>
+      <c r="L46" s="94"/>
+      <c r="M46" s="111"/>
+      <c r="N46">
+        <v>0.5</v>
+      </c>
+      <c r="O46" s="31">
+        <v>75</v>
+      </c>
+      <c r="P46" s="94" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
+      <c r="B47" s="81" t="s">
+        <v>284</v>
+      </c>
+      <c r="C47" s="95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D47" s="24"/>
+      <c r="F47" s="92"/>
+      <c r="G47" s="24"/>
+      <c r="I47" s="92"/>
+      <c r="J47" s="24"/>
+      <c r="L47" s="94"/>
+      <c r="M47" s="111"/>
+      <c r="N47">
+        <v>1</v>
+      </c>
+      <c r="O47" s="31">
+        <v>100</v>
+      </c>
+      <c r="P47" s="92"/>
+    </row>
+    <row r="48" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B48" s="90" t="s">
+        <v>288</v>
+      </c>
+      <c r="C48" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="F48" s="92"/>
+      <c r="I48" s="92"/>
+      <c r="L48" s="94"/>
+      <c r="M48" s="111"/>
+      <c r="N48"/>
+      <c r="P48" s="94" t="s">
+        <v>285</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="M8:M45"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="B6:B7"/>
@@ -6803,217 +7002,234 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
+    <mergeCell ref="M8:M48"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B6:B7 B23:B45">
-    <cfRule type="expression" dxfId="47" priority="27">
+  <conditionalFormatting sqref="B2 B6:B7 B23:B41">
+    <cfRule type="expression" dxfId="62" priority="38">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C44">
-    <cfRule type="expression" dxfId="46" priority="16">
+    <cfRule type="expression" dxfId="61" priority="27">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="17">
+    <cfRule type="expression" dxfId="60" priority="28">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="18">
+    <cfRule type="expression" dxfId="59" priority="29">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8 B23:B24">
-    <cfRule type="expression" dxfId="43" priority="230">
+    <cfRule type="expression" dxfId="58" priority="241">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14 B32:B33">
-    <cfRule type="expression" dxfId="42" priority="232">
+    <cfRule type="expression" dxfId="57" priority="243">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="41" priority="248">
+    <cfRule type="expression" dxfId="56" priority="259">
       <formula>MAX($E34,$H34,$K34)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="40" priority="269">
+    <cfRule type="expression" dxfId="55" priority="280">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B12">
-    <cfRule type="expression" dxfId="39" priority="3">
+    <cfRule type="expression" dxfId="54" priority="14">
       <formula>MAX($E17,$H17,$K17)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B33">
-    <cfRule type="expression" dxfId="38" priority="1">
+    <cfRule type="expression" dxfId="53" priority="12">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:B16">
-    <cfRule type="expression" dxfId="37" priority="318">
+    <cfRule type="expression" dxfId="52" priority="329">
       <formula>MAX($E34,$H34,$K34)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="36" priority="349">
+    <cfRule type="expression" dxfId="51" priority="360">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="350">
+    <cfRule type="expression" dxfId="50" priority="361">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14 B16:B18">
-    <cfRule type="expression" dxfId="34" priority="355">
+    <cfRule type="expression" dxfId="49" priority="366">
       <formula>MAX($E36,$H36,$K36)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:B19">
-    <cfRule type="expression" dxfId="33" priority="356">
+    <cfRule type="expression" dxfId="48" priority="367">
       <formula>MAX($E36,$H36,$K36)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:B21">
-    <cfRule type="expression" dxfId="32" priority="388">
+    <cfRule type="expression" dxfId="47" priority="399">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="31" priority="437">
+    <cfRule type="expression" dxfId="46" priority="448">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="438">
+    <cfRule type="expression" dxfId="45" priority="449">
       <formula>MAX($E4,$H4,$K4)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="expression" dxfId="29" priority="497">
+    <cfRule type="expression" dxfId="44" priority="508">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="expression" dxfId="28" priority="502">
+    <cfRule type="expression" dxfId="43" priority="513">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B31">
-    <cfRule type="expression" dxfId="27" priority="510">
+    <cfRule type="expression" dxfId="42" priority="521">
       <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="511">
+    <cfRule type="expression" dxfId="41" priority="522">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="expression" dxfId="25" priority="520">
+    <cfRule type="expression" dxfId="40" priority="531">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="521">
+    <cfRule type="expression" dxfId="39" priority="532">
       <formula>MAX($E16,$H16,$K16)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="23" priority="531">
+    <cfRule type="expression" dxfId="38" priority="542">
       <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="expression" dxfId="22" priority="533">
+    <cfRule type="expression" dxfId="37" priority="544">
       <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12 B16">
-    <cfRule type="expression" dxfId="21" priority="538">
+    <cfRule type="expression" dxfId="36" priority="549">
       <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="539">
+    <cfRule type="expression" dxfId="35" priority="550">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25 B27:B29">
-    <cfRule type="expression" dxfId="19" priority="581">
+    <cfRule type="expression" dxfId="34" priority="592">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="582">
+    <cfRule type="expression" dxfId="33" priority="593">
       <formula>MAX($E38,$H38,$K38)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="17" priority="592">
+    <cfRule type="expression" dxfId="32" priority="603">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23">
-    <cfRule type="expression" dxfId="16" priority="598">
+    <cfRule type="expression" dxfId="31" priority="609">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:B24">
-    <cfRule type="expression" dxfId="15" priority="608">
+    <cfRule type="expression" dxfId="30" priority="619">
       <formula>MAX($E44,$H44,$K44)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24 B27">
-    <cfRule type="expression" dxfId="14" priority="610">
+    <cfRule type="expression" dxfId="29" priority="621">
       <formula>MAX($E40,$H40,$K40)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20 B22">
-    <cfRule type="expression" dxfId="13" priority="618">
+    <cfRule type="expression" dxfId="28" priority="629">
       <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="619">
+    <cfRule type="expression" dxfId="27" priority="630">
       <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="expression" dxfId="11" priority="622">
+    <cfRule type="expression" dxfId="26" priority="633">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26">
-    <cfRule type="expression" dxfId="10" priority="623">
+    <cfRule type="expression" dxfId="25" priority="634">
       <formula>MAX($E10,$H10,$K10)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="624">
+    <cfRule type="expression" dxfId="24" priority="635">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:B15 B17:B19">
-    <cfRule type="expression" dxfId="8" priority="655">
+    <cfRule type="expression" dxfId="23" priority="666">
       <formula>MAX($E36,$H36,$K36)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="656">
+    <cfRule type="expression" dxfId="22" priority="667">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:B26 B28:B31">
-    <cfRule type="expression" dxfId="6" priority="659">
+    <cfRule type="expression" dxfId="21" priority="670">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:B33">
-    <cfRule type="expression" dxfId="5" priority="666">
+    <cfRule type="expression" dxfId="20" priority="677">
       <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="667">
+    <cfRule type="expression" dxfId="19" priority="678">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:B11">
-    <cfRule type="expression" dxfId="3" priority="679">
+    <cfRule type="expression" dxfId="18" priority="690">
       <formula>MAX($E34,$H34,$K34)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="680">
+    <cfRule type="expression" dxfId="17" priority="691">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B24">
-    <cfRule type="expression" dxfId="1" priority="681">
+    <cfRule type="expression" dxfId="16" priority="692">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="682">
+    <cfRule type="expression" dxfId="15" priority="693">
       <formula>MAX($E40,$H40,$K40)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C45:C47">
+    <cfRule type="expression" dxfId="11" priority="2">
+      <formula>$C45="Charlotte/Eddy"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="3">
+      <formula>$C45="Charlotte"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="4">
+      <formula>$C45="Eddy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B41:B48">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>MAX($E41,$H41,$K41)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Plusieurs fix interface + refont systeme de notifications
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82D00F7-D4AB-41A5-AAF9-EA7341C98BD1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7D17FC-1F75-4E49-AE89-4DBBCD22DDF1}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,17 +27,22 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="292">
   <si>
     <t>Planification globale</t>
   </si>
@@ -906,6 +911,15 @@
   </si>
   <si>
     <t>Debug reccomencer un jeu quand on vient d'en finir un</t>
+  </si>
+  <si>
+    <t>Ajout une page option avec les niveaux de l ia</t>
+  </si>
+  <si>
+    <t>Refonte du système de notification avec retour mouvement valide</t>
+  </si>
+  <si>
+    <t>Divers fix aspect interface</t>
   </si>
 </sst>
 </file>
@@ -1710,146 +1724,28 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="86">
+  <dxfs count="76">
     <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -1892,6 +1788,39 @@
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -2684,26 +2613,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" customWidth="1"/>
-    <col min="4" max="4" width="15.81640625" customWidth="1"/>
-    <col min="5" max="5" width="42.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" customWidth="1"/>
+    <col min="5" max="5" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="47" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2717,7 +2646,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2731,7 +2660,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2745,7 +2674,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2759,7 +2688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2773,7 +2702,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2787,7 +2716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2801,7 +2730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2815,7 +2744,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2829,7 +2758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2843,7 +2772,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2857,7 +2786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2871,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2885,7 +2814,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2899,7 +2828,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2913,7 +2842,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2927,7 +2856,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2941,7 +2870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2955,7 +2884,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2969,7 +2898,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2983,7 +2912,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2997,7 +2926,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -3011,7 +2940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -3025,7 +2954,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -3039,7 +2968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -3053,7 +2982,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -3067,7 +2996,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -3081,7 +3010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -3095,7 +3024,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -3109,7 +3038,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -3123,7 +3052,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -3137,7 +3066,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -3151,7 +3080,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -3165,8 +3094,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -3178,7 +3107,7 @@
   </sheetData>
   <autoFilter ref="B5:E37" xr:uid="{93133217-C8F5-4788-AEEB-7509B70AEF5D}"/>
   <conditionalFormatting sqref="B6:B7">
-    <cfRule type="expression" dxfId="85" priority="1">
+    <cfRule type="expression" dxfId="75" priority="1">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3201,32 +3130,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="27.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
-    <col min="5" max="5" width="19.81640625" customWidth="1"/>
-    <col min="6" max="6" width="18.81640625" customWidth="1"/>
-    <col min="7" max="7" width="9.81640625" customWidth="1"/>
-    <col min="8" max="8" width="16.1796875" customWidth="1"/>
-    <col min="9" max="9" width="18.81640625" customWidth="1"/>
-    <col min="10" max="10" width="9.54296875" customWidth="1"/>
-    <col min="11" max="11" width="16.1796875" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
-    <col min="15" max="15" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="18.77734375" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.21875" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -3256,7 +3185,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -3310,7 +3239,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -3337,7 +3266,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -3359,7 +3288,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -3386,7 +3315,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -3419,7 +3348,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -3456,7 +3385,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -3493,7 +3422,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -3525,7 +3454,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3553,7 +3482,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3580,15 +3509,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.35">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3604,24 +3533,24 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" customWidth="1"/>
-    <col min="2" max="2" width="77.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.54296875" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.81640625" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B3" s="99" t="s">
         <v>6</v>
       </c>
@@ -3636,8 +3565,8 @@
       <c r="K3" s="100"/>
       <c r="L3" s="101"/>
     </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
       <c r="B5" s="102" t="s">
         <v>1</v>
       </c>
@@ -3672,7 +3601,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B6" s="103"/>
       <c r="C6" s="105"/>
       <c r="D6" s="42" t="s">
@@ -3697,7 +3626,7 @@
       </c>
       <c r="L6" s="107"/>
     </row>
-    <row r="7" spans="2:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3720,7 +3649,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3739,7 +3668,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3758,7 +3687,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3777,7 +3706,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3796,7 +3725,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3815,7 +3744,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3834,7 +3763,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3853,7 +3782,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3872,7 +3801,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3891,7 +3820,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3910,7 +3839,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3929,7 +3858,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3948,7 +3877,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3967,7 +3896,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3988,7 +3917,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -4007,7 +3936,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -4028,7 +3957,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -4047,7 +3976,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -4066,7 +3995,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -4087,7 +4016,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -4108,7 +4037,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -4129,7 +4058,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -4148,7 +4077,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -4167,7 +4096,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -4186,7 +4115,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -4205,7 +4134,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -4224,7 +4153,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -4243,7 +4172,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -4262,7 +4191,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -4281,7 +4210,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -4300,7 +4229,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -4319,7 +4248,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -4338,7 +4267,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -4357,7 +4286,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -4376,7 +4305,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -4395,7 +4324,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -4414,7 +4343,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -4433,7 +4362,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -4452,7 +4381,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -4471,7 +4400,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -4490,7 +4419,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -4520,67 +4449,67 @@
     <mergeCell ref="L5:L6"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B43">
-    <cfRule type="expression" dxfId="84" priority="7">
+    <cfRule type="expression" dxfId="74" priority="7">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B42">
-    <cfRule type="expression" dxfId="83" priority="1">
+    <cfRule type="expression" dxfId="73" priority="1">
       <formula>MAX($E30,$K30,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="expression" dxfId="82" priority="32">
+    <cfRule type="expression" dxfId="72" priority="32">
       <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="38">
+    <cfRule type="expression" dxfId="71" priority="38">
       <formula>MAX($E46,$K46,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45 B47:B48">
-    <cfRule type="expression" dxfId="80" priority="30">
+    <cfRule type="expression" dxfId="70" priority="30">
       <formula>MAX($E45,$K45,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45:B1048576">
-    <cfRule type="expression" dxfId="79" priority="6">
+    <cfRule type="expression" dxfId="69" priority="6">
       <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C45">
-    <cfRule type="expression" dxfId="78" priority="25">
+    <cfRule type="expression" dxfId="68" priority="25">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="27">
+    <cfRule type="expression" dxfId="67" priority="27">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="76" priority="8">
+    <cfRule type="expression" dxfId="66" priority="8">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42:C1048576">
-    <cfRule type="expression" dxfId="75" priority="13">
+    <cfRule type="expression" dxfId="65" priority="13">
       <formula>$C42="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="14">
+    <cfRule type="expression" dxfId="64" priority="14">
       <formula>$C42="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C47">
-    <cfRule type="expression" dxfId="73" priority="20">
+    <cfRule type="expression" dxfId="63" priority="20">
       <formula>$C47="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="21">
+    <cfRule type="expression" dxfId="62" priority="21">
       <formula>$C47="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C48">
-    <cfRule type="expression" dxfId="71" priority="9">
+    <cfRule type="expression" dxfId="61" priority="9">
       <formula>$C48="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="10">
+    <cfRule type="expression" dxfId="60" priority="10">
       <formula>$C48="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4595,23 +4524,23 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="21.81640625" customWidth="1"/>
-    <col min="5" max="5" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1796875" customWidth="1"/>
+    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.81640625" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.77734375" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.453125" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.5" thickBot="1" x14ac:dyDescent="1.05">
+    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B1" s="99" t="s">
         <v>16</v>
       </c>
@@ -4626,8 +4555,8 @@
       <c r="K1" s="100"/>
       <c r="L1" s="101"/>
     </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
       <c r="B4" s="102" t="s">
         <v>1</v>
       </c>
@@ -4662,7 +4591,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B5" s="103"/>
       <c r="C5" s="105"/>
       <c r="D5" s="42" t="s">
@@ -4687,7 +4616,7 @@
       </c>
       <c r="L5" s="107"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4705,7 +4634,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4723,7 +4652,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4741,7 +4670,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4759,7 +4688,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4777,7 +4706,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4795,7 +4724,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4813,7 +4742,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4831,7 +4760,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4849,7 +4778,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4867,7 +4796,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4885,7 +4814,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4903,7 +4832,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4921,7 +4850,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4939,7 +4868,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4958,7 +4887,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4977,7 +4906,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4996,7 +4925,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -5015,7 +4944,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -5034,7 +4963,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -5053,7 +4982,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -5072,7 +5001,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -5091,7 +5020,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -5110,7 +5039,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -5129,7 +5058,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -5148,7 +5077,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -5167,7 +5096,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -5186,7 +5115,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -5205,7 +5134,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -5226,7 +5155,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -5246,7 +5175,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -5266,7 +5195,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -5286,7 +5215,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -5306,7 +5235,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -5326,7 +5255,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -5346,7 +5275,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -5368,7 +5297,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -5388,7 +5317,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -5408,7 +5337,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -5428,7 +5357,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -5446,7 +5375,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -5464,7 +5393,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="58" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -5489,7 +5418,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -5507,7 +5436,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -5525,7 +5454,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5548,7 +5477,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5571,7 +5500,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5589,7 +5518,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5607,7 +5536,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5624,7 +5553,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5642,7 +5571,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5659,7 +5588,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5682,7 +5611,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5709,7 +5638,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5727,7 +5656,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5760,23 +5689,23 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B1 B4:B60">
-    <cfRule type="expression" dxfId="69" priority="49">
+    <cfRule type="expression" dxfId="59" priority="49">
       <formula>MAX($E1,$H1,$K1)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="expression" dxfId="68" priority="89">
+    <cfRule type="expression" dxfId="58" priority="89">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1 C4:C60">
-    <cfRule type="expression" dxfId="67" priority="46">
+    <cfRule type="expression" dxfId="57" priority="46">
       <formula>$C1="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="47">
+    <cfRule type="expression" dxfId="56" priority="47">
       <formula>$C1="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="48">
+    <cfRule type="expression" dxfId="55" priority="48">
       <formula>$C1="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5791,21 +5720,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="81.54296875" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="81.5546875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.81640625" customWidth="1"/>
-    <col min="5" max="5" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="5" max="5" width="28.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46" x14ac:dyDescent="1">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5819,7 +5748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="87" t="s">
         <v>226</v>
       </c>
@@ -5833,7 +5762,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="73" t="s">
         <v>240</v>
       </c>
@@ -5847,7 +5776,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="88" t="s">
         <v>241</v>
       </c>
@@ -5861,7 +5790,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="88" t="s">
         <v>230</v>
       </c>
@@ -5875,7 +5804,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="73" t="s">
         <v>233</v>
       </c>
@@ -5889,7 +5818,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="88" t="s">
         <v>179</v>
       </c>
@@ -5903,7 +5832,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="84" t="s">
         <v>68</v>
       </c>
@@ -5915,10 +5844,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="64" priority="157">
+    <cfRule type="expression" dxfId="54" priority="157">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="158">
+    <cfRule type="expression" dxfId="53" priority="158">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5932,28 +5861,28 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:P48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:P51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.81640625" customWidth="1"/>
-    <col min="2" max="2" width="67.7265625" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" style="31" customWidth="1"/>
-    <col min="4" max="4" width="20.1796875" style="31" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.81640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.36328125" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.54296875" style="93" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7265625" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.1796875" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.08984375" style="31" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.54296875" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.77734375" customWidth="1"/>
+    <col min="2" max="2" width="67.77734375" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="31" customWidth="1"/>
+    <col min="4" max="4" width="20.21875" style="31" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.77734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" style="93" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5546875" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="46" x14ac:dyDescent="1">
+    <row r="2" spans="2:16" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B2" s="108" t="s">
         <v>17</v>
       </c>
@@ -5972,8 +5901,8 @@
       <c r="O2" s="109"/>
       <c r="P2" s="109"/>
     </row>
-    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.4">
       <c r="B6" s="102" t="s">
         <v>1</v>
       </c>
@@ -6004,7 +5933,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="112" t="s">
+      <c r="L6" s="110" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="43">
@@ -6020,7 +5949,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="21.5" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="2:16" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B7" s="103"/>
       <c r="C7" s="105"/>
       <c r="D7" s="91" t="s">
@@ -6043,7 +5972,7 @@
       <c r="K7" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="113"/>
+      <c r="L7" s="111"/>
       <c r="M7" s="98" t="s">
         <v>201</v>
       </c>
@@ -6055,7 +5984,7 @@
       </c>
       <c r="P7" s="107"/>
     </row>
-    <row r="8" spans="2:16" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:16" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="81" t="s">
         <v>68</v>
       </c>
@@ -6073,13 +6002,13 @@
       <c r="I8" s="92"/>
       <c r="J8" s="24"/>
       <c r="L8" s="94"/>
-      <c r="M8" s="110" t="s">
+      <c r="M8" s="112" t="s">
         <v>278</v>
       </c>
       <c r="N8"/>
       <c r="P8" s="92"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="81" t="s">
         <v>256</v>
       </c>
@@ -6097,11 +6026,11 @@
       <c r="I9" s="92"/>
       <c r="J9" s="24"/>
       <c r="L9" s="94"/>
-      <c r="M9" s="111"/>
+      <c r="M9" s="113"/>
       <c r="N9"/>
       <c r="P9" s="92"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
         <v>245</v>
       </c>
@@ -6119,11 +6048,11 @@
       <c r="I10" s="92"/>
       <c r="J10" s="24"/>
       <c r="L10" s="94"/>
-      <c r="M10" s="111"/>
+      <c r="M10" s="113"/>
       <c r="N10"/>
       <c r="P10" s="92"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
         <v>244</v>
       </c>
@@ -6141,11 +6070,11 @@
       <c r="I11" s="92"/>
       <c r="J11" s="24"/>
       <c r="L11" s="94"/>
-      <c r="M11" s="111"/>
+      <c r="M11" s="113"/>
       <c r="N11"/>
       <c r="P11" s="92"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
         <v>257</v>
       </c>
@@ -6163,11 +6092,11 @@
       <c r="I12" s="92"/>
       <c r="J12" s="24"/>
       <c r="L12" s="94"/>
-      <c r="M12" s="111"/>
+      <c r="M12" s="113"/>
       <c r="N12"/>
       <c r="P12" s="92"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
@@ -6185,11 +6114,11 @@
       <c r="I13" s="92"/>
       <c r="J13" s="24"/>
       <c r="L13" s="94"/>
-      <c r="M13" s="111"/>
+      <c r="M13" s="113"/>
       <c r="N13"/>
       <c r="P13" s="92"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
@@ -6207,11 +6136,11 @@
       <c r="I14" s="92"/>
       <c r="J14" s="24"/>
       <c r="L14" s="94"/>
-      <c r="M14" s="111"/>
+      <c r="M14" s="113"/>
       <c r="N14"/>
       <c r="P14" s="92"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
@@ -6229,11 +6158,11 @@
       <c r="I15" s="92"/>
       <c r="J15" s="24"/>
       <c r="L15" s="94"/>
-      <c r="M15" s="111"/>
+      <c r="M15" s="113"/>
       <c r="N15"/>
       <c r="P15" s="92"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
@@ -6251,11 +6180,11 @@
       <c r="I16" s="92"/>
       <c r="J16" s="24"/>
       <c r="L16" s="94"/>
-      <c r="M16" s="111"/>
+      <c r="M16" s="113"/>
       <c r="N16"/>
       <c r="P16" s="92"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
@@ -6273,11 +6202,11 @@
       <c r="I17" s="92"/>
       <c r="J17" s="24"/>
       <c r="L17" s="94"/>
-      <c r="M17" s="111"/>
+      <c r="M17" s="113"/>
       <c r="N17"/>
       <c r="P17" s="92"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
@@ -6295,11 +6224,11 @@
       <c r="I18" s="92"/>
       <c r="J18" s="24"/>
       <c r="L18" s="94"/>
-      <c r="M18" s="111"/>
+      <c r="M18" s="113"/>
       <c r="N18"/>
       <c r="P18" s="92"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
@@ -6317,11 +6246,11 @@
       <c r="I19" s="92"/>
       <c r="J19" s="24"/>
       <c r="L19" s="94"/>
-      <c r="M19" s="111"/>
+      <c r="M19" s="113"/>
       <c r="N19"/>
       <c r="P19" s="92"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
@@ -6339,11 +6268,11 @@
       <c r="I20" s="92"/>
       <c r="J20" s="24"/>
       <c r="L20" s="94"/>
-      <c r="M20" s="111"/>
+      <c r="M20" s="113"/>
       <c r="N20"/>
       <c r="P20" s="92"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
@@ -6361,11 +6290,11 @@
       <c r="I21" s="92"/>
       <c r="J21" s="24"/>
       <c r="L21" s="94"/>
-      <c r="M21" s="111"/>
+      <c r="M21" s="113"/>
       <c r="N21"/>
       <c r="P21" s="92"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" s="81" t="s">
         <v>255</v>
       </c>
@@ -6383,11 +6312,11 @@
       <c r="I22" s="92"/>
       <c r="J22" s="24"/>
       <c r="L22" s="94"/>
-      <c r="M22" s="111"/>
+      <c r="M22" s="113"/>
       <c r="N22"/>
       <c r="P22" s="92"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="82" t="s">
         <v>258</v>
       </c>
@@ -6405,11 +6334,11 @@
       <c r="I23" s="92"/>
       <c r="J23" s="24"/>
       <c r="L23" s="94"/>
-      <c r="M23" s="111"/>
+      <c r="M23" s="113"/>
       <c r="N23"/>
       <c r="P23" s="92"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="82" t="s">
         <v>259</v>
       </c>
@@ -6422,11 +6351,11 @@
       <c r="I24" s="92"/>
       <c r="J24" s="24"/>
       <c r="L24" s="94"/>
-      <c r="M24" s="111"/>
+      <c r="M24" s="113"/>
       <c r="N24"/>
       <c r="P24" s="92"/>
     </row>
-    <row r="25" spans="2:16" ht="31.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:16" ht="31.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="83" t="s">
         <v>260</v>
       </c>
@@ -6444,11 +6373,11 @@
         <v>100</v>
       </c>
       <c r="L25" s="94"/>
-      <c r="M25" s="111"/>
+      <c r="M25" s="113"/>
       <c r="N25"/>
       <c r="P25" s="92"/>
     </row>
-    <row r="26" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="83" t="s">
         <v>261</v>
       </c>
@@ -6466,11 +6395,11 @@
         <v>100</v>
       </c>
       <c r="L26" s="94"/>
-      <c r="M26" s="111"/>
+      <c r="M26" s="113"/>
       <c r="N26"/>
       <c r="P26" s="92"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B27" s="83" t="s">
         <v>262</v>
       </c>
@@ -6488,11 +6417,11 @@
         <v>100</v>
       </c>
       <c r="L27" s="94"/>
-      <c r="M27" s="111"/>
+      <c r="M27" s="113"/>
       <c r="N27"/>
       <c r="P27" s="92"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B28" s="83" t="s">
         <v>263</v>
       </c>
@@ -6510,11 +6439,11 @@
         <v>100</v>
       </c>
       <c r="L28" s="94"/>
-      <c r="M28" s="111"/>
+      <c r="M28" s="113"/>
       <c r="N28"/>
       <c r="P28" s="92"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B29" s="83" t="s">
         <v>264</v>
       </c>
@@ -6532,11 +6461,11 @@
         <v>100</v>
       </c>
       <c r="L29" s="94"/>
-      <c r="M29" s="111"/>
+      <c r="M29" s="113"/>
       <c r="N29"/>
       <c r="P29" s="92"/>
     </row>
-    <row r="30" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B30" s="83" t="s">
         <v>265</v>
       </c>
@@ -6554,11 +6483,11 @@
         <v>100</v>
       </c>
       <c r="L30" s="94"/>
-      <c r="M30" s="111"/>
+      <c r="M30" s="113"/>
       <c r="N30"/>
       <c r="P30" s="92"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B31" s="83" t="s">
         <v>280</v>
       </c>
@@ -6570,8 +6499,11 @@
       <c r="G31" s="24"/>
       <c r="I31" s="92"/>
       <c r="J31" s="24"/>
+      <c r="K31" s="31">
+        <v>100</v>
+      </c>
       <c r="L31" s="94"/>
-      <c r="M31" s="111"/>
+      <c r="M31" s="113"/>
       <c r="N31">
         <v>2</v>
       </c>
@@ -6580,7 +6512,7 @@
       </c>
       <c r="P31" s="92"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B32" s="83" t="s">
         <v>279</v>
       </c>
@@ -6593,7 +6525,7 @@
       <c r="I32" s="92"/>
       <c r="J32" s="24"/>
       <c r="L32" s="94"/>
-      <c r="M32" s="111"/>
+      <c r="M32" s="113"/>
       <c r="N32">
         <v>1</v>
       </c>
@@ -6602,7 +6534,7 @@
       </c>
       <c r="P32" s="92"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="83" t="s">
         <v>281</v>
       </c>
@@ -6615,7 +6547,7 @@
       <c r="I33" s="92"/>
       <c r="J33" s="24"/>
       <c r="L33" s="94"/>
-      <c r="M33" s="111"/>
+      <c r="M33" s="113"/>
       <c r="N33">
         <v>2</v>
       </c>
@@ -6624,111 +6556,101 @@
       </c>
       <c r="P33" s="92"/>
     </row>
-    <row r="34" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B34" s="29" t="s">
-        <v>215</v>
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B34" s="83" t="s">
+        <v>289</v>
       </c>
       <c r="C34" s="95" t="s">
-        <v>103</v>
-      </c>
-      <c r="D34" s="24">
-        <v>2</v>
-      </c>
-      <c r="E34" s="31">
-        <v>50</v>
-      </c>
-      <c r="F34" s="94" t="s">
-        <v>272</v>
-      </c>
-      <c r="G34" s="24">
-        <v>2</v>
-      </c>
-      <c r="H34" s="31">
-        <v>100</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="D34" s="24"/>
+      <c r="F34" s="92"/>
+      <c r="G34" s="24"/>
       <c r="I34" s="92"/>
-      <c r="J34" s="24"/>
       <c r="L34" s="94"/>
-      <c r="M34" s="111"/>
-      <c r="N34"/>
+      <c r="M34" s="113"/>
+      <c r="N34">
+        <v>1.5</v>
+      </c>
+      <c r="O34" s="31">
+        <v>100</v>
+      </c>
       <c r="P34" s="92"/>
     </row>
-    <row r="35" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B35" s="29" t="s">
-        <v>216</v>
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B35" s="83" t="s">
+        <v>290</v>
       </c>
       <c r="C35" s="95" t="s">
-        <v>103</v>
-      </c>
-      <c r="D35" s="24">
-        <v>1</v>
-      </c>
-      <c r="E35" s="31">
-        <v>25</v>
-      </c>
-      <c r="F35" s="94" t="s">
-        <v>273</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="D35" s="24"/>
+      <c r="F35" s="92"/>
       <c r="G35" s="24"/>
       <c r="I35" s="92"/>
-      <c r="J35" s="24">
-        <v>4</v>
-      </c>
-      <c r="K35" s="31">
-        <v>100</v>
-      </c>
       <c r="L35" s="94"/>
-      <c r="M35" s="111"/>
-      <c r="N35"/>
+      <c r="M35" s="113"/>
+      <c r="N35">
+        <v>2.5</v>
+      </c>
+      <c r="O35" s="31">
+        <v>100</v>
+      </c>
       <c r="P35" s="92"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B36" s="29" t="s">
-        <v>217</v>
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B36" s="83" t="s">
+        <v>291</v>
       </c>
       <c r="C36" s="95" t="s">
-        <v>103</v>
-      </c>
-      <c r="D36" s="24">
-        <v>5</v>
-      </c>
-      <c r="E36" s="31">
-        <v>100</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="D36" s="24"/>
       <c r="F36" s="92"/>
       <c r="G36" s="24"/>
       <c r="I36" s="92"/>
-      <c r="J36" s="24"/>
       <c r="L36" s="94"/>
-      <c r="M36" s="111"/>
-      <c r="N36"/>
+      <c r="M36" s="113"/>
+      <c r="N36">
+        <v>1.5</v>
+      </c>
+      <c r="O36" s="31">
+        <v>100</v>
+      </c>
       <c r="P36" s="92"/>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C37" s="95" t="s">
         <v>103</v>
       </c>
       <c r="D37" s="24">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E37" s="31">
-        <v>100</v>
-      </c>
-      <c r="F37" s="92"/>
-      <c r="G37" s="24"/>
+        <v>50</v>
+      </c>
+      <c r="F37" s="94" t="s">
+        <v>272</v>
+      </c>
+      <c r="G37" s="24">
+        <v>2</v>
+      </c>
+      <c r="H37" s="31">
+        <v>100</v>
+      </c>
       <c r="I37" s="92"/>
       <c r="J37" s="24"/>
       <c r="L37" s="94"/>
-      <c r="M37" s="111"/>
+      <c r="M37" s="113"/>
       <c r="N37"/>
       <c r="P37" s="92"/>
     </row>
-    <row r="38" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C38" s="95" t="s">
         <v>103</v>
@@ -6739,201 +6661,191 @@
       <c r="E38" s="31">
         <v>25</v>
       </c>
-      <c r="F38" s="92" t="s">
-        <v>271</v>
-      </c>
-      <c r="G38" s="24">
-        <v>2</v>
-      </c>
-      <c r="H38" s="31">
-        <v>75</v>
-      </c>
-      <c r="I38" s="94" t="s">
-        <v>270</v>
-      </c>
+      <c r="F38" s="94" t="s">
+        <v>273</v>
+      </c>
+      <c r="G38" s="24"/>
+      <c r="I38" s="92"/>
       <c r="J38" s="24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K38" s="31">
         <v>100</v>
       </c>
-      <c r="L38" s="94" t="s">
-        <v>282</v>
-      </c>
-      <c r="M38" s="111"/>
+      <c r="L38" s="94"/>
+      <c r="M38" s="113"/>
       <c r="N38"/>
       <c r="P38" s="92"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C39" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="D39" s="24"/>
+      <c r="D39" s="24">
+        <v>5</v>
+      </c>
+      <c r="E39" s="31">
+        <v>100</v>
+      </c>
       <c r="F39" s="92"/>
-      <c r="G39" s="24">
-        <v>3</v>
-      </c>
-      <c r="H39" s="31">
-        <v>100</v>
-      </c>
+      <c r="G39" s="24"/>
       <c r="I39" s="92"/>
       <c r="J39" s="24"/>
       <c r="L39" s="94"/>
-      <c r="M39" s="111"/>
+      <c r="M39" s="113"/>
       <c r="N39"/>
       <c r="P39" s="92"/>
     </row>
-    <row r="40" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B40" s="90" t="s">
-        <v>266</v>
-      </c>
-      <c r="C40" s="96" t="s">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B40" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="C40" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="G40" s="24">
+      <c r="D40" s="24">
         <v>1.5</v>
       </c>
-      <c r="H40" s="31">
-        <v>100</v>
-      </c>
-      <c r="I40" s="93" t="s">
-        <v>269</v>
-      </c>
+      <c r="E40" s="31">
+        <v>100</v>
+      </c>
+      <c r="F40" s="92"/>
+      <c r="G40" s="24"/>
+      <c r="I40" s="92"/>
       <c r="J40" s="24"/>
       <c r="L40" s="94"/>
-      <c r="M40" s="111"/>
+      <c r="M40" s="113"/>
       <c r="N40"/>
       <c r="P40" s="92"/>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B41" s="90" t="s">
-        <v>267</v>
-      </c>
-      <c r="C41" s="96" t="s">
+    <row r="41" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B41" s="29" t="s">
+        <v>222</v>
+      </c>
+      <c r="C41" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="G41" s="24"/>
+      <c r="D41" s="24">
+        <v>1</v>
+      </c>
+      <c r="E41" s="31">
+        <v>25</v>
+      </c>
+      <c r="F41" s="92" t="s">
+        <v>271</v>
+      </c>
+      <c r="G41" s="24">
+        <v>2</v>
+      </c>
+      <c r="H41" s="31">
+        <v>75</v>
+      </c>
+      <c r="I41" s="94" t="s">
+        <v>270</v>
+      </c>
       <c r="J41" s="24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K41" s="31">
         <v>100</v>
       </c>
-      <c r="L41" s="94"/>
-      <c r="M41" s="111"/>
+      <c r="L41" s="94" t="s">
+        <v>282</v>
+      </c>
+      <c r="M41" s="113"/>
       <c r="N41"/>
       <c r="P41" s="92"/>
     </row>
-    <row r="42" spans="2:16" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="B42" s="90" t="s">
-        <v>268</v>
-      </c>
-      <c r="C42" s="96" t="s">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B42" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="C42" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="G42" s="24"/>
-      <c r="J42" s="24">
-        <v>4</v>
-      </c>
-      <c r="K42" s="31">
-        <v>90</v>
-      </c>
-      <c r="L42" s="94" t="s">
-        <v>275</v>
-      </c>
-      <c r="M42" s="111"/>
+      <c r="D42" s="24"/>
+      <c r="F42" s="92"/>
+      <c r="G42" s="24">
+        <v>3</v>
+      </c>
+      <c r="H42" s="31">
+        <v>100</v>
+      </c>
+      <c r="I42" s="92"/>
+      <c r="J42" s="24"/>
+      <c r="L42" s="94"/>
+      <c r="M42" s="113"/>
       <c r="N42"/>
       <c r="P42" s="92"/>
     </row>
-    <row r="43" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:16" ht="72" x14ac:dyDescent="0.3">
       <c r="B43" s="90" t="s">
-        <v>239</v>
-      </c>
-      <c r="C43" s="95" t="s">
+        <v>266</v>
+      </c>
+      <c r="C43" s="96" t="s">
         <v>103</v>
       </c>
-      <c r="D43" s="24"/>
-      <c r="F43" s="92"/>
-      <c r="G43" s="24"/>
-      <c r="I43" s="92"/>
-      <c r="J43" s="24">
+      <c r="G43" s="24">
         <v>1.5</v>
       </c>
-      <c r="K43" s="31">
-        <v>100</v>
-      </c>
-      <c r="L43" s="94" t="s">
-        <v>274</v>
-      </c>
-      <c r="M43" s="111"/>
+      <c r="H43" s="31">
+        <v>100</v>
+      </c>
+      <c r="I43" s="93" t="s">
+        <v>269</v>
+      </c>
+      <c r="J43" s="24"/>
+      <c r="L43" s="94"/>
+      <c r="M43" s="113"/>
       <c r="N43"/>
       <c r="P43" s="92"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B44" s="90" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C44" s="96" t="s">
         <v>103</v>
       </c>
-      <c r="D44" s="31">
-        <v>1</v>
-      </c>
-      <c r="E44" s="31">
-        <v>10</v>
-      </c>
-      <c r="G44" s="24">
-        <v>2</v>
-      </c>
-      <c r="H44" s="31">
-        <v>30</v>
-      </c>
+      <c r="G44" s="24"/>
       <c r="J44" s="24">
         <v>2</v>
       </c>
       <c r="K44" s="31">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="L44" s="94"/>
-      <c r="M44" s="111"/>
-      <c r="N44">
+      <c r="M44" s="113"/>
+      <c r="N44"/>
+      <c r="P44" s="92"/>
+    </row>
+    <row r="45" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="B45" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="C45" s="96" t="s">
+        <v>103</v>
+      </c>
+      <c r="G45" s="24"/>
+      <c r="J45" s="24">
         <v>4</v>
       </c>
-      <c r="O44" s="31">
-        <v>75</v>
-      </c>
-      <c r="P44" s="92"/>
-    </row>
-    <row r="45" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B45" s="90" t="s">
-        <v>277</v>
-      </c>
-      <c r="C45" s="95" t="s">
-        <v>103</v>
-      </c>
-      <c r="D45" s="24"/>
-      <c r="F45" s="92"/>
-      <c r="G45" s="24"/>
-      <c r="I45" s="92"/>
-      <c r="J45" s="24">
-        <v>1</v>
-      </c>
       <c r="K45" s="31">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="L45" s="94" t="s">
-        <v>283</v>
-      </c>
-      <c r="M45" s="111"/>
+        <v>275</v>
+      </c>
+      <c r="M45" s="113"/>
       <c r="N45"/>
       <c r="P45" s="92"/>
     </row>
-    <row r="46" spans="2:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B46" s="90" t="s">
-        <v>287</v>
+        <v>239</v>
       </c>
       <c r="C46" s="95" t="s">
         <v>103</v>
@@ -6942,59 +6854,143 @@
       <c r="F46" s="92"/>
       <c r="G46" s="24"/>
       <c r="I46" s="92"/>
-      <c r="J46" s="24"/>
-      <c r="L46" s="94"/>
-      <c r="M46" s="111"/>
-      <c r="N46">
+      <c r="J46" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="K46" s="31">
+        <v>100</v>
+      </c>
+      <c r="L46" s="94" t="s">
+        <v>274</v>
+      </c>
+      <c r="M46" s="113"/>
+      <c r="N46"/>
+      <c r="P46" s="92"/>
+    </row>
+    <row r="47" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B47" s="90" t="s">
+        <v>276</v>
+      </c>
+      <c r="C47" s="96" t="s">
+        <v>103</v>
+      </c>
+      <c r="D47" s="31">
+        <v>1</v>
+      </c>
+      <c r="E47" s="31">
+        <v>10</v>
+      </c>
+      <c r="G47" s="24">
+        <v>2</v>
+      </c>
+      <c r="H47" s="31">
+        <v>30</v>
+      </c>
+      <c r="J47" s="24">
+        <v>2</v>
+      </c>
+      <c r="K47" s="31">
+        <v>50</v>
+      </c>
+      <c r="L47" s="94"/>
+      <c r="M47" s="113"/>
+      <c r="N47">
+        <v>4</v>
+      </c>
+      <c r="O47" s="31">
+        <v>75</v>
+      </c>
+      <c r="P47" s="92"/>
+    </row>
+    <row r="48" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B48" s="90" t="s">
+        <v>277</v>
+      </c>
+      <c r="C48" s="95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D48" s="24"/>
+      <c r="F48" s="92"/>
+      <c r="G48" s="24"/>
+      <c r="I48" s="92"/>
+      <c r="J48" s="24">
+        <v>1</v>
+      </c>
+      <c r="K48" s="31">
+        <v>75</v>
+      </c>
+      <c r="L48" s="94" t="s">
+        <v>283</v>
+      </c>
+      <c r="M48" s="113"/>
+      <c r="N48"/>
+      <c r="P48" s="92"/>
+    </row>
+    <row r="49" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B49" s="90" t="s">
+        <v>287</v>
+      </c>
+      <c r="C49" s="95" t="s">
+        <v>103</v>
+      </c>
+      <c r="D49" s="24"/>
+      <c r="F49" s="92"/>
+      <c r="G49" s="24"/>
+      <c r="I49" s="92"/>
+      <c r="J49" s="24"/>
+      <c r="L49" s="94"/>
+      <c r="M49" s="113"/>
+      <c r="N49">
         <v>0.5</v>
       </c>
-      <c r="O46" s="31">
+      <c r="O49" s="31">
         <v>75</v>
       </c>
-      <c r="P46" s="94" t="s">
+      <c r="P49" s="94" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B47" s="81" t="s">
+    <row r="50" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B50" s="81" t="s">
         <v>284</v>
       </c>
-      <c r="C47" s="95" t="s">
+      <c r="C50" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="D47" s="24"/>
-      <c r="F47" s="92"/>
-      <c r="G47" s="24"/>
-      <c r="I47" s="92"/>
-      <c r="J47" s="24"/>
-      <c r="L47" s="94"/>
-      <c r="M47" s="111"/>
-      <c r="N47">
+      <c r="D50" s="24"/>
+      <c r="F50" s="92"/>
+      <c r="G50" s="24"/>
+      <c r="I50" s="92"/>
+      <c r="J50" s="24"/>
+      <c r="L50" s="94"/>
+      <c r="M50" s="113"/>
+      <c r="N50">
         <v>1</v>
       </c>
-      <c r="O47" s="31">
-        <v>100</v>
-      </c>
-      <c r="P47" s="92"/>
-    </row>
-    <row r="48" spans="2:16" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B48" s="90" t="s">
+      <c r="O50" s="31">
+        <v>100</v>
+      </c>
+      <c r="P50" s="92"/>
+    </row>
+    <row r="51" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+      <c r="B51" s="90" t="s">
         <v>288</v>
       </c>
-      <c r="C48" s="31" t="s">
+      <c r="C51" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="F48" s="92"/>
-      <c r="I48" s="92"/>
-      <c r="L48" s="94"/>
-      <c r="M48" s="111"/>
-      <c r="N48"/>
-      <c r="P48" s="94" t="s">
+      <c r="F51" s="92"/>
+      <c r="I51" s="92"/>
+      <c r="L51" s="94"/>
+      <c r="M51" s="113"/>
+      <c r="N51"/>
+      <c r="P51" s="94" t="s">
         <v>285</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="M8:M51"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="B6:B7"/>
@@ -7002,234 +6998,238 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="L6:L7"/>
-    <mergeCell ref="M8:M48"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 B6:B7 B23:B41">
-    <cfRule type="expression" dxfId="62" priority="38">
+  <conditionalFormatting sqref="B2 B6:B7 B23:B44">
+    <cfRule type="expression" dxfId="52" priority="38">
       <formula>MAX($E2,$H2,$K2)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C44">
-    <cfRule type="expression" dxfId="61" priority="27">
+  <conditionalFormatting sqref="C6:C47">
+    <cfRule type="expression" dxfId="51" priority="27">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="28">
+    <cfRule type="expression" dxfId="50" priority="28">
       <formula>$C6="Charlotte"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="29">
+    <cfRule type="expression" dxfId="49" priority="29">
       <formula>$C6="Eddy"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B8 B23:B24">
-    <cfRule type="expression" dxfId="58" priority="241">
+  <conditionalFormatting sqref="B8">
+    <cfRule type="expression" dxfId="48" priority="241">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14 B32:B33">
-    <cfRule type="expression" dxfId="57" priority="243">
+  <conditionalFormatting sqref="B14">
+    <cfRule type="expression" dxfId="47" priority="243">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
-    <cfRule type="expression" dxfId="56" priority="259">
-      <formula>MAX($E34,$H34,$K34)=100</formula>
+    <cfRule type="expression" dxfId="46" priority="259">
+      <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="55" priority="280">
+    <cfRule type="expression" dxfId="45" priority="280">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B12">
-    <cfRule type="expression" dxfId="54" priority="14">
+    <cfRule type="expression" dxfId="44" priority="14">
       <formula>MAX($E17,$H17,$K17)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B33">
-    <cfRule type="expression" dxfId="53" priority="12">
+  <conditionalFormatting sqref="B23:B36">
+    <cfRule type="expression" dxfId="43" priority="12">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:B16">
-    <cfRule type="expression" dxfId="52" priority="329">
-      <formula>MAX($E34,$H34,$K34)=100</formula>
+    <cfRule type="expression" dxfId="42" priority="329">
+      <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="expression" dxfId="51" priority="360">
+    <cfRule type="expression" dxfId="41" priority="360">
       <formula>MAX($E25,$H25,$K25)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="361">
+    <cfRule type="expression" dxfId="40" priority="361">
       <formula>MAX($E5,$H5,$K5)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14 B16:B18">
-    <cfRule type="expression" dxfId="49" priority="366">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="39" priority="366">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:B19">
-    <cfRule type="expression" dxfId="48" priority="367">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="38" priority="367">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:B21">
-    <cfRule type="expression" dxfId="47" priority="399">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
+  <conditionalFormatting sqref="B20:B21 B23:B24">
+    <cfRule type="expression" dxfId="37" priority="399">
+      <formula>MAX($E40,$H40,$K40)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8">
-    <cfRule type="expression" dxfId="46" priority="448">
+    <cfRule type="expression" dxfId="36" priority="448">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="449">
+    <cfRule type="expression" dxfId="35" priority="449">
       <formula>MAX($E4,$H4,$K4)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="expression" dxfId="44" priority="508">
+    <cfRule type="expression" dxfId="34" priority="508">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="expression" dxfId="43" priority="513">
+    <cfRule type="expression" dxfId="33" priority="513">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:B31">
-    <cfRule type="expression" dxfId="42" priority="521">
+    <cfRule type="expression" dxfId="32" priority="521">
       <formula>MAX($E14,$H14,$K14)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="522">
+    <cfRule type="expression" dxfId="31" priority="522">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="expression" dxfId="40" priority="531">
+    <cfRule type="expression" dxfId="30" priority="531">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="532">
+    <cfRule type="expression" dxfId="29" priority="532">
       <formula>MAX($E16,$H16,$K16)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="expression" dxfId="38" priority="542">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
+    <cfRule type="expression" dxfId="28" priority="542">
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="expression" dxfId="37" priority="544">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
+    <cfRule type="expression" dxfId="27" priority="544">
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12 B16">
-    <cfRule type="expression" dxfId="36" priority="549">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
+    <cfRule type="expression" dxfId="26" priority="549">
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="550">
+    <cfRule type="expression" dxfId="25" priority="550">
       <formula>MAX($E8,$H8,$K8)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25 B27:B29">
-    <cfRule type="expression" dxfId="34" priority="592">
+    <cfRule type="expression" dxfId="24" priority="592">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="593">
-      <formula>MAX($E38,$H38,$K38)=100</formula>
+    <cfRule type="expression" dxfId="23" priority="593">
+      <formula>MAX($E41,$H41,$K41)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="expression" dxfId="32" priority="603">
+    <cfRule type="expression" dxfId="22" priority="603">
+      <formula>MAX($E46,$H46,$K46)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B23">
+    <cfRule type="expression" dxfId="21" priority="609">
+      <formula>MAX($E46,$H46,$K46)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B21:B24">
+    <cfRule type="expression" dxfId="20" priority="619">
+      <formula>MAX($E47,$H47,$K47)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B24 B27">
+    <cfRule type="expression" dxfId="19" priority="621">
       <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23">
-    <cfRule type="expression" dxfId="31" priority="609">
-      <formula>MAX($E43,$H43,$K43)=100</formula>
+  <conditionalFormatting sqref="B20 B22">
+    <cfRule type="expression" dxfId="18" priority="629">
+      <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21:B24">
-    <cfRule type="expression" dxfId="30" priority="619">
-      <formula>MAX($E44,$H44,$K44)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B24 B27">
-    <cfRule type="expression" dxfId="29" priority="621">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20 B22">
-    <cfRule type="expression" dxfId="28" priority="629">
-      <formula>MAX($E42,$H42,$K42)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="630">
+    <cfRule type="expression" dxfId="17" priority="630">
       <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="expression" dxfId="26" priority="633">
-      <formula>MAX($E43,$H43,$K43)=100</formula>
+    <cfRule type="expression" dxfId="16" priority="633">
+      <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26">
-    <cfRule type="expression" dxfId="25" priority="634">
+    <cfRule type="expression" dxfId="15" priority="634">
       <formula>MAX($E10,$H10,$K10)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="24" priority="635">
-      <formula>MAX($E43,$H43,$K43)=100</formula>
+    <cfRule type="expression" dxfId="14" priority="635">
+      <formula>MAX($E46,$H46,$K46)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:B26 B28:B31">
+    <cfRule type="expression" dxfId="13" priority="670">
+      <formula>MAX($E40,$H40,$K40)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:B36">
+    <cfRule type="expression" dxfId="12" priority="677">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="678">
+      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C48:C50">
+    <cfRule type="expression" dxfId="10" priority="2">
+      <formula>$C48="Charlotte/Eddy"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="3">
+      <formula>$C48="Charlotte"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="4">
+      <formula>$C48="Eddy"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B44:B51">
+    <cfRule type="expression" dxfId="7" priority="1">
+      <formula>MAX($E44,$H44,$K44)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:B36">
+    <cfRule type="expression" dxfId="6" priority="695">
+      <formula>MAX($E46,$H46,$K46)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:B15 B17:B19">
-    <cfRule type="expression" dxfId="23" priority="666">
-      <formula>MAX($E36,$H36,$K36)=100</formula>
+    <cfRule type="expression" dxfId="5" priority="727">
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="22" priority="667">
+    <cfRule type="expression" dxfId="4" priority="728">
       <formula>MAX($E9,$H9,$K9)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B25:B26 B28:B31">
-    <cfRule type="expression" dxfId="21" priority="670">
+  <conditionalFormatting sqref="B10:B11">
+    <cfRule type="expression" dxfId="3" priority="745">
       <formula>MAX($E37,$H37,$K37)=100</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B32:B33">
-    <cfRule type="expression" dxfId="20" priority="677">
-      <formula>MAX($E15,$H15,$K15)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="678">
-      <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10:B11">
-    <cfRule type="expression" dxfId="18" priority="690">
-      <formula>MAX($E34,$H34,$K34)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="691">
+    <cfRule type="expression" dxfId="2" priority="746">
       <formula>MAX($E6,$H6,$K6)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B24">
-    <cfRule type="expression" dxfId="16" priority="692">
+    <cfRule type="expression" dxfId="1" priority="747">
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="693">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C45:C47">
-    <cfRule type="expression" dxfId="11" priority="2">
-      <formula>$C45="Charlotte/Eddy"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="3">
-      <formula>$C45="Charlotte"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="4">
-      <formula>$C45="Eddy"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B41:B48">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>MAX($E41,$H41,$K41)=100</formula>
+    <cfRule type="expression" dxfId="0" priority="748">
+      <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7243,28 +7243,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" customWidth="1"/>
-    <col min="2" max="2" width="93.1796875" customWidth="1"/>
+    <col min="1" max="1" width="3.21875" customWidth="1"/>
+    <col min="2" max="2" width="93.21875" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="42.81640625" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.77734375" customWidth="1"/>
+    <col min="6" max="6" width="42.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.9" customHeight="1" x14ac:dyDescent="1">
+    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="47" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="2:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -7281,7 +7281,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -7294,7 +7294,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -7307,7 +7307,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -7320,7 +7320,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -7333,7 +7333,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -7346,7 +7346,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -7359,7 +7359,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -7372,7 +7372,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -7385,7 +7385,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -7398,7 +7398,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -7411,7 +7411,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -7424,7 +7424,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -7437,7 +7437,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -7450,7 +7450,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -7463,7 +7463,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -7476,7 +7476,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -7489,7 +7489,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -7502,7 +7502,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -7515,7 +7515,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -7528,7 +7528,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -7541,7 +7541,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -7554,7 +7554,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -7567,7 +7567,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -7580,7 +7580,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -7593,7 +7593,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -7606,7 +7606,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -7619,7 +7619,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -7632,7 +7632,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -7645,7 +7645,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -7658,7 +7658,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -7671,7 +7671,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -7684,7 +7684,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -7697,7 +7697,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -7710,7 +7710,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -7723,7 +7723,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -7736,7 +7736,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -7749,7 +7749,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -7762,7 +7762,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -7775,7 +7775,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -7788,7 +7788,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -7801,7 +7801,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -7814,7 +7814,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -7827,7 +7827,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -7840,7 +7840,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -7853,7 +7853,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -7866,7 +7866,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -7879,7 +7879,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -7892,7 +7892,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -7905,7 +7905,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -7918,7 +7918,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -7931,7 +7931,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -7944,7 +7944,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -7957,7 +7957,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -7970,7 +7970,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -7983,7 +7983,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -7996,7 +7996,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -8009,7 +8009,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -8022,7 +8022,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -8035,7 +8035,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -8048,7 +8048,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -8059,7 +8059,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -8070,7 +8070,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -8081,7 +8081,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -8092,7 +8092,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -8103,7 +8103,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -8114,7 +8114,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -8125,7 +8125,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -8136,7 +8136,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -8147,7 +8147,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>106</v>
       </c>
@@ -8158,7 +8158,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>107</v>
       </c>
@@ -8169,182 +8169,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Ajout fleche last  move + nom reel du joueur adverse+ simplifier timer
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8388B779-1C7F-47CB-91F1-D1707B550C01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C165DBAF-A721-4F81-A2CC-AF9EC8C572A1}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,12 +35,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -48,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="295">
   <si>
     <t>Planification globale</t>
   </si>
@@ -929,6 +923,12 @@
   </si>
   <si>
     <t>Augmenter le nombre d'itérations par tour de l'IA</t>
+  </si>
+  <si>
+    <t>Ajouter une fleche avec le sens du dernier coup joué</t>
+  </si>
+  <si>
+    <t>Ajouter le vrai nom du joueur au lieu de hardcoder + faire clignoter nom du joueur qui joue</t>
   </si>
 </sst>
 </file>
@@ -1692,23 +1692,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1723,19 +1714,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1744,20 +1744,15 @@
   <dxfs count="59">
     <dxf>
       <fill>
-        <gradientFill degree="45">
-          <stop position="0">
-            <color rgb="FFFCFDCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FFCCFFFF"/>
-          </stop>
-        </gradientFill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1771,15 +1766,20 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor rgb="FFCCFFFF"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
+        <gradientFill degree="45">
+          <stop position="0">
+            <color rgb="FFFCFDCF"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFCCFFFF"/>
+          </stop>
+        </gradientFill>
       </fill>
     </dxf>
     <dxf>
@@ -2490,26 +2490,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="42.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="42.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2537,7 +2537,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2677,7 +2677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2775,7 +2775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -2971,8 +2971,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -3007,32 +3007,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
-    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -3062,7 +3062,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -3116,7 +3116,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -3143,7 +3143,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -3165,7 +3165,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -3192,7 +3192,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -3225,7 +3225,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -3299,7 +3299,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3359,7 +3359,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3386,15 +3386,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3410,44 +3410,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="77.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B3" s="107" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B3" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="108"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="109"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B5" s="101" t="s">
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="96"/>
+      <c r="L3" s="97"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="103" t="s">
+      <c r="C5" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3456,7 +3456,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="99" t="s">
+      <c r="F5" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3465,7 +3465,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="99" t="s">
+      <c r="I5" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3474,36 +3474,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="99" t="s">
+      <c r="L5" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="102"/>
-      <c r="C6" s="104"/>
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="99"/>
+      <c r="C6" s="101"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="100"/>
+      <c r="F6" s="103"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="100"/>
+      <c r="I6" s="103"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="100"/>
-    </row>
-    <row r="7" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L6" s="103"/>
+    </row>
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3526,7 +3526,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3545,7 +3545,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3564,7 +3564,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3583,7 +3583,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3602,7 +3602,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3621,7 +3621,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3640,7 +3640,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3659,7 +3659,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3678,7 +3678,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3697,7 +3697,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3716,7 +3716,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3735,7 +3735,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3754,7 +3754,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3773,7 +3773,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3813,7 +3813,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3853,7 +3853,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3872,7 +3872,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3914,7 +3914,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3954,7 +3954,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -3973,7 +3973,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -4239,7 +4239,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -4296,7 +4296,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -4401,43 +4401,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.6640625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B1" s="107" t="s">
+    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B1" s="95" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="109"/>
-    </row>
-    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B4" s="101" t="s">
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="97"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4446,7 +4446,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4455,7 +4455,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="99" t="s">
+      <c r="I4" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4464,36 +4464,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="99" t="s">
+      <c r="L4" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="102"/>
-      <c r="C5" s="104"/>
+    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="99"/>
+      <c r="C5" s="101"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="100"/>
+      <c r="F5" s="103"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="100"/>
+      <c r="I5" s="103"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="100"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="103"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4511,7 +4511,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4529,7 +4529,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4547,7 +4547,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4565,7 +4565,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4583,7 +4583,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4601,7 +4601,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4619,7 +4619,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4637,7 +4637,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4655,7 +4655,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4673,7 +4673,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4691,7 +4691,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4709,7 +4709,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4727,7 +4727,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4745,7 +4745,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4764,7 +4764,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4783,7 +4783,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4802,7 +4802,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -4821,7 +4821,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -4840,7 +4840,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -4859,7 +4859,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -4878,7 +4878,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -4897,7 +4897,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -4916,7 +4916,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -4935,7 +4935,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -4954,7 +4954,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -4973,7 +4973,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -4992,7 +4992,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -5011,7 +5011,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -5174,7 +5174,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -5194,7 +5194,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -5214,7 +5214,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -5252,7 +5252,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -5270,7 +5270,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -5295,7 +5295,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -5313,7 +5313,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -5331,7 +5331,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5354,7 +5354,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5395,7 +5395,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5413,7 +5413,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5430,7 +5430,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5448,7 +5448,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5465,7 +5465,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5515,7 +5515,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5533,7 +5533,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5597,21 +5597,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="81.5703125" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="81.5546875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5625,7 +5625,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="85" t="s">
         <v>226</v>
       </c>
@@ -5639,7 +5639,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="73" t="s">
         <v>240</v>
       </c>
@@ -5653,7 +5653,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="86" t="s">
         <v>241</v>
       </c>
@@ -5667,7 +5667,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="86" t="s">
         <v>230</v>
       </c>
@@ -5681,7 +5681,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="73" t="s">
         <v>233</v>
       </c>
@@ -5695,7 +5695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>179</v>
       </c>
@@ -5709,7 +5709,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="82" t="s">
         <v>68</v>
       </c>
@@ -5735,50 +5735,50 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:P65"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:P67"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="67.7109375" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="31" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" style="31" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" style="90" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.5703125" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="67.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="31" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="31" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.6640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" style="90" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5546875" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="B2" s="97" t="s">
+    <row r="2" spans="2:16" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="B2" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="98"/>
-    </row>
-    <row r="5" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.35">
-      <c r="B6" s="101" t="s">
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="107"/>
+    </row>
+    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="103" t="s">
+      <c r="C6" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="88" t="s">
@@ -5787,7 +5787,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="99" t="s">
+      <c r="F6" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5796,7 +5796,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="99" t="s">
+      <c r="I6" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="60" t="s">
@@ -5805,7 +5805,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="105" t="s">
+      <c r="L6" s="108" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="43">
@@ -5817,34 +5817,34 @@
       <c r="O6" s="43">
         <v>46167</v>
       </c>
-      <c r="P6" s="99" t="s">
+      <c r="P6" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="102"/>
-      <c r="C7" s="104"/>
+    <row r="7" spans="2:16" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="99"/>
+      <c r="C7" s="101"/>
       <c r="D7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="100"/>
+      <c r="F7" s="103"/>
       <c r="G7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="100"/>
+      <c r="I7" s="103"/>
       <c r="J7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="106"/>
+      <c r="L7" s="109"/>
       <c r="M7" s="94" t="s">
         <v>201</v>
       </c>
@@ -5854,9 +5854,9 @@
       <c r="O7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="100"/>
-    </row>
-    <row r="8" spans="2:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P7" s="103"/>
+    </row>
+    <row r="8" spans="2:16" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="79" t="s">
         <v>68</v>
       </c>
@@ -5874,13 +5874,13 @@
       <c r="I8" s="89"/>
       <c r="J8" s="24"/>
       <c r="L8" s="91"/>
-      <c r="M8" s="95" t="s">
+      <c r="M8" s="104" t="s">
         <v>278</v>
       </c>
       <c r="N8"/>
       <c r="P8" s="89"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="79" t="s">
         <v>256</v>
       </c>
@@ -5898,11 +5898,11 @@
       <c r="I9" s="89"/>
       <c r="J9" s="24"/>
       <c r="L9" s="91"/>
-      <c r="M9" s="96"/>
+      <c r="M9" s="105"/>
       <c r="N9"/>
       <c r="P9" s="89"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
         <v>245</v>
       </c>
@@ -5920,11 +5920,11 @@
       <c r="I10" s="89"/>
       <c r="J10" s="24"/>
       <c r="L10" s="91"/>
-      <c r="M10" s="96"/>
+      <c r="M10" s="105"/>
       <c r="N10"/>
       <c r="P10" s="89"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
         <v>244</v>
       </c>
@@ -5942,11 +5942,11 @@
       <c r="I11" s="89"/>
       <c r="J11" s="24"/>
       <c r="L11" s="91"/>
-      <c r="M11" s="96"/>
+      <c r="M11" s="105"/>
       <c r="N11"/>
       <c r="P11" s="89"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
         <v>257</v>
       </c>
@@ -5963,11 +5963,11 @@
       <c r="I12" s="89"/>
       <c r="J12" s="24"/>
       <c r="L12" s="91"/>
-      <c r="M12" s="96"/>
+      <c r="M12" s="105"/>
       <c r="N12"/>
       <c r="P12" s="89"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
@@ -5984,11 +5984,11 @@
       <c r="I13" s="89"/>
       <c r="J13" s="24"/>
       <c r="L13" s="91"/>
-      <c r="M13" s="96"/>
+      <c r="M13" s="105"/>
       <c r="N13"/>
       <c r="P13" s="89"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
@@ -6005,11 +6005,11 @@
       <c r="I14" s="89"/>
       <c r="J14" s="24"/>
       <c r="L14" s="91"/>
-      <c r="M14" s="96"/>
+      <c r="M14" s="105"/>
       <c r="N14"/>
       <c r="P14" s="89"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
@@ -6026,11 +6026,11 @@
       <c r="I15" s="89"/>
       <c r="J15" s="24"/>
       <c r="L15" s="91"/>
-      <c r="M15" s="96"/>
+      <c r="M15" s="105"/>
       <c r="N15"/>
       <c r="P15" s="89"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
@@ -6047,11 +6047,11 @@
       <c r="I16" s="89"/>
       <c r="J16" s="24"/>
       <c r="L16" s="91"/>
-      <c r="M16" s="96"/>
+      <c r="M16" s="105"/>
       <c r="N16"/>
       <c r="P16" s="89"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
@@ -6067,11 +6067,11 @@
       <c r="I17" s="89"/>
       <c r="J17" s="24"/>
       <c r="L17" s="91"/>
-      <c r="M17" s="96"/>
+      <c r="M17" s="105"/>
       <c r="N17"/>
       <c r="P17" s="89"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
@@ -6087,11 +6087,11 @@
       <c r="I18" s="89"/>
       <c r="J18" s="24"/>
       <c r="L18" s="91"/>
-      <c r="M18" s="96"/>
+      <c r="M18" s="105"/>
       <c r="N18"/>
       <c r="P18" s="89"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
@@ -6107,11 +6107,11 @@
       <c r="I19" s="89"/>
       <c r="J19" s="24"/>
       <c r="L19" s="91"/>
-      <c r="M19" s="96"/>
+      <c r="M19" s="105"/>
       <c r="N19"/>
       <c r="P19" s="89"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
@@ -6127,11 +6127,11 @@
       <c r="I20" s="89"/>
       <c r="J20" s="24"/>
       <c r="L20" s="91"/>
-      <c r="M20" s="96"/>
+      <c r="M20" s="105"/>
       <c r="N20"/>
       <c r="P20" s="89"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
@@ -6147,11 +6147,11 @@
       <c r="I21" s="89"/>
       <c r="J21" s="24"/>
       <c r="L21" s="91"/>
-      <c r="M21" s="96"/>
+      <c r="M21" s="105"/>
       <c r="N21"/>
       <c r="P21" s="89"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" s="79" t="s">
         <v>255</v>
       </c>
@@ -6167,11 +6167,11 @@
       <c r="I22" s="89"/>
       <c r="J22" s="24"/>
       <c r="L22" s="91"/>
-      <c r="M22" s="96"/>
+      <c r="M22" s="105"/>
       <c r="N22"/>
       <c r="P22" s="89"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="80" t="s">
         <v>258</v>
       </c>
@@ -6189,11 +6189,11 @@
       <c r="I23" s="89"/>
       <c r="J23" s="24"/>
       <c r="L23" s="91"/>
-      <c r="M23" s="96"/>
+      <c r="M23" s="105"/>
       <c r="N23"/>
       <c r="P23" s="89"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="80" t="s">
         <v>259</v>
       </c>
@@ -6206,11 +6206,11 @@
       <c r="I24" s="89"/>
       <c r="J24" s="24"/>
       <c r="L24" s="91"/>
-      <c r="M24" s="96"/>
+      <c r="M24" s="105"/>
       <c r="N24"/>
       <c r="P24" s="89"/>
     </row>
-    <row r="25" spans="2:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="81" t="s">
         <v>260</v>
       </c>
@@ -6228,11 +6228,11 @@
         <v>100</v>
       </c>
       <c r="L25" s="91"/>
-      <c r="M25" s="96"/>
+      <c r="M25" s="105"/>
       <c r="N25"/>
       <c r="P25" s="89"/>
     </row>
-    <row r="26" spans="2:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="81" t="s">
         <v>261</v>
       </c>
@@ -6250,11 +6250,11 @@
         <v>100</v>
       </c>
       <c r="L26" s="91"/>
-      <c r="M26" s="96"/>
+      <c r="M26" s="105"/>
       <c r="N26"/>
       <c r="P26" s="89"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B27" s="81" t="s">
         <v>262</v>
       </c>
@@ -6272,11 +6272,11 @@
         <v>100</v>
       </c>
       <c r="L27" s="91"/>
-      <c r="M27" s="96"/>
+      <c r="M27" s="105"/>
       <c r="N27"/>
       <c r="P27" s="89"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B28" s="81" t="s">
         <v>263</v>
       </c>
@@ -6294,11 +6294,11 @@
         <v>100</v>
       </c>
       <c r="L28" s="91"/>
-      <c r="M28" s="96"/>
+      <c r="M28" s="105"/>
       <c r="N28"/>
       <c r="P28" s="89"/>
     </row>
-    <row r="29" spans="2:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B29" s="81" t="s">
         <v>264</v>
       </c>
@@ -6316,11 +6316,11 @@
         <v>100</v>
       </c>
       <c r="L29" s="91"/>
-      <c r="M29" s="96"/>
+      <c r="M29" s="105"/>
       <c r="N29"/>
       <c r="P29" s="89"/>
     </row>
-    <row r="30" spans="2:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B30" s="81" t="s">
         <v>265</v>
       </c>
@@ -6338,11 +6338,11 @@
         <v>100</v>
       </c>
       <c r="L30" s="91"/>
-      <c r="M30" s="96"/>
+      <c r="M30" s="105"/>
       <c r="N30"/>
       <c r="P30" s="89"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B31" s="81" t="s">
         <v>280</v>
       </c>
@@ -6358,7 +6358,7 @@
         <v>100</v>
       </c>
       <c r="L31" s="91"/>
-      <c r="M31" s="96"/>
+      <c r="M31" s="105"/>
       <c r="N31">
         <v>2</v>
       </c>
@@ -6367,7 +6367,7 @@
       </c>
       <c r="P31" s="89"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B32" s="81" t="s">
         <v>279</v>
       </c>
@@ -6380,7 +6380,7 @@
       <c r="I32" s="89"/>
       <c r="J32" s="24"/>
       <c r="L32" s="91"/>
-      <c r="M32" s="96"/>
+      <c r="M32" s="105"/>
       <c r="N32">
         <v>1</v>
       </c>
@@ -6389,7 +6389,7 @@
       </c>
       <c r="P32" s="89"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B33" s="81" t="s">
         <v>281</v>
       </c>
@@ -6402,7 +6402,7 @@
       <c r="I33" s="89"/>
       <c r="J33" s="24"/>
       <c r="L33" s="91"/>
-      <c r="M33" s="96"/>
+      <c r="M33" s="105"/>
       <c r="N33">
         <v>2</v>
       </c>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="P33" s="89"/>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B34" s="81" t="s">
         <v>289</v>
       </c>
@@ -6423,7 +6423,7 @@
       <c r="G34" s="24"/>
       <c r="I34" s="89"/>
       <c r="L34" s="91"/>
-      <c r="M34" s="96"/>
+      <c r="M34" s="105"/>
       <c r="N34">
         <v>1.5</v>
       </c>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="P34" s="89"/>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B35" s="81" t="s">
         <v>290</v>
       </c>
@@ -6444,7 +6444,7 @@
       <c r="G35" s="24"/>
       <c r="I35" s="89"/>
       <c r="L35" s="91"/>
-      <c r="M35" s="96"/>
+      <c r="M35" s="105"/>
       <c r="N35">
         <v>2.5</v>
       </c>
@@ -6453,7 +6453,7 @@
       </c>
       <c r="P35" s="89"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B36" s="81" t="s">
         <v>291</v>
       </c>
@@ -6465,7 +6465,7 @@
       <c r="G36" s="24"/>
       <c r="I36" s="89"/>
       <c r="L36" s="91"/>
-      <c r="M36" s="96"/>
+      <c r="M36" s="105"/>
       <c r="N36">
         <v>1.5</v>
       </c>
@@ -6474,297 +6474,280 @@
       </c>
       <c r="P36" s="89"/>
     </row>
-    <row r="37" spans="2:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="B37" s="29" t="s">
-        <v>215</v>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B37" s="81" t="s">
+        <v>293</v>
       </c>
       <c r="C37" s="92" t="s">
-        <v>103</v>
-      </c>
-      <c r="D37" s="24">
-        <v>2</v>
-      </c>
-      <c r="E37" s="31">
-        <v>50</v>
-      </c>
-      <c r="F37" s="91" t="s">
-        <v>272</v>
-      </c>
-      <c r="G37" s="24">
-        <v>2</v>
-      </c>
-      <c r="H37" s="31">
-        <v>100</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="D37" s="24"/>
+      <c r="F37" s="89"/>
+      <c r="G37" s="24"/>
       <c r="I37" s="89"/>
-      <c r="J37" s="24"/>
       <c r="L37" s="91"/>
-      <c r="M37" s="96"/>
-      <c r="N37"/>
+      <c r="M37" s="105"/>
+      <c r="N37">
+        <v>1.5</v>
+      </c>
+      <c r="O37" s="31">
+        <v>100</v>
+      </c>
       <c r="P37" s="89"/>
     </row>
-    <row r="38" spans="2:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="B38" s="29" t="s">
-        <v>216</v>
+    <row r="38" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B38" s="81" t="s">
+        <v>294</v>
       </c>
       <c r="C38" s="92" t="s">
-        <v>103</v>
-      </c>
-      <c r="D38" s="24">
-        <v>1</v>
-      </c>
-      <c r="E38" s="31">
-        <v>25</v>
-      </c>
-      <c r="F38" s="91" t="s">
-        <v>273</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="D38" s="24"/>
+      <c r="F38" s="89"/>
       <c r="G38" s="24"/>
       <c r="I38" s="89"/>
-      <c r="J38" s="24">
-        <v>4</v>
-      </c>
-      <c r="K38" s="31">
-        <v>100</v>
-      </c>
       <c r="L38" s="91"/>
-      <c r="M38" s="96"/>
-      <c r="N38"/>
+      <c r="M38" s="105"/>
+      <c r="N38">
+        <v>0.75</v>
+      </c>
+      <c r="O38" s="31">
+        <v>100</v>
+      </c>
       <c r="P38" s="89"/>
     </row>
-    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C39" s="92" t="s">
         <v>103</v>
       </c>
       <c r="D39" s="24">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E39" s="31">
-        <v>100</v>
-      </c>
-      <c r="F39" s="89"/>
-      <c r="G39" s="24"/>
+        <v>50</v>
+      </c>
+      <c r="F39" s="91" t="s">
+        <v>272</v>
+      </c>
+      <c r="G39" s="24">
+        <v>2</v>
+      </c>
+      <c r="H39" s="31">
+        <v>100</v>
+      </c>
       <c r="I39" s="89"/>
       <c r="J39" s="24"/>
       <c r="L39" s="91"/>
-      <c r="M39" s="96"/>
+      <c r="M39" s="105"/>
       <c r="N39"/>
       <c r="P39" s="89"/>
     </row>
-    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C40" s="92" t="s">
         <v>103</v>
       </c>
       <c r="D40" s="24">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E40" s="31">
-        <v>100</v>
-      </c>
-      <c r="F40" s="89"/>
+        <v>25</v>
+      </c>
+      <c r="F40" s="91" t="s">
+        <v>273</v>
+      </c>
       <c r="G40" s="24"/>
       <c r="I40" s="89"/>
-      <c r="J40" s="24"/>
+      <c r="J40" s="24">
+        <v>4</v>
+      </c>
+      <c r="K40" s="31">
+        <v>100</v>
+      </c>
       <c r="L40" s="91"/>
-      <c r="M40" s="96"/>
+      <c r="M40" s="105"/>
       <c r="N40"/>
       <c r="P40" s="89"/>
     </row>
-    <row r="41" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C41" s="92" t="s">
         <v>103</v>
       </c>
       <c r="D41" s="24">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E41" s="31">
-        <v>25</v>
-      </c>
-      <c r="F41" s="89" t="s">
-        <v>271</v>
-      </c>
-      <c r="G41" s="24">
-        <v>2</v>
-      </c>
-      <c r="H41" s="31">
-        <v>75</v>
-      </c>
-      <c r="I41" s="91" t="s">
-        <v>270</v>
-      </c>
-      <c r="J41" s="24">
-        <v>1</v>
-      </c>
-      <c r="K41" s="31">
-        <v>100</v>
-      </c>
-      <c r="L41" s="91" t="s">
-        <v>282</v>
-      </c>
-      <c r="M41" s="96"/>
+        <v>100</v>
+      </c>
+      <c r="F41" s="89"/>
+      <c r="G41" s="24"/>
+      <c r="I41" s="89"/>
+      <c r="J41" s="24"/>
+      <c r="L41" s="91"/>
+      <c r="M41" s="105"/>
       <c r="N41"/>
       <c r="P41" s="89"/>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C42" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="D42" s="24"/>
+      <c r="D42" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="E42" s="31">
+        <v>100</v>
+      </c>
       <c r="F42" s="89"/>
-      <c r="G42" s="24">
-        <v>3</v>
-      </c>
-      <c r="H42" s="31">
-        <v>100</v>
-      </c>
+      <c r="G42" s="24"/>
       <c r="I42" s="89"/>
       <c r="J42" s="24"/>
       <c r="L42" s="91"/>
-      <c r="M42" s="96"/>
+      <c r="M42" s="105"/>
       <c r="N42"/>
       <c r="P42" s="89"/>
     </row>
-    <row r="43" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
-        <v>266</v>
+        <v>222</v>
       </c>
       <c r="C43" s="92" t="s">
         <v>103</v>
       </c>
+      <c r="D43" s="24">
+        <v>1</v>
+      </c>
+      <c r="E43" s="31">
+        <v>25</v>
+      </c>
+      <c r="F43" s="89" t="s">
+        <v>271</v>
+      </c>
       <c r="G43" s="24">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H43" s="31">
-        <v>100</v>
-      </c>
-      <c r="I43" s="90" t="s">
-        <v>269</v>
-      </c>
-      <c r="J43" s="24"/>
-      <c r="L43" s="91"/>
-      <c r="M43" s="96"/>
+        <v>75</v>
+      </c>
+      <c r="I43" s="91" t="s">
+        <v>270</v>
+      </c>
+      <c r="J43" s="24">
+        <v>1</v>
+      </c>
+      <c r="K43" s="31">
+        <v>100</v>
+      </c>
+      <c r="L43" s="91" t="s">
+        <v>282</v>
+      </c>
+      <c r="M43" s="105"/>
       <c r="N43"/>
       <c r="P43" s="89"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
-        <v>267</v>
+        <v>221</v>
       </c>
       <c r="C44" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="G44" s="24"/>
-      <c r="J44" s="24">
-        <v>2</v>
-      </c>
-      <c r="K44" s="31">
-        <v>100</v>
-      </c>
+      <c r="D44" s="24"/>
+      <c r="F44" s="89"/>
+      <c r="G44" s="24">
+        <v>3</v>
+      </c>
+      <c r="H44" s="31">
+        <v>100</v>
+      </c>
+      <c r="I44" s="89"/>
+      <c r="J44" s="24"/>
       <c r="L44" s="91"/>
-      <c r="M44" s="96"/>
+      <c r="M44" s="105"/>
       <c r="N44"/>
       <c r="P44" s="89"/>
     </row>
-    <row r="45" spans="2:16" ht="165" x14ac:dyDescent="0.25">
-      <c r="B45" s="79" t="s">
-        <v>268</v>
+    <row r="45" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+      <c r="B45" s="29" t="s">
+        <v>266</v>
       </c>
       <c r="C45" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="G45" s="24"/>
-      <c r="J45" s="24">
-        <v>4</v>
-      </c>
-      <c r="K45" s="31">
-        <v>90</v>
-      </c>
-      <c r="L45" s="91" t="s">
-        <v>275</v>
-      </c>
-      <c r="M45" s="96"/>
-      <c r="N45">
-        <v>1</v>
-      </c>
-      <c r="O45" s="31">
-        <v>100</v>
-      </c>
+      <c r="G45" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="H45" s="31">
+        <v>100</v>
+      </c>
+      <c r="I45" s="90" t="s">
+        <v>269</v>
+      </c>
+      <c r="J45" s="24"/>
+      <c r="L45" s="91"/>
+      <c r="M45" s="105"/>
+      <c r="N45"/>
       <c r="P45" s="89"/>
     </row>
-    <row r="46" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
-        <v>239</v>
+        <v>267</v>
       </c>
       <c r="C46" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="D46" s="24"/>
-      <c r="F46" s="89"/>
       <c r="G46" s="24"/>
-      <c r="I46" s="89"/>
       <c r="J46" s="24">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K46" s="31">
         <v>100</v>
       </c>
-      <c r="L46" s="91" t="s">
-        <v>274</v>
-      </c>
-      <c r="M46" s="96"/>
+      <c r="L46" s="91"/>
+      <c r="M46" s="105"/>
       <c r="N46"/>
       <c r="P46" s="89"/>
     </row>
-    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B47" s="29" t="s">
-        <v>276</v>
+    <row r="47" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="B47" s="79" t="s">
+        <v>268</v>
       </c>
       <c r="C47" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="D47" s="31">
+      <c r="G47" s="24"/>
+      <c r="J47" s="24">
+        <v>4</v>
+      </c>
+      <c r="K47" s="31">
+        <v>90</v>
+      </c>
+      <c r="L47" s="91" t="s">
+        <v>275</v>
+      </c>
+      <c r="M47" s="105"/>
+      <c r="N47">
         <v>1</v>
       </c>
-      <c r="E47" s="31">
-        <v>10</v>
-      </c>
-      <c r="G47" s="24">
-        <v>2</v>
-      </c>
-      <c r="H47" s="31">
-        <v>30</v>
-      </c>
-      <c r="J47" s="24">
-        <v>2</v>
-      </c>
-      <c r="K47" s="31">
-        <v>50</v>
-      </c>
-      <c r="L47" s="91"/>
-      <c r="M47" s="96"/>
-      <c r="N47">
-        <v>4</v>
-      </c>
       <c r="O47" s="31">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="P47" s="89"/>
     </row>
-    <row r="48" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B48" s="29" t="s">
-        <v>277</v>
+        <v>239</v>
       </c>
       <c r="C48" s="92" t="s">
         <v>103</v>
@@ -6774,45 +6757,56 @@
       <c r="G48" s="24"/>
       <c r="I48" s="89"/>
       <c r="J48" s="24">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K48" s="31">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="L48" s="91" t="s">
-        <v>283</v>
-      </c>
-      <c r="M48" s="96"/>
+        <v>274</v>
+      </c>
+      <c r="M48" s="105"/>
       <c r="N48"/>
       <c r="P48" s="89"/>
     </row>
-    <row r="49" spans="2:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="B49" s="79" t="s">
-        <v>287</v>
+    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B49" s="29" t="s">
+        <v>276</v>
       </c>
       <c r="C49" s="92" t="s">
         <v>103</v>
       </c>
-      <c r="D49" s="24"/>
-      <c r="F49" s="89"/>
-      <c r="G49" s="24"/>
-      <c r="I49" s="89"/>
-      <c r="J49" s="24"/>
+      <c r="D49" s="31">
+        <v>1</v>
+      </c>
+      <c r="E49" s="31">
+        <v>10</v>
+      </c>
+      <c r="G49" s="24">
+        <v>2</v>
+      </c>
+      <c r="H49" s="31">
+        <v>30</v>
+      </c>
+      <c r="J49" s="24">
+        <v>2</v>
+      </c>
+      <c r="K49" s="31">
+        <v>50</v>
+      </c>
       <c r="L49" s="91"/>
-      <c r="M49" s="96"/>
+      <c r="M49" s="105"/>
       <c r="N49">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="O49" s="31">
-        <v>100</v>
-      </c>
-      <c r="P49" s="91" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B50" s="79" t="s">
-        <v>284</v>
+        <v>75</v>
+      </c>
+      <c r="P49" s="89"/>
+    </row>
+    <row r="50" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B50" s="29" t="s">
+        <v>277</v>
       </c>
       <c r="C50" s="92" t="s">
         <v>103</v>
@@ -6821,80 +6815,128 @@
       <c r="F50" s="89"/>
       <c r="G50" s="24"/>
       <c r="I50" s="89"/>
-      <c r="J50" s="24"/>
-      <c r="L50" s="91"/>
-      <c r="M50" s="96"/>
-      <c r="N50">
+      <c r="J50" s="24">
         <v>1</v>
       </c>
-      <c r="O50" s="31">
-        <v>100</v>
-      </c>
+      <c r="K50" s="31">
+        <v>75</v>
+      </c>
+      <c r="L50" s="91" t="s">
+        <v>283</v>
+      </c>
+      <c r="M50" s="105"/>
+      <c r="N50"/>
       <c r="P50" s="89"/>
     </row>
-    <row r="51" spans="2:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="B51" s="29" t="s">
+    <row r="51" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B51" s="79" t="s">
+        <v>287</v>
+      </c>
+      <c r="C51" s="92" t="s">
+        <v>103</v>
+      </c>
+      <c r="D51" s="24"/>
+      <c r="F51" s="89"/>
+      <c r="G51" s="24"/>
+      <c r="I51" s="89"/>
+      <c r="J51" s="24"/>
+      <c r="L51" s="91"/>
+      <c r="M51" s="105"/>
+      <c r="N51">
+        <v>0.5</v>
+      </c>
+      <c r="O51" s="31">
+        <v>100</v>
+      </c>
+      <c r="P51" s="91" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B52" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="C52" s="92" t="s">
+        <v>103</v>
+      </c>
+      <c r="D52" s="24"/>
+      <c r="F52" s="89"/>
+      <c r="G52" s="24"/>
+      <c r="I52" s="89"/>
+      <c r="J52" s="24"/>
+      <c r="L52" s="91"/>
+      <c r="M52" s="105"/>
+      <c r="N52">
+        <v>1</v>
+      </c>
+      <c r="O52" s="31">
+        <v>100</v>
+      </c>
+      <c r="P52" s="89"/>
+    </row>
+    <row r="53" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+      <c r="B53" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="C51" s="31" t="s">
+      <c r="C53" s="31" t="s">
         <v>103</v>
       </c>
-      <c r="F51" s="89"/>
-      <c r="I51" s="89"/>
-      <c r="L51" s="91"/>
-      <c r="M51" s="96"/>
-      <c r="N51"/>
-      <c r="P51" s="91" t="s">
+      <c r="F53" s="89"/>
+      <c r="I53" s="89"/>
+      <c r="L53" s="91"/>
+      <c r="M53" s="105"/>
+      <c r="N53"/>
+      <c r="P53" s="91" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B52" s="29" t="s">
+    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="B54" s="29" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B53" s="29"/>
-    </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B54" s="29"/>
-    </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B55" s="29"/>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B56" s="29"/>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B57" s="29"/>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B58" s="29"/>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B59" s="29"/>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B60" s="29"/>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B61" s="29"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B62" s="29"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B63" s="29"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B64" s="29"/>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B65" s="29"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B66" s="29"/>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B67" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="M8:M51"/>
+    <mergeCell ref="M8:M53"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="B6:B7"/>
@@ -6933,22 +6975,22 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:B10">
     <cfRule type="expression" dxfId="30" priority="259">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:B14 B16:B18">
     <cfRule type="expression" dxfId="29" priority="366">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
     <cfRule type="expression" dxfId="28" priority="542">
-      <formula>MAX($E42,$H42,$K42)=100</formula>
+      <formula>MAX($E44,$H44,$K44)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12 B16">
     <cfRule type="expression" dxfId="27" priority="549">
-      <formula>MAX($E42,$H42,$K42)=100</formula>
+      <formula>MAX($E44,$H44,$K44)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
@@ -6958,7 +7000,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:B15 B17:B19">
     <cfRule type="expression" dxfId="25" priority="727">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
+      <formula>MAX($E41,$H41,$K41)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14">
@@ -6968,22 +7010,22 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
     <cfRule type="expression" dxfId="23" priority="603">
-      <formula>MAX($E46,$H46,$K46)=100</formula>
+      <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:B16">
     <cfRule type="expression" dxfId="22" priority="329">
-      <formula>MAX($E37,$H37,$K37)=100</formula>
+      <formula>MAX($E39,$H39,$K39)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B17">
+  <conditionalFormatting sqref="B17 B22">
     <cfRule type="expression" dxfId="21" priority="544">
-      <formula>MAX($E42,$H42,$K42)=100</formula>
+      <formula>MAX($E44,$H44,$K44)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:B19">
     <cfRule type="expression" dxfId="20" priority="367">
-      <formula>MAX($E39,$H39,$K39)=100</formula>
+      <formula>MAX($E41,$H41,$K41)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:B21">
@@ -6991,14 +7033,14 @@
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20 B22">
+  <conditionalFormatting sqref="B20">
     <cfRule type="expression" dxfId="18" priority="629">
-      <formula>MAX($E45,$H45,$K45)=100</formula>
+      <formula>MAX($E47,$H47,$K47)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:B21 B23:B24">
     <cfRule type="expression" dxfId="17" priority="399">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:B22">
@@ -7008,17 +7050,17 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:B24">
     <cfRule type="expression" dxfId="15" priority="619">
-      <formula>MAX($E47,$H47,$K47)=100</formula>
+      <formula>MAX($E49,$H49,$K49)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
     <cfRule type="expression" dxfId="14" priority="633">
-      <formula>MAX($E46,$H46,$K46)=100</formula>
+      <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23">
     <cfRule type="expression" dxfId="13" priority="609">
-      <formula>MAX($E46,$H46,$K46)=100</formula>
+      <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:B24">
@@ -7026,29 +7068,29 @@
       <formula>MAX($E11,$H11,$K11)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B36">
+  <conditionalFormatting sqref="B23:B38">
     <cfRule type="expression" dxfId="11" priority="12">
       <formula>MAX(#REF!,#REF!,#REF!)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:B65">
+  <conditionalFormatting sqref="B23:B67">
     <cfRule type="expression" dxfId="10" priority="1">
       <formula>MAX($E23,$H23,$K23)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24 B27">
     <cfRule type="expression" dxfId="9" priority="621">
-      <formula>MAX($E43,$H43,$K43)=100</formula>
+      <formula>MAX($E45,$H45,$K45)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25 B27:B29">
     <cfRule type="expression" dxfId="8" priority="593">
-      <formula>MAX($E41,$H41,$K41)=100</formula>
+      <formula>MAX($E43,$H43,$K43)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:B26 B28:B31">
     <cfRule type="expression" dxfId="7" priority="670">
-      <formula>MAX($E40,$H40,$K40)=100</formula>
+      <formula>MAX($E42,$H42,$K42)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:B31">
@@ -7058,26 +7100,26 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B26">
     <cfRule type="expression" dxfId="5" priority="635">
-      <formula>MAX($E46,$H46,$K46)=100</formula>
+      <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32:B36">
-    <cfRule type="expression" dxfId="4" priority="695">
-      <formula>MAX($E46,$H46,$K46)=100</formula>
+  <conditionalFormatting sqref="C6:C52">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="677">
-      <formula>MAX($E15,$H15,$K15)=100</formula>
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>$C6="Charlotte"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C50">
     <cfRule type="expression" dxfId="2" priority="4">
       <formula>$C6="Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
-      <formula>$C6="Charlotte"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:B38">
+    <cfRule type="expression" dxfId="1" priority="766">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>$C6="Charlotte/Eddy"</formula>
+    <cfRule type="expression" dxfId="0" priority="767">
+      <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7091,28 +7133,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
-    <col min="2" max="2" width="93.28515625" customWidth="1"/>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
+    <col min="2" max="2" width="93.33203125" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="42.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.6">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -7129,7 +7171,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -7142,7 +7184,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -7155,7 +7197,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -7168,7 +7210,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -7181,7 +7223,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -7194,7 +7236,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -7207,7 +7249,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -7220,7 +7262,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -7233,7 +7275,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -7246,7 +7288,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -7259,7 +7301,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -7272,7 +7314,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -7285,7 +7327,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -7298,7 +7340,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -7311,7 +7353,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -7324,7 +7366,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -7337,7 +7379,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -7350,7 +7392,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -7363,7 +7405,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -7376,7 +7418,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -7389,7 +7431,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -7402,7 +7444,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -7415,7 +7457,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -7428,7 +7470,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -7441,7 +7483,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -7454,7 +7496,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -7467,7 +7509,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -7480,7 +7522,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -7493,7 +7535,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -7506,7 +7548,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -7519,7 +7561,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -7532,7 +7574,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -7545,7 +7587,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -7558,7 +7600,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -7571,7 +7613,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -7584,7 +7626,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -7597,7 +7639,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -7610,7 +7652,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -7623,7 +7665,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -7636,7 +7678,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -7649,7 +7691,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -7662,7 +7704,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -7675,7 +7717,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -7688,7 +7730,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -7701,7 +7743,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -7714,7 +7756,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -7727,7 +7769,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -7740,7 +7782,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -7753,7 +7795,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -7766,7 +7808,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -7779,7 +7821,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -7792,7 +7834,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -7805,7 +7847,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -7818,7 +7860,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -7831,7 +7873,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -7844,7 +7886,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -7857,7 +7899,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -7870,7 +7912,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -7883,7 +7925,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -7896,7 +7938,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -7907,7 +7949,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -7918,7 +7960,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -7929,7 +7971,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -7940,7 +7982,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -7951,7 +7993,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -7962,7 +8004,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -7973,7 +8015,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -7984,7 +8026,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -7995,7 +8037,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B74" s="3" t="s">
         <v>106</v>
       </c>
@@ -8006,7 +8048,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B75" s="3" t="s">
         <v>107</v>
       </c>
@@ -8017,182 +8059,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
arrangé les cls d'authentification perdues après redémarrage
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C165DBAF-A721-4F81-A2CC-AF9EC8C572A1}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E45BC96-B1C2-422B-BADA-3B289994C7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,6 +35,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -42,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="298">
   <si>
     <t>Planification globale</t>
   </si>
@@ -929,6 +935,15 @@
   </si>
   <si>
     <t>Ajouter le vrai nom du joueur au lieu de hardcoder + faire clignoter nom du joueur qui joue</t>
+  </si>
+  <si>
+    <t>Passé d'environs 1000 à environs 2000. Retiré le deepcopy</t>
+  </si>
+  <si>
+    <t>Authentification key recconue après redémarrage du serveur</t>
+  </si>
+  <si>
+    <t>User n'a plus à se reconnecter, mais les parties en cours sont perdues et restent affichées</t>
   </si>
 </sst>
 </file>
@@ -1692,14 +1707,23 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1714,28 +1738,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1745,14 +1760,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
+          <bgColor rgb="FFCCFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1760,13 +1768,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFCFDCF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1780,6 +1781,20 @@
             <color rgb="FFCCFFFF"/>
           </stop>
         </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -2490,26 +2505,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
-    <col min="5" max="5" width="42.6640625" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="42.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
+    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2523,7 +2538,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2537,7 +2552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2551,7 +2566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2565,7 +2580,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2579,7 +2594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2593,7 +2608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2607,7 +2622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2621,7 +2636,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2635,7 +2650,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2649,7 +2664,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2663,7 +2678,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2677,7 +2692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2691,7 +2706,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2705,7 +2720,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2719,7 +2734,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2733,7 +2748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2747,7 +2762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2761,7 +2776,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2775,7 +2790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2789,7 +2804,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2803,7 +2818,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -2817,7 +2832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -2831,7 +2846,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -2845,7 +2860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -2859,7 +2874,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -2873,7 +2888,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -2887,7 +2902,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -2901,7 +2916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -2915,7 +2930,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -2929,7 +2944,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -2943,7 +2958,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -2957,7 +2972,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -2971,8 +2986,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -3007,32 +3022,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5546875" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.6640625" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" customWidth="1"/>
-    <col min="8" max="8" width="16.33203125" customWidth="1"/>
-    <col min="9" max="9" width="18.6640625" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" customWidth="1"/>
-    <col min="11" max="11" width="16.33203125" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
-    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19.7109375" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" customWidth="1"/>
+    <col min="8" max="8" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" customWidth="1"/>
+    <col min="10" max="10" width="9.5703125" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" customWidth="1"/>
+    <col min="12" max="12" width="18.5703125" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" customWidth="1"/>
+    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="1:18" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -3062,7 +3077,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -3116,7 +3131,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -3143,7 +3158,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -3165,7 +3180,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -3192,7 +3207,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -3225,7 +3240,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -3262,7 +3277,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -3299,7 +3314,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -3331,7 +3346,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3359,7 +3374,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3386,15 +3401,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.25">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.25">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.25">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3410,44 +3425,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
-    <col min="2" max="2" width="77.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
+    <col min="2" max="2" width="77.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.5703125" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B3" s="95" t="s">
+    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="B3" s="107" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="97"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="B5" s="98" t="s">
+      <c r="C3" s="108"/>
+      <c r="D3" s="108"/>
+      <c r="E3" s="108"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="108"/>
+      <c r="H3" s="108"/>
+      <c r="I3" s="108"/>
+      <c r="J3" s="108"/>
+      <c r="K3" s="108"/>
+      <c r="L3" s="109"/>
+    </row>
+    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="B5" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="100" t="s">
+      <c r="C5" s="103" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3456,7 +3471,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="102" t="s">
+      <c r="F5" s="99" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3465,7 +3480,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="102" t="s">
+      <c r="I5" s="99" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3474,36 +3489,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="102" t="s">
+      <c r="L5" s="99" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="99"/>
-      <c r="C6" s="101"/>
+    <row r="6" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="102"/>
+      <c r="C6" s="104"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="103"/>
+      <c r="F6" s="100"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="103"/>
+      <c r="I6" s="100"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="103"/>
-    </row>
-    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="L6" s="100"/>
+    </row>
+    <row r="7" spans="2:12" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3526,7 +3541,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3545,7 +3560,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3564,7 +3579,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3583,7 +3598,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3602,7 +3617,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3621,7 +3636,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3640,7 +3655,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3659,7 +3674,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3678,7 +3693,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3697,7 +3712,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3716,7 +3731,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3735,7 +3750,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3754,7 +3769,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3773,7 +3788,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3794,7 +3809,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3813,7 +3828,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3834,7 +3849,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3853,7 +3868,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3872,7 +3887,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3893,7 +3908,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3914,7 +3929,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3935,7 +3950,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3954,7 +3969,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -3973,7 +3988,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -3992,7 +4007,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -4011,7 +4026,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -4030,7 +4045,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -4049,7 +4064,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -4068,7 +4083,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -4087,7 +4102,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -4106,7 +4121,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -4125,7 +4140,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -4144,7 +4159,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -4163,7 +4178,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -4182,7 +4197,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -4201,7 +4216,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -4220,7 +4235,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -4239,7 +4254,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -4258,7 +4273,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -4277,7 +4292,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -4296,7 +4311,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -4401,43 +4416,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.33203125" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.6640625" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.7109375" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.44140625" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B1" s="95" t="s">
+    <row r="1" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
+      <c r="B1" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="97"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
-      <c r="B4" s="98" t="s">
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="109"/>
+    </row>
+    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="B4" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="100" t="s">
+      <c r="C4" s="103" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4446,7 +4461,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="102" t="s">
+      <c r="F4" s="99" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4455,7 +4470,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="102" t="s">
+      <c r="I4" s="99" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4464,36 +4479,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="102" t="s">
+      <c r="L4" s="99" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="99"/>
-      <c r="C5" s="101"/>
+    <row r="5" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="102"/>
+      <c r="C5" s="104"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="103"/>
+      <c r="F5" s="100"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="103"/>
+      <c r="I5" s="100"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="103"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
+      <c r="L5" s="100"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4511,7 +4526,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4529,7 +4544,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4547,7 +4562,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4565,7 +4580,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4583,7 +4598,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4601,7 +4616,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4619,7 +4634,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4637,7 +4652,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4655,7 +4670,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4673,7 +4688,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4691,7 +4706,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4709,7 +4724,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4727,7 +4742,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4745,7 +4760,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4764,7 +4779,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4783,7 +4798,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4802,7 +4817,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -4821,7 +4836,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -4840,7 +4855,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -4859,7 +4874,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -4878,7 +4893,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -4897,7 +4912,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -4916,7 +4931,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -4935,7 +4950,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -4954,7 +4969,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -4973,7 +4988,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -4992,7 +5007,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -5011,7 +5026,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -5032,7 +5047,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -5052,7 +5067,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -5072,7 +5087,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -5092,7 +5107,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -5112,7 +5127,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -5132,7 +5147,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -5152,7 +5167,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -5174,7 +5189,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -5194,7 +5209,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -5214,7 +5229,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -5234,7 +5249,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -5252,7 +5267,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -5270,7 +5285,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:12" ht="60" x14ac:dyDescent="0.25">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -5295,7 +5310,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -5313,7 +5328,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -5331,7 +5346,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5354,7 +5369,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5377,7 +5392,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5395,7 +5410,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5413,7 +5428,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5430,7 +5445,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5448,7 +5463,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5465,7 +5480,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5488,7 +5503,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:12" ht="45" x14ac:dyDescent="0.25">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5515,7 +5530,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5533,7 +5548,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5597,21 +5612,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" customWidth="1"/>
-    <col min="2" max="2" width="81.5546875" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="81.5703125" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.6640625" customWidth="1"/>
-    <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" customWidth="1"/>
+    <col min="5" max="5" width="28.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:5" ht="46.5" x14ac:dyDescent="0.7">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:5" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5625,7 +5640,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B4" s="85" t="s">
         <v>226</v>
       </c>
@@ -5639,7 +5654,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:5" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="73" t="s">
         <v>240</v>
       </c>
@@ -5653,7 +5668,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B6" s="86" t="s">
         <v>241</v>
       </c>
@@ -5667,7 +5682,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="86" t="s">
         <v>230</v>
       </c>
@@ -5681,7 +5696,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
       <c r="B8" s="73" t="s">
         <v>233</v>
       </c>
@@ -5695,7 +5710,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5" ht="60" x14ac:dyDescent="0.25">
       <c r="B9" s="86" t="s">
         <v>179</v>
       </c>
@@ -5709,7 +5724,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="82" t="s">
         <v>68</v>
       </c>
@@ -5736,49 +5751,49 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B2:P67"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" customWidth="1"/>
-    <col min="2" max="2" width="67.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" style="31" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="31" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5546875" style="90" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="2" max="2" width="67.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" style="31" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" style="31" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.5703125" style="90" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5703125" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="46.2" x14ac:dyDescent="0.85">
-      <c r="B2" s="106" t="s">
+    <row r="2" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
+      <c r="B2" s="97" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
-      <c r="H2" s="107"/>
-      <c r="I2" s="107"/>
-      <c r="J2" s="107"/>
-      <c r="K2" s="107"/>
-      <c r="L2" s="107"/>
-      <c r="M2" s="107"/>
-      <c r="N2" s="107"/>
-      <c r="O2" s="107"/>
-      <c r="P2" s="107"/>
-    </row>
-    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.4">
-      <c r="B6" s="98" t="s">
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="98"/>
+      <c r="O2" s="98"/>
+      <c r="P2" s="98"/>
+    </row>
+    <row r="5" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.35">
+      <c r="B6" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="C6" s="103" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="88" t="s">
@@ -5787,7 +5802,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="102" t="s">
+      <c r="F6" s="99" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5796,7 +5811,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="102" t="s">
+      <c r="I6" s="99" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="60" t="s">
@@ -5805,7 +5820,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="108" t="s">
+      <c r="L6" s="105" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="43">
@@ -5817,34 +5832,34 @@
       <c r="O6" s="43">
         <v>46167</v>
       </c>
-      <c r="P6" s="102" t="s">
+      <c r="P6" s="99" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="99"/>
-      <c r="C7" s="101"/>
+    <row r="7" spans="2:16" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="102"/>
+      <c r="C7" s="104"/>
       <c r="D7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="103"/>
+      <c r="F7" s="100"/>
       <c r="G7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="103"/>
+      <c r="I7" s="100"/>
       <c r="J7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="109"/>
+      <c r="L7" s="106"/>
       <c r="M7" s="94" t="s">
         <v>201</v>
       </c>
@@ -5854,9 +5869,9 @@
       <c r="O7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="103"/>
-    </row>
-    <row r="8" spans="2:16" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P7" s="100"/>
+    </row>
+    <row r="8" spans="2:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="79" t="s">
         <v>68</v>
       </c>
@@ -5874,13 +5889,13 @@
       <c r="I8" s="89"/>
       <c r="J8" s="24"/>
       <c r="L8" s="91"/>
-      <c r="M8" s="104" t="s">
+      <c r="M8" s="95" t="s">
         <v>278</v>
       </c>
       <c r="N8"/>
       <c r="P8" s="89"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B9" s="79" t="s">
         <v>256</v>
       </c>
@@ -5898,11 +5913,11 @@
       <c r="I9" s="89"/>
       <c r="J9" s="24"/>
       <c r="L9" s="91"/>
-      <c r="M9" s="105"/>
+      <c r="M9" s="96"/>
       <c r="N9"/>
       <c r="P9" s="89"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B10" s="79" t="s">
         <v>245</v>
       </c>
@@ -5920,11 +5935,11 @@
       <c r="I10" s="89"/>
       <c r="J10" s="24"/>
       <c r="L10" s="91"/>
-      <c r="M10" s="105"/>
+      <c r="M10" s="96"/>
       <c r="N10"/>
       <c r="P10" s="89"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="79" t="s">
         <v>244</v>
       </c>
@@ -5942,11 +5957,11 @@
       <c r="I11" s="89"/>
       <c r="J11" s="24"/>
       <c r="L11" s="91"/>
-      <c r="M11" s="105"/>
+      <c r="M11" s="96"/>
       <c r="N11"/>
       <c r="P11" s="89"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="79" t="s">
         <v>257</v>
       </c>
@@ -5963,11 +5978,11 @@
       <c r="I12" s="89"/>
       <c r="J12" s="24"/>
       <c r="L12" s="91"/>
-      <c r="M12" s="105"/>
+      <c r="M12" s="96"/>
       <c r="N12"/>
       <c r="P12" s="89"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
@@ -5984,11 +5999,11 @@
       <c r="I13" s="89"/>
       <c r="J13" s="24"/>
       <c r="L13" s="91"/>
-      <c r="M13" s="105"/>
+      <c r="M13" s="96"/>
       <c r="N13"/>
       <c r="P13" s="89"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
@@ -6005,11 +6020,11 @@
       <c r="I14" s="89"/>
       <c r="J14" s="24"/>
       <c r="L14" s="91"/>
-      <c r="M14" s="105"/>
+      <c r="M14" s="96"/>
       <c r="N14"/>
       <c r="P14" s="89"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
@@ -6026,11 +6041,11 @@
       <c r="I15" s="89"/>
       <c r="J15" s="24"/>
       <c r="L15" s="91"/>
-      <c r="M15" s="105"/>
+      <c r="M15" s="96"/>
       <c r="N15"/>
       <c r="P15" s="89"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
@@ -6047,11 +6062,11 @@
       <c r="I16" s="89"/>
       <c r="J16" s="24"/>
       <c r="L16" s="91"/>
-      <c r="M16" s="105"/>
+      <c r="M16" s="96"/>
       <c r="N16"/>
       <c r="P16" s="89"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
@@ -6067,11 +6082,11 @@
       <c r="I17" s="89"/>
       <c r="J17" s="24"/>
       <c r="L17" s="91"/>
-      <c r="M17" s="105"/>
+      <c r="M17" s="96"/>
       <c r="N17"/>
       <c r="P17" s="89"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
@@ -6087,11 +6102,11 @@
       <c r="I18" s="89"/>
       <c r="J18" s="24"/>
       <c r="L18" s="91"/>
-      <c r="M18" s="105"/>
+      <c r="M18" s="96"/>
       <c r="N18"/>
       <c r="P18" s="89"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
@@ -6107,11 +6122,11 @@
       <c r="I19" s="89"/>
       <c r="J19" s="24"/>
       <c r="L19" s="91"/>
-      <c r="M19" s="105"/>
+      <c r="M19" s="96"/>
       <c r="N19"/>
       <c r="P19" s="89"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
@@ -6127,11 +6142,11 @@
       <c r="I20" s="89"/>
       <c r="J20" s="24"/>
       <c r="L20" s="91"/>
-      <c r="M20" s="105"/>
+      <c r="M20" s="96"/>
       <c r="N20"/>
       <c r="P20" s="89"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
@@ -6147,11 +6162,11 @@
       <c r="I21" s="89"/>
       <c r="J21" s="24"/>
       <c r="L21" s="91"/>
-      <c r="M21" s="105"/>
+      <c r="M21" s="96"/>
       <c r="N21"/>
       <c r="P21" s="89"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="79" t="s">
         <v>255</v>
       </c>
@@ -6167,11 +6182,11 @@
       <c r="I22" s="89"/>
       <c r="J22" s="24"/>
       <c r="L22" s="91"/>
-      <c r="M22" s="105"/>
+      <c r="M22" s="96"/>
       <c r="N22"/>
       <c r="P22" s="89"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="80" t="s">
         <v>258</v>
       </c>
@@ -6189,11 +6204,11 @@
       <c r="I23" s="89"/>
       <c r="J23" s="24"/>
       <c r="L23" s="91"/>
-      <c r="M23" s="105"/>
+      <c r="M23" s="96"/>
       <c r="N23"/>
       <c r="P23" s="89"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="80" t="s">
         <v>259</v>
       </c>
@@ -6206,11 +6221,11 @@
       <c r="I24" s="89"/>
       <c r="J24" s="24"/>
       <c r="L24" s="91"/>
-      <c r="M24" s="105"/>
+      <c r="M24" s="96"/>
       <c r="N24"/>
       <c r="P24" s="89"/>
     </row>
-    <row r="25" spans="2:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="81" t="s">
         <v>260</v>
       </c>
@@ -6228,11 +6243,11 @@
         <v>100</v>
       </c>
       <c r="L25" s="91"/>
-      <c r="M25" s="105"/>
+      <c r="M25" s="96"/>
       <c r="N25"/>
       <c r="P25" s="89"/>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:16" ht="30" x14ac:dyDescent="0.25">
       <c r="B26" s="81" t="s">
         <v>261</v>
       </c>
@@ -6250,11 +6265,11 @@
         <v>100</v>
       </c>
       <c r="L26" s="91"/>
-      <c r="M26" s="105"/>
+      <c r="M26" s="96"/>
       <c r="N26"/>
       <c r="P26" s="89"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B27" s="81" t="s">
         <v>262</v>
       </c>
@@ -6272,11 +6287,11 @@
         <v>100</v>
       </c>
       <c r="L27" s="91"/>
-      <c r="M27" s="105"/>
+      <c r="M27" s="96"/>
       <c r="N27"/>
       <c r="P27" s="89"/>
     </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="81" t="s">
         <v>263</v>
       </c>
@@ -6294,11 +6309,11 @@
         <v>100</v>
       </c>
       <c r="L28" s="91"/>
-      <c r="M28" s="105"/>
+      <c r="M28" s="96"/>
       <c r="N28"/>
       <c r="P28" s="89"/>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:16" ht="30" x14ac:dyDescent="0.25">
       <c r="B29" s="81" t="s">
         <v>264</v>
       </c>
@@ -6316,11 +6331,11 @@
         <v>100</v>
       </c>
       <c r="L29" s="91"/>
-      <c r="M29" s="105"/>
+      <c r="M29" s="96"/>
       <c r="N29"/>
       <c r="P29" s="89"/>
     </row>
-    <row r="30" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:16" ht="30" x14ac:dyDescent="0.25">
       <c r="B30" s="81" t="s">
         <v>265</v>
       </c>
@@ -6338,11 +6353,11 @@
         <v>100</v>
       </c>
       <c r="L30" s="91"/>
-      <c r="M30" s="105"/>
+      <c r="M30" s="96"/>
       <c r="N30"/>
       <c r="P30" s="89"/>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B31" s="81" t="s">
         <v>280</v>
       </c>
@@ -6358,7 +6373,7 @@
         <v>100</v>
       </c>
       <c r="L31" s="91"/>
-      <c r="M31" s="105"/>
+      <c r="M31" s="96"/>
       <c r="N31">
         <v>2</v>
       </c>
@@ -6367,7 +6382,7 @@
       </c>
       <c r="P31" s="89"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B32" s="81" t="s">
         <v>279</v>
       </c>
@@ -6380,7 +6395,7 @@
       <c r="I32" s="89"/>
       <c r="J32" s="24"/>
       <c r="L32" s="91"/>
-      <c r="M32" s="105"/>
+      <c r="M32" s="96"/>
       <c r="N32">
         <v>1</v>
       </c>
@@ -6389,7 +6404,7 @@
       </c>
       <c r="P32" s="89"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B33" s="81" t="s">
         <v>281</v>
       </c>
@@ -6402,7 +6417,7 @@
       <c r="I33" s="89"/>
       <c r="J33" s="24"/>
       <c r="L33" s="91"/>
-      <c r="M33" s="105"/>
+      <c r="M33" s="96"/>
       <c r="N33">
         <v>2</v>
       </c>
@@ -6411,7 +6426,7 @@
       </c>
       <c r="P33" s="89"/>
     </row>
-    <row r="34" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B34" s="81" t="s">
         <v>289</v>
       </c>
@@ -6423,7 +6438,7 @@
       <c r="G34" s="24"/>
       <c r="I34" s="89"/>
       <c r="L34" s="91"/>
-      <c r="M34" s="105"/>
+      <c r="M34" s="96"/>
       <c r="N34">
         <v>1.5</v>
       </c>
@@ -6432,7 +6447,7 @@
       </c>
       <c r="P34" s="89"/>
     </row>
-    <row r="35" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B35" s="81" t="s">
         <v>290</v>
       </c>
@@ -6444,7 +6459,7 @@
       <c r="G35" s="24"/>
       <c r="I35" s="89"/>
       <c r="L35" s="91"/>
-      <c r="M35" s="105"/>
+      <c r="M35" s="96"/>
       <c r="N35">
         <v>2.5</v>
       </c>
@@ -6453,7 +6468,7 @@
       </c>
       <c r="P35" s="89"/>
     </row>
-    <row r="36" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B36" s="81" t="s">
         <v>291</v>
       </c>
@@ -6465,7 +6480,7 @@
       <c r="G36" s="24"/>
       <c r="I36" s="89"/>
       <c r="L36" s="91"/>
-      <c r="M36" s="105"/>
+      <c r="M36" s="96"/>
       <c r="N36">
         <v>1.5</v>
       </c>
@@ -6474,7 +6489,7 @@
       </c>
       <c r="P36" s="89"/>
     </row>
-    <row r="37" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B37" s="81" t="s">
         <v>293</v>
       </c>
@@ -6486,7 +6501,7 @@
       <c r="G37" s="24"/>
       <c r="I37" s="89"/>
       <c r="L37" s="91"/>
-      <c r="M37" s="105"/>
+      <c r="M37" s="96"/>
       <c r="N37">
         <v>1.5</v>
       </c>
@@ -6495,7 +6510,7 @@
       </c>
       <c r="P37" s="89"/>
     </row>
-    <row r="38" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:16" ht="30" x14ac:dyDescent="0.25">
       <c r="B38" s="81" t="s">
         <v>294</v>
       </c>
@@ -6507,7 +6522,7 @@
       <c r="G38" s="24"/>
       <c r="I38" s="89"/>
       <c r="L38" s="91"/>
-      <c r="M38" s="105"/>
+      <c r="M38" s="96"/>
       <c r="N38">
         <v>0.75</v>
       </c>
@@ -6516,7 +6531,7 @@
       </c>
       <c r="P38" s="89"/>
     </row>
-    <row r="39" spans="2:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:16" ht="45" x14ac:dyDescent="0.25">
       <c r="B39" s="29" t="s">
         <v>215</v>
       </c>
@@ -6541,11 +6556,11 @@
       <c r="I39" s="89"/>
       <c r="J39" s="24"/>
       <c r="L39" s="91"/>
-      <c r="M39" s="105"/>
+      <c r="M39" s="96"/>
       <c r="N39"/>
       <c r="P39" s="89"/>
     </row>
-    <row r="40" spans="2:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:16" ht="30" x14ac:dyDescent="0.25">
       <c r="B40" s="29" t="s">
         <v>216</v>
       </c>
@@ -6570,11 +6585,11 @@
         <v>100</v>
       </c>
       <c r="L40" s="91"/>
-      <c r="M40" s="105"/>
+      <c r="M40" s="96"/>
       <c r="N40"/>
       <c r="P40" s="89"/>
     </row>
-    <row r="41" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B41" s="29" t="s">
         <v>217</v>
       </c>
@@ -6592,11 +6607,11 @@
       <c r="I41" s="89"/>
       <c r="J41" s="24"/>
       <c r="L41" s="91"/>
-      <c r="M41" s="105"/>
+      <c r="M41" s="96"/>
       <c r="N41"/>
       <c r="P41" s="89"/>
     </row>
-    <row r="42" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B42" s="29" t="s">
         <v>218</v>
       </c>
@@ -6614,11 +6629,11 @@
       <c r="I42" s="89"/>
       <c r="J42" s="24"/>
       <c r="L42" s="91"/>
-      <c r="M42" s="105"/>
+      <c r="M42" s="96"/>
       <c r="N42"/>
       <c r="P42" s="89"/>
     </row>
-    <row r="43" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:16" ht="75" x14ac:dyDescent="0.25">
       <c r="B43" s="29" t="s">
         <v>222</v>
       </c>
@@ -6652,11 +6667,11 @@
       <c r="L43" s="91" t="s">
         <v>282</v>
       </c>
-      <c r="M43" s="105"/>
+      <c r="M43" s="96"/>
       <c r="N43"/>
       <c r="P43" s="89"/>
     </row>
-    <row r="44" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B44" s="29" t="s">
         <v>221</v>
       </c>
@@ -6674,11 +6689,11 @@
       <c r="I44" s="89"/>
       <c r="J44" s="24"/>
       <c r="L44" s="91"/>
-      <c r="M44" s="105"/>
+      <c r="M44" s="96"/>
       <c r="N44"/>
       <c r="P44" s="89"/>
     </row>
-    <row r="45" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:16" ht="75" x14ac:dyDescent="0.25">
       <c r="B45" s="29" t="s">
         <v>266</v>
       </c>
@@ -6696,11 +6711,11 @@
       </c>
       <c r="J45" s="24"/>
       <c r="L45" s="91"/>
-      <c r="M45" s="105"/>
+      <c r="M45" s="96"/>
       <c r="N45"/>
       <c r="P45" s="89"/>
     </row>
-    <row r="46" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B46" s="29" t="s">
         <v>267</v>
       </c>
@@ -6715,11 +6730,11 @@
         <v>100</v>
       </c>
       <c r="L46" s="91"/>
-      <c r="M46" s="105"/>
+      <c r="M46" s="96"/>
       <c r="N46"/>
       <c r="P46" s="89"/>
     </row>
-    <row r="47" spans="2:16" ht="158.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:16" ht="165" x14ac:dyDescent="0.25">
       <c r="B47" s="79" t="s">
         <v>268</v>
       </c>
@@ -6736,7 +6751,7 @@
       <c r="L47" s="91" t="s">
         <v>275</v>
       </c>
-      <c r="M47" s="105"/>
+      <c r="M47" s="96"/>
       <c r="N47">
         <v>1</v>
       </c>
@@ -6745,7 +6760,7 @@
       </c>
       <c r="P47" s="89"/>
     </row>
-    <row r="48" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:16" ht="75" x14ac:dyDescent="0.25">
       <c r="B48" s="29" t="s">
         <v>239</v>
       </c>
@@ -6765,11 +6780,11 @@
       <c r="L48" s="91" t="s">
         <v>274</v>
       </c>
-      <c r="M48" s="105"/>
+      <c r="M48" s="96"/>
       <c r="N48"/>
       <c r="P48" s="89"/>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B49" s="29" t="s">
         <v>276</v>
       </c>
@@ -6795,7 +6810,7 @@
         <v>50</v>
       </c>
       <c r="L49" s="91"/>
-      <c r="M49" s="105"/>
+      <c r="M49" s="96"/>
       <c r="N49">
         <v>4</v>
       </c>
@@ -6804,7 +6819,7 @@
       </c>
       <c r="P49" s="89"/>
     </row>
-    <row r="50" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:16" ht="75" x14ac:dyDescent="0.25">
       <c r="B50" s="29" t="s">
         <v>277</v>
       </c>
@@ -6824,11 +6839,11 @@
       <c r="L50" s="91" t="s">
         <v>283</v>
       </c>
-      <c r="M50" s="105"/>
+      <c r="M50" s="96"/>
       <c r="N50"/>
       <c r="P50" s="89"/>
     </row>
-    <row r="51" spans="2:16" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:16" ht="60" x14ac:dyDescent="0.25">
       <c r="B51" s="79" t="s">
         <v>287</v>
       </c>
@@ -6841,7 +6856,7 @@
       <c r="I51" s="89"/>
       <c r="J51" s="24"/>
       <c r="L51" s="91"/>
-      <c r="M51" s="105"/>
+      <c r="M51" s="96"/>
       <c r="N51">
         <v>0.5</v>
       </c>
@@ -6852,7 +6867,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B52" s="79" t="s">
         <v>284</v>
       </c>
@@ -6865,7 +6880,7 @@
       <c r="I52" s="89"/>
       <c r="J52" s="24"/>
       <c r="L52" s="91"/>
-      <c r="M52" s="105"/>
+      <c r="M52" s="96"/>
       <c r="N52">
         <v>1</v>
       </c>
@@ -6874,64 +6889,90 @@
       </c>
       <c r="P52" s="89"/>
     </row>
-    <row r="53" spans="2:16" ht="72" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:16" ht="90" x14ac:dyDescent="0.25">
       <c r="B53" s="29" t="s">
         <v>288</v>
       </c>
-      <c r="C53" s="31" t="s">
+      <c r="C53" s="92" t="s">
         <v>103</v>
       </c>
       <c r="F53" s="89"/>
       <c r="I53" s="89"/>
       <c r="L53" s="91"/>
-      <c r="M53" s="105"/>
+      <c r="M53" s="96"/>
       <c r="N53"/>
       <c r="P53" s="91" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:16" ht="45" x14ac:dyDescent="0.25">
       <c r="B54" s="29" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B55" s="29"/>
-    </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="C54" s="92" t="s">
+        <v>103</v>
+      </c>
+      <c r="N54" s="31">
+        <v>5</v>
+      </c>
+      <c r="O54" s="31">
+        <v>80</v>
+      </c>
+      <c r="P54" s="90" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="55" spans="2:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="B55" s="79" t="s">
+        <v>296</v>
+      </c>
+      <c r="C55" s="92" t="s">
+        <v>103</v>
+      </c>
+      <c r="N55" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="O55" s="31">
+        <v>100</v>
+      </c>
+      <c r="P55" s="90" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="56" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B56" s="29"/>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B57" s="29"/>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B58" s="29"/>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B59" s="29"/>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B60" s="29"/>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B61" s="29"/>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B62" s="29"/>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B63" s="29"/>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B64" s="29"/>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="29"/>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="29"/>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="29"/>
     </row>
   </sheetData>
@@ -7103,23 +7144,23 @@
       <formula>MAX($E48,$H48,$K48)=100</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C52">
-    <cfRule type="expression" dxfId="4" priority="2">
+  <conditionalFormatting sqref="B32:B38">
+    <cfRule type="expression" dxfId="4" priority="766">
+      <formula>MAX($E15,$H15,$K15)=100</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="767">
+      <formula>MAX($E48,$H48,$K48)=100</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:C55">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>$C6="Charlotte/Eddy"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$C6="Charlotte"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="1" priority="4">
       <formula>$C6="Eddy"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B32:B38">
-    <cfRule type="expression" dxfId="1" priority="766">
-      <formula>MAX($E15,$H15,$K15)=100</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="767">
-      <formula>MAX($E48,$H48,$K48)=100</formula>
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>$C6="Charlotte"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7133,28 +7174,28 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:F101"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
-    <col min="2" max="2" width="93.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" customWidth="1"/>
+    <col min="2" max="2" width="93.28515625" customWidth="1"/>
     <col min="3" max="3" width="33" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="42.6640625" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
+    <row r="1" spans="2:6" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:6" ht="46.95" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="5" spans="2:6" ht="46.9" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B5" s="2" t="s">
         <v>62</v>
       </c>
@@ -7171,7 +7212,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
@@ -7184,7 +7225,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>21</v>
       </c>
@@ -7197,7 +7238,7 @@
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -7210,7 +7251,7 @@
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>24</v>
       </c>
@@ -7223,7 +7264,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>25</v>
       </c>
@@ -7236,7 +7277,7 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -7249,7 +7290,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
@@ -7262,7 +7303,7 @@
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
@@ -7275,7 +7316,7 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
@@ -7288,7 +7329,7 @@
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>34</v>
       </c>
@@ -7301,7 +7342,7 @@
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
@@ -7314,7 +7355,7 @@
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>71</v>
       </c>
@@ -7327,7 +7368,7 @@
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>36</v>
       </c>
@@ -7340,7 +7381,7 @@
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
@@ -7353,7 +7394,7 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
@@ -7366,7 +7407,7 @@
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>41</v>
       </c>
@@ -7379,7 +7420,7 @@
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>42</v>
       </c>
@@ -7392,7 +7433,7 @@
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
@@ -7405,7 +7446,7 @@
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="3" t="s">
         <v>39</v>
       </c>
@@ -7418,7 +7459,7 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -7431,7 +7472,7 @@
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
         <v>43</v>
       </c>
@@ -7444,7 +7485,7 @@
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
         <v>45</v>
       </c>
@@ -7457,7 +7498,7 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
         <v>80</v>
       </c>
@@ -7470,7 +7511,7 @@
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="3" t="s">
         <v>46</v>
       </c>
@@ -7483,7 +7524,7 @@
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="3" t="s">
         <v>47</v>
       </c>
@@ -7496,7 +7537,7 @@
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="3" t="s">
         <v>70</v>
       </c>
@@ -7509,7 +7550,7 @@
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="s">
         <v>48</v>
       </c>
@@ -7522,7 +7563,7 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
@@ -7535,7 +7576,7 @@
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="3" t="s">
         <v>60</v>
       </c>
@@ -7548,7 +7589,7 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="3" t="s">
         <v>51</v>
       </c>
@@ -7561,7 +7602,7 @@
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
         <v>53</v>
       </c>
@@ -7574,7 +7615,7 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="3" t="s">
         <v>52</v>
       </c>
@@ -7587,7 +7628,7 @@
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -7600,7 +7641,7 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
         <v>55</v>
       </c>
@@ -7613,7 +7654,7 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
         <v>56</v>
       </c>
@@ -7626,7 +7667,7 @@
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="3" t="s">
         <v>57</v>
       </c>
@@ -7639,7 +7680,7 @@
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="3" t="s">
         <v>58</v>
       </c>
@@ -7652,7 +7693,7 @@
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="3" t="s">
         <v>59</v>
       </c>
@@ -7665,7 +7706,7 @@
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" s="3" t="s">
         <v>61</v>
       </c>
@@ -7678,7 +7719,7 @@
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="3" t="s">
         <v>63</v>
       </c>
@@ -7691,7 +7732,7 @@
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
         <v>64</v>
       </c>
@@ -7704,7 +7745,7 @@
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" s="3" t="s">
         <v>65</v>
       </c>
@@ -7717,7 +7758,7 @@
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
         <v>86</v>
       </c>
@@ -7730,7 +7771,7 @@
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="3" t="s">
         <v>67</v>
       </c>
@@ -7743,7 +7784,7 @@
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
         <v>68</v>
       </c>
@@ -7756,7 +7797,7 @@
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="3" t="s">
         <v>69</v>
       </c>
@@ -7769,7 +7810,7 @@
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
         <v>72</v>
       </c>
@@ -7782,7 +7823,7 @@
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53" s="3" t="s">
         <v>73</v>
       </c>
@@ -7795,7 +7836,7 @@
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
         <v>74</v>
       </c>
@@ -7808,7 +7849,7 @@
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="3" t="s">
         <v>85</v>
       </c>
@@ -7821,7 +7862,7 @@
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="3" t="s">
         <v>76</v>
       </c>
@@ -7834,7 +7875,7 @@
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57" s="3" t="s">
         <v>77</v>
       </c>
@@ -7847,7 +7888,7 @@
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
         <v>78</v>
       </c>
@@ -7860,7 +7901,7 @@
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59" s="3" t="s">
         <v>79</v>
       </c>
@@ -7873,7 +7914,7 @@
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
         <v>81</v>
       </c>
@@ -7886,7 +7927,7 @@
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
         <v>82</v>
       </c>
@@ -7899,7 +7940,7 @@
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="3" t="s">
         <v>83</v>
       </c>
@@ -7912,7 +7953,7 @@
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B63" s="3" t="s">
         <v>84</v>
       </c>
@@ -7925,7 +7966,7 @@
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B64" s="3" t="s">
         <v>75</v>
       </c>
@@ -7938,7 +7979,7 @@
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
         <v>92</v>
       </c>
@@ -7949,7 +7990,7 @@
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
@@ -7960,7 +8001,7 @@
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" s="3" t="s">
         <v>94</v>
       </c>
@@ -7971,7 +8012,7 @@
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
         <v>95</v>
       </c>
@@ -7982,7 +8023,7 @@
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" s="3" t="s">
         <v>96</v>
       </c>
@@ -7993,7 +8034,7 @@
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" s="3" t="s">
         <v>97</v>
       </c>
@@ -8004,7 +8045,7 @@
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" s="3" t="s">
         <v>98</v>
       </c>
@@ -8015,7 +8056,7 @@
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" s="3" t="s">
         <v>99</v>
       </c>
@@ -8026,7 +8067,7 @@
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" s="3" t="s">
         <v>100</v>
       </c>
@@ -8037,7 +8078,7 @@
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" s="3" t="s">
         <v>106</v>
       </c>
@@ -8048,7 +8089,7 @@
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="3" t="s">
         <v>107</v>
       </c>
@@ -8059,182 +8100,182 @@
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="3"/>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="3"/>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
       <c r="D81" s="3"/>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
       <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
       <c r="D83" s="3"/>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
       <c r="D84" s="3"/>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3"/>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3"/>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3"/>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>

</xml_diff>

<commit_message>
Ajout client responsive sur hd et fhd
</commit_message>
<xml_diff>
--- a/doc/C61_-_Document_de_planification_L_Attaque.xlsx
+++ b/doc/C61_-_Document_de_planification_L_Attaque.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\L-Attaque\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_projet\L-Attaque\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9856A3B3-31D9-42BD-9E66-8CC20E3A03F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D46FF9-1C1D-4B30-B7C9-49FCD4C2D5CB}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="5" xr2:uid="{0139C51A-36D8-4FB0-B647-CB90E1DC24D3}"/>
   </bookViews>
   <sheets>
     <sheet name="Planification" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Planification trop détaillée'!$B$5:$F$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 3'!$B$4:$L$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,12 +35,6 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -48,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="301">
   <si>
     <t>Planification globale</t>
   </si>
@@ -950,6 +944,9 @@
   </si>
   <si>
     <t>Tweaker les valeurs de l'algorithme pour qu'il fonctionne mieux</t>
+  </si>
+  <si>
+    <t>Ajouter responsive sur hd et fhd</t>
   </si>
 </sst>
 </file>
@@ -1713,23 +1710,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1744,19 +1732,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1766,7 +1763,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFCCFFFF"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1774,6 +1778,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFCFDCF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1787,20 +1798,6 @@
             <color rgb="FFCCFFFF"/>
           </stop>
         </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -2511,26 +2508,26 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.28515625" customWidth="1"/>
+    <col min="1" max="1" width="3.33203125" customWidth="1"/>
     <col min="2" max="2" width="116" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" customWidth="1"/>
-    <col min="5" max="5" width="42.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="42.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="44.85" customHeight="1" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="46.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:5" ht="46.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
@@ -2544,7 +2541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="48" t="s">
         <v>138</v>
       </c>
@@ -2558,7 +2555,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="52" t="s">
         <v>108</v>
       </c>
@@ -2572,7 +2569,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B8" s="53" t="s">
         <v>109</v>
       </c>
@@ -2586,7 +2583,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" s="53" t="s">
         <v>110</v>
       </c>
@@ -2600,7 +2597,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" s="53" t="s">
         <v>111</v>
       </c>
@@ -2614,7 +2611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B11" s="53" t="s">
         <v>113</v>
       </c>
@@ -2628,7 +2625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="53" t="s">
         <v>114</v>
       </c>
@@ -2642,7 +2639,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B13" s="53" t="s">
         <v>115</v>
       </c>
@@ -2656,7 +2653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="53" t="s">
         <v>142</v>
       </c>
@@ -2670,7 +2667,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B15" s="53" t="s">
         <v>118</v>
       </c>
@@ -2684,7 +2681,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B16" s="53" t="s">
         <v>119</v>
       </c>
@@ -2698,7 +2695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" s="53" t="s">
         <v>121</v>
       </c>
@@ -2712,7 +2709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" s="53" t="s">
         <v>127</v>
       </c>
@@ -2726,7 +2723,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" s="49" t="s">
         <v>116</v>
       </c>
@@ -2740,7 +2737,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" s="49" t="s">
         <v>117</v>
       </c>
@@ -2754,7 +2751,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" s="49" t="s">
         <v>122</v>
       </c>
@@ -2768,7 +2765,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" s="49" t="s">
         <v>123</v>
       </c>
@@ -2782,7 +2779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" s="49" t="s">
         <v>124</v>
       </c>
@@ -2796,7 +2793,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" s="49" t="s">
         <v>126</v>
       </c>
@@ -2810,7 +2807,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B25" s="49" t="s">
         <v>130</v>
       </c>
@@ -2824,7 +2821,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B26" s="49" t="s">
         <v>131</v>
       </c>
@@ -2838,7 +2835,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B27" s="49" t="s">
         <v>132</v>
       </c>
@@ -2852,7 +2849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B28" s="54" t="s">
         <v>125</v>
       </c>
@@ -2866,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B29" s="54" t="s">
         <v>128</v>
       </c>
@@ -2880,7 +2877,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B30" s="54" t="s">
         <v>120</v>
       </c>
@@ -2894,7 +2891,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="54" t="s">
         <v>129</v>
       </c>
@@ -2908,7 +2905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="54" t="s">
         <v>133</v>
       </c>
@@ -2922,7 +2919,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="54" t="s">
         <v>134</v>
       </c>
@@ -2936,7 +2933,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="54" t="s">
         <v>135</v>
       </c>
@@ -2950,7 +2947,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="54" t="s">
         <v>136</v>
       </c>
@@ -2964,7 +2961,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="54" t="s">
         <v>137</v>
       </c>
@@ -2978,7 +2975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="56" t="s">
         <v>112</v>
       </c>
@@ -2992,8 +2989,8 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="D39" s="32" t="s">
         <v>143</v>
       </c>
@@ -3028,32 +3025,32 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:S26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" customWidth="1"/>
-    <col min="9" max="9" width="18.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
-    <col min="15" max="15" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="15" max="15" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:18" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="5"/>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -3083,7 +3080,7 @@
       <c r="Q3" s="4"/>
       <c r="R3" s="6"/>
     </row>
-    <row r="4" spans="1:18" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5"/>
       <c r="B4" s="4" t="s">
         <v>1</v>
@@ -3137,7 +3134,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
         <v>93</v>
       </c>
@@ -3164,7 +3161,7 @@
       <c r="Q5" s="9"/>
       <c r="R5" s="10"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
         <v>92</v>
       </c>
@@ -3186,7 +3183,7 @@
       <c r="P6" s="24"/>
       <c r="R6" s="11"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
         <v>94</v>
       </c>
@@ -3213,7 +3210,7 @@
       <c r="P7" s="24"/>
       <c r="R7" s="11"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B8" s="19" t="s">
         <v>100</v>
       </c>
@@ -3246,7 +3243,7 @@
       <c r="P8" s="24"/>
       <c r="R8" s="11"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
         <v>95</v>
       </c>
@@ -3283,7 +3280,7 @@
       </c>
       <c r="R9" s="21"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
@@ -3320,7 +3317,7 @@
       </c>
       <c r="R10" s="21"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B11" s="19" t="s">
         <v>97</v>
       </c>
@@ -3352,7 +3349,7 @@
       </c>
       <c r="R11" s="21"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B12" s="19" t="s">
         <v>98</v>
       </c>
@@ -3380,7 +3377,7 @@
       <c r="P12" s="24"/>
       <c r="R12" s="11"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="38" t="s">
         <v>96</v>
       </c>
@@ -3407,15 +3404,15 @@
       <c r="Q13" s="37"/>
       <c r="R13" s="13"/>
     </row>
-    <row r="21" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:19" x14ac:dyDescent="0.3">
       <c r="J21" s="15"/>
     </row>
-    <row r="25" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M25" s="15"/>
       <c r="P25" s="15"/>
       <c r="S25" s="15"/>
     </row>
-    <row r="26" spans="10:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:19" x14ac:dyDescent="0.3">
       <c r="M26" s="15"/>
       <c r="P26" s="15"/>
       <c r="S26" s="15"/>
@@ -3431,44 +3428,44 @@
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="B2:L48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="2" width="77.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="77.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="74" customWidth="1"/>
-    <col min="10" max="10" width="16.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B3" s="107" t="s">
+    <row r="2" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B3" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="108"/>
-      <c r="I3" s="108"/>
-      <c r="J3" s="108"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="109"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B5" s="101" t="s">
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
+      <c r="J3" s="96"/>
+      <c r="K3" s="96"/>
+      <c r="L3" s="97"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B5" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="103" t="s">
+      <c r="C5" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="42" t="s">
@@ -3477,7 +3474,7 @@
       <c r="E5" s="43">
         <v>46083</v>
       </c>
-      <c r="F5" s="99" t="s">
+      <c r="F5" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="45" t="s">
@@ -3486,7 +3483,7 @@
       <c r="H5" s="43">
         <v>46090</v>
       </c>
-      <c r="I5" s="99" t="s">
+      <c r="I5" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J5" s="45" t="s">
@@ -3495,36 +3492,36 @@
       <c r="K5" s="43">
         <v>46104</v>
       </c>
-      <c r="L5" s="99" t="s">
+      <c r="L5" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="102"/>
-      <c r="C6" s="104"/>
+    <row r="6" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="99"/>
+      <c r="C6" s="101"/>
       <c r="D6" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="100"/>
+      <c r="F6" s="103"/>
       <c r="G6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="H6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="100"/>
+      <c r="I6" s="103"/>
       <c r="J6" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K6" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="100"/>
-    </row>
-    <row r="7" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="L6" s="103"/>
+    </row>
+    <row r="7" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="28" t="s">
         <v>22</v>
       </c>
@@ -3547,7 +3544,7 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>33</v>
       </c>
@@ -3566,7 +3563,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>34</v>
       </c>
@@ -3585,7 +3582,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>73</v>
       </c>
@@ -3604,7 +3601,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>151</v>
       </c>
@@ -3623,7 +3620,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>23</v>
       </c>
@@ -3642,7 +3639,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>24</v>
       </c>
@@ -3661,7 +3658,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>25</v>
       </c>
@@ -3680,7 +3677,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>149</v>
       </c>
@@ -3699,7 +3696,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>27</v>
       </c>
@@ -3718,7 +3715,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>28</v>
       </c>
@@ -3737,7 +3734,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>147</v>
       </c>
@@ -3756,7 +3753,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>148</v>
       </c>
@@ -3775,7 +3772,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="46" t="s">
         <v>156</v>
       </c>
@@ -3794,7 +3791,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>89</v>
       </c>
@@ -3815,7 +3812,7 @@
       </c>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>49</v>
       </c>
@@ -3834,7 +3831,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>88</v>
       </c>
@@ -3855,7 +3852,7 @@
       </c>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>72</v>
       </c>
@@ -3874,7 +3871,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>78</v>
       </c>
@@ -3893,7 +3890,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>90</v>
       </c>
@@ -3914,7 +3911,7 @@
       </c>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>91</v>
       </c>
@@ -3935,7 +3932,7 @@
       </c>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>77</v>
       </c>
@@ -3956,7 +3953,7 @@
       </c>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>74</v>
       </c>
@@ -3975,7 +3972,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>171</v>
       </c>
@@ -3994,7 +3991,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>40</v>
       </c>
@@ -4013,7 +4010,7 @@
       </c>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>41</v>
       </c>
@@ -4032,7 +4029,7 @@
       </c>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>150</v>
       </c>
@@ -4051,7 +4048,7 @@
       </c>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>153</v>
       </c>
@@ -4070,7 +4067,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>71</v>
       </c>
@@ -4089,7 +4086,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>36</v>
       </c>
@@ -4108,7 +4105,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>37</v>
       </c>
@@ -4127,7 +4124,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>167</v>
       </c>
@@ -4146,7 +4143,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>168</v>
       </c>
@@ -4165,7 +4162,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>165</v>
       </c>
@@ -4184,7 +4181,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>166</v>
       </c>
@@ -4203,7 +4200,7 @@
       </c>
       <c r="L41" s="11"/>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>163</v>
       </c>
@@ -4222,7 +4219,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>162</v>
       </c>
@@ -4241,7 +4238,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>158</v>
       </c>
@@ -4260,7 +4257,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="29" t="s">
         <v>157</v>
       </c>
@@ -4279,7 +4276,7 @@
       </c>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="29" t="s">
         <v>161</v>
       </c>
@@ -4298,7 +4295,7 @@
       </c>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B47" s="29" t="s">
         <v>169</v>
       </c>
@@ -4317,7 +4314,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>160</v>
       </c>
@@ -4422,43 +4419,43 @@
     <tabColor theme="8"/>
   </sheetPr>
   <dimension ref="B1:L60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
     <col min="2" max="2" width="89" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="16" style="31" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="52.7109375" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.6640625" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="69.42578125" customWidth="1"/>
+    <col min="11" max="11" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="69.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="B1" s="107" t="s">
+    <row r="1" spans="2:12" ht="46.8" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B1" s="95" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="109"/>
-    </row>
-    <row r="3" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="B4" s="101" t="s">
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="97"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:12" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="103" t="s">
+      <c r="C4" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="42" t="s">
@@ -4467,7 +4464,7 @@
       <c r="E4" s="43">
         <v>46111</v>
       </c>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="60" t="s">
@@ -4476,7 +4473,7 @@
       <c r="H4" s="43">
         <v>46125</v>
       </c>
-      <c r="I4" s="99" t="s">
+      <c r="I4" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J4" s="45" t="s">
@@ -4485,36 +4482,36 @@
       <c r="K4" s="43">
         <v>46132</v>
       </c>
-      <c r="L4" s="99" t="s">
+      <c r="L4" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="102"/>
-      <c r="C5" s="104"/>
+    <row r="5" spans="2:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="99"/>
+      <c r="C5" s="101"/>
       <c r="D5" s="42" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="100"/>
+      <c r="F5" s="103"/>
       <c r="G5" s="59" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="100"/>
+      <c r="I5" s="103"/>
       <c r="J5" s="44" t="s">
         <v>10</v>
       </c>
       <c r="K5" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="L5" s="100"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="103"/>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="29" t="s">
         <v>174</v>
       </c>
@@ -4532,7 +4529,7 @@
       <c r="I6" s="11"/>
       <c r="L6" s="11"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="29" t="s">
         <v>175</v>
       </c>
@@ -4550,7 +4547,7 @@
       <c r="I7" s="11"/>
       <c r="L7" s="11"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="29" t="s">
         <v>176</v>
       </c>
@@ -4568,7 +4565,7 @@
       <c r="I8" s="11"/>
       <c r="L8" s="11"/>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="29" t="s">
         <v>159</v>
       </c>
@@ -4586,7 +4583,7 @@
       <c r="I9" s="11"/>
       <c r="L9" s="11"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="29" t="s">
         <v>173</v>
       </c>
@@ -4604,7 +4601,7 @@
       <c r="I10" s="11"/>
       <c r="L10" s="11"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="29" t="s">
         <v>172</v>
       </c>
@@ -4622,7 +4619,7 @@
       <c r="I11" s="11"/>
       <c r="L11" s="11"/>
     </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="29" t="s">
         <v>164</v>
       </c>
@@ -4640,7 +4637,7 @@
       <c r="I12" s="11"/>
       <c r="L12" s="11"/>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>170</v>
       </c>
@@ -4658,7 +4655,7 @@
       <c r="I13" s="11"/>
       <c r="L13" s="11"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>177</v>
       </c>
@@ -4676,7 +4673,7 @@
       <c r="I14" s="11"/>
       <c r="L14" s="11"/>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>178</v>
       </c>
@@ -4694,7 +4691,7 @@
       <c r="I15" s="11"/>
       <c r="L15" s="11"/>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>180</v>
       </c>
@@ -4712,7 +4709,7 @@
       <c r="I16" s="11"/>
       <c r="L16" s="11"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>182</v>
       </c>
@@ -4730,7 +4727,7 @@
       <c r="I17" s="11"/>
       <c r="L17" s="11"/>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>183</v>
       </c>
@@ -4748,7 +4745,7 @@
       <c r="I18" s="11"/>
       <c r="L18" s="11"/>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>184</v>
       </c>
@@ -4766,7 +4763,7 @@
       <c r="I19" s="11"/>
       <c r="L19" s="11"/>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>195</v>
       </c>
@@ -4785,7 +4782,7 @@
       <c r="I20" s="11"/>
       <c r="L20" s="11"/>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>185</v>
       </c>
@@ -4804,7 +4801,7 @@
       <c r="I21" s="11"/>
       <c r="L21" s="11"/>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B22" s="29" t="s">
         <v>196</v>
       </c>
@@ -4823,7 +4820,7 @@
       <c r="I22" s="11"/>
       <c r="L22" s="11"/>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B23" s="29" t="s">
         <v>192</v>
       </c>
@@ -4842,7 +4839,7 @@
       <c r="I23" s="11"/>
       <c r="L23" s="11"/>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B24" s="29" t="s">
         <v>186</v>
       </c>
@@ -4861,7 +4858,7 @@
       <c r="I24" s="11"/>
       <c r="L24" s="11"/>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B25" s="29" t="s">
         <v>198</v>
       </c>
@@ -4880,7 +4877,7 @@
       <c r="I25" s="11"/>
       <c r="L25" s="11"/>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B26" s="29" t="s">
         <v>187</v>
       </c>
@@ -4899,7 +4896,7 @@
       <c r="I26" s="11"/>
       <c r="L26" s="11"/>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>188</v>
       </c>
@@ -4918,7 +4915,7 @@
       <c r="I27" s="11"/>
       <c r="L27" s="11"/>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B28" s="29" t="s">
         <v>189</v>
       </c>
@@ -4937,7 +4934,7 @@
       <c r="I28" s="11"/>
       <c r="L28" s="11"/>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B29" s="29" t="s">
         <v>190</v>
       </c>
@@ -4956,7 +4953,7 @@
       <c r="I29" s="11"/>
       <c r="L29" s="11"/>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B30" s="29" t="s">
         <v>194</v>
       </c>
@@ -4975,7 +4972,7 @@
       <c r="I30" s="11"/>
       <c r="L30" s="11"/>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B31" s="29" t="s">
         <v>191</v>
       </c>
@@ -4994,7 +4991,7 @@
       <c r="I31" s="11"/>
       <c r="L31" s="11"/>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="29" t="s">
         <v>193</v>
       </c>
@@ -5013,7 +5010,7 @@
       <c r="I32" s="11"/>
       <c r="L32" s="11"/>
     </row>
-    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B33" s="29" t="s">
         <v>197</v>
       </c>
@@ -5032,7 +5029,7 @@
       <c r="I33" s="11"/>
       <c r="L33" s="11"/>
     </row>
-    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B34" s="29" t="s">
         <v>199</v>
       </c>
@@ -5053,7 +5050,7 @@
       </c>
       <c r="L34" s="11"/>
     </row>
-    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B35" s="29" t="s">
         <v>203</v>
       </c>
@@ -5073,7 +5070,7 @@
       </c>
       <c r="L35" s="11"/>
     </row>
-    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B36" s="29" t="s">
         <v>202</v>
       </c>
@@ -5093,7 +5090,7 @@
       </c>
       <c r="L36" s="11"/>
     </row>
-    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B37" s="29" t="s">
         <v>204</v>
       </c>
@@ -5113,7 +5110,7 @@
       </c>
       <c r="L37" s="11"/>
     </row>
-    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B38" s="29" t="s">
         <v>205</v>
       </c>
@@ -5133,7 +5130,7 @@
       </c>
       <c r="L38" s="11"/>
     </row>
-    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B39" s="29" t="s">
         <v>206</v>
       </c>
@@ -5153,7 +5150,7 @@
       </c>
       <c r="L39" s="11"/>
     </row>
-    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B40" s="29" t="s">
         <v>207</v>
       </c>
@@ -5173,7 +5170,7 @@
       </c>
       <c r="L40" s="11"/>
     </row>
-    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B41" s="29" t="s">
         <v>208</v>
       </c>
@@ -5195,7 +5192,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B42" s="29" t="s">
         <v>54</v>
       </c>
@@ -5215,7 +5212,7 @@
       </c>
       <c r="L42" s="11"/>
     </row>
-    <row r="43" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B43" s="29" t="s">
         <v>210</v>
       </c>
@@ -5235,7 +5232,7 @@
       </c>
       <c r="L43" s="11"/>
     </row>
-    <row r="44" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B44" s="29" t="s">
         <v>209</v>
       </c>
@@ -5255,7 +5252,7 @@
       </c>
       <c r="L44" s="11"/>
     </row>
-    <row r="45" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B45" s="58" t="s">
         <v>181</v>
       </c>
@@ -5273,7 +5270,7 @@
       <c r="I45" s="11"/>
       <c r="L45" s="11"/>
     </row>
-    <row r="46" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B46" s="58" t="s">
         <v>84</v>
       </c>
@@ -5291,7 +5288,7 @@
       <c r="I46" s="11"/>
       <c r="L46" s="11"/>
     </row>
-    <row r="47" spans="2:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B47" s="58" t="s">
         <v>83</v>
       </c>
@@ -5316,7 +5313,7 @@
       </c>
       <c r="L47" s="11"/>
     </row>
-    <row r="48" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B48" s="58" t="s">
         <v>81</v>
       </c>
@@ -5334,7 +5331,7 @@
       <c r="I48" s="11"/>
       <c r="L48" s="11"/>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B49" s="58" t="s">
         <v>60</v>
       </c>
@@ -5352,7 +5349,7 @@
       <c r="I49" s="11"/>
       <c r="L49" s="11"/>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B50" s="58" t="s">
         <v>223</v>
       </c>
@@ -5375,7 +5372,7 @@
       <c r="I50" s="11"/>
       <c r="L50" s="11"/>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B51" s="58" t="s">
         <v>219</v>
       </c>
@@ -5398,7 +5395,7 @@
       </c>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B52" s="58" t="s">
         <v>56</v>
       </c>
@@ -5416,7 +5413,7 @@
       <c r="I52" s="11"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B53" s="58" t="s">
         <v>57</v>
       </c>
@@ -5434,7 +5431,7 @@
       <c r="I53" s="11"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B54" s="58" t="s">
         <v>55</v>
       </c>
@@ -5451,7 +5448,7 @@
       <c r="I54" s="11"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B55" s="58" t="s">
         <v>58</v>
       </c>
@@ -5469,7 +5466,7 @@
       <c r="I55" s="11"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B56" s="58" t="s">
         <v>243</v>
       </c>
@@ -5486,7 +5483,7 @@
       <c r="I56" s="11"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B57" s="58" t="s">
         <v>220</v>
       </c>
@@ -5509,7 +5506,7 @@
       </c>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="2:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B58" s="58" t="s">
         <v>200</v>
       </c>
@@ -5536,7 +5533,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B59" s="58" t="s">
         <v>211</v>
       </c>
@@ -5554,7 +5551,7 @@
       </c>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B60" s="64" t="s">
         <v>212</v>
       </c>
@@ -5618,21 +5615,21 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="B1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="81.5703125" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="81.5546875" customWidth="1"/>
     <col min="3" max="3" width="81" style="61" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" customWidth="1"/>
-    <col min="5" max="5" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.6640625" customWidth="1"/>
+    <col min="5" max="5" width="28.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="46.5" x14ac:dyDescent="0.7">
+    <row r="1" spans="2:5" ht="46.2" x14ac:dyDescent="0.85">
       <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:5" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:5" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B3" s="8" t="s">
         <v>224</v>
       </c>
@@ -5646,7 +5643,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="85" t="s">
         <v>226</v>
       </c>
@@ -5660,7 +5657,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="73" t="s">
         <v>240</v>
       </c>
@@ -5674,7 +5671,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="86" t="s">
         <v>241</v>
       </c>
@@ -5688,7 +5685,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="86" t="s">
         <v>230</v>
       </c>
@@ -5702,7 +5699,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="73" t="s">
         <v>233</v>
       </c>
@@ -5716,7 +5713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B9" s="86" t="s">
         <v>179</v>
       </c>
@@ -5730,7 +5727,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="82" t="s">
         <v>68</v>
       </c>
@@ -5756,50 +5753,50 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B2:P67"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:P68"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.7109375" customWidth="1"/>
-    <col min="2" max="2" width="67.7109375" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="31" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" style="31" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="35.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="15.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.5703125" style="90" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" style="31" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.6640625" customWidth="1"/>
+    <col min="2" max="2" width="67.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" style="31" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="31" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.6640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="15.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.5546875" style="90" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.109375" style="31" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22" style="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="B2" s="97" t="s">
+    <row r="2" spans="2:16" ht="46.2" x14ac:dyDescent="0.85">
+      <c r="B2" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="98"/>
-    </row>
-    <row r="5" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.35">
-      <c r="B6" s="101" t="s">
+      <c r="C2" s="107"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="107"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107"/>
+      <c r="O2" s="107"/>
+      <c r="P2" s="107"/>
+    </row>
+    <row r="5" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:16" ht="21" x14ac:dyDescent="0.4">
+      <c r="B6" s="98" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="103" t="s">
+      <c r="C6" s="100" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="88" t="s">
@@ -5808,7 +5805,7 @@
       <c r="E6" s="43">
         <v>46139</v>
       </c>
-      <c r="F6" s="99" t="s">
+      <c r="F6" s="102" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="60" t="s">
@@ -5817,7 +5814,7 @@
       <c r="H6" s="43">
         <v>46146</v>
       </c>
-      <c r="I6" s="99" t="s">
+      <c r="I6" s="102" t="s">
         <v>12</v>
       </c>
       <c r="J6" s="60" t="s">
@@ -5826,7 +5823,7 @@
       <c r="K6" s="43">
         <v>46153</v>
       </c>
-      <c r="L6" s="105" t="s">
+      <c r="L6" s="108" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="43">
@@ -5838,34 +5835,34 @@
       <c r="O6" s="43">
         <v>46167</v>
       </c>
-      <c r="P6" s="99" t="s">
+      <c r="P6" s="102" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:16" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="102"/>
-      <c r="C7" s="104"/>
+    <row r="7" spans="2:16" ht="21.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="99"/>
+      <c r="C7" s="101"/>
       <c r="D7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="100"/>
+      <c r="F7" s="103"/>
       <c r="G7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="H7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="100"/>
+      <c r="I7" s="103"/>
       <c r="J7" s="88" t="s">
         <v>10</v>
       </c>
       <c r="K7" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="106"/>
+      <c r="L7" s="109"/>
       <c r="M7" s="94" t="s">
         <v>201</v>
       </c>
@@ -5875,9 +5872,9 @@
       <c r="O7" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="P7" s="100"/>
-    </row>
-    <row r="8" spans="2:16" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P7" s="103"/>
+    </row>
+    <row r="8" spans="2:16" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="79" t="s">
         <v>68</v>
       </c>
@@ -5895,13 +5892,13 @@
       <c r="I8" s="89"/>
       <c r="J8" s="24"/>
       <c r="L8" s="91"/>
-      <c r="M8" s="95" t="s">
+      <c r="M8" s="104" t="s">
         <v>278</v>
       </c>
       <c r="N8"/>
       <c r="P8" s="89"/>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="79" t="s">
         <v>256</v>
       </c>
@@ -5919,11 +5916,11 @@
       <c r="I9" s="89"/>
       <c r="J9" s="24"/>
       <c r="L9" s="91"/>
-      <c r="M9" s="96"/>
+      <c r="M9" s="105"/>
       <c r="N9"/>
       <c r="P9" s="89"/>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
         <v>245</v>
       </c>
@@ -5941,11 +5938,11 @@
       <c r="I10" s="89"/>
       <c r="J10" s="24"/>
       <c r="L10" s="91"/>
-      <c r="M10" s="96"/>
+      <c r="M10" s="105"/>
       <c r="N10"/>
       <c r="P10" s="89"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
         <v>244</v>
       </c>
@@ -5963,11 +5960,11 @@
       <c r="I11" s="89"/>
       <c r="J11" s="24"/>
       <c r="L11" s="91"/>
-      <c r="M11" s="96"/>
+      <c r="M11" s="105"/>
       <c r="N11"/>
       <c r="P11" s="89"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
         <v>257</v>
       </c>
@@ -5984,11 +5981,11 @@
       <c r="I12" s="89"/>
       <c r="J12" s="24"/>
       <c r="L12" s="91"/>
-      <c r="M12" s="96"/>
+      <c r="M12" s="105"/>
       <c r="N12"/>
       <c r="P12" s="89"/>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B13" s="29" t="s">
         <v>246</v>
       </c>
@@ -6005,11 +6002,11 @@
       <c r="I13" s="89"/>
       <c r="J13" s="24"/>
       <c r="L13" s="91"/>
-      <c r="M13" s="96"/>
+      <c r="M13" s="105"/>
       <c r="N13"/>
       <c r="P13" s="89"/>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B14" s="29" t="s">
         <v>247</v>
       </c>
@@ -6026,11 +6023,11 @@
       <c r="I14" s="89"/>
       <c r="J14" s="24"/>
       <c r="L14" s="91"/>
-      <c r="M14" s="96"/>
+      <c r="M14" s="105"/>
       <c r="N14"/>
       <c r="P14" s="89"/>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B15" s="29" t="s">
         <v>254</v>
       </c>
@@ -6047,11 +6044,11 @@
       <c r="I15" s="89"/>
       <c r="J15" s="24"/>
       <c r="L15" s="91"/>
-      <c r="M15" s="96"/>
+      <c r="M15" s="105"/>
       <c r="N15"/>
       <c r="P15" s="89"/>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B16" s="29" t="s">
         <v>248</v>
       </c>
@@ -6068,11 +6065,11 @@
       <c r="I16" s="89"/>
       <c r="J16" s="24"/>
       <c r="L16" s="91"/>
-      <c r="M16" s="96"/>
+      <c r="M16" s="105"/>
       <c r="N16"/>
       <c r="P16" s="89"/>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B17" s="29" t="s">
         <v>249</v>
       </c>
@@ -6088,11 +6085,11 @@
       <c r="I17" s="89"/>
       <c r="J17" s="24"/>
       <c r="L17" s="91"/>
-      <c r="M17" s="96"/>
+      <c r="M17" s="105"/>
       <c r="N17"/>
       <c r="P17" s="89"/>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B18" s="29" t="s">
         <v>250</v>
       </c>
@@ -6108,11 +6105,11 @@
       <c r="I18" s="89"/>
       <c r="J18" s="24"/>
       <c r="L18" s="91"/>
-      <c r="M18" s="96"/>
+      <c r="M18" s="105"/>
       <c r="N18"/>
       <c r="P18" s="89"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B19" s="29" t="s">
         <v>251</v>
       </c>
@@ -6128,11 +6125,11 @@
       <c r="I19" s="89"/>
       <c r="J19" s="24"/>
       <c r="L19" s="91"/>
-      <c r="M19" s="96"/>
+      <c r="M19" s="105"/>
       <c r="N19"/>
       <c r="P19" s="89"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B20" s="29" t="s">
         <v>252</v>
       </c>
@@ -6148,11 +6145,11 @@
       <c r="I20" s="89"/>
       <c r="J20" s="24"/>
       <c r="L20" s="91"/>
-      <c r="M20" s="96"/>
+      <c r="M20" s="105"/>
       <c r="N20"/>
       <c r="P20" s="89"/>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B21" s="29" t="s">
         <v>253</v>
       </c>
@@ -6168,11 +6165,11 @@
       <c r="I21" s="89"/>
       <c r="J21" s="24"/>
       <c r="L21" s="91"/>
-      <c r="M21" s="96"/>
+      <c r="M21" s="105"/>
       <c r="N21"/>
       <c r="P21" s="89"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B22" s="79" t="s">
         <v>255</v>
       </c>
@@ -6188,11 +6185,11 @@
       <c r="I22" s="89"/>
       <c r="J22" s="24"/>
       <c r="L22" s="91"/>
-      <c r="M22" s="96"/>
+      <c r="M22" s="105"/>
       <c r="N22"/>
       <c r="P22" s="89"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B23" s="80" t="s">
         <v>258</v>
       </c>
@@ -6210,11 +6207,11 @@
       <c r="I23" s="89"/>
       <c r="J23" s="24"/>
       <c r="L23" s="91"/>
-      <c r="M23" s="96"/>
+      <c r="M23" s="105"/>
       <c r="N23"/>
       <c r="P23" s="89"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B24" s="80" t="s">
         <v>259</v>
       </c>
@@ -6227,11 +6224,11 @@
       <c r="I24" s="89"/>
       <c r="J24" s="24"/>
       <c r="L24" s="91"/>
-      <c r="M24" s="96"/>
+      <c r="M24" s="105"/>
       <c r="N24"/>
       <c r="P24" s="89"/>
     </row>
-    <row r="25" spans="2:16" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="81" t="s">
         <v>260</v>
       </c>
@@ -6249,11 +6246,11 @@
         <v>100</v>
       </c>
       <c r="L25" s="91"/>
-      <c r="M25" s="96"/>
+      <c r="M25" s="105"/>
       <c r="N25"/>
       <c r="P25" s="89"/>
     </row>
-    <row r="26" spans="2:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B26" s="81" t="s">
         <v>261</v>
       </c>
@@ -6271,11 +6268,11 @@
         <v>100</v>
       </c>
       <c r="L26" s="91"/>
-      <c r="M26" s="96"/>
+      <c r="M26" s="105"/>
       <c r="N26"/>
       <c r="P26" s="89"/>
     </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B27" s="81" t="s